<commit_message>
+ Add Attribute for Character. Edit animation system (using CrossFade instead of Trigger)
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,8 @@
     <sheet name="Armor" sheetId="4" r:id="rId4"/>
     <sheet name="Character" sheetId="5" r:id="rId5"/>
     <sheet name="CharacterStat" sheetId="6" r:id="rId6"/>
-    <sheet name="CharacterUpgrade" sheetId="7" r:id="rId7"/>
+    <sheet name="CharacterAttribute" sheetId="8" r:id="rId7"/>
+    <sheet name="CharacterUpgrade" sheetId="7" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$104</definedName>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="315">
   <si>
     <t>ID</t>
   </si>
@@ -958,6 +959,21 @@
   </si>
   <si>
     <t>crit_dmg_res</t>
+  </si>
+  <si>
+    <t>Enemy1</t>
+  </si>
+  <si>
+    <t>AttributeType</t>
+  </si>
+  <si>
+    <t>StatLink</t>
+  </si>
+  <si>
+    <t>StartPercent</t>
+  </si>
+  <si>
+    <t>1.0</t>
   </si>
 </sst>
 </file>
@@ -4152,7 +4168,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -4413,6 +4429,29 @@
         <v>287</v>
       </c>
     </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>310</v>
+      </c>
+      <c r="B12" t="s">
+        <v>202</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="D12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E12" t="s">
+        <v>287</v>
+      </c>
+      <c r="F12" t="s">
+        <v>287</v>
+      </c>
+      <c r="G12" t="s">
+        <v>287</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4420,9 +4459,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4841,6 +4881,44 @@
         <v>0</v>
       </c>
       <c r="L11" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>310</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="8">
+        <v>2500</v>
+      </c>
+      <c r="E12" s="8">
+        <v>1650</v>
+      </c>
+      <c r="F12" s="8">
+        <v>280</v>
+      </c>
+      <c r="G12" s="8">
+        <v>1</v>
+      </c>
+      <c r="H12" s="8">
+        <v>0</v>
+      </c>
+      <c r="I12" s="8">
+        <v>0</v>
+      </c>
+      <c r="J12" s="8">
+        <v>0</v>
+      </c>
+      <c r="K12" s="8">
+        <v>0</v>
+      </c>
+      <c r="L12" s="8">
         <v>0</v>
       </c>
     </row>
@@ -4851,7 +4929,263 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>311</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>288</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>292</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>294</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>295</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>296</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>297</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>298</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>299</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>300</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>310</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -5014,6 +5348,20 @@
         <v>33</v>
       </c>
     </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>310</v>
+      </c>
+      <c r="B12" s="8">
+        <v>175</v>
+      </c>
+      <c r="C12" s="8">
+        <v>115</v>
+      </c>
+      <c r="D12" s="8">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
+ Make Skill set for Natra and HongHaiNhi
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="6"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
     <sheet name="CharacterUpgrade" sheetId="7" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$105</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="319">
   <si>
     <t>ID</t>
   </si>
@@ -974,6 +974,18 @@
   </si>
   <si>
     <t>1.0</t>
+  </si>
+  <si>
+    <t>FireLance_Ring_Damasl</t>
+  </si>
+  <si>
+    <t>STR_FIRELANCE_RING_DAMASL_NAME</t>
+  </si>
+  <si>
+    <t>STR_FIRELANCE_RING_DAMASL_DES</t>
+  </si>
+  <si>
+    <t>STR_FIRELANCE_RING_DAMASL_SKILL</t>
   </si>
 </sst>
 </file>
@@ -1418,7 +1430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G114"/>
+  <dimension ref="A1:G115"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
@@ -1732,77 +1744,77 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
-        <v>79</v>
+      <c r="A16" s="12" t="s">
+        <v>315</v>
       </c>
       <c r="B16" t="s">
-        <v>86</v>
+        <v>316</v>
       </c>
       <c r="C16" t="s">
-        <v>93</v>
+        <v>317</v>
       </c>
       <c r="D16" t="s">
-        <v>100</v>
+        <v>318</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>66</v>
+        <v>62</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D17" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F17" s="6" t="s">
-        <v>67</v>
+      <c r="F17" s="5" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D18" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F18" s="4" t="s">
-        <v>65</v>
+      <c r="F18" s="6" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C19" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D19" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>106</v>
@@ -1813,79 +1825,79 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D20" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F20" s="2" t="s">
-        <v>63</v>
+      <c r="F20" s="4" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B21" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D21" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F21" s="3" t="s">
-        <v>64</v>
+      <c r="F21" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B22" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C22" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D22" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F22" s="2" t="s">
-        <v>63</v>
+      <c r="F22" s="3" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>107</v>
+      <c r="A23" s="11" t="s">
+        <v>85</v>
       </c>
       <c r="B23" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="C23" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="D23" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>63</v>
@@ -1893,16 +1905,16 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B24" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C24" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>123</v>
@@ -1913,16 +1925,16 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B25" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C25" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D25" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>123</v>
@@ -1933,16 +1945,16 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B26" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C26" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D26" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>123</v>
@@ -1952,20 +1964,20 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
-        <v>124</v>
+      <c r="A27" t="s">
+        <v>110</v>
       </c>
       <c r="B27" t="s">
-        <v>152</v>
+        <v>114</v>
       </c>
       <c r="C27" t="s">
-        <v>180</v>
+        <v>118</v>
       </c>
       <c r="D27" t="s">
-        <v>187</v>
+        <v>122</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>188</v>
+        <v>123</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>63</v>
@@ -1973,13 +1985,13 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B28" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C28" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D28" t="s">
         <v>187</v>
@@ -1993,13 +2005,13 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B29" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C29" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D29" t="s">
         <v>187</v>
@@ -2013,13 +2025,13 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B30" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C30" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D30" t="s">
         <v>187</v>
@@ -2033,13 +2045,13 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B31" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C31" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D31" t="s">
         <v>187</v>
@@ -2053,13 +2065,13 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B32" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C32" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D32" t="s">
         <v>187</v>
@@ -2073,13 +2085,13 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B33" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C33" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D33" t="s">
         <v>187</v>
@@ -2093,13 +2105,13 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B34" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C34" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="D34" t="s">
         <v>187</v>
@@ -2107,19 +2119,19 @@
       <c r="E34" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="F34" s="5" t="s">
-        <v>66</v>
+      <c r="F34" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B35" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C35" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D35" t="s">
         <v>187</v>
@@ -2133,13 +2145,13 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B36" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C36" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D36" t="s">
         <v>187</v>
@@ -2153,13 +2165,13 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B37" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D37" t="s">
         <v>187</v>
@@ -2173,13 +2185,13 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B38" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C38" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D38" t="s">
         <v>187</v>
@@ -2193,13 +2205,13 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B39" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C39" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D39" t="s">
         <v>187</v>
@@ -2213,13 +2225,13 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B40" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C40" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D40" t="s">
         <v>187</v>
@@ -2233,13 +2245,13 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B41" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C41" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="D41" t="s">
         <v>187</v>
@@ -2247,19 +2259,19 @@
       <c r="E41" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="F41" s="3" t="s">
-        <v>64</v>
+      <c r="F41" s="5" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B42" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C42" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D42" t="s">
         <v>187</v>
@@ -2273,13 +2285,13 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B43" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C43" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D43" t="s">
         <v>187</v>
@@ -2293,13 +2305,13 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="13" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B44" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C44" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D44" t="s">
         <v>187</v>
@@ -2313,13 +2325,13 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B45" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C45" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D45" t="s">
         <v>187</v>
@@ -2333,13 +2345,13 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B46" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C46" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D46" t="s">
         <v>187</v>
@@ -2353,13 +2365,13 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="13" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B47" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C47" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D47" t="s">
         <v>187</v>
@@ -2373,13 +2385,13 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B48" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C48" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="D48" t="s">
         <v>187</v>
@@ -2387,19 +2399,19 @@
       <c r="E48" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="F48" s="6" t="s">
-        <v>67</v>
+      <c r="F48" s="3" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B49" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C49" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D49" t="s">
         <v>187</v>
@@ -2413,13 +2425,13 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="13" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B50" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C50" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D50" t="s">
         <v>187</v>
@@ -2433,13 +2445,13 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B51" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C51" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D51" t="s">
         <v>187</v>
@@ -2453,13 +2465,13 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B52" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C52" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D52" t="s">
         <v>187</v>
@@ -2473,13 +2485,13 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="13" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B53" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C53" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D53" t="s">
         <v>187</v>
@@ -2493,13 +2505,13 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="13" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B54" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C54" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D54" t="s">
         <v>187</v>
@@ -2512,20 +2524,20 @@
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="15" t="s">
-        <v>189</v>
+      <c r="A55" s="13" t="s">
+        <v>151</v>
       </c>
       <c r="B55" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="C55" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="D55" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="F55" s="6" t="s">
         <v>67</v>
@@ -2533,10 +2545,10 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B56" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C56" t="s">
         <v>194</v>
@@ -2547,16 +2559,16 @@
       <c r="E56" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="F56" s="3" t="s">
-        <v>64</v>
+      <c r="F56" s="6" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B57" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C57" t="s">
         <v>194</v>
@@ -2567,16 +2579,16 @@
       <c r="E57" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="F57" s="5" t="s">
-        <v>66</v>
+      <c r="F57" s="3" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B58" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C58" t="s">
         <v>194</v>
@@ -2587,22 +2599,25 @@
       <c r="E58" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="F58" s="2" t="s">
-        <v>63</v>
+      <c r="F58" s="5" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="12" t="s">
-        <v>285</v>
+      <c r="A59" s="15" t="s">
+        <v>192</v>
       </c>
       <c r="B59" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C59" t="s">
-        <v>201</v>
+        <v>194</v>
+      </c>
+      <c r="D59" t="s">
+        <v>195</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="F59" s="2" t="s">
         <v>63</v>
@@ -2610,10 +2625,10 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="12" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="B60" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C60" t="s">
         <v>201</v>
@@ -2621,16 +2636,16 @@
       <c r="E60" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F60" s="11" t="s">
-        <v>67</v>
+      <c r="F60" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="12" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B61" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C61" t="s">
         <v>201</v>
@@ -2638,16 +2653,16 @@
       <c r="E61" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F61" s="16" t="s">
-        <v>66</v>
+      <c r="F61" s="11" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="12" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B62" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C62" t="s">
         <v>201</v>
@@ -2655,16 +2670,16 @@
       <c r="E62" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F62" s="3" t="s">
-        <v>64</v>
+      <c r="F62" s="16" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="12" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B63" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C63" t="s">
         <v>201</v>
@@ -2678,10 +2693,10 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="12" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B64" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C64" t="s">
         <v>201</v>
@@ -2689,16 +2704,16 @@
       <c r="E64" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F64" s="2" t="s">
-        <v>63</v>
+      <c r="F64" s="3" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="12" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B65" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C65" t="s">
         <v>201</v>
@@ -2706,16 +2721,16 @@
       <c r="E65" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F65" s="14" t="s">
-        <v>65</v>
+      <c r="F65" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="12" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B66" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C66" t="s">
         <v>201</v>
@@ -2723,16 +2738,16 @@
       <c r="E66" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F66" s="2" t="s">
-        <v>63</v>
+      <c r="F66" s="14" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="12" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B67" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C67" t="s">
         <v>201</v>
@@ -2746,10 +2761,10 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="12" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B68" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C68" t="s">
         <v>201</v>
@@ -2762,25 +2777,28 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="17" t="s">
-        <v>212</v>
+      <c r="A69" s="12" t="s">
+        <v>300</v>
       </c>
       <c r="B69" t="s">
-        <v>248</v>
+        <v>210</v>
+      </c>
+      <c r="C69" t="s">
+        <v>201</v>
       </c>
       <c r="E69" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="F69" s="14" t="s">
-        <v>65</v>
+        <v>211</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="17" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B70" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E70" s="7" t="s">
         <v>254</v>
@@ -2791,10 +2809,10 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="17" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B71" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E71" s="7" t="s">
         <v>254</v>
@@ -2805,10 +2823,10 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="17" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B72" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E72" s="7" t="s">
         <v>254</v>
@@ -2819,10 +2837,10 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="17" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B73" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E73" s="7" t="s">
         <v>254</v>
@@ -2833,10 +2851,10 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="17" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B74" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E74" s="7" t="s">
         <v>254</v>
@@ -2847,10 +2865,10 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B75" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="E75" s="7" t="s">
         <v>254</v>
@@ -2861,10 +2879,10 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="17" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B76" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E76" s="7" t="s">
         <v>254</v>
@@ -2875,10 +2893,10 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="17" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B77" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E77" s="7" t="s">
         <v>254</v>
@@ -2889,10 +2907,10 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="17" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B78" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E78" s="7" t="s">
         <v>254</v>
@@ -2903,10 +2921,10 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="17" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B79" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E79" s="7" t="s">
         <v>254</v>
@@ -2917,10 +2935,10 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="17" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B80" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E80" s="7" t="s">
         <v>254</v>
@@ -2931,10 +2949,10 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="17" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B81" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="E81" s="7" t="s">
         <v>254</v>
@@ -2945,10 +2963,10 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="17" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B82" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E82" s="7" t="s">
         <v>254</v>
@@ -2959,10 +2977,10 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="17" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B83" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E83" s="7" t="s">
         <v>254</v>
@@ -2973,10 +2991,10 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="17" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B84" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E84" s="7" t="s">
         <v>254</v>
@@ -2987,10 +3005,10 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="17" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B85" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E85" s="7" t="s">
         <v>254</v>
@@ -3001,10 +3019,10 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="17" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B86" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E86" s="7" t="s">
         <v>254</v>
@@ -3015,10 +3033,10 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="17" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B87" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="E87" s="7" t="s">
         <v>254</v>
@@ -3029,10 +3047,10 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="17" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B88" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E88" s="7" t="s">
         <v>254</v>
@@ -3043,10 +3061,10 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="17" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B89" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E89" s="7" t="s">
         <v>254</v>
@@ -3057,10 +3075,10 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="17" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B90" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E90" s="7" t="s">
         <v>254</v>
@@ -3071,10 +3089,10 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="17" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B91" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E91" s="7" t="s">
         <v>254</v>
@@ -3085,10 +3103,10 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="17" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B92" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E92" s="7" t="s">
         <v>254</v>
@@ -3099,10 +3117,10 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="17" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B93" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="E93" s="7" t="s">
         <v>254</v>
@@ -3113,10 +3131,10 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="17" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B94" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E94" s="7" t="s">
         <v>254</v>
@@ -3127,10 +3145,10 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="17" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B95" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E95" s="7" t="s">
         <v>254</v>
@@ -3141,10 +3159,10 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="17" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B96" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E96" s="7" t="s">
         <v>254</v>
@@ -3155,10 +3173,10 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="17" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B97" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E97" s="7" t="s">
         <v>254</v>
@@ -3169,10 +3187,10 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="17" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B98" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E98" s="7" t="s">
         <v>254</v>
@@ -3183,10 +3201,10 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="17" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B99" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="E99" s="7" t="s">
         <v>254</v>
@@ -3197,10 +3215,10 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="17" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B100" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E100" s="7" t="s">
         <v>254</v>
@@ -3211,10 +3229,10 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="17" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B101" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E101" s="7" t="s">
         <v>254</v>
@@ -3225,10 +3243,10 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="17" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B102" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E102" s="7" t="s">
         <v>254</v>
@@ -3239,10 +3257,10 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="17" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B103" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E103" s="7" t="s">
         <v>254</v>
@@ -3253,10 +3271,10 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="17" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B104" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E104" s="7" t="s">
         <v>254</v>
@@ -3266,11 +3284,14 @@
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A105" s="11" t="s">
-        <v>258</v>
+      <c r="A105" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="B105" t="s">
+        <v>253</v>
       </c>
       <c r="E105" s="7" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="F105" s="14" t="s">
         <v>65</v>
@@ -3278,7 +3299,7 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="11" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E106" s="7" t="s">
         <v>267</v>
@@ -3289,7 +3310,7 @@
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="11" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E107" s="7" t="s">
         <v>267</v>
@@ -3300,7 +3321,7 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="11" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E108" s="7" t="s">
         <v>267</v>
@@ -3311,7 +3332,7 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="11" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E109" s="7" t="s">
         <v>267</v>
@@ -3322,7 +3343,7 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E110" s="7" t="s">
         <v>267</v>
@@ -3333,7 +3354,7 @@
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E111" s="7" t="s">
         <v>267</v>
@@ -3344,7 +3365,7 @@
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E112" s="7" t="s">
         <v>267</v>
@@ -3355,7 +3376,7 @@
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E113" s="7" t="s">
         <v>267</v>
@@ -3365,10 +3386,21 @@
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E114" s="7"/>
+      <c r="A114" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="E114" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="F114" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E115" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A104"/>
+  <autoFilter ref="A1:A105"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3432,7 +3464,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
@@ -3737,6 +3769,26 @@
       </c>
       <c r="F15" s="10">
         <v>210</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>315</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="9">
+        <v>685</v>
+      </c>
+      <c r="D16" s="9">
+        <v>165</v>
+      </c>
+      <c r="E16" s="10">
+        <v>420</v>
+      </c>
+      <c r="F16" s="10">
+        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -4895,7 +4947,7 @@
         <v>75</v>
       </c>
       <c r="D12" s="8">
-        <v>2500</v>
+        <v>6000</v>
       </c>
       <c r="E12" s="8">
         <v>1650</v>

</xml_diff>

<commit_message>
+ Make skill set for ZhuBaJie and LittleWhiteDragon and edit Attributes and Stats  of character.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="322">
   <si>
     <t>ID</t>
   </si>
@@ -986,6 +986,15 @@
   </si>
   <si>
     <t>STR_FIRELANCE_RING_DAMASL_SKILL</t>
+  </si>
+  <si>
+    <t>TheBoySage</t>
+  </si>
+  <si>
+    <t>STR_THE_BOY_SAGE</t>
+  </si>
+  <si>
+    <t>0.8</t>
   </si>
 </sst>
 </file>
@@ -4220,7 +4229,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -4504,6 +4513,29 @@
         <v>287</v>
       </c>
     </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>319</v>
+      </c>
+      <c r="B13" t="s">
+        <v>320</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="D13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E13" t="s">
+        <v>287</v>
+      </c>
+      <c r="F13" t="s">
+        <v>287</v>
+      </c>
+      <c r="G13" t="s">
+        <v>287</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4511,7 +4543,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -4971,6 +5003,44 @@
         <v>0</v>
       </c>
       <c r="L12" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>319</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="8">
+        <v>2650</v>
+      </c>
+      <c r="E13" s="8">
+        <v>2400</v>
+      </c>
+      <c r="F13" s="8">
+        <v>325</v>
+      </c>
+      <c r="G13" s="8">
+        <v>1</v>
+      </c>
+      <c r="H13" s="8">
+        <v>20</v>
+      </c>
+      <c r="I13" s="8">
+        <v>0</v>
+      </c>
+      <c r="J13" s="8">
+        <v>0</v>
+      </c>
+      <c r="K13" s="8">
+        <v>0</v>
+      </c>
+      <c r="L13" s="8">
         <v>0</v>
       </c>
     </row>
@@ -5086,7 +5156,7 @@
         <v>69</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
+ Config Battle Data.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="6"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="1" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -15,6 +15,8 @@
     <sheet name="CharacterStat" sheetId="6" r:id="rId6"/>
     <sheet name="CharacterAttribute" sheetId="8" r:id="rId7"/>
     <sheet name="CharacterUpgrade" sheetId="7" r:id="rId8"/>
+    <sheet name="BattleConfig" sheetId="9" r:id="rId9"/>
+    <sheet name="StageEnemies" sheetId="10" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$105</definedName>
@@ -29,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1049" uniqueCount="341">
   <si>
     <t>ID</t>
   </si>
@@ -995,6 +997,63 @@
   </si>
   <si>
     <t>0.8</t>
+  </si>
+  <si>
+    <t>GoldHornKing</t>
+  </si>
+  <si>
+    <t>SilverHornKing</t>
+  </si>
+  <si>
+    <t>YellowWindMonster</t>
+  </si>
+  <si>
+    <t>GoldfishDemon</t>
+  </si>
+  <si>
+    <t>STR_GOLD_HORN_KING</t>
+  </si>
+  <si>
+    <t>STR_SILVER_HORN_KING</t>
+  </si>
+  <si>
+    <t>STR_YELLOW_WIND_MONSTER</t>
+  </si>
+  <si>
+    <t>STR_GOLD_FISH_DEMON</t>
+  </si>
+  <si>
+    <t>Tutorial_Default</t>
+  </si>
+  <si>
+    <t>BackGrouind</t>
+  </si>
+  <si>
+    <t>Default</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_TUTORIAL</t>
+  </si>
+  <si>
+    <t>Reward</t>
+  </si>
+  <si>
+    <t>Default_01</t>
+  </si>
+  <si>
+    <t>BattleID</t>
+  </si>
+  <si>
+    <t>Slot</t>
+  </si>
+  <si>
+    <t>Enemy_ID</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VanguardTiger </t>
   </si>
 </sst>
 </file>
@@ -1010,7 +1069,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1095,6 +1154,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1108,7 +1173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1159,6 +1224,7 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3414,6 +3480,77 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.140625" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>336</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>337</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>338</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="B2" s="7">
+        <v>1</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>340</v>
+      </c>
+      <c r="D2" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="B3" s="7">
+        <v>2</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>340</v>
+      </c>
+      <c r="D3" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="B4" s="7">
+        <v>3</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>340</v>
+      </c>
+      <c r="D4" s="7">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C5"/>
@@ -4229,7 +4366,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -4491,8 +4628,8 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>310</v>
+      <c r="A12" s="24" t="s">
+        <v>340</v>
       </c>
       <c r="B12" t="s">
         <v>202</v>
@@ -4514,7 +4651,7 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="A13" s="24" t="s">
         <v>319</v>
       </c>
       <c r="B13" t="s">
@@ -4533,6 +4670,98 @@
         <v>287</v>
       </c>
       <c r="G13" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="24" t="s">
+        <v>322</v>
+      </c>
+      <c r="B14" t="s">
+        <v>326</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="D14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E14" t="s">
+        <v>287</v>
+      </c>
+      <c r="F14" t="s">
+        <v>287</v>
+      </c>
+      <c r="G14" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="24" t="s">
+        <v>323</v>
+      </c>
+      <c r="B15" t="s">
+        <v>327</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="D15" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15" t="s">
+        <v>287</v>
+      </c>
+      <c r="F15" t="s">
+        <v>287</v>
+      </c>
+      <c r="G15" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="24" t="s">
+        <v>324</v>
+      </c>
+      <c r="B16" t="s">
+        <v>328</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="D16" t="s">
+        <v>74</v>
+      </c>
+      <c r="E16" t="s">
+        <v>287</v>
+      </c>
+      <c r="F16" t="s">
+        <v>287</v>
+      </c>
+      <c r="G16" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="24" t="s">
+        <v>325</v>
+      </c>
+      <c r="B17" t="s">
+        <v>329</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="D17" t="s">
+        <v>74</v>
+      </c>
+      <c r="E17" t="s">
+        <v>287</v>
+      </c>
+      <c r="F17" t="s">
+        <v>287</v>
+      </c>
+      <c r="G17" t="s">
         <v>287</v>
       </c>
     </row>
@@ -4543,7 +4772,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -4969,8 +5198,8 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>310</v>
+      <c r="A12" s="24" t="s">
+        <v>340</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>289</v>
@@ -5007,7 +5236,7 @@
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="A13" s="24" t="s">
         <v>319</v>
       </c>
       <c r="B13" s="16" t="s">
@@ -5041,6 +5270,158 @@
         <v>0</v>
       </c>
       <c r="L13" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="24" t="s">
+        <v>322</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" s="8">
+        <v>2650</v>
+      </c>
+      <c r="E14" s="8">
+        <v>2400</v>
+      </c>
+      <c r="F14" s="8">
+        <v>325</v>
+      </c>
+      <c r="G14" s="8">
+        <v>1</v>
+      </c>
+      <c r="H14" s="8">
+        <v>20</v>
+      </c>
+      <c r="I14" s="8">
+        <v>0</v>
+      </c>
+      <c r="J14" s="8">
+        <v>0</v>
+      </c>
+      <c r="K14" s="8">
+        <v>0</v>
+      </c>
+      <c r="L14" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="24" t="s">
+        <v>323</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" s="8">
+        <v>2650</v>
+      </c>
+      <c r="E15" s="8">
+        <v>2400</v>
+      </c>
+      <c r="F15" s="8">
+        <v>325</v>
+      </c>
+      <c r="G15" s="8">
+        <v>1</v>
+      </c>
+      <c r="H15" s="8">
+        <v>20</v>
+      </c>
+      <c r="I15" s="8">
+        <v>0</v>
+      </c>
+      <c r="J15" s="8">
+        <v>0</v>
+      </c>
+      <c r="K15" s="8">
+        <v>0</v>
+      </c>
+      <c r="L15" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" s="24" t="s">
+        <v>324</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="C16" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="8">
+        <v>2650</v>
+      </c>
+      <c r="E16" s="8">
+        <v>2400</v>
+      </c>
+      <c r="F16" s="8">
+        <v>325</v>
+      </c>
+      <c r="G16" s="8">
+        <v>1</v>
+      </c>
+      <c r="H16" s="8">
+        <v>20</v>
+      </c>
+      <c r="I16" s="8">
+        <v>0</v>
+      </c>
+      <c r="J16" s="8">
+        <v>0</v>
+      </c>
+      <c r="K16" s="8">
+        <v>0</v>
+      </c>
+      <c r="L16" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" s="24" t="s">
+        <v>325</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" s="8">
+        <v>2650</v>
+      </c>
+      <c r="E17" s="8">
+        <v>2400</v>
+      </c>
+      <c r="F17" s="8">
+        <v>325</v>
+      </c>
+      <c r="G17" s="8">
+        <v>1</v>
+      </c>
+      <c r="H17" s="8">
+        <v>20</v>
+      </c>
+      <c r="I17" s="8">
+        <v>0</v>
+      </c>
+      <c r="J17" s="8">
+        <v>0</v>
+      </c>
+      <c r="K17" s="8">
+        <v>0</v>
+      </c>
+      <c r="L17" s="8">
         <v>0</v>
       </c>
     </row>
@@ -5051,7 +5432,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -5280,8 +5661,8 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>310</v>
+      <c r="A12" s="24" t="s">
+        <v>340</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>289</v>
@@ -5296,6 +5677,106 @@
         <v>69</v>
       </c>
       <c r="F12" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="24" t="s">
+        <v>319</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="24" t="s">
+        <v>322</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="24" t="s">
+        <v>323</v>
+      </c>
+      <c r="B15" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="24" t="s">
+        <v>324</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="24" t="s">
+        <v>325</v>
+      </c>
+      <c r="B17" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F17" s="7" t="s">
         <v>314</v>
       </c>
     </row>
@@ -5307,7 +5788,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -5484,6 +5965,121 @@
         <v>20</v>
       </c>
     </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="24" t="s">
+        <v>319</v>
+      </c>
+      <c r="B13" s="8">
+        <v>175</v>
+      </c>
+      <c r="C13" s="8">
+        <v>115</v>
+      </c>
+      <c r="D13" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="24" t="s">
+        <v>322</v>
+      </c>
+      <c r="B14" s="8">
+        <v>175</v>
+      </c>
+      <c r="C14" s="8">
+        <v>115</v>
+      </c>
+      <c r="D14" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="24" t="s">
+        <v>323</v>
+      </c>
+      <c r="B15" s="8">
+        <v>175</v>
+      </c>
+      <c r="C15" s="8">
+        <v>115</v>
+      </c>
+      <c r="D15" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="24" t="s">
+        <v>324</v>
+      </c>
+      <c r="B16" s="8">
+        <v>175</v>
+      </c>
+      <c r="C16" s="8">
+        <v>115</v>
+      </c>
+      <c r="D16" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="24" t="s">
+        <v>325</v>
+      </c>
+      <c r="B17" s="8">
+        <v>175</v>
+      </c>
+      <c r="C17" s="8">
+        <v>115</v>
+      </c>
+      <c r="D17" s="8">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>331</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>335</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
+ Make UI for Battle Scene and add icon skill for all characters.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="1" activeTab="9"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="1" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="StageEnemies" sheetId="10" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$111</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1049" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="342">
   <si>
     <t>ID</t>
   </si>
@@ -1054,6 +1054,9 @@
   </si>
   <si>
     <t xml:space="preserve">VanguardTiger </t>
+  </si>
+  <si>
+    <t>STR_VANGUARD_TIGER</t>
   </si>
 </sst>
 </file>
@@ -1505,7 +1508,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
@@ -2869,92 +2872,110 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" s="17" t="s">
-        <v>212</v>
+      <c r="A70" s="24" t="s">
+        <v>340</v>
       </c>
       <c r="B70" t="s">
-        <v>248</v>
+        <v>341</v>
+      </c>
+      <c r="C70" t="s">
+        <v>201</v>
       </c>
       <c r="E70" s="7" t="s">
-        <v>254</v>
+        <v>211</v>
       </c>
       <c r="F70" s="14" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" s="17" t="s">
-        <v>213</v>
+      <c r="A71" s="24" t="s">
+        <v>319</v>
       </c>
       <c r="B71" t="s">
-        <v>249</v>
+        <v>320</v>
+      </c>
+      <c r="C71" t="s">
+        <v>201</v>
       </c>
       <c r="E71" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="F71" s="14" t="s">
-        <v>65</v>
+        <v>211</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" s="17" t="s">
-        <v>214</v>
+      <c r="A72" s="24" t="s">
+        <v>322</v>
       </c>
       <c r="B72" t="s">
-        <v>250</v>
+        <v>326</v>
+      </c>
+      <c r="C72" t="s">
+        <v>201</v>
       </c>
       <c r="E72" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="F72" s="14" t="s">
-        <v>65</v>
+        <v>211</v>
+      </c>
+      <c r="F72" s="16" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A73" s="17" t="s">
-        <v>215</v>
+      <c r="A73" s="24" t="s">
+        <v>323</v>
       </c>
       <c r="B73" t="s">
-        <v>251</v>
+        <v>327</v>
+      </c>
+      <c r="C73" t="s">
+        <v>201</v>
       </c>
       <c r="E73" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="F73" s="14" t="s">
-        <v>65</v>
+        <v>211</v>
+      </c>
+      <c r="F73" s="16" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A74" s="17" t="s">
-        <v>216</v>
+      <c r="A74" s="24" t="s">
+        <v>324</v>
       </c>
       <c r="B74" t="s">
-        <v>252</v>
+        <v>328</v>
+      </c>
+      <c r="C74" t="s">
+        <v>201</v>
       </c>
       <c r="E74" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="F74" s="14" t="s">
-        <v>65</v>
+        <v>211</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A75" s="17" t="s">
-        <v>217</v>
+      <c r="A75" s="24" t="s">
+        <v>325</v>
       </c>
       <c r="B75" t="s">
-        <v>253</v>
+        <v>329</v>
+      </c>
+      <c r="C75" t="s">
+        <v>201</v>
       </c>
       <c r="E75" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="F75" s="14" t="s">
-        <v>65</v>
+        <v>211</v>
+      </c>
+      <c r="F75" s="16" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="17" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="B76" t="s">
         <v>248</v>
@@ -2968,7 +2989,7 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="17" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="B77" t="s">
         <v>249</v>
@@ -2982,7 +3003,7 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="17" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="B78" t="s">
         <v>250</v>
@@ -2996,7 +3017,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="17" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="B79" t="s">
         <v>251</v>
@@ -3010,7 +3031,7 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="17" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="B80" t="s">
         <v>252</v>
@@ -3024,7 +3045,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="17" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="B81" t="s">
         <v>253</v>
@@ -3038,7 +3059,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="17" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="B82" t="s">
         <v>248</v>
@@ -3052,7 +3073,7 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="17" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="B83" t="s">
         <v>249</v>
@@ -3066,7 +3087,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="17" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="B84" t="s">
         <v>250</v>
@@ -3080,7 +3101,7 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="17" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="B85" t="s">
         <v>251</v>
@@ -3094,7 +3115,7 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="17" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="B86" t="s">
         <v>252</v>
@@ -3108,7 +3129,7 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="17" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="B87" t="s">
         <v>253</v>
@@ -3122,7 +3143,7 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="17" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="B88" t="s">
         <v>248</v>
@@ -3136,7 +3157,7 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="17" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B89" t="s">
         <v>249</v>
@@ -3150,7 +3171,7 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="17" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="B90" t="s">
         <v>250</v>
@@ -3164,7 +3185,7 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="17" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="B91" t="s">
         <v>251</v>
@@ -3178,7 +3199,7 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="17" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="B92" t="s">
         <v>252</v>
@@ -3192,7 +3213,7 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="17" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="B93" t="s">
         <v>253</v>
@@ -3206,7 +3227,7 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="17" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B94" t="s">
         <v>248</v>
@@ -3220,7 +3241,7 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="17" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="B95" t="s">
         <v>249</v>
@@ -3234,7 +3255,7 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="17" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="B96" t="s">
         <v>250</v>
@@ -3248,7 +3269,7 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="17" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="B97" t="s">
         <v>251</v>
@@ -3262,7 +3283,7 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="17" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="B98" t="s">
         <v>252</v>
@@ -3276,7 +3297,7 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="17" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B99" t="s">
         <v>253</v>
@@ -3290,7 +3311,7 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="17" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B100" t="s">
         <v>248</v>
@@ -3304,7 +3325,7 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="17" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="B101" t="s">
         <v>249</v>
@@ -3318,7 +3339,7 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="17" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="B102" t="s">
         <v>250</v>
@@ -3332,7 +3353,7 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="17" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="B103" t="s">
         <v>251</v>
@@ -3346,7 +3367,7 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="17" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="B104" t="s">
         <v>252</v>
@@ -3360,7 +3381,7 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="17" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="B105" t="s">
         <v>253</v>
@@ -3373,66 +3394,84 @@
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A106" s="11" t="s">
-        <v>258</v>
+      <c r="A106" s="17" t="s">
+        <v>242</v>
+      </c>
+      <c r="B106" t="s">
+        <v>248</v>
       </c>
       <c r="E106" s="7" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="F106" s="14" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A107" s="11" t="s">
-        <v>259</v>
+      <c r="A107" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="B107" t="s">
+        <v>249</v>
       </c>
       <c r="E107" s="7" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="F107" s="14" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A108" s="11" t="s">
-        <v>260</v>
+      <c r="A108" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="B108" t="s">
+        <v>250</v>
       </c>
       <c r="E108" s="7" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="F108" s="14" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A109" s="11" t="s">
-        <v>261</v>
+      <c r="A109" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="B109" t="s">
+        <v>251</v>
       </c>
       <c r="E109" s="7" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="F109" s="14" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A110" s="11" t="s">
-        <v>262</v>
+      <c r="A110" s="17" t="s">
+        <v>246</v>
+      </c>
+      <c r="B110" t="s">
+        <v>252</v>
       </c>
       <c r="E110" s="7" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="F110" s="14" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A111" s="11" t="s">
-        <v>263</v>
+      <c r="A111" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="B111" t="s">
+        <v>253</v>
       </c>
       <c r="E111" s="7" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="F111" s="14" t="s">
         <v>65</v>
@@ -3440,7 +3479,7 @@
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="11" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="E112" s="7" t="s">
         <v>267</v>
@@ -3451,7 +3490,7 @@
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="E113" s="7" t="s">
         <v>267</v>
@@ -3462,7 +3501,7 @@
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="11" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="E114" s="7" t="s">
         <v>267</v>
@@ -3472,17 +3511,83 @@
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E115" s="7"/>
+      <c r="A115" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="E115" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="F115" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" s="11" t="s">
+        <v>262</v>
+      </c>
+      <c r="E116" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="F116" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="E117" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="F117" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="E118" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="F118" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="E119" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="F119" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="E120" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="F120" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E121" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A105"/>
+  <autoFilter ref="A1:A111"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" customWidth="1"/>
@@ -3543,6 +3648,20 @@
         <v>340</v>
       </c>
       <c r="D4" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="B5" s="7">
+        <v>5</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>324</v>
+      </c>
+      <c r="D5" s="7">
         <v>5</v>
       </c>
     </row>
@@ -4632,7 +4751,7 @@
         <v>340</v>
       </c>
       <c r="B12" t="s">
-        <v>202</v>
+        <v>341</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>289</v>
@@ -4657,8 +4776,8 @@
       <c r="B13" t="s">
         <v>320</v>
       </c>
-      <c r="C13" s="16" t="s">
-        <v>291</v>
+      <c r="C13" s="2" t="s">
+        <v>286</v>
       </c>
       <c r="D13" t="s">
         <v>74</v>
@@ -4726,8 +4845,8 @@
       <c r="B16" t="s">
         <v>328</v>
       </c>
-      <c r="C16" s="16" t="s">
-        <v>291</v>
+      <c r="C16" s="2" t="s">
+        <v>286</v>
       </c>
       <c r="D16" t="s">
         <v>74</v>
@@ -5239,8 +5358,8 @@
       <c r="A13" s="24" t="s">
         <v>319</v>
       </c>
-      <c r="B13" s="16" t="s">
-        <v>291</v>
+      <c r="B13" s="2" t="s">
+        <v>286</v>
       </c>
       <c r="C13" s="23" t="s">
         <v>74</v>
@@ -5353,8 +5472,8 @@
       <c r="A16" s="24" t="s">
         <v>324</v>
       </c>
-      <c r="B16" s="16" t="s">
-        <v>291</v>
+      <c r="B16" s="2" t="s">
+        <v>286</v>
       </c>
       <c r="C16" s="23" t="s">
         <v>74</v>
@@ -5667,8 +5786,8 @@
       <c r="B12" s="19" t="s">
         <v>289</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>75</v>
+      <c r="C12" s="20" t="s">
+        <v>73</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>301</v>
@@ -5684,11 +5803,11 @@
       <c r="A13" s="24" t="s">
         <v>319</v>
       </c>
-      <c r="B13" s="19" t="s">
-        <v>289</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>75</v>
+      <c r="B13" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>74</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>301</v>
@@ -5704,8 +5823,8 @@
       <c r="A14" s="24" t="s">
         <v>322</v>
       </c>
-      <c r="B14" s="19" t="s">
-        <v>289</v>
+      <c r="B14" s="16" t="s">
+        <v>291</v>
       </c>
       <c r="C14" s="12" t="s">
         <v>75</v>
@@ -5724,8 +5843,8 @@
       <c r="A15" s="24" t="s">
         <v>323</v>
       </c>
-      <c r="B15" s="19" t="s">
-        <v>289</v>
+      <c r="B15" s="16" t="s">
+        <v>291</v>
       </c>
       <c r="C15" s="12" t="s">
         <v>75</v>
@@ -5744,11 +5863,11 @@
       <c r="A16" s="24" t="s">
         <v>324</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>289</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>75</v>
+      <c r="B16" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C16" s="23" t="s">
+        <v>74</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>301</v>
@@ -5764,11 +5883,11 @@
       <c r="A17" s="24" t="s">
         <v>325</v>
       </c>
-      <c r="B17" s="19" t="s">
-        <v>289</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>75</v>
+      <c r="B17" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>73</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>301</v>
@@ -6070,7 +6189,7 @@
       <c r="A2" s="7" t="s">
         <v>330</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" t="s">
         <v>333</v>
       </c>
       <c r="C2" s="7" t="s">

</xml_diff>

<commit_message>
+ Battle Setup State (Init character and enemy and init skill for character)
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="354">
   <si>
     <t>ID</t>
   </si>
@@ -879,24 +879,12 @@
     <t>Ring</t>
   </si>
   <si>
-    <t>FirstSkill</t>
-  </si>
-  <si>
-    <t>SecondSkill</t>
-  </si>
-  <si>
-    <t>ThirdSkill</t>
-  </si>
-  <si>
     <t>SunWukong</t>
   </si>
   <si>
     <t>UR</t>
   </si>
   <si>
-    <t>null</t>
-  </si>
-  <si>
     <t>TangSanZang</t>
   </si>
   <si>
@@ -996,9 +984,6 @@
     <t>STR_THE_BOY_SAGE</t>
   </si>
   <si>
-    <t>0.8</t>
-  </si>
-  <si>
     <t>GoldHornKing</t>
   </si>
   <si>
@@ -1057,6 +1042,57 @@
   </si>
   <si>
     <t>STR_VANGUARD_TIGER</t>
+  </si>
+  <si>
+    <t>Melee</t>
+  </si>
+  <si>
+    <t>Range</t>
+  </si>
+  <si>
+    <t>Summon</t>
+  </si>
+  <si>
+    <t>BuffShield</t>
+  </si>
+  <si>
+    <t>Healing</t>
+  </si>
+  <si>
+    <t>ThunderBall</t>
+  </si>
+  <si>
+    <t>FireRing</t>
+  </si>
+  <si>
+    <t>FireBall</t>
+  </si>
+  <si>
+    <t>EmpowerAttack</t>
+  </si>
+  <si>
+    <t>Torando</t>
+  </si>
+  <si>
+    <t>Suriken</t>
+  </si>
+  <si>
+    <t>PosionBall</t>
+  </si>
+  <si>
+    <t>DivineWind</t>
+  </si>
+  <si>
+    <t>Base</t>
+  </si>
+  <si>
+    <t>Major</t>
+  </si>
+  <si>
+    <t>Ultimate</t>
+  </si>
+  <si>
+    <t>None</t>
   </si>
 </sst>
 </file>
@@ -1072,7 +1108,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1163,6 +1199,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1176,7 +1218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1228,6 +1270,13 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1823,16 +1872,16 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="B16" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="C16" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D16" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>62</v>
@@ -2703,7 +2752,7 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="12" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="B60" t="s">
         <v>200</v>
@@ -2720,7 +2769,7 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="12" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="B61" t="s">
         <v>202</v>
@@ -2737,7 +2786,7 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="12" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="B62" t="s">
         <v>203</v>
@@ -2754,7 +2803,7 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="12" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B63" t="s">
         <v>204</v>
@@ -2771,7 +2820,7 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="12" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="B64" t="s">
         <v>205</v>
@@ -2788,7 +2837,7 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="12" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="B65" t="s">
         <v>206</v>
@@ -2805,7 +2854,7 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="12" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="B66" t="s">
         <v>207</v>
@@ -2822,7 +2871,7 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="12" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="B67" t="s">
         <v>208</v>
@@ -2839,7 +2888,7 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="12" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B68" t="s">
         <v>209</v>
@@ -2856,7 +2905,7 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="12" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="B69" t="s">
         <v>210</v>
@@ -2873,10 +2922,10 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="24" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="B70" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C70" t="s">
         <v>201</v>
@@ -2890,10 +2939,10 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="24" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B71" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C71" t="s">
         <v>201</v>
@@ -2907,10 +2956,10 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="24" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="B72" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="C72" t="s">
         <v>201</v>
@@ -2924,10 +2973,10 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="24" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="B73" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="C73" t="s">
         <v>201</v>
@@ -2941,10 +2990,10 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="24" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B74" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="C74" t="s">
         <v>201</v>
@@ -2958,10 +3007,10 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="24" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="B75" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="C75" t="s">
         <v>201</v>
@@ -3587,7 +3636,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" customWidth="1"/>
@@ -3597,27 +3646,27 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="B2" s="7">
         <v>1</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D2" s="7">
         <v>5</v>
@@ -3625,13 +3674,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="B3" s="7">
         <v>2</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D3" s="7">
         <v>5</v>
@@ -3639,29 +3688,15 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="B4" s="7">
         <v>3</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="D4" s="7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="B5" s="7">
-        <v>5</v>
-      </c>
-      <c r="C5" s="24" t="s">
-        <v>324</v>
-      </c>
-      <c r="D5" s="7">
         <v>5</v>
       </c>
     </row>
@@ -4038,7 +4073,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>73</v>
@@ -4491,6 +4526,9 @@
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -4507,381 +4545,381 @@
         <v>68</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>282</v>
+        <v>350</v>
       </c>
       <c r="F1" s="18" t="s">
-        <v>283</v>
+        <v>351</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>284</v>
+        <v>352</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="B2" t="s">
         <v>200</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="D2" t="s">
+        <v>283</v>
+      </c>
+      <c r="D2" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="E2" t="s">
-        <v>287</v>
-      </c>
-      <c r="F2" t="s">
-        <v>287</v>
-      </c>
-      <c r="G2" t="s">
-        <v>287</v>
+      <c r="E2" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="B3" t="s">
         <v>202</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>289</v>
-      </c>
-      <c r="D3" t="s">
+        <v>285</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E3" t="s">
-        <v>287</v>
-      </c>
-      <c r="F3" t="s">
-        <v>287</v>
-      </c>
-      <c r="G3" t="s">
-        <v>287</v>
+      <c r="E3" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="B4" t="s">
         <v>203</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="D4" t="s">
+        <v>287</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E4" t="s">
-        <v>287</v>
-      </c>
-      <c r="F4" t="s">
-        <v>287</v>
-      </c>
-      <c r="G4" t="s">
-        <v>287</v>
+      <c r="E4" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B5" t="s">
         <v>204</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="D5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="E5" t="s">
-        <v>287</v>
-      </c>
-      <c r="F5" t="s">
-        <v>287</v>
-      </c>
-      <c r="G5" t="s">
-        <v>287</v>
+      <c r="E5" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>341</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>294</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="A6" s="25" t="s">
+        <v>290</v>
+      </c>
+      <c r="B6" s="25" t="s">
         <v>205</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="C6" s="26" t="s">
+        <v>289</v>
+      </c>
+      <c r="D6" s="27" t="s">
         <v>78</v>
       </c>
-      <c r="E6" t="s">
-        <v>287</v>
-      </c>
-      <c r="F6" t="s">
-        <v>287</v>
-      </c>
-      <c r="G6" t="s">
-        <v>287</v>
+      <c r="E6" s="27" t="s">
+        <v>337</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>353</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="B7" t="s">
         <v>206</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="D7" t="s">
+        <v>287</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E7" t="s">
-        <v>287</v>
-      </c>
-      <c r="F7" t="s">
-        <v>287</v>
-      </c>
-      <c r="G7" t="s">
-        <v>287</v>
+      <c r="E7" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="B8" t="s">
         <v>207</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="D8" t="s">
-        <v>297</v>
-      </c>
-      <c r="E8" t="s">
-        <v>287</v>
-      </c>
-      <c r="F8" t="s">
-        <v>287</v>
-      </c>
-      <c r="G8" t="s">
-        <v>287</v>
+      <c r="E8" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="B9" t="s">
         <v>208</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="D9" t="s">
+        <v>287</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E9" t="s">
-        <v>287</v>
-      </c>
-      <c r="F9" t="s">
-        <v>287</v>
-      </c>
-      <c r="G9" t="s">
-        <v>287</v>
+      <c r="E9" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>348</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>299</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="A10" s="25" t="s">
+        <v>295</v>
+      </c>
+      <c r="B10" s="25" t="s">
         <v>209</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="C10" s="26" t="s">
+        <v>283</v>
+      </c>
+      <c r="D10" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="E10" t="s">
-        <v>287</v>
-      </c>
-      <c r="F10" t="s">
-        <v>287</v>
-      </c>
-      <c r="G10" t="s">
-        <v>287</v>
+      <c r="E10" s="27" t="s">
+        <v>337</v>
+      </c>
+      <c r="F10" s="27" t="s">
+        <v>353</v>
+      </c>
+      <c r="G10" s="27" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>300</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="A11" s="25" t="s">
+        <v>296</v>
+      </c>
+      <c r="B11" s="25" t="s">
         <v>210</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="C11" s="26" t="s">
+        <v>283</v>
+      </c>
+      <c r="D11" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="E11" t="s">
-        <v>287</v>
-      </c>
-      <c r="F11" t="s">
-        <v>287</v>
-      </c>
-      <c r="G11" t="s">
-        <v>287</v>
+      <c r="E11" s="27" t="s">
+        <v>338</v>
+      </c>
+      <c r="F11" s="27" t="s">
+        <v>353</v>
+      </c>
+      <c r="G11" s="27" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="B12" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>289</v>
-      </c>
-      <c r="D12" t="s">
+        <v>285</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E12" t="s">
-        <v>287</v>
-      </c>
-      <c r="F12" t="s">
-        <v>287</v>
-      </c>
-      <c r="G12" t="s">
-        <v>287</v>
+      <c r="E12" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>353</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="24" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B13" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="D13" t="s">
+        <v>283</v>
+      </c>
+      <c r="D13" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E13" t="s">
-        <v>287</v>
-      </c>
-      <c r="F13" t="s">
-        <v>287</v>
-      </c>
-      <c r="G13" t="s">
-        <v>287</v>
+      <c r="E13" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="B14" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="D14" t="s">
+        <v>287</v>
+      </c>
+      <c r="D14" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E14" t="s">
-        <v>287</v>
-      </c>
-      <c r="F14" t="s">
-        <v>287</v>
-      </c>
-      <c r="G14" t="s">
-        <v>287</v>
+      <c r="E14" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="B15" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="D15" t="s">
+        <v>287</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E15" t="s">
-        <v>287</v>
-      </c>
-      <c r="F15" t="s">
-        <v>287</v>
-      </c>
-      <c r="G15" t="s">
-        <v>287</v>
+      <c r="E15" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B16" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="D16" t="s">
+        <v>283</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E16" t="s">
-        <v>287</v>
-      </c>
-      <c r="F16" t="s">
-        <v>287</v>
-      </c>
-      <c r="G16" t="s">
-        <v>287</v>
+      <c r="E16" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="B17" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="D17" t="s">
+        <v>287</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E17" t="s">
-        <v>287</v>
-      </c>
-      <c r="F17" t="s">
-        <v>287</v>
-      </c>
-      <c r="G17" t="s">
-        <v>287</v>
+      <c r="E17" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -4909,39 +4947,39 @@
         <v>68</v>
       </c>
       <c r="D1" s="18" t="s">
+        <v>297</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>298</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>300</v>
+      </c>
+      <c r="H1" s="18" t="s">
         <v>301</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="I1" s="18" t="s">
         <v>302</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="J1" s="18" t="s">
         <v>303</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="K1" s="18" t="s">
         <v>304</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="L1" s="18" t="s">
         <v>305</v>
-      </c>
-      <c r="I1" s="18" t="s">
-        <v>306</v>
-      </c>
-      <c r="J1" s="18" t="s">
-        <v>307</v>
-      </c>
-      <c r="K1" s="18" t="s">
-        <v>308</v>
-      </c>
-      <c r="L1" s="18" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C2" s="20" t="s">
         <v>73</v>
@@ -4976,10 +5014,10 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="C3" s="12" t="s">
         <v>75</v>
@@ -5014,10 +5052,10 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C4" s="21" t="s">
         <v>76</v>
@@ -5052,10 +5090,10 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="C5" s="22" t="s">
         <v>78</v>
@@ -5090,10 +5128,10 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>78</v>
@@ -5128,10 +5166,10 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C7" s="23" t="s">
         <v>74</v>
@@ -5166,13 +5204,13 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C8" s="13" t="s">
         <v>293</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>297</v>
       </c>
       <c r="D8" s="8">
         <v>2750</v>
@@ -5204,10 +5242,10 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C9" s="21" t="s">
         <v>76</v>
@@ -5242,10 +5280,10 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C10" s="21" t="s">
         <v>76</v>
@@ -5280,10 +5318,10 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>75</v>
@@ -5318,10 +5356,10 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>75</v>
@@ -5356,10 +5394,10 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="24" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C13" s="23" t="s">
         <v>74</v>
@@ -5394,10 +5432,10 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C14" s="23" t="s">
         <v>74</v>
@@ -5432,10 +5470,10 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C15" s="23" t="s">
         <v>74</v>
@@ -5470,16 +5508,16 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C16" s="23" t="s">
         <v>74</v>
       </c>
       <c r="D16" s="8">
-        <v>2650</v>
+        <v>6000</v>
       </c>
       <c r="E16" s="8">
         <v>2400</v>
@@ -5508,10 +5546,10 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C17" s="23" t="s">
         <v>74</v>
@@ -5570,333 +5608,333 @@
         <v>68</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="F1" s="18" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C2" s="20" t="s">
         <v>73</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="C3" s="12" t="s">
         <v>75</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C4" s="21" t="s">
         <v>76</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="C5" s="22" t="s">
         <v>78</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>78</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C7" s="23" t="s">
         <v>74</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C8" s="13" t="s">
         <v>293</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="D8" s="7" t="s">
         <v>297</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>301</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C9" s="21" t="s">
         <v>76</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C10" s="21" t="s">
         <v>76</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>75</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="C12" s="20" t="s">
         <v>73</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="24" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C13" s="23" t="s">
         <v>74</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C14" s="12" t="s">
         <v>75</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C15" s="12" t="s">
         <v>75</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C16" s="23" t="s">
         <v>74</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="C17" s="20" t="s">
         <v>73</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
   </sheetData>
@@ -5921,18 +5959,18 @@
         <v>0</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="B2" s="8">
         <v>375</v>
@@ -5946,7 +5984,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="B3" s="8">
         <v>175</v>
@@ -5960,7 +5998,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="B4" s="8">
         <v>350</v>
@@ -5974,7 +6012,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B5" s="8">
         <v>232</v>
@@ -5988,7 +6026,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="B6" s="8">
         <v>234</v>
@@ -6002,7 +6040,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="B7" s="8">
         <v>238</v>
@@ -6016,7 +6054,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="B8" s="8">
         <v>220</v>
@@ -6030,7 +6068,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="B9" s="8">
         <v>425</v>
@@ -6044,7 +6082,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B10" s="8">
         <v>370</v>
@@ -6058,7 +6096,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="B11" s="8">
         <v>300</v>
@@ -6072,7 +6110,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="B12" s="8">
         <v>175</v>
@@ -6086,7 +6124,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="24" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B13" s="8">
         <v>175</v>
@@ -6100,7 +6138,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="B14" s="8">
         <v>175</v>
@@ -6114,7 +6152,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="B15" s="8">
         <v>175</v>
@@ -6128,7 +6166,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B16" s="8">
         <v>175</v>
@@ -6142,7 +6180,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="B17" s="8">
         <v>175</v>
@@ -6179,24 +6217,24 @@
         <v>1</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="B2" t="s">
+        <v>328</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>330</v>
-      </c>
-      <c r="B2" t="s">
-        <v>333</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Fix skill bug for all character in battle.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="1" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="1" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1085" uniqueCount="355">
   <si>
     <t>ID</t>
   </si>
@@ -1093,6 +1093,9 @@
   </si>
   <si>
     <t>None</t>
+  </si>
+  <si>
+    <t>MajorAttack</t>
   </si>
 </sst>
 </file>
@@ -3636,7 +3639,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" customWidth="1"/>
@@ -3697,6 +3700,48 @@
         <v>335</v>
       </c>
       <c r="D4" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="B5" s="7">
+        <v>4</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>335</v>
+      </c>
+      <c r="D5" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="B6" s="7">
+        <v>5</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>335</v>
+      </c>
+      <c r="D6" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="B7" s="7">
+        <v>6</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>335</v>
+      </c>
+      <c r="D7" s="7">
         <v>5</v>
       </c>
     </row>
@@ -4847,7 +4892,7 @@
         <v>337</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>345</v>
+        <v>354</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>345</v>
@@ -4916,7 +4961,7 @@
         <v>337</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>345</v>
+        <v>354</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>345</v>
@@ -5365,7 +5410,7 @@
         <v>75</v>
       </c>
       <c r="D12" s="8">
-        <v>6000</v>
+        <v>2500</v>
       </c>
       <c r="E12" s="8">
         <v>1650</v>

</xml_diff>

<commit_message>
+ Action Queue for character skill and make Action Point System (Speed of character) to order turn.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="1" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="1" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -933,9 +933,6 @@
     <t>def</t>
   </si>
   <si>
-    <t>spd</t>
-  </si>
-  <si>
     <t>def_shred</t>
   </si>
   <si>
@@ -1096,6 +1093,9 @@
   </si>
   <si>
     <t>MajorAttack</t>
+  </si>
+  <si>
+    <t>speed</t>
   </si>
 </sst>
 </file>
@@ -1875,16 +1875,16 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="B16" t="s">
         <v>311</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>312</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>313</v>
-      </c>
-      <c r="D16" t="s">
-        <v>314</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>62</v>
@@ -2925,10 +2925,10 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="24" t="s">
+        <v>334</v>
+      </c>
+      <c r="B70" t="s">
         <v>335</v>
-      </c>
-      <c r="B70" t="s">
-        <v>336</v>
       </c>
       <c r="C70" t="s">
         <v>201</v>
@@ -2942,10 +2942,10 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="24" t="s">
+        <v>314</v>
+      </c>
+      <c r="B71" t="s">
         <v>315</v>
-      </c>
-      <c r="B71" t="s">
-        <v>316</v>
       </c>
       <c r="C71" t="s">
         <v>201</v>
@@ -2959,10 +2959,10 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="24" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B72" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C72" t="s">
         <v>201</v>
@@ -2976,10 +2976,10 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="24" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B73" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C73" t="s">
         <v>201</v>
@@ -2993,10 +2993,10 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="24" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B74" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C74" t="s">
         <v>201</v>
@@ -3010,10 +3010,10 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="24" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B75" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C75" t="s">
         <v>201</v>
@@ -3649,27 +3649,27 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
+        <v>330</v>
+      </c>
+      <c r="B1" s="18" t="s">
         <v>331</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="C1" s="18" t="s">
         <v>332</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="D1" s="18" t="s">
         <v>333</v>
-      </c>
-      <c r="D1" s="18" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B2" s="7">
         <v>1</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D2" s="7">
         <v>5</v>
@@ -3677,13 +3677,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B3" s="7">
         <v>2</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D3" s="7">
         <v>5</v>
@@ -3691,13 +3691,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B4" s="7">
         <v>3</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D4" s="7">
         <v>5</v>
@@ -3705,13 +3705,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B5" s="7">
         <v>4</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D5" s="7">
         <v>5</v>
@@ -3719,13 +3719,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B6" s="7">
         <v>5</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D6" s="7">
         <v>5</v>
@@ -3733,13 +3733,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B7" s="7">
         <v>6</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D7" s="7">
         <v>5</v>
@@ -4118,7 +4118,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>73</v>
@@ -4590,13 +4590,13 @@
         <v>68</v>
       </c>
       <c r="E1" s="18" t="s">
+        <v>349</v>
+      </c>
+      <c r="F1" s="18" t="s">
         <v>350</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="G1" s="18" t="s">
         <v>351</v>
-      </c>
-      <c r="G1" s="18" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -4613,13 +4613,13 @@
         <v>73</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -4636,13 +4636,13 @@
         <v>75</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -4659,13 +4659,13 @@
         <v>76</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -4682,13 +4682,13 @@
         <v>78</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -4705,13 +4705,13 @@
         <v>78</v>
       </c>
       <c r="E6" s="27" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="G6" s="27" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -4728,13 +4728,13 @@
         <v>74</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -4751,13 +4751,13 @@
         <v>293</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -4774,13 +4774,13 @@
         <v>76</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -4797,13 +4797,13 @@
         <v>73</v>
       </c>
       <c r="E10" s="27" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F10" s="27" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="G10" s="27" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -4820,21 +4820,21 @@
         <v>75</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F11" s="27" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="G11" s="27" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
+        <v>334</v>
+      </c>
+      <c r="B12" t="s">
         <v>335</v>
-      </c>
-      <c r="B12" t="s">
-        <v>336</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>285</v>
@@ -4843,21 +4843,21 @@
         <v>75</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="24" t="s">
+        <v>314</v>
+      </c>
+      <c r="B13" t="s">
         <v>315</v>
-      </c>
-      <c r="B13" t="s">
-        <v>316</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>283</v>
@@ -4866,21 +4866,21 @@
         <v>74</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F13" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="G13" s="7" t="s">
         <v>344</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B14" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>287</v>
@@ -4889,21 +4889,21 @@
         <v>74</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>287</v>
@@ -4912,21 +4912,21 @@
         <v>74</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B16" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>283</v>
@@ -4935,21 +4935,21 @@
         <v>74</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B17" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>287</v>
@@ -4958,13 +4958,13 @@
         <v>74</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -5001,22 +5001,22 @@
         <v>299</v>
       </c>
       <c r="G1" s="18" t="s">
+        <v>354</v>
+      </c>
+      <c r="H1" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="I1" s="18" t="s">
         <v>301</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="J1" s="18" t="s">
         <v>302</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="K1" s="18" t="s">
         <v>303</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="L1" s="18" t="s">
         <v>304</v>
-      </c>
-      <c r="L1" s="18" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -5039,7 +5039,7 @@
         <v>400</v>
       </c>
       <c r="G2" s="8">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="H2" s="8">
         <v>0</v>
@@ -5077,7 +5077,7 @@
         <v>280</v>
       </c>
       <c r="G3" s="8">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="H3" s="8">
         <v>0</v>
@@ -5115,7 +5115,7 @@
         <v>400</v>
       </c>
       <c r="G4" s="8">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="H4" s="8">
         <v>0</v>
@@ -5153,7 +5153,7 @@
         <v>300</v>
       </c>
       <c r="G5" s="8">
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="H5" s="8">
         <v>0</v>
@@ -5191,7 +5191,7 @@
         <v>340</v>
       </c>
       <c r="G6" s="8">
-        <v>1</v>
+        <v>95</v>
       </c>
       <c r="H6" s="8">
         <v>0</v>
@@ -5229,7 +5229,7 @@
         <v>325</v>
       </c>
       <c r="G7" s="8">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="H7" s="8">
         <v>20</v>
@@ -5267,7 +5267,7 @@
         <v>300</v>
       </c>
       <c r="G8" s="8">
-        <v>2</v>
+        <v>105</v>
       </c>
       <c r="H8" s="8">
         <v>0</v>
@@ -5305,7 +5305,7 @@
         <v>420</v>
       </c>
       <c r="G9" s="8">
-        <v>1</v>
+        <v>110</v>
       </c>
       <c r="H9" s="8">
         <v>0</v>
@@ -5343,7 +5343,7 @@
         <v>350</v>
       </c>
       <c r="G10" s="8">
-        <v>1</v>
+        <v>115</v>
       </c>
       <c r="H10" s="8">
         <v>0</v>
@@ -5381,7 +5381,7 @@
         <v>330</v>
       </c>
       <c r="G11" s="8">
-        <v>1</v>
+        <v>120</v>
       </c>
       <c r="H11" s="8">
         <v>0</v>
@@ -5401,7 +5401,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>285</v>
@@ -5419,7 +5419,7 @@
         <v>280</v>
       </c>
       <c r="G12" s="8">
-        <v>1</v>
+        <v>125</v>
       </c>
       <c r="H12" s="8">
         <v>0</v>
@@ -5439,7 +5439,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="24" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>283</v>
@@ -5457,7 +5457,7 @@
         <v>325</v>
       </c>
       <c r="G13" s="8">
-        <v>1</v>
+        <v>130</v>
       </c>
       <c r="H13" s="8">
         <v>20</v>
@@ -5477,7 +5477,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B14" s="16" t="s">
         <v>287</v>
@@ -5495,7 +5495,7 @@
         <v>325</v>
       </c>
       <c r="G14" s="8">
-        <v>1</v>
+        <v>135</v>
       </c>
       <c r="H14" s="8">
         <v>20</v>
@@ -5515,7 +5515,7 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B15" s="16" t="s">
         <v>287</v>
@@ -5533,7 +5533,7 @@
         <v>325</v>
       </c>
       <c r="G15" s="8">
-        <v>1</v>
+        <v>140</v>
       </c>
       <c r="H15" s="8">
         <v>20</v>
@@ -5553,7 +5553,7 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>283</v>
@@ -5571,7 +5571,7 @@
         <v>325</v>
       </c>
       <c r="G16" s="8">
-        <v>1</v>
+        <v>145</v>
       </c>
       <c r="H16" s="8">
         <v>20</v>
@@ -5591,7 +5591,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B17" s="16" t="s">
         <v>287</v>
@@ -5609,7 +5609,7 @@
         <v>325</v>
       </c>
       <c r="G17" s="8">
-        <v>1</v>
+        <v>150</v>
       </c>
       <c r="H17" s="8">
         <v>20</v>
@@ -5653,13 +5653,13 @@
         <v>68</v>
       </c>
       <c r="D1" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="E1" s="18" t="s">
         <v>307</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="F1" s="18" t="s">
         <v>308</v>
-      </c>
-      <c r="F1" s="18" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -5679,7 +5679,7 @@
         <v>69</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -5699,7 +5699,7 @@
         <v>69</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -5719,7 +5719,7 @@
         <v>69</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -5739,7 +5739,7 @@
         <v>69</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -5759,7 +5759,7 @@
         <v>69</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -5779,7 +5779,7 @@
         <v>69</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -5799,7 +5799,7 @@
         <v>69</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -5819,7 +5819,7 @@
         <v>69</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -5839,7 +5839,7 @@
         <v>69</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -5859,12 +5859,12 @@
         <v>69</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>285</v>
@@ -5879,12 +5879,12 @@
         <v>69</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="24" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>283</v>
@@ -5899,12 +5899,12 @@
         <v>69</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B14" s="16" t="s">
         <v>287</v>
@@ -5919,12 +5919,12 @@
         <v>69</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B15" s="16" t="s">
         <v>287</v>
@@ -5939,12 +5939,12 @@
         <v>69</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>283</v>
@@ -5959,12 +5959,12 @@
         <v>69</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B17" s="16" t="s">
         <v>287</v>
@@ -5979,7 +5979,7 @@
         <v>69</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>
@@ -6155,7 +6155,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B12" s="8">
         <v>175</v>
@@ -6169,7 +6169,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="24" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B13" s="8">
         <v>175</v>
@@ -6183,7 +6183,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B14" s="8">
         <v>175</v>
@@ -6197,7 +6197,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B15" s="8">
         <v>175</v>
@@ -6211,7 +6211,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B16" s="8">
         <v>175</v>
@@ -6225,7 +6225,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B17" s="8">
         <v>175</v>
@@ -6262,24 +6262,24 @@
         <v>1</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Config skill Data and handle damage in Skill Runtime
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -12,11 +12,12 @@
     <sheet name="Weapon" sheetId="2" r:id="rId3"/>
     <sheet name="Armor" sheetId="4" r:id="rId4"/>
     <sheet name="Character" sheetId="5" r:id="rId5"/>
-    <sheet name="CharacterStat" sheetId="6" r:id="rId6"/>
-    <sheet name="CharacterAttribute" sheetId="8" r:id="rId7"/>
-    <sheet name="CharacterUpgrade" sheetId="7" r:id="rId8"/>
-    <sheet name="BattleConfig" sheetId="9" r:id="rId9"/>
-    <sheet name="StageEnemies" sheetId="10" r:id="rId10"/>
+    <sheet name="SkillConfig" sheetId="11" r:id="rId6"/>
+    <sheet name="CharacterStat" sheetId="6" r:id="rId7"/>
+    <sheet name="CharacterAttribute" sheetId="8" r:id="rId8"/>
+    <sheet name="CharacterUpgrade" sheetId="7" r:id="rId9"/>
+    <sheet name="BattleConfig" sheetId="9" r:id="rId10"/>
+    <sheet name="StageEnemies" sheetId="10" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$111</definedName>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1085" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1166" uniqueCount="409">
   <si>
     <t>ID</t>
   </si>
@@ -1096,6 +1097,168 @@
   </si>
   <si>
     <t>speed</t>
+  </si>
+  <si>
+    <t>DamageMultiplier</t>
+  </si>
+  <si>
+    <t>SunWukong_B</t>
+  </si>
+  <si>
+    <t>SunWukong_M</t>
+  </si>
+  <si>
+    <t>SunWukong_U</t>
+  </si>
+  <si>
+    <t>TangSanZang_B</t>
+  </si>
+  <si>
+    <t>TangSanZang_M</t>
+  </si>
+  <si>
+    <t>TangSanZang_U</t>
+  </si>
+  <si>
+    <t>ZhuBaJie_B</t>
+  </si>
+  <si>
+    <t>ZhuBaJie_M</t>
+  </si>
+  <si>
+    <t>ZhuBaJie_U</t>
+  </si>
+  <si>
+    <t>ShaWujing_B</t>
+  </si>
+  <si>
+    <t>ShaWujing_M</t>
+  </si>
+  <si>
+    <t>ShaWujing_U</t>
+  </si>
+  <si>
+    <t>DragonKing_B</t>
+  </si>
+  <si>
+    <t>DragonKing_M</t>
+  </si>
+  <si>
+    <t>DragonKing_U</t>
+  </si>
+  <si>
+    <t>ThirdPrinceNezha_B</t>
+  </si>
+  <si>
+    <t>ThirdPrinceNezha_M</t>
+  </si>
+  <si>
+    <t>ThirdPrinceNezha_U</t>
+  </si>
+  <si>
+    <t>LittleWhiteDragon_B</t>
+  </si>
+  <si>
+    <t>LittleWhiteDragon_M</t>
+  </si>
+  <si>
+    <t>LittleWhiteDragon_U</t>
+  </si>
+  <si>
+    <t>ErlangShen_B</t>
+  </si>
+  <si>
+    <t>ErlangShen_M</t>
+  </si>
+  <si>
+    <t>Des</t>
+  </si>
+  <si>
+    <t>ErlangShen_U</t>
+  </si>
+  <si>
+    <t>BullDemonKing_B</t>
+  </si>
+  <si>
+    <t>BullDemonKing_M</t>
+  </si>
+  <si>
+    <t>BullDemonKing_U</t>
+  </si>
+  <si>
+    <t>GuanyinBodhisattva_B</t>
+  </si>
+  <si>
+    <t>GuanyinBodhisattva_M</t>
+  </si>
+  <si>
+    <t>GuanyinBodhisattva_U</t>
+  </si>
+  <si>
+    <t>VanguardTiger_B</t>
+  </si>
+  <si>
+    <t>TheBoySage_B</t>
+  </si>
+  <si>
+    <t>TheBoySage_M</t>
+  </si>
+  <si>
+    <t>TheBoySage_U</t>
+  </si>
+  <si>
+    <t>GoldHornKing_B</t>
+  </si>
+  <si>
+    <t>GoldHornKing_M</t>
+  </si>
+  <si>
+    <t>GoldHornKing_U</t>
+  </si>
+  <si>
+    <t>SilverHornKing_U</t>
+  </si>
+  <si>
+    <t>SilverHornKing_B</t>
+  </si>
+  <si>
+    <t>SilverHornKing_M</t>
+  </si>
+  <si>
+    <t>YellowWindMonster_B</t>
+  </si>
+  <si>
+    <t>YellowWindMonster_M</t>
+  </si>
+  <si>
+    <t>YellowWindMonster_U</t>
+  </si>
+  <si>
+    <t>GoldfishDemon_B</t>
+  </si>
+  <si>
+    <t>GoldfishDemon_M</t>
+  </si>
+  <si>
+    <t>GoldfishDemon_U</t>
+  </si>
+  <si>
+    <t>1.5</t>
+  </si>
+  <si>
+    <t>1.8</t>
+  </si>
+  <si>
+    <t>MaxCooldown</t>
+  </si>
+  <si>
+    <t>VanguardTiger</t>
+  </si>
+  <si>
+    <t>None_Skill</t>
+  </si>
+  <si>
+    <t>FlatDamage</t>
   </si>
 </sst>
 </file>
@@ -1221,7 +1384,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1279,6 +1442,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3639,7 +3812,52 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="B2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>329</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" customWidth="1"/>
@@ -3708,40 +3926,12 @@
         <v>324</v>
       </c>
       <c r="B5" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>334</v>
+        <v>318</v>
       </c>
       <c r="D5" s="7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>324</v>
-      </c>
-      <c r="B6" s="7">
-        <v>5</v>
-      </c>
-      <c r="C6" s="24" t="s">
-        <v>334</v>
-      </c>
-      <c r="D6" s="7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>324</v>
-      </c>
-      <c r="B7" s="7">
-        <v>6</v>
-      </c>
-      <c r="C7" s="24" t="s">
-        <v>334</v>
-      </c>
-      <c r="D7" s="7">
         <v>5</v>
       </c>
     </row>
@@ -4571,8 +4761,8 @@
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4612,14 +4802,17 @@
       <c r="D2" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="E2" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>338</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>344</v>
+      <c r="E2" s="8" t="str">
+        <f>A2&amp;"_B"</f>
+        <v>SunWukong_B</v>
+      </c>
+      <c r="F2" s="8" t="str">
+        <f>A2&amp;"_M"</f>
+        <v>SunWukong_M</v>
+      </c>
+      <c r="G2" s="8" t="str">
+        <f>A2&amp;"_U"</f>
+        <v>SunWukong_U</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -4635,14 +4828,17 @@
       <c r="D3" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E3" s="8" t="s">
-        <v>337</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>344</v>
+      <c r="E3" s="8" t="str">
+        <f t="shared" ref="E3:E17" si="0">A3&amp;"_B"</f>
+        <v>TangSanZang_B</v>
+      </c>
+      <c r="F3" s="8" t="str">
+        <f t="shared" ref="F3:F17" si="1">A3&amp;"_M"</f>
+        <v>TangSanZang_M</v>
+      </c>
+      <c r="G3" s="8" t="str">
+        <f t="shared" ref="G3:G17" si="2">A3&amp;"_U"</f>
+        <v>TangSanZang_U</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -4658,14 +4854,17 @@
       <c r="D4" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>344</v>
+      <c r="E4" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>ZhuBaJie_B</v>
+      </c>
+      <c r="F4" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>ZhuBaJie_M</v>
+      </c>
+      <c r="G4" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>ZhuBaJie_U</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -4681,14 +4880,17 @@
       <c r="D5" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="E5" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>340</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>344</v>
+      <c r="E5" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>ShaWujing_B</v>
+      </c>
+      <c r="F5" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>ShaWujing_M</v>
+      </c>
+      <c r="G5" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>ShaWujing_U</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -4704,14 +4906,17 @@
       <c r="D6" s="27" t="s">
         <v>78</v>
       </c>
-      <c r="E6" s="27" t="s">
-        <v>336</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>352</v>
-      </c>
-      <c r="G6" s="27" t="s">
-        <v>352</v>
+      <c r="E6" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>DragonKing_B</v>
+      </c>
+      <c r="F6" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>DragonKing_M</v>
+      </c>
+      <c r="G6" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>DragonKing_U</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -4727,14 +4932,17 @@
       <c r="D7" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E7" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>342</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>344</v>
+      <c r="E7" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>ThirdPrinceNezha_B</v>
+      </c>
+      <c r="F7" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>ThirdPrinceNezha_M</v>
+      </c>
+      <c r="G7" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>ThirdPrinceNezha_U</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -4750,14 +4958,17 @@
       <c r="D8" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>344</v>
+      <c r="E8" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>LittleWhiteDragon_B</v>
+      </c>
+      <c r="F8" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>LittleWhiteDragon_M</v>
+      </c>
+      <c r="G8" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>LittleWhiteDragon_U</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -4773,14 +4984,17 @@
       <c r="D9" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E9" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>347</v>
+      <c r="E9" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>BullDemonKing_B</v>
+      </c>
+      <c r="F9" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>BullDemonKing_M</v>
+      </c>
+      <c r="G9" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>BullDemonKing_U</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -4796,14 +5010,17 @@
       <c r="D10" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="E10" s="27" t="s">
-        <v>336</v>
-      </c>
-      <c r="F10" s="27" t="s">
-        <v>352</v>
-      </c>
-      <c r="G10" s="27" t="s">
-        <v>352</v>
+      <c r="E10" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>ErlangShen_B</v>
+      </c>
+      <c r="F10" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>ErlangShen_M</v>
+      </c>
+      <c r="G10" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>ErlangShen_U</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -4819,19 +5036,22 @@
       <c r="D11" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="E11" s="27" t="s">
-        <v>337</v>
-      </c>
-      <c r="F11" s="27" t="s">
-        <v>352</v>
-      </c>
-      <c r="G11" s="27" t="s">
-        <v>352</v>
+      <c r="E11" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>GuanyinBodhisattva_B</v>
+      </c>
+      <c r="F11" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>GuanyinBodhisattva_M</v>
+      </c>
+      <c r="G11" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>GuanyinBodhisattva_U</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="24" t="s">
-        <v>334</v>
+      <c r="A12" s="13" t="s">
+        <v>406</v>
       </c>
       <c r="B12" t="s">
         <v>335</v>
@@ -4842,14 +5062,15 @@
       <c r="D12" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E12" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>352</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>352</v>
+      <c r="E12" s="8" t="str">
+        <f>A12&amp;"_B"</f>
+        <v>VanguardTiger_B</v>
+      </c>
+      <c r="F12" s="29" t="s">
+        <v>407</v>
+      </c>
+      <c r="G12" s="29" t="s">
+        <v>407</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -4865,14 +5086,17 @@
       <c r="D13" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E13" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>343</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>344</v>
+      <c r="E13" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>TheBoySage_B</v>
+      </c>
+      <c r="F13" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>TheBoySage_M</v>
+      </c>
+      <c r="G13" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>TheBoySage_U</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -4888,14 +5112,17 @@
       <c r="D14" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E14" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>353</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>344</v>
+      <c r="E14" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>GoldHornKing_B</v>
+      </c>
+      <c r="F14" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>GoldHornKing_M</v>
+      </c>
+      <c r="G14" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>GoldHornKing_U</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -4911,14 +5138,17 @@
       <c r="D15" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E15" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>345</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>344</v>
+      <c r="E15" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>SilverHornKing_B</v>
+      </c>
+      <c r="F15" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>SilverHornKing_M</v>
+      </c>
+      <c r="G15" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>SilverHornKing_U</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -4934,14 +5164,17 @@
       <c r="D16" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E16" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>346</v>
-      </c>
-      <c r="G16" s="8" t="s">
-        <v>348</v>
+      <c r="E16" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>YellowWindMonster_B</v>
+      </c>
+      <c r="F16" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>YellowWindMonster_M</v>
+      </c>
+      <c r="G16" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>YellowWindMonster_U</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -4957,14 +5190,17 @@
       <c r="D17" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E17" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>353</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>344</v>
+      <c r="E17" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>GoldfishDemon_B</v>
+      </c>
+      <c r="F17" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>GoldfishDemon_M</v>
+      </c>
+      <c r="G17" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>GoldfishDemon_U</v>
       </c>
     </row>
   </sheetData>
@@ -4973,6 +5209,1224 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G48"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.85546875" customWidth="1"/>
+    <col min="2" max="2" width="29" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" customWidth="1"/>
+    <col min="6" max="6" width="23.42578125" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>379</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>405</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>356</v>
+      </c>
+      <c r="B2" t="str">
+        <f>A2&amp;"_Name"</f>
+        <v>SunWukong_B_Name</v>
+      </c>
+      <c r="C2" t="str">
+        <f>A2&amp;"_Des"</f>
+        <v>SunWukong_B_Des</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="E2" s="8">
+        <v>1</v>
+      </c>
+      <c r="F2" s="8">
+        <v>0</v>
+      </c>
+      <c r="G2" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>357</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" ref="B3:B48" si="0">A3&amp;"_Name"</f>
+        <v>SunWukong_M_Name</v>
+      </c>
+      <c r="C3" t="str">
+        <f t="shared" ref="C3:C48" si="1">A3&amp;"_Des"</f>
+        <v>SunWukong_M_Des</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F3" s="8">
+        <v>4</v>
+      </c>
+      <c r="G3" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>358</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>SunWukong_U_Name</v>
+      </c>
+      <c r="C4" t="str">
+        <f t="shared" si="1"/>
+        <v>SunWukong_U_Des</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F4" s="8">
+        <v>5</v>
+      </c>
+      <c r="G4" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>359</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>TangSanZang_B_Name</v>
+      </c>
+      <c r="C5" t="str">
+        <f t="shared" si="1"/>
+        <v>TangSanZang_B_Des</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="E5" s="8">
+        <v>1</v>
+      </c>
+      <c r="F5" s="8">
+        <v>0</v>
+      </c>
+      <c r="G5" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>360</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>TangSanZang_M_Name</v>
+      </c>
+      <c r="C6" t="str">
+        <f t="shared" si="1"/>
+        <v>TangSanZang_M_Des</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F6" s="8">
+        <v>4</v>
+      </c>
+      <c r="G6" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>361</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>TangSanZang_U_Name</v>
+      </c>
+      <c r="C7" t="str">
+        <f t="shared" si="1"/>
+        <v>TangSanZang_U_Des</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F7" s="8">
+        <v>5</v>
+      </c>
+      <c r="G7" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>362</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>ZhuBaJie_B_Name</v>
+      </c>
+      <c r="C8" t="str">
+        <f t="shared" si="1"/>
+        <v>ZhuBaJie_B_Des</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="E8" s="8">
+        <v>1</v>
+      </c>
+      <c r="F8" s="8">
+        <v>0</v>
+      </c>
+      <c r="G8" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>363</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>ZhuBaJie_M_Name</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="1"/>
+        <v>ZhuBaJie_M_Des</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F9" s="8">
+        <v>4</v>
+      </c>
+      <c r="G9" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>364</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>ZhuBaJie_U_Name</v>
+      </c>
+      <c r="C10" t="str">
+        <f t="shared" si="1"/>
+        <v>ZhuBaJie_U_Des</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F10" s="8">
+        <v>5</v>
+      </c>
+      <c r="G10" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>ShaWujing_B_Name</v>
+      </c>
+      <c r="C11" t="str">
+        <f t="shared" si="1"/>
+        <v>ShaWujing_B_Des</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="E11" s="8">
+        <v>1</v>
+      </c>
+      <c r="F11" s="8">
+        <v>0</v>
+      </c>
+      <c r="G11" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>ShaWujing_M_Name</v>
+      </c>
+      <c r="C12" t="str">
+        <f t="shared" si="1"/>
+        <v>ShaWujing_M_Des</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F12" s="8">
+        <v>4</v>
+      </c>
+      <c r="G12" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>ShaWujing_U_Name</v>
+      </c>
+      <c r="C13" t="str">
+        <f t="shared" si="1"/>
+        <v>ShaWujing_U_Des</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F13" s="8">
+        <v>5</v>
+      </c>
+      <c r="G13" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="25" t="s">
+        <v>368</v>
+      </c>
+      <c r="B14" t="str">
+        <f t="shared" si="0"/>
+        <v>DragonKing_B_Name</v>
+      </c>
+      <c r="C14" t="str">
+        <f t="shared" si="1"/>
+        <v>DragonKing_B_Des</v>
+      </c>
+      <c r="D14" s="27" t="s">
+        <v>336</v>
+      </c>
+      <c r="E14" s="8">
+        <v>1</v>
+      </c>
+      <c r="F14" s="8">
+        <v>0</v>
+      </c>
+      <c r="G14" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="25" t="s">
+        <v>369</v>
+      </c>
+      <c r="B15" t="str">
+        <f t="shared" si="0"/>
+        <v>DragonKing_M_Name</v>
+      </c>
+      <c r="C15" t="str">
+        <f t="shared" si="1"/>
+        <v>DragonKing_M_Des</v>
+      </c>
+      <c r="D15" s="27" t="s">
+        <v>352</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F15" s="8">
+        <v>4</v>
+      </c>
+      <c r="G15" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="25" t="s">
+        <v>370</v>
+      </c>
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>DragonKing_U_Name</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="1"/>
+        <v>DragonKing_U_Des</v>
+      </c>
+      <c r="D16" s="27" t="s">
+        <v>352</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F16" s="8">
+        <v>5</v>
+      </c>
+      <c r="G16" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>371</v>
+      </c>
+      <c r="B17" t="str">
+        <f t="shared" si="0"/>
+        <v>ThirdPrinceNezha_B_Name</v>
+      </c>
+      <c r="C17" t="str">
+        <f t="shared" si="1"/>
+        <v>ThirdPrinceNezha_B_Des</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="E17" s="8">
+        <v>1</v>
+      </c>
+      <c r="F17" s="8">
+        <v>0</v>
+      </c>
+      <c r="G17" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>372</v>
+      </c>
+      <c r="B18" t="str">
+        <f t="shared" si="0"/>
+        <v>ThirdPrinceNezha_M_Name</v>
+      </c>
+      <c r="C18" t="str">
+        <f t="shared" si="1"/>
+        <v>ThirdPrinceNezha_M_Des</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F18" s="8">
+        <v>4</v>
+      </c>
+      <c r="G18" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>373</v>
+      </c>
+      <c r="B19" t="str">
+        <f t="shared" si="0"/>
+        <v>ThirdPrinceNezha_U_Name</v>
+      </c>
+      <c r="C19" t="str">
+        <f t="shared" si="1"/>
+        <v>ThirdPrinceNezha_U_Des</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F19" s="8">
+        <v>5</v>
+      </c>
+      <c r="G19" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>374</v>
+      </c>
+      <c r="B20" t="str">
+        <f t="shared" si="0"/>
+        <v>LittleWhiteDragon_B_Name</v>
+      </c>
+      <c r="C20" t="str">
+        <f t="shared" si="1"/>
+        <v>LittleWhiteDragon_B_Des</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="E20" s="8">
+        <v>1</v>
+      </c>
+      <c r="F20" s="8">
+        <v>0</v>
+      </c>
+      <c r="G20" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="B21" t="str">
+        <f t="shared" si="0"/>
+        <v>LittleWhiteDragon_M_Name</v>
+      </c>
+      <c r="C21" t="str">
+        <f t="shared" si="1"/>
+        <v>LittleWhiteDragon_M_Des</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F21" s="8">
+        <v>4</v>
+      </c>
+      <c r="G21" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>376</v>
+      </c>
+      <c r="B22" t="str">
+        <f t="shared" si="0"/>
+        <v>LittleWhiteDragon_U_Name</v>
+      </c>
+      <c r="C22" t="str">
+        <f t="shared" si="1"/>
+        <v>LittleWhiteDragon_U_Des</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F22" s="8">
+        <v>5</v>
+      </c>
+      <c r="G22" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>381</v>
+      </c>
+      <c r="B23" t="str">
+        <f t="shared" si="0"/>
+        <v>BullDemonKing_B_Name</v>
+      </c>
+      <c r="C23" t="str">
+        <f t="shared" si="1"/>
+        <v>BullDemonKing_B_Des</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="E23" s="8">
+        <v>1</v>
+      </c>
+      <c r="F23" s="8">
+        <v>0</v>
+      </c>
+      <c r="G23" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>382</v>
+      </c>
+      <c r="B24" t="str">
+        <f t="shared" si="0"/>
+        <v>BullDemonKing_M_Name</v>
+      </c>
+      <c r="C24" t="str">
+        <f t="shared" si="1"/>
+        <v>BullDemonKing_M_Des</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F24" s="8">
+        <v>4</v>
+      </c>
+      <c r="G24" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>383</v>
+      </c>
+      <c r="B25" t="str">
+        <f t="shared" si="0"/>
+        <v>BullDemonKing_U_Name</v>
+      </c>
+      <c r="C25" t="str">
+        <f t="shared" si="1"/>
+        <v>BullDemonKing_U_Des</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F25" s="8">
+        <v>5</v>
+      </c>
+      <c r="G25" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="25" t="s">
+        <v>377</v>
+      </c>
+      <c r="B26" t="str">
+        <f t="shared" si="0"/>
+        <v>ErlangShen_B_Name</v>
+      </c>
+      <c r="C26" t="str">
+        <f t="shared" si="1"/>
+        <v>ErlangShen_B_Des</v>
+      </c>
+      <c r="D26" s="27" t="s">
+        <v>336</v>
+      </c>
+      <c r="E26" s="8">
+        <v>1</v>
+      </c>
+      <c r="F26" s="8">
+        <v>0</v>
+      </c>
+      <c r="G26" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="25" t="s">
+        <v>378</v>
+      </c>
+      <c r="B27" t="str">
+        <f t="shared" si="0"/>
+        <v>ErlangShen_M_Name</v>
+      </c>
+      <c r="C27" t="str">
+        <f t="shared" si="1"/>
+        <v>ErlangShen_M_Des</v>
+      </c>
+      <c r="D27" s="27" t="s">
+        <v>352</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F27" s="8">
+        <v>4</v>
+      </c>
+      <c r="G27" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="25" t="s">
+        <v>380</v>
+      </c>
+      <c r="B28" t="str">
+        <f t="shared" si="0"/>
+        <v>ErlangShen_U_Name</v>
+      </c>
+      <c r="C28" t="str">
+        <f t="shared" si="1"/>
+        <v>ErlangShen_U_Des</v>
+      </c>
+      <c r="D28" s="27" t="s">
+        <v>352</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F28" s="8">
+        <v>5</v>
+      </c>
+      <c r="G28" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="25" t="s">
+        <v>384</v>
+      </c>
+      <c r="B29" t="str">
+        <f t="shared" si="0"/>
+        <v>GuanyinBodhisattva_B_Name</v>
+      </c>
+      <c r="C29" t="str">
+        <f t="shared" si="1"/>
+        <v>GuanyinBodhisattva_B_Des</v>
+      </c>
+      <c r="D29" s="27" t="s">
+        <v>337</v>
+      </c>
+      <c r="E29" s="8">
+        <v>1</v>
+      </c>
+      <c r="F29" s="8">
+        <v>0</v>
+      </c>
+      <c r="G29" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="25" t="s">
+        <v>385</v>
+      </c>
+      <c r="B30" t="str">
+        <f t="shared" si="0"/>
+        <v>GuanyinBodhisattva_M_Name</v>
+      </c>
+      <c r="C30" t="str">
+        <f t="shared" si="1"/>
+        <v>GuanyinBodhisattva_M_Des</v>
+      </c>
+      <c r="D30" s="27" t="s">
+        <v>352</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F30" s="8">
+        <v>4</v>
+      </c>
+      <c r="G30" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="25" t="s">
+        <v>386</v>
+      </c>
+      <c r="B31" t="str">
+        <f t="shared" si="0"/>
+        <v>GuanyinBodhisattva_U_Name</v>
+      </c>
+      <c r="C31" t="str">
+        <f t="shared" si="1"/>
+        <v>GuanyinBodhisattva_U_Des</v>
+      </c>
+      <c r="D31" s="27" t="s">
+        <v>352</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F31" s="8">
+        <v>5</v>
+      </c>
+      <c r="G31" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="13" t="s">
+        <v>387</v>
+      </c>
+      <c r="B32" t="str">
+        <f t="shared" si="0"/>
+        <v>VanguardTiger_B_Name</v>
+      </c>
+      <c r="C32" t="str">
+        <f t="shared" si="1"/>
+        <v>VanguardTiger_B_Des</v>
+      </c>
+      <c r="D32" s="30" t="s">
+        <v>336</v>
+      </c>
+      <c r="E32" s="8">
+        <v>1</v>
+      </c>
+      <c r="F32" s="8">
+        <v>0</v>
+      </c>
+      <c r="G32" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="B33" t="str">
+        <f t="shared" si="0"/>
+        <v>TheBoySage_B_Name</v>
+      </c>
+      <c r="C33" t="str">
+        <f t="shared" si="1"/>
+        <v>TheBoySage_B_Des</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="E33" s="8">
+        <v>1</v>
+      </c>
+      <c r="F33" s="8">
+        <v>0</v>
+      </c>
+      <c r="G33" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="B34" t="str">
+        <f t="shared" si="0"/>
+        <v>TheBoySage_M_Name</v>
+      </c>
+      <c r="C34" t="str">
+        <f t="shared" si="1"/>
+        <v>TheBoySage_M_Des</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F34" s="8">
+        <v>4</v>
+      </c>
+      <c r="G34" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="s">
+        <v>390</v>
+      </c>
+      <c r="B35" t="str">
+        <f t="shared" si="0"/>
+        <v>TheBoySage_U_Name</v>
+      </c>
+      <c r="C35" t="str">
+        <f t="shared" si="1"/>
+        <v>TheBoySage_U_Des</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F35" s="8">
+        <v>5</v>
+      </c>
+      <c r="G35" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>391</v>
+      </c>
+      <c r="B36" t="str">
+        <f t="shared" si="0"/>
+        <v>GoldHornKing_B_Name</v>
+      </c>
+      <c r="C36" t="str">
+        <f t="shared" si="1"/>
+        <v>GoldHornKing_B_Des</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="E36" s="8">
+        <v>1</v>
+      </c>
+      <c r="F36" s="8">
+        <v>0</v>
+      </c>
+      <c r="G36" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>392</v>
+      </c>
+      <c r="B37" t="str">
+        <f t="shared" si="0"/>
+        <v>GoldHornKing_M_Name</v>
+      </c>
+      <c r="C37" t="str">
+        <f t="shared" si="1"/>
+        <v>GoldHornKing_M_Des</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>353</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F37" s="8">
+        <v>4</v>
+      </c>
+      <c r="G37" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>393</v>
+      </c>
+      <c r="B38" t="str">
+        <f t="shared" si="0"/>
+        <v>GoldHornKing_U_Name</v>
+      </c>
+      <c r="C38" t="str">
+        <f t="shared" si="1"/>
+        <v>GoldHornKing_U_Des</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F38" s="8">
+        <v>5</v>
+      </c>
+      <c r="G38" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="12" t="s">
+        <v>395</v>
+      </c>
+      <c r="B39" t="str">
+        <f t="shared" si="0"/>
+        <v>SilverHornKing_B_Name</v>
+      </c>
+      <c r="C39" t="str">
+        <f t="shared" si="1"/>
+        <v>SilverHornKing_B_Des</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="E39" s="8">
+        <v>1</v>
+      </c>
+      <c r="F39" s="8">
+        <v>0</v>
+      </c>
+      <c r="G39" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="12" t="s">
+        <v>396</v>
+      </c>
+      <c r="B40" t="str">
+        <f t="shared" si="0"/>
+        <v>SilverHornKing_M_Name</v>
+      </c>
+      <c r="C40" t="str">
+        <f t="shared" si="1"/>
+        <v>SilverHornKing_M_Des</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F40" s="8">
+        <v>4</v>
+      </c>
+      <c r="G40" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="12" t="s">
+        <v>394</v>
+      </c>
+      <c r="B41" t="str">
+        <f t="shared" si="0"/>
+        <v>SilverHornKing_U_Name</v>
+      </c>
+      <c r="C41" t="str">
+        <f t="shared" si="1"/>
+        <v>SilverHornKing_U_Des</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F41" s="8">
+        <v>5</v>
+      </c>
+      <c r="G41" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="28" t="s">
+        <v>397</v>
+      </c>
+      <c r="B42" t="str">
+        <f t="shared" si="0"/>
+        <v>YellowWindMonster_B_Name</v>
+      </c>
+      <c r="C42" t="str">
+        <f t="shared" si="1"/>
+        <v>YellowWindMonster_B_Des</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="E42" s="8">
+        <v>1</v>
+      </c>
+      <c r="F42" s="8">
+        <v>0</v>
+      </c>
+      <c r="G42" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="28" t="s">
+        <v>398</v>
+      </c>
+      <c r="B43" t="str">
+        <f t="shared" si="0"/>
+        <v>YellowWindMonster_M_Name</v>
+      </c>
+      <c r="C43" t="str">
+        <f t="shared" si="1"/>
+        <v>YellowWindMonster_M_Des</v>
+      </c>
+      <c r="D43" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F43" s="8">
+        <v>4</v>
+      </c>
+      <c r="G43" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="28" t="s">
+        <v>399</v>
+      </c>
+      <c r="B44" t="str">
+        <f t="shared" si="0"/>
+        <v>YellowWindMonster_U_Name</v>
+      </c>
+      <c r="C44" t="str">
+        <f t="shared" si="1"/>
+        <v>YellowWindMonster_U_Des</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F44" s="8">
+        <v>5</v>
+      </c>
+      <c r="G44" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="12" t="s">
+        <v>400</v>
+      </c>
+      <c r="B45" t="str">
+        <f t="shared" si="0"/>
+        <v>GoldfishDemon_B_Name</v>
+      </c>
+      <c r="C45" t="str">
+        <f t="shared" si="1"/>
+        <v>GoldfishDemon_B_Des</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="E45" s="8">
+        <v>1</v>
+      </c>
+      <c r="F45" s="8">
+        <v>0</v>
+      </c>
+      <c r="G45" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="12" t="s">
+        <v>401</v>
+      </c>
+      <c r="B46" t="str">
+        <f t="shared" si="0"/>
+        <v>GoldfishDemon_M_Name</v>
+      </c>
+      <c r="C46" t="str">
+        <f t="shared" si="1"/>
+        <v>GoldfishDemon_M_Des</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="F46" s="8">
+        <v>4</v>
+      </c>
+      <c r="G46" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="12" t="s">
+        <v>402</v>
+      </c>
+      <c r="B47" t="str">
+        <f t="shared" si="0"/>
+        <v>GoldfishDemon_U_Name</v>
+      </c>
+      <c r="C47" t="str">
+        <f t="shared" si="1"/>
+        <v>GoldfishDemon_U_Des</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="E47" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="F47" s="8">
+        <v>5</v>
+      </c>
+      <c r="G47" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="31" t="s">
+        <v>407</v>
+      </c>
+      <c r="B48" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>None_Skill_Name</v>
+      </c>
+      <c r="C48" s="8" t="str">
+        <f t="shared" si="1"/>
+        <v>None_Skill_Des</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>352</v>
+      </c>
+      <c r="E48" s="8">
+        <v>0</v>
+      </c>
+      <c r="F48" s="8">
+        <v>0</v>
+      </c>
+      <c r="G48" s="8">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5229,7 +6683,7 @@
         <v>325</v>
       </c>
       <c r="G7" s="8">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="H7" s="8">
         <v>20</v>
@@ -5267,7 +6721,7 @@
         <v>300</v>
       </c>
       <c r="G8" s="8">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="H8" s="8">
         <v>0</v>
@@ -5305,7 +6759,7 @@
         <v>420</v>
       </c>
       <c r="G9" s="8">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="H9" s="8">
         <v>0</v>
@@ -5343,7 +6797,7 @@
         <v>350</v>
       </c>
       <c r="G10" s="8">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="H10" s="8">
         <v>0</v>
@@ -5381,7 +6835,7 @@
         <v>330</v>
       </c>
       <c r="G11" s="8">
-        <v>120</v>
+        <v>95</v>
       </c>
       <c r="H11" s="8">
         <v>0</v>
@@ -5419,7 +6873,7 @@
         <v>280</v>
       </c>
       <c r="G12" s="8">
-        <v>125</v>
+        <v>70</v>
       </c>
       <c r="H12" s="8">
         <v>0</v>
@@ -5457,7 +6911,7 @@
         <v>325</v>
       </c>
       <c r="G13" s="8">
-        <v>130</v>
+        <v>80</v>
       </c>
       <c r="H13" s="8">
         <v>20</v>
@@ -5495,7 +6949,7 @@
         <v>325</v>
       </c>
       <c r="G14" s="8">
-        <v>135</v>
+        <v>80</v>
       </c>
       <c r="H14" s="8">
         <v>20</v>
@@ -5533,7 +6987,7 @@
         <v>325</v>
       </c>
       <c r="G15" s="8">
-        <v>140</v>
+        <v>80</v>
       </c>
       <c r="H15" s="8">
         <v>20</v>
@@ -5562,7 +7016,7 @@
         <v>74</v>
       </c>
       <c r="D16" s="8">
-        <v>6000</v>
+        <v>3900</v>
       </c>
       <c r="E16" s="8">
         <v>2400</v>
@@ -5571,7 +7025,7 @@
         <v>325</v>
       </c>
       <c r="G16" s="8">
-        <v>145</v>
+        <v>80</v>
       </c>
       <c r="H16" s="8">
         <v>20</v>
@@ -5609,7 +7063,7 @@
         <v>325</v>
       </c>
       <c r="G17" s="8">
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="H17" s="8">
         <v>20</v>
@@ -5632,7 +7086,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5988,7 +7442,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6240,49 +7694,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" customWidth="1"/>
-    <col min="3" max="3" width="21.28515625" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" customWidth="1"/>
-    <col min="5" max="5" width="23.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="D1" s="18" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>324</v>
-      </c>
-      <c r="B2" t="s">
-        <v>327</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>326</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>329</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
+ Make Target System for Action State.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="1" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="2" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1166" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1214" uniqueCount="412">
   <si>
     <t>ID</t>
   </si>
@@ -1259,6 +1259,15 @@
   </si>
   <si>
     <t>FlatDamage</t>
+  </si>
+  <si>
+    <t>TargetType</t>
+  </si>
+  <si>
+    <t>SingleEnemy</t>
+  </si>
+  <si>
+    <t>Selft</t>
   </si>
 </sst>
 </file>
@@ -5210,7 +5219,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" customWidth="1"/>
@@ -5220,9 +5229,10 @@
     <col min="5" max="5" width="17.7109375" customWidth="1"/>
     <col min="6" max="6" width="23.42578125" customWidth="1"/>
     <col min="7" max="7" width="16.85546875" customWidth="1"/>
+    <col min="8" max="8" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
@@ -5244,8 +5254,11 @@
       <c r="G1" s="18" t="s">
         <v>408</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="18" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>356</v>
       </c>
@@ -5269,8 +5282,11 @@
       <c r="G2" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>357</v>
       </c>
@@ -5294,8 +5310,11 @@
       <c r="G3" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>358</v>
       </c>
@@ -5319,8 +5338,11 @@
       <c r="G4" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>359</v>
       </c>
@@ -5344,8 +5366,11 @@
       <c r="G5" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
         <v>360</v>
       </c>
@@ -5369,8 +5394,11 @@
       <c r="G6" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H6" s="8" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
         <v>361</v>
       </c>
@@ -5394,8 +5422,11 @@
       <c r="G7" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H7" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>362</v>
       </c>
@@ -5419,8 +5450,11 @@
       <c r="G8" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H8" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>363</v>
       </c>
@@ -5444,8 +5478,11 @@
       <c r="G9" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H9" s="8" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>364</v>
       </c>
@@ -5469,8 +5506,11 @@
       <c r="G10" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H10" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
         <v>365</v>
       </c>
@@ -5494,8 +5534,11 @@
       <c r="G11" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H11" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>366</v>
       </c>
@@ -5519,8 +5562,11 @@
       <c r="G12" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H12" s="8" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
         <v>367</v>
       </c>
@@ -5544,8 +5590,11 @@
       <c r="G13" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H13" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
         <v>368</v>
       </c>
@@ -5569,8 +5618,11 @@
       <c r="G14" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H14" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="25" t="s">
         <v>369</v>
       </c>
@@ -5594,8 +5646,11 @@
       <c r="G15" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H15" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="25" t="s">
         <v>370</v>
       </c>
@@ -5619,8 +5674,11 @@
       <c r="G16" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H16" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>371</v>
       </c>
@@ -5644,8 +5702,11 @@
       <c r="G17" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H17" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>372</v>
       </c>
@@ -5669,8 +5730,11 @@
       <c r="G18" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H18" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>373</v>
       </c>
@@ -5694,8 +5758,11 @@
       <c r="G19" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H19" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
         <v>374</v>
       </c>
@@ -5719,8 +5786,11 @@
       <c r="G20" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H20" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
         <v>375</v>
       </c>
@@ -5744,8 +5814,11 @@
       <c r="G21" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H21" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
         <v>376</v>
       </c>
@@ -5769,8 +5842,11 @@
       <c r="G22" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H22" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>381</v>
       </c>
@@ -5794,8 +5870,11 @@
       <c r="G23" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H23" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>382</v>
       </c>
@@ -5819,8 +5898,11 @@
       <c r="G24" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H24" s="8" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>383</v>
       </c>
@@ -5844,8 +5926,11 @@
       <c r="G25" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H25" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
         <v>377</v>
       </c>
@@ -5869,8 +5954,11 @@
       <c r="G26" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H26" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="25" t="s">
         <v>378</v>
       </c>
@@ -5894,8 +5982,11 @@
       <c r="G27" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H27" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="25" t="s">
         <v>380</v>
       </c>
@@ -5919,8 +6010,11 @@
       <c r="G28" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H28" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="25" t="s">
         <v>384</v>
       </c>
@@ -5944,8 +6038,11 @@
       <c r="G29" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H29" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="25" t="s">
         <v>385</v>
       </c>
@@ -5969,8 +6066,11 @@
       <c r="G30" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H30" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="25" t="s">
         <v>386</v>
       </c>
@@ -5994,8 +6094,11 @@
       <c r="G31" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H31" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
         <v>387</v>
       </c>
@@ -6019,8 +6122,11 @@
       <c r="G32" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H32" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
         <v>388</v>
       </c>
@@ -6044,8 +6150,11 @@
       <c r="G33" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H33" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
         <v>389</v>
       </c>
@@ -6069,8 +6178,11 @@
       <c r="G34" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H34" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
         <v>390</v>
       </c>
@@ -6094,8 +6206,11 @@
       <c r="G35" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H35" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>391</v>
       </c>
@@ -6119,8 +6234,11 @@
       <c r="G36" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H36" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>392</v>
       </c>
@@ -6144,8 +6262,11 @@
       <c r="G37" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H37" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>393</v>
       </c>
@@ -6169,8 +6290,11 @@
       <c r="G38" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H38" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
         <v>395</v>
       </c>
@@ -6194,8 +6318,11 @@
       <c r="G39" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H39" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
         <v>396</v>
       </c>
@@ -6219,8 +6346,11 @@
       <c r="G40" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H40" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
         <v>394</v>
       </c>
@@ -6244,8 +6374,11 @@
       <c r="G41" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H41" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="28" t="s">
         <v>397</v>
       </c>
@@ -6269,8 +6402,11 @@
       <c r="G42" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H42" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="28" t="s">
         <v>398</v>
       </c>
@@ -6294,8 +6430,11 @@
       <c r="G43" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H43" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="28" t="s">
         <v>399</v>
       </c>
@@ -6319,8 +6458,11 @@
       <c r="G44" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H44" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
         <v>400</v>
       </c>
@@ -6344,8 +6486,11 @@
       <c r="G45" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H45" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="12" t="s">
         <v>401</v>
       </c>
@@ -6369,8 +6514,11 @@
       <c r="G46" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H46" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="12" t="s">
         <v>402</v>
       </c>
@@ -6394,8 +6542,11 @@
       <c r="G47" s="8">
         <v>100</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H47" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>407</v>
       </c>
@@ -6418,6 +6569,9 @@
       </c>
       <c r="G48" s="8">
         <v>100</v>
+      </c>
+      <c r="H48" s="8" t="s">
+        <v>410</v>
       </c>
     </row>
   </sheetData>
@@ -6531,7 +6685,7 @@
         <v>280</v>
       </c>
       <c r="G3" s="8">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="H3" s="8">
         <v>0</v>

</xml_diff>

<commit_message>
+ Update health bar to calculate hp and shield. And make skill AOE or Single target.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1214" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="413">
   <si>
     <t>ID</t>
   </si>
@@ -1267,7 +1267,10 @@
     <t>SingleEnemy</t>
   </si>
   <si>
-    <t>Selft</t>
+    <t>Self</t>
+  </si>
+  <si>
+    <t>AllEnemies</t>
   </si>
 </sst>
 </file>
@@ -5301,8 +5304,8 @@
       <c r="D3" s="8" t="s">
         <v>338</v>
       </c>
-      <c r="E3" s="8" t="s">
-        <v>403</v>
+      <c r="E3" s="8">
+        <v>1</v>
       </c>
       <c r="F3" s="8">
         <v>4</v>
@@ -5311,7 +5314,7 @@
         <v>100</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -6647,7 +6650,7 @@
         <v>400</v>
       </c>
       <c r="G2" s="8">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="H2" s="8">
         <v>0</v>
@@ -6685,7 +6688,7 @@
         <v>280</v>
       </c>
       <c r="G3" s="8">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="H3" s="8">
         <v>0</v>

</xml_diff>

<commit_message>
+ Config skill effect and make factory effect skill
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -13,11 +13,12 @@
     <sheet name="Armor" sheetId="4" r:id="rId4"/>
     <sheet name="Character" sheetId="5" r:id="rId5"/>
     <sheet name="SkillConfig" sheetId="11" r:id="rId6"/>
-    <sheet name="CharacterStat" sheetId="6" r:id="rId7"/>
-    <sheet name="CharacterAttribute" sheetId="8" r:id="rId8"/>
-    <sheet name="CharacterUpgrade" sheetId="7" r:id="rId9"/>
-    <sheet name="BattleConfig" sheetId="9" r:id="rId10"/>
-    <sheet name="StageEnemies" sheetId="10" r:id="rId11"/>
+    <sheet name="EffectConfig" sheetId="12" r:id="rId7"/>
+    <sheet name="CharacterStat" sheetId="6" r:id="rId8"/>
+    <sheet name="CharacterAttribute" sheetId="8" r:id="rId9"/>
+    <sheet name="CharacterUpgrade" sheetId="7" r:id="rId10"/>
+    <sheet name="BattleConfig" sheetId="9" r:id="rId11"/>
+    <sheet name="StageEnemies" sheetId="10" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$111</definedName>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1312" uniqueCount="449">
   <si>
     <t>ID</t>
   </si>
@@ -1009,9 +1010,6 @@
     <t>Tutorial_Default</t>
   </si>
   <si>
-    <t>BackGrouind</t>
-  </si>
-  <si>
     <t>Default</t>
   </si>
   <si>
@@ -1075,9 +1073,6 @@
     <t>Suriken</t>
   </si>
   <si>
-    <t>PosionBall</t>
-  </si>
-  <si>
     <t>DivineWind</t>
   </si>
   <si>
@@ -1271,6 +1266,120 @@
   </si>
   <si>
     <t>AllEnemies</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>MaxStack</t>
+  </si>
+  <si>
+    <t>Poison</t>
+  </si>
+  <si>
+    <t>EFF_Posion_def</t>
+  </si>
+  <si>
+    <t>EFF_Stun_def</t>
+  </si>
+  <si>
+    <t>TargetStat</t>
+  </si>
+  <si>
+    <t>EFF_BufATK_def</t>
+  </si>
+  <si>
+    <t>EFF_BufDEF_def</t>
+  </si>
+  <si>
+    <t>EFF_BufSpd_def</t>
+  </si>
+  <si>
+    <t>DEF</t>
+  </si>
+  <si>
+    <t>SPEED</t>
+  </si>
+  <si>
+    <t>Stun</t>
+  </si>
+  <si>
+    <t>StatBuff</t>
+  </si>
+  <si>
+    <t>EFF_DefSpd_def</t>
+  </si>
+  <si>
+    <t>StatDebuff</t>
+  </si>
+  <si>
+    <t>EFF_ResetDef</t>
+  </si>
+  <si>
+    <t>RESIST_DEBUFF_NAME</t>
+  </si>
+  <si>
+    <t>RESIST_DEBUFF_DES</t>
+  </si>
+  <si>
+    <t>BUFF_DEF_NAME</t>
+  </si>
+  <si>
+    <t>BUFF_DEF_DES</t>
+  </si>
+  <si>
+    <t>BUFF_ATTACK_NAME</t>
+  </si>
+  <si>
+    <t>BUFF_ATTACK_DES</t>
+  </si>
+  <si>
+    <t>DEBUFF_STUN_NAME</t>
+  </si>
+  <si>
+    <t>DEBUFF_STUN_DES</t>
+  </si>
+  <si>
+    <t>BUFF_SPEED_NAME</t>
+  </si>
+  <si>
+    <t>BUFF_SPEED_DES</t>
+  </si>
+  <si>
+    <t>DEBUFF_SPEED_NAME</t>
+  </si>
+  <si>
+    <t>DEBUFF_SPEED_DES</t>
+  </si>
+  <si>
+    <t>EFF_POSION_NAME</t>
+  </si>
+  <si>
+    <t>EFF_POSION_DES</t>
+  </si>
+  <si>
+    <t>ResetDebuff</t>
+  </si>
+  <si>
+    <t>Effect</t>
+  </si>
+  <si>
+    <t>BackGround</t>
+  </si>
+  <si>
+    <t>ModifyType</t>
+  </si>
+  <si>
+    <t>Percent</t>
+  </si>
+  <si>
+    <t>Constant</t>
+  </si>
+  <si>
+    <t>PoisonBall</t>
   </si>
 </sst>
 </file>
@@ -3110,10 +3219,10 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="24" t="s">
+        <v>333</v>
+      </c>
+      <c r="B70" t="s">
         <v>334</v>
-      </c>
-      <c r="B70" t="s">
-        <v>335</v>
       </c>
       <c r="C70" t="s">
         <v>201</v>
@@ -3823,6 +3932,260 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>297</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>298</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B2" s="8">
+        <v>375</v>
+      </c>
+      <c r="C2" s="8">
+        <v>200</v>
+      </c>
+      <c r="D2" s="8">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>284</v>
+      </c>
+      <c r="B3" s="8">
+        <v>175</v>
+      </c>
+      <c r="C3" s="8">
+        <v>115</v>
+      </c>
+      <c r="D3" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>286</v>
+      </c>
+      <c r="B4" s="8">
+        <v>350</v>
+      </c>
+      <c r="C4" s="8">
+        <v>121</v>
+      </c>
+      <c r="D4" s="8">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>288</v>
+      </c>
+      <c r="B5" s="8">
+        <v>232</v>
+      </c>
+      <c r="C5" s="8">
+        <v>110</v>
+      </c>
+      <c r="D5" s="8">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>290</v>
+      </c>
+      <c r="B6" s="8">
+        <v>234</v>
+      </c>
+      <c r="C6" s="8">
+        <v>105</v>
+      </c>
+      <c r="D6" s="8">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>291</v>
+      </c>
+      <c r="B7" s="8">
+        <v>238</v>
+      </c>
+      <c r="C7" s="8">
+        <v>216</v>
+      </c>
+      <c r="D7" s="8">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>292</v>
+      </c>
+      <c r="B8" s="8">
+        <v>220</v>
+      </c>
+      <c r="C8" s="8">
+        <v>144</v>
+      </c>
+      <c r="D8" s="8">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>294</v>
+      </c>
+      <c r="B9" s="8">
+        <v>425</v>
+      </c>
+      <c r="C9" s="8">
+        <v>150</v>
+      </c>
+      <c r="D9" s="8">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>295</v>
+      </c>
+      <c r="B10" s="8">
+        <v>370</v>
+      </c>
+      <c r="C10" s="8">
+        <v>210</v>
+      </c>
+      <c r="D10" s="8">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>296</v>
+      </c>
+      <c r="B11" s="8">
+        <v>300</v>
+      </c>
+      <c r="C11" s="8">
+        <v>195</v>
+      </c>
+      <c r="D11" s="8">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>305</v>
+      </c>
+      <c r="B12" s="8">
+        <v>175</v>
+      </c>
+      <c r="C12" s="8">
+        <v>115</v>
+      </c>
+      <c r="D12" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="24" t="s">
+        <v>314</v>
+      </c>
+      <c r="B13" s="8">
+        <v>175</v>
+      </c>
+      <c r="C13" s="8">
+        <v>115</v>
+      </c>
+      <c r="D13" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="24" t="s">
+        <v>316</v>
+      </c>
+      <c r="B14" s="8">
+        <v>175</v>
+      </c>
+      <c r="C14" s="8">
+        <v>115</v>
+      </c>
+      <c r="D14" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="24" t="s">
+        <v>317</v>
+      </c>
+      <c r="B15" s="8">
+        <v>175</v>
+      </c>
+      <c r="C15" s="8">
+        <v>115</v>
+      </c>
+      <c r="D15" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="24" t="s">
+        <v>318</v>
+      </c>
+      <c r="B16" s="8">
+        <v>175</v>
+      </c>
+      <c r="C16" s="8">
+        <v>115</v>
+      </c>
+      <c r="D16" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="24" t="s">
+        <v>319</v>
+      </c>
+      <c r="B17" s="8">
+        <v>175</v>
+      </c>
+      <c r="C17" s="8">
+        <v>115</v>
+      </c>
+      <c r="D17" s="8">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3842,10 +4205,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>325</v>
+        <v>444</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -3853,13 +4216,13 @@
         <v>324</v>
       </c>
       <c r="B2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
   </sheetData>
@@ -3867,7 +4230,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3879,16 +4242,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
+        <v>329</v>
+      </c>
+      <c r="B1" s="18" t="s">
         <v>330</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="C1" s="18" t="s">
         <v>331</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="D1" s="18" t="s">
         <v>332</v>
-      </c>
-      <c r="D1" s="18" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -3899,7 +4262,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D2" s="7">
         <v>5</v>
@@ -3913,7 +4276,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D3" s="7">
         <v>5</v>
@@ -3927,7 +4290,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D4" s="7">
         <v>5</v>
@@ -4792,13 +5155,13 @@
         <v>68</v>
       </c>
       <c r="E1" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>348</v>
+      </c>
+      <c r="G1" s="18" t="s">
         <v>349</v>
-      </c>
-      <c r="F1" s="18" t="s">
-        <v>350</v>
-      </c>
-      <c r="G1" s="18" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -5063,10 +5426,10 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B12" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>285</v>
@@ -5079,10 +5442,10 @@
         <v>VanguardTiger_B</v>
       </c>
       <c r="F12" s="29" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -5222,7 +5585,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" customWidth="1"/>
@@ -5233,9 +5596,10 @@
     <col min="6" max="6" width="23.42578125" customWidth="1"/>
     <col min="7" max="7" width="16.85546875" customWidth="1"/>
     <col min="8" max="8" width="16.5703125" customWidth="1"/>
+    <col min="9" max="9" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
@@ -5243,27 +5607,30 @@
         <v>1</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="D1" s="18" t="s">
         <v>68</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F1" s="18" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="H1" s="18" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>407</v>
+      </c>
+      <c r="I1" s="18" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B2" t="str">
         <f>A2&amp;"_Name"</f>
@@ -5274,7 +5641,7 @@
         <v>SunWukong_B_Des</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E2" s="8">
         <v>1</v>
@@ -5286,12 +5653,15 @@
         <v>100</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" ref="B3:B48" si="0">A3&amp;"_Name"</f>
@@ -5302,7 +5672,7 @@
         <v>SunWukong_M_Des</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E3" s="8">
         <v>1</v>
@@ -5314,12 +5684,15 @@
         <v>100</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
@@ -5330,10 +5703,10 @@
         <v>SunWukong_U_Des</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F4" s="8">
         <v>5</v>
@@ -5342,12 +5715,15 @@
         <v>100</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
@@ -5358,7 +5734,7 @@
         <v>TangSanZang_B_Des</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E5" s="8">
         <v>1</v>
@@ -5370,12 +5746,15 @@
         <v>100</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
@@ -5386,10 +5765,10 @@
         <v>TangSanZang_M_Des</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F6" s="8">
         <v>4</v>
@@ -5398,12 +5777,15 @@
         <v>100</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>409</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
@@ -5414,10 +5796,10 @@
         <v>TangSanZang_U_Des</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F7" s="8">
         <v>5</v>
@@ -5426,12 +5808,15 @@
         <v>100</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I7" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
@@ -5442,7 +5827,7 @@
         <v>ZhuBaJie_B_Des</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E8" s="8">
         <v>1</v>
@@ -5454,12 +5839,15 @@
         <v>100</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
@@ -5470,10 +5858,10 @@
         <v>ZhuBaJie_M_Des</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F9" s="8">
         <v>4</v>
@@ -5482,12 +5870,15 @@
         <v>100</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>409</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -5498,10 +5889,10 @@
         <v>ZhuBaJie_U_Des</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F10" s="8">
         <v>5</v>
@@ -5510,12 +5901,15 @@
         <v>100</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I10" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
@@ -5526,7 +5920,7 @@
         <v>ShaWujing_B_Des</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E11" s="8">
         <v>1</v>
@@ -5538,12 +5932,15 @@
         <v>100</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
@@ -5554,10 +5951,10 @@
         <v>ShaWujing_M_Des</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F12" s="8">
         <v>4</v>
@@ -5566,12 +5963,15 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+        <v>409</v>
+      </c>
+      <c r="I12" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
@@ -5582,10 +5982,10 @@
         <v>ShaWujing_U_Des</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F13" s="8">
         <v>5</v>
@@ -5594,12 +5994,15 @@
         <v>100</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
@@ -5610,7 +6013,7 @@
         <v>DragonKing_B_Des</v>
       </c>
       <c r="D14" s="27" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E14" s="8">
         <v>1</v>
@@ -5622,12 +6025,15 @@
         <v>100</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="25" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
@@ -5638,10 +6044,10 @@
         <v>DragonKing_M_Des</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F15" s="8">
         <v>4</v>
@@ -5650,12 +6056,15 @@
         <v>100</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="25" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
@@ -5666,10 +6075,10 @@
         <v>DragonKing_U_Des</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F16" s="8">
         <v>5</v>
@@ -5678,12 +6087,15 @@
         <v>100</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
@@ -5694,7 +6106,7 @@
         <v>ThirdPrinceNezha_B_Des</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E17" s="8">
         <v>1</v>
@@ -5706,12 +6118,15 @@
         <v>100</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
@@ -5722,10 +6137,10 @@
         <v>ThirdPrinceNezha_M_Des</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F18" s="8">
         <v>4</v>
@@ -5734,12 +6149,15 @@
         <v>100</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="0"/>
@@ -5750,10 +6168,10 @@
         <v>ThirdPrinceNezha_U_Des</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F19" s="8">
         <v>5</v>
@@ -5762,12 +6180,15 @@
         <v>100</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I19" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="0"/>
@@ -5778,7 +6199,7 @@
         <v>LittleWhiteDragon_B_Des</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E20" s="8">
         <v>1</v>
@@ -5790,12 +6211,15 @@
         <v>100</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
@@ -5806,10 +6230,10 @@
         <v>LittleWhiteDragon_M_Des</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F21" s="8">
         <v>4</v>
@@ -5818,12 +6242,15 @@
         <v>100</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
@@ -5834,10 +6261,10 @@
         <v>LittleWhiteDragon_U_Des</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F22" s="8">
         <v>5</v>
@@ -5846,12 +6273,15 @@
         <v>100</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
@@ -5862,7 +6292,7 @@
         <v>BullDemonKing_B_Des</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E23" s="8">
         <v>1</v>
@@ -5874,12 +6304,15 @@
         <v>100</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="0"/>
@@ -5890,10 +6323,10 @@
         <v>BullDemonKing_M_Des</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F24" s="8">
         <v>4</v>
@@ -5902,12 +6335,15 @@
         <v>100</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+        <v>409</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
@@ -5918,10 +6354,10 @@
         <v>BullDemonKing_U_Des</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>347</v>
+        <v>448</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F25" s="8">
         <v>5</v>
@@ -5930,12 +6366,15 @@
         <v>100</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I25" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
@@ -5946,7 +6385,7 @@
         <v>ErlangShen_B_Des</v>
       </c>
       <c r="D26" s="27" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E26" s="8">
         <v>1</v>
@@ -5958,12 +6397,15 @@
         <v>100</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="25" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="0"/>
@@ -5974,10 +6416,10 @@
         <v>ErlangShen_M_Des</v>
       </c>
       <c r="D27" s="27" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F27" s="8">
         <v>4</v>
@@ -5986,12 +6428,15 @@
         <v>100</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="25" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="0"/>
@@ -6002,10 +6447,10 @@
         <v>ErlangShen_U_Des</v>
       </c>
       <c r="D28" s="27" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F28" s="8">
         <v>5</v>
@@ -6014,12 +6459,15 @@
         <v>100</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="25" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="0"/>
@@ -6030,7 +6478,7 @@
         <v>GuanyinBodhisattva_B_Des</v>
       </c>
       <c r="D29" s="27" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E29" s="8">
         <v>1</v>
@@ -6042,12 +6490,15 @@
         <v>100</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="25" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="0"/>
@@ -6058,10 +6509,10 @@
         <v>GuanyinBodhisattva_M_Des</v>
       </c>
       <c r="D30" s="27" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F30" s="8">
         <v>4</v>
@@ -6070,12 +6521,15 @@
         <v>100</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="25" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="0"/>
@@ -6086,10 +6540,10 @@
         <v>GuanyinBodhisattva_U_Des</v>
       </c>
       <c r="D31" s="27" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F31" s="8">
         <v>5</v>
@@ -6098,12 +6552,15 @@
         <v>100</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="0"/>
@@ -6114,7 +6571,7 @@
         <v>VanguardTiger_B_Des</v>
       </c>
       <c r="D32" s="30" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E32" s="8">
         <v>1</v>
@@ -6126,12 +6583,15 @@
         <v>100</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I32" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="0"/>
@@ -6142,7 +6602,7 @@
         <v>TheBoySage_B_Des</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E33" s="8">
         <v>1</v>
@@ -6154,12 +6614,15 @@
         <v>100</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="0"/>
@@ -6170,10 +6633,10 @@
         <v>TheBoySage_M_Des</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F34" s="8">
         <v>4</v>
@@ -6182,12 +6645,15 @@
         <v>100</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I34" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="0"/>
@@ -6198,10 +6664,10 @@
         <v>TheBoySage_U_Des</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F35" s="8">
         <v>5</v>
@@ -6210,12 +6676,15 @@
         <v>100</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="0"/>
@@ -6226,7 +6695,7 @@
         <v>GoldHornKing_B_Des</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E36" s="8">
         <v>1</v>
@@ -6238,12 +6707,15 @@
         <v>100</v>
       </c>
       <c r="H36" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I36" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="0"/>
@@ -6254,10 +6726,10 @@
         <v>GoldHornKing_M_Des</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F37" s="8">
         <v>4</v>
@@ -6266,12 +6738,15 @@
         <v>100</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I37" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="0"/>
@@ -6282,10 +6757,10 @@
         <v>GoldHornKing_U_Des</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F38" s="8">
         <v>5</v>
@@ -6294,12 +6769,15 @@
         <v>100</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I38" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="0"/>
@@ -6310,7 +6788,7 @@
         <v>SilverHornKing_B_Des</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E39" s="8">
         <v>1</v>
@@ -6322,12 +6800,15 @@
         <v>100</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I39" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="0"/>
@@ -6338,10 +6819,10 @@
         <v>SilverHornKing_M_Des</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F40" s="8">
         <v>4</v>
@@ -6350,12 +6831,15 @@
         <v>100</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I40" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="0"/>
@@ -6366,10 +6850,10 @@
         <v>SilverHornKing_U_Des</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F41" s="8">
         <v>5</v>
@@ -6378,12 +6862,15 @@
         <v>100</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I41" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="28" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="0"/>
@@ -6394,7 +6881,7 @@
         <v>YellowWindMonster_B_Des</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E42" s="8">
         <v>1</v>
@@ -6406,12 +6893,15 @@
         <v>100</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I42" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="28" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="0"/>
@@ -6422,10 +6912,10 @@
         <v>YellowWindMonster_M_Des</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F43" s="8">
         <v>4</v>
@@ -6434,12 +6924,15 @@
         <v>100</v>
       </c>
       <c r="H43" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I43" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="28" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="0"/>
@@ -6450,10 +6943,10 @@
         <v>YellowWindMonster_U_Des</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F44" s="8">
         <v>5</v>
@@ -6462,12 +6955,15 @@
         <v>100</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I44" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="0"/>
@@ -6478,7 +6974,7 @@
         <v>GoldfishDemon_B_Des</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E45" s="8">
         <v>1</v>
@@ -6490,12 +6986,15 @@
         <v>100</v>
       </c>
       <c r="H45" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I45" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="12" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="0"/>
@@ -6506,10 +7005,10 @@
         <v>GoldfishDemon_M_Des</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="F46" s="8">
         <v>4</v>
@@ -6518,12 +7017,15 @@
         <v>100</v>
       </c>
       <c r="H46" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I46" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="12" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="0"/>
@@ -6534,10 +7036,10 @@
         <v>GoldfishDemon_U_Des</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="F47" s="8">
         <v>5</v>
@@ -6546,12 +7048,15 @@
         <v>100</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+      <c r="I47" s="7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B48" s="8" t="str">
         <f t="shared" si="0"/>
@@ -6562,7 +7067,7 @@
         <v>None_Skill_Des</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E48" s="8">
         <v>0</v>
@@ -6574,7 +7079,10 @@
         <v>100</v>
       </c>
       <c r="H48" s="8" t="s">
-        <v>410</v>
+        <v>408</v>
+      </c>
+      <c r="I48" s="7" t="s">
+        <v>350</v>
       </c>
     </row>
   </sheetData>
@@ -6584,6 +7092,258 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.28515625" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5703125" customWidth="1"/>
+    <col min="5" max="6" width="16.5703125" style="7" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" style="7" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" style="7" customWidth="1"/>
+    <col min="9" max="9" width="18.28515625" style="7" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>377</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>417</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>445</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>411</v>
+      </c>
+      <c r="H1" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="I1" s="18" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B2" t="s">
+        <v>440</v>
+      </c>
+      <c r="C2" t="s">
+        <v>441</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>414</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="G2" s="7">
+        <v>2</v>
+      </c>
+      <c r="H2" s="7">
+        <v>100</v>
+      </c>
+      <c r="I2" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>416</v>
+      </c>
+      <c r="B3" t="s">
+        <v>434</v>
+      </c>
+      <c r="C3" t="s">
+        <v>435</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>423</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="G3" s="7">
+        <v>1</v>
+      </c>
+      <c r="H3" s="7">
+        <v>100</v>
+      </c>
+      <c r="I3" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>418</v>
+      </c>
+      <c r="B4" t="s">
+        <v>432</v>
+      </c>
+      <c r="C4" t="s">
+        <v>433</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="G4" s="7">
+        <v>2</v>
+      </c>
+      <c r="H4" s="7">
+        <v>100</v>
+      </c>
+      <c r="I4" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>419</v>
+      </c>
+      <c r="B5" t="s">
+        <v>430</v>
+      </c>
+      <c r="C5" t="s">
+        <v>431</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>421</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="G5" s="7">
+        <v>2</v>
+      </c>
+      <c r="H5" s="7">
+        <v>100</v>
+      </c>
+      <c r="I5" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>420</v>
+      </c>
+      <c r="B6" t="s">
+        <v>436</v>
+      </c>
+      <c r="C6" t="s">
+        <v>437</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>422</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>446</v>
+      </c>
+      <c r="G6" s="7">
+        <v>2</v>
+      </c>
+      <c r="H6" s="7">
+        <v>20</v>
+      </c>
+      <c r="I6" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>425</v>
+      </c>
+      <c r="B7" t="s">
+        <v>438</v>
+      </c>
+      <c r="C7" t="s">
+        <v>439</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>426</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>422</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>446</v>
+      </c>
+      <c r="G7" s="7">
+        <v>2</v>
+      </c>
+      <c r="H7" s="7">
+        <v>-20</v>
+      </c>
+      <c r="I7" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>427</v>
+      </c>
+      <c r="B8" t="s">
+        <v>428</v>
+      </c>
+      <c r="C8" t="s">
+        <v>429</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="G8" s="7">
+        <v>1</v>
+      </c>
+      <c r="H8" s="7">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6612,7 +7372,7 @@
         <v>299</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="H1" s="18" t="s">
         <v>300</v>
@@ -6755,7 +7515,7 @@
         <v>78</v>
       </c>
       <c r="D5" s="8">
-        <v>2900</v>
+        <v>3200</v>
       </c>
       <c r="E5" s="8">
         <v>1380</v>
@@ -7012,7 +7772,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>285</v>
@@ -7243,7 +8003,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7475,7 +8235,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>285</v>
@@ -7597,258 +8357,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="18" t="s">
-        <v>297</v>
-      </c>
-      <c r="C1" s="18" t="s">
-        <v>298</v>
-      </c>
-      <c r="D1" s="18" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>282</v>
-      </c>
-      <c r="B2" s="8">
-        <v>375</v>
-      </c>
-      <c r="C2" s="8">
-        <v>200</v>
-      </c>
-      <c r="D2" s="8">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>284</v>
-      </c>
-      <c r="B3" s="8">
-        <v>175</v>
-      </c>
-      <c r="C3" s="8">
-        <v>115</v>
-      </c>
-      <c r="D3" s="8">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>286</v>
-      </c>
-      <c r="B4" s="8">
-        <v>350</v>
-      </c>
-      <c r="C4" s="8">
-        <v>121</v>
-      </c>
-      <c r="D4" s="8">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>288</v>
-      </c>
-      <c r="B5" s="8">
-        <v>232</v>
-      </c>
-      <c r="C5" s="8">
-        <v>110</v>
-      </c>
-      <c r="D5" s="8">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>290</v>
-      </c>
-      <c r="B6" s="8">
-        <v>234</v>
-      </c>
-      <c r="C6" s="8">
-        <v>105</v>
-      </c>
-      <c r="D6" s="8">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>291</v>
-      </c>
-      <c r="B7" s="8">
-        <v>238</v>
-      </c>
-      <c r="C7" s="8">
-        <v>216</v>
-      </c>
-      <c r="D7" s="8">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>292</v>
-      </c>
-      <c r="B8" s="8">
-        <v>220</v>
-      </c>
-      <c r="C8" s="8">
-        <v>144</v>
-      </c>
-      <c r="D8" s="8">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>294</v>
-      </c>
-      <c r="B9" s="8">
-        <v>425</v>
-      </c>
-      <c r="C9" s="8">
-        <v>150</v>
-      </c>
-      <c r="D9" s="8">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>295</v>
-      </c>
-      <c r="B10" s="8">
-        <v>370</v>
-      </c>
-      <c r="C10" s="8">
-        <v>210</v>
-      </c>
-      <c r="D10" s="8">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>296</v>
-      </c>
-      <c r="B11" s="8">
-        <v>300</v>
-      </c>
-      <c r="C11" s="8">
-        <v>195</v>
-      </c>
-      <c r="D11" s="8">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>305</v>
-      </c>
-      <c r="B12" s="8">
-        <v>175</v>
-      </c>
-      <c r="C12" s="8">
-        <v>115</v>
-      </c>
-      <c r="D12" s="8">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="24" t="s">
-        <v>314</v>
-      </c>
-      <c r="B13" s="8">
-        <v>175</v>
-      </c>
-      <c r="C13" s="8">
-        <v>115</v>
-      </c>
-      <c r="D13" s="8">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="24" t="s">
-        <v>316</v>
-      </c>
-      <c r="B14" s="8">
-        <v>175</v>
-      </c>
-      <c r="C14" s="8">
-        <v>115</v>
-      </c>
-      <c r="D14" s="8">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="24" t="s">
-        <v>317</v>
-      </c>
-      <c r="B15" s="8">
-        <v>175</v>
-      </c>
-      <c r="C15" s="8">
-        <v>115</v>
-      </c>
-      <c r="D15" s="8">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="24" t="s">
-        <v>318</v>
-      </c>
-      <c r="B16" s="8">
-        <v>175</v>
-      </c>
-      <c r="C16" s="8">
-        <v>115</v>
-      </c>
-      <c r="D16" s="8">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="24" t="s">
-        <v>319</v>
-      </c>
-      <c r="B17" s="8">
-        <v>175</v>
-      </c>
-      <c r="C17" s="8">
-        <v>115</v>
-      </c>
-      <c r="D17" s="8">
-        <v>20</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
+ Handel Effect UI in battle Scene.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="2" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="2" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1312" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1312" uniqueCount="450">
   <si>
     <t>ID</t>
   </si>
@@ -1380,6 +1380,9 @@
   </si>
   <si>
     <t>PoisonBall</t>
+  </si>
+  <si>
+    <t>StatModifier</t>
   </si>
 </sst>
 </file>
@@ -5597,6 +5600,7 @@
     <col min="7" max="7" width="16.85546875" customWidth="1"/>
     <col min="8" max="8" width="16.5703125" customWidth="1"/>
     <col min="9" max="9" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5774,7 +5778,7 @@
         <v>4</v>
       </c>
       <c r="G6" s="8">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H6" s="8" t="s">
         <v>409</v>
@@ -5903,8 +5907,8 @@
       <c r="H10" s="8" t="s">
         <v>408</v>
       </c>
-      <c r="I10" t="s">
-        <v>419</v>
+      <c r="I10" s="7" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -5960,13 +5964,13 @@
         <v>4</v>
       </c>
       <c r="G12" s="8">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>409</v>
       </c>
       <c r="I12" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -6323,7 +6327,7 @@
         <v>BullDemonKing_M_Des</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>338</v>
+        <v>449</v>
       </c>
       <c r="E24" s="8" t="s">
         <v>401</v>
@@ -6332,13 +6336,13 @@
         <v>4</v>
       </c>
       <c r="G24" s="8">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H24" s="8" t="s">
         <v>409</v>
       </c>
-      <c r="I24" s="7" t="s">
-        <v>350</v>
+      <c r="I24" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -6918,10 +6922,10 @@
         <v>401</v>
       </c>
       <c r="F43" s="8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G43" s="8">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="H43" s="8" t="s">
         <v>408</v>
@@ -6949,7 +6953,7 @@
         <v>402</v>
       </c>
       <c r="F44" s="8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G44" s="8">
         <v>100</v>
@@ -7155,13 +7159,13 @@
         <v>350</v>
       </c>
       <c r="G2" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H2" s="7">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I2" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -7216,7 +7220,7 @@
         <v>2</v>
       </c>
       <c r="H4" s="7">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="I4" s="7">
         <v>1</v>
@@ -7245,7 +7249,7 @@
         <v>2</v>
       </c>
       <c r="H5" s="7">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I5" s="7">
         <v>1</v>
@@ -7477,7 +7481,7 @@
         <v>76</v>
       </c>
       <c r="D4" s="8">
-        <v>3900</v>
+        <v>3200</v>
       </c>
       <c r="E4" s="8">
         <v>1350</v>
@@ -7515,7 +7519,7 @@
         <v>78</v>
       </c>
       <c r="D5" s="8">
-        <v>3200</v>
+        <v>3900</v>
       </c>
       <c r="E5" s="8">
         <v>1380</v>
@@ -7781,10 +7785,10 @@
         <v>75</v>
       </c>
       <c r="D12" s="8">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="E12" s="8">
-        <v>1650</v>
+        <v>2650</v>
       </c>
       <c r="F12" s="8">
         <v>280</v>
@@ -7933,7 +7937,7 @@
         <v>74</v>
       </c>
       <c r="D16" s="8">
-        <v>3900</v>
+        <v>4900</v>
       </c>
       <c r="E16" s="8">
         <v>2400</v>
@@ -7942,7 +7946,7 @@
         <v>325</v>
       </c>
       <c r="G16" s="8">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="H16" s="8">
         <v>20</v>

</xml_diff>

<commit_message>
+ Add audio manager, and make skill audio for character
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="2" activeTab="6"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="3" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1312" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="469">
   <si>
     <t>ID</t>
   </si>
@@ -1383,6 +1383,63 @@
   </si>
   <si>
     <t>StatModifier</t>
+  </si>
+  <si>
+    <t>Boss</t>
+  </si>
+  <si>
+    <t>Sound</t>
+  </si>
+  <si>
+    <t>SunWukong_Attack</t>
+  </si>
+  <si>
+    <t>TangSanZang_Attack</t>
+  </si>
+  <si>
+    <t>SunWukong_Main</t>
+  </si>
+  <si>
+    <t>Wind_Blow</t>
+  </si>
+  <si>
+    <t>VanguardTiger_Attack</t>
+  </si>
+  <si>
+    <t>TangSanZang_Major</t>
+  </si>
+  <si>
+    <t>ZhuBaJie_Major</t>
+  </si>
+  <si>
+    <t>ShaWujing_Major</t>
+  </si>
+  <si>
+    <t>LittleWhiteDragon_Major</t>
+  </si>
+  <si>
+    <t>TangSanZang_Main</t>
+  </si>
+  <si>
+    <t>Battle_Test</t>
+  </si>
+  <si>
+    <t>ZhuBaJie_Attack</t>
+  </si>
+  <si>
+    <t>ShaWujing_Attack</t>
+  </si>
+  <si>
+    <t>LittleWhiteDragon_Attack</t>
+  </si>
+  <si>
+    <t>ZhuBaJie_Main</t>
+  </si>
+  <si>
+    <t>ShaWujing_Main</t>
+  </si>
+  <si>
+    <t>LittleWhiteDragon_Main</t>
   </si>
 </sst>
 </file>
@@ -1508,7 +1565,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1575,6 +1632,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -4190,10 +4250,10 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" customWidth="1"/>
     <col min="2" max="2" width="21.140625" customWidth="1"/>
     <col min="3" max="3" width="21.28515625" customWidth="1"/>
     <col min="4" max="4" width="15.5703125" customWidth="1"/>
@@ -4228,6 +4288,20 @@
         <v>328</v>
       </c>
     </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="B3" t="s">
+        <v>326</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>328</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4235,7 +4309,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" customWidth="1"/>
@@ -4243,7 +4317,7 @@
     <col min="3" max="3" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
         <v>329</v>
       </c>
@@ -4256,8 +4330,11 @@
       <c r="D1" s="18" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="18" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>324</v>
       </c>
@@ -4270,8 +4347,11 @@
       <c r="D2" s="7">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>324</v>
       </c>
@@ -4284,8 +4364,11 @@
       <c r="D3" s="7">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>324</v>
       </c>
@@ -4298,19 +4381,110 @@
       <c r="D4" s="7">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>324</v>
       </c>
       <c r="B5" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D5" s="7">
         <v>5</v>
+      </c>
+      <c r="E5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="B6" s="5">
+        <v>5</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>318</v>
+      </c>
+      <c r="D6" s="5">
+        <v>5</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="B7" s="7">
+        <v>6</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>317</v>
+      </c>
+      <c r="D7" s="7">
+        <v>5</v>
+      </c>
+      <c r="E7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="B8" s="7">
+        <v>1</v>
+      </c>
+      <c r="C8" s="24" t="s">
+        <v>333</v>
+      </c>
+      <c r="D8" s="7">
+        <v>5</v>
+      </c>
+      <c r="E8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="B9" s="7">
+        <v>2</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>333</v>
+      </c>
+      <c r="D9" s="7">
+        <v>5</v>
+      </c>
+      <c r="E9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="B10" s="7">
+        <v>3</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>333</v>
+      </c>
+      <c r="D10" s="7">
+        <v>5</v>
+      </c>
+      <c r="E10" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5142,6 +5316,7 @@
     <col min="5" max="5" width="21.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18.5703125" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -5588,7 +5763,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" customWidth="1"/>
@@ -5600,10 +5775,10 @@
     <col min="7" max="7" width="16.85546875" customWidth="1"/>
     <col min="8" max="8" width="16.5703125" customWidth="1"/>
     <col min="9" max="9" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.140625" customWidth="1"/>
+    <col min="10" max="10" width="24.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
@@ -5631,8 +5806,11 @@
       <c r="I1" s="18" t="s">
         <v>443</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="18" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>354</v>
       </c>
@@ -5662,8 +5840,11 @@
       <c r="I2" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J2" s="32" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>355</v>
       </c>
@@ -5693,8 +5874,11 @@
       <c r="I3" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J3" s="32" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>356</v>
       </c>
@@ -5724,8 +5908,11 @@
       <c r="I4" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J4" s="32" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>357</v>
       </c>
@@ -5755,8 +5942,11 @@
       <c r="I5" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J5" s="32" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
         <v>358</v>
       </c>
@@ -5786,8 +5976,11 @@
       <c r="I6" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J6" s="32" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
         <v>359</v>
       </c>
@@ -5817,8 +6010,11 @@
       <c r="I7" t="s">
         <v>416</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J7" s="32" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>360</v>
       </c>
@@ -5848,8 +6044,11 @@
       <c r="I8" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J8" s="32" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>361</v>
       </c>
@@ -5879,8 +6078,11 @@
       <c r="I9" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J9" s="32" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>362</v>
       </c>
@@ -5910,8 +6112,11 @@
       <c r="I10" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J10" s="32" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
         <v>363</v>
       </c>
@@ -5941,8 +6146,11 @@
       <c r="I11" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J11" s="32" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>364</v>
       </c>
@@ -5972,8 +6180,11 @@
       <c r="I12" t="s">
         <v>419</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J12" s="32" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
         <v>365</v>
       </c>
@@ -6003,8 +6214,11 @@
       <c r="I13" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J13" s="32" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
         <v>366</v>
       </c>
@@ -6035,7 +6249,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="25" t="s">
         <v>367</v>
       </c>
@@ -6066,7 +6280,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="25" t="s">
         <v>368</v>
       </c>
@@ -6097,7 +6311,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>369</v>
       </c>
@@ -6128,7 +6342,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>370</v>
       </c>
@@ -6159,7 +6373,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>371</v>
       </c>
@@ -6190,7 +6404,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
         <v>372</v>
       </c>
@@ -6220,8 +6434,11 @@
       <c r="I20" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J20" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
         <v>373</v>
       </c>
@@ -6251,8 +6468,11 @@
       <c r="I21" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J21" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
         <v>374</v>
       </c>
@@ -6282,8 +6502,11 @@
       <c r="I22" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J22" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>379</v>
       </c>
@@ -6314,7 +6537,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>380</v>
       </c>
@@ -6345,7 +6568,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>381</v>
       </c>
@@ -6376,7 +6599,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
         <v>375</v>
       </c>
@@ -6407,7 +6630,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="25" t="s">
         <v>376</v>
       </c>
@@ -6438,7 +6661,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="25" t="s">
         <v>378</v>
       </c>
@@ -6469,7 +6692,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="25" t="s">
         <v>382</v>
       </c>
@@ -6500,7 +6723,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="25" t="s">
         <v>383</v>
       </c>
@@ -6531,7 +6754,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="25" t="s">
         <v>384</v>
       </c>
@@ -6562,7 +6785,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
         <v>385</v>
       </c>
@@ -6591,6 +6814,9 @@
       </c>
       <c r="I32" s="7" t="s">
         <v>350</v>
+      </c>
+      <c r="J32" t="s">
+        <v>456</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
+ Make Effect Stat Modifier & SFX
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1371" uniqueCount="488">
   <si>
     <t>ID</t>
   </si>
@@ -1440,6 +1440,63 @@
   </si>
   <si>
     <t>LittleWhiteDragon_Main</t>
+  </si>
+  <si>
+    <t>ThirdPrinceNezha_Attack</t>
+  </si>
+  <si>
+    <t>TheBoySage_Attack</t>
+  </si>
+  <si>
+    <t>ThirdPrinceNezha_Main</t>
+  </si>
+  <si>
+    <t>ThirdPrinceNezha_Major</t>
+  </si>
+  <si>
+    <t>BullDemonKing_Major</t>
+  </si>
+  <si>
+    <t>TheBoySage_Major</t>
+  </si>
+  <si>
+    <t>YellowWindMonster_Attack</t>
+  </si>
+  <si>
+    <t>TheBoySage_Main</t>
+  </si>
+  <si>
+    <t>YellowWindMonster_Major</t>
+  </si>
+  <si>
+    <t>YellowWindMonster_Main</t>
+  </si>
+  <si>
+    <t>BullDemonKing_Main</t>
+  </si>
+  <si>
+    <t>SilverHornKing_Attack</t>
+  </si>
+  <si>
+    <t>GoldfishDemon_Attack</t>
+  </si>
+  <si>
+    <t>SilverHornKing_Major</t>
+  </si>
+  <si>
+    <t>GoldfishDemon_Major</t>
+  </si>
+  <si>
+    <t>GoldHornKing_Attack</t>
+  </si>
+  <si>
+    <t>GoldHornKing_Major</t>
+  </si>
+  <si>
+    <t>GoldHornKing_Main</t>
+  </si>
+  <si>
+    <t>GoldfishDemon_Main</t>
   </si>
 </sst>
 </file>
@@ -4309,7 +4366,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" customWidth="1"/>
@@ -4461,7 +4518,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>333</v>
+        <v>314</v>
       </c>
       <c r="D9" s="7">
         <v>5</v>
@@ -4478,12 +4535,63 @@
         <v>3</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>333</v>
+        <v>319</v>
       </c>
       <c r="D10" s="7">
         <v>5</v>
       </c>
       <c r="E10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="B11" s="7">
+        <v>5</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>318</v>
+      </c>
+      <c r="D11" s="7">
+        <v>5</v>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="B12" s="7">
+        <v>4</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>316</v>
+      </c>
+      <c r="D12" s="7">
+        <v>5</v>
+      </c>
+      <c r="E12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="B13" s="7">
+        <v>6</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>317</v>
+      </c>
+      <c r="D13" s="7">
+        <v>5</v>
+      </c>
+      <c r="E13" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5863,7 +5971,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G3" s="8">
         <v>100</v>
@@ -5897,7 +6005,7 @@
         <v>402</v>
       </c>
       <c r="F4" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G4" s="8">
         <v>100</v>
@@ -5965,7 +6073,7 @@
         <v>401</v>
       </c>
       <c r="F6" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G6" s="8">
         <v>0</v>
@@ -5999,7 +6107,7 @@
         <v>402</v>
       </c>
       <c r="F7" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G7" s="8">
         <v>100</v>
@@ -6067,7 +6175,7 @@
         <v>401</v>
       </c>
       <c r="F9" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G9" s="8">
         <v>100</v>
@@ -6101,7 +6209,7 @@
         <v>402</v>
       </c>
       <c r="F10" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G10" s="8">
         <v>100</v>
@@ -6169,7 +6277,7 @@
         <v>401</v>
       </c>
       <c r="F12" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G12" s="8">
         <v>0</v>
@@ -6203,7 +6311,7 @@
         <v>402</v>
       </c>
       <c r="F13" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G13" s="8">
         <v>100</v>
@@ -6268,7 +6376,7 @@
         <v>401</v>
       </c>
       <c r="F15" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G15" s="8">
         <v>100</v>
@@ -6299,7 +6407,7 @@
         <v>402</v>
       </c>
       <c r="F16" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G16" s="8">
         <v>100</v>
@@ -6341,6 +6449,9 @@
       <c r="I17" s="7" t="s">
         <v>350</v>
       </c>
+      <c r="J17" t="s">
+        <v>469</v>
+      </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -6361,7 +6472,7 @@
         <v>401</v>
       </c>
       <c r="F18" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G18" s="8">
         <v>100</v>
@@ -6371,6 +6482,9 @@
       </c>
       <c r="I18" s="7" t="s">
         <v>350</v>
+      </c>
+      <c r="J18" t="s">
+        <v>472</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -6392,7 +6506,7 @@
         <v>402</v>
       </c>
       <c r="F19" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G19" s="8">
         <v>100</v>
@@ -6400,8 +6514,11 @@
       <c r="H19" s="8" t="s">
         <v>408</v>
       </c>
-      <c r="I19" t="s">
-        <v>420</v>
+      <c r="I19" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="J19" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -6457,7 +6574,7 @@
         <v>401</v>
       </c>
       <c r="F21" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G21" s="8">
         <v>100</v>
@@ -6491,7 +6608,7 @@
         <v>402</v>
       </c>
       <c r="F22" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G22" s="8">
         <v>100</v>
@@ -6536,6 +6653,9 @@
       <c r="I23" s="7" t="s">
         <v>350</v>
       </c>
+      <c r="J23" t="s">
+        <v>456</v>
+      </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
@@ -6556,7 +6676,7 @@
         <v>401</v>
       </c>
       <c r="F24" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G24" s="8">
         <v>0</v>
@@ -6566,6 +6686,9 @@
       </c>
       <c r="I24" t="s">
         <v>418</v>
+      </c>
+      <c r="J24" s="8" t="s">
+        <v>473</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -6587,7 +6710,7 @@
         <v>402</v>
       </c>
       <c r="F25" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G25" s="8">
         <v>100</v>
@@ -6597,6 +6720,9 @@
       </c>
       <c r="I25" t="s">
         <v>415</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>479</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -6649,7 +6775,7 @@
         <v>401</v>
       </c>
       <c r="F27" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G27" s="8">
         <v>100</v>
@@ -6680,7 +6806,7 @@
         <v>402</v>
       </c>
       <c r="F28" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G28" s="8">
         <v>100</v>
@@ -6742,7 +6868,7 @@
         <v>401</v>
       </c>
       <c r="F30" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G30" s="8">
         <v>100</v>
@@ -6773,7 +6899,7 @@
         <v>402</v>
       </c>
       <c r="F31" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G31" s="8">
         <v>100</v>
@@ -6819,7 +6945,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
         <v>386</v>
       </c>
@@ -6849,8 +6975,11 @@
       <c r="I33" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J33" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
         <v>387</v>
       </c>
@@ -6869,7 +6998,7 @@
         <v>401</v>
       </c>
       <c r="F34" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G34" s="8">
         <v>100</v>
@@ -6880,8 +7009,11 @@
       <c r="I34" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J34" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
         <v>388</v>
       </c>
@@ -6900,7 +7032,7 @@
         <v>402</v>
       </c>
       <c r="F35" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G35" s="8">
         <v>100</v>
@@ -6911,8 +7043,11 @@
       <c r="I35" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J35" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>389</v>
       </c>
@@ -6942,8 +7077,11 @@
       <c r="I36" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J36" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>390</v>
       </c>
@@ -6962,7 +7100,7 @@
         <v>401</v>
       </c>
       <c r="F37" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G37" s="8">
         <v>100</v>
@@ -6973,8 +7111,11 @@
       <c r="I37" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J37" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>391</v>
       </c>
@@ -6993,7 +7134,7 @@
         <v>402</v>
       </c>
       <c r="F38" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G38" s="8">
         <v>100</v>
@@ -7004,8 +7145,11 @@
       <c r="I38" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J38" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
         <v>393</v>
       </c>
@@ -7035,8 +7179,11 @@
       <c r="I39" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J39" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
         <v>394</v>
       </c>
@@ -7055,7 +7202,7 @@
         <v>401</v>
       </c>
       <c r="F40" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G40" s="8">
         <v>100</v>
@@ -7066,8 +7213,11 @@
       <c r="I40" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J40" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
         <v>392</v>
       </c>
@@ -7086,7 +7236,7 @@
         <v>402</v>
       </c>
       <c r="F41" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G41" s="8">
         <v>100</v>
@@ -7097,8 +7247,11 @@
       <c r="I41" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J41" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="28" t="s">
         <v>395</v>
       </c>
@@ -7128,8 +7281,11 @@
       <c r="I42" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J42" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="28" t="s">
         <v>396</v>
       </c>
@@ -7148,7 +7304,7 @@
         <v>401</v>
       </c>
       <c r="F43" s="8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G43" s="8">
         <v>1000</v>
@@ -7156,11 +7312,14 @@
       <c r="H43" s="8" t="s">
         <v>408</v>
       </c>
-      <c r="I43" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I43" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="J43" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="28" t="s">
         <v>397</v>
       </c>
@@ -7179,7 +7338,7 @@
         <v>402</v>
       </c>
       <c r="F44" s="8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G44" s="8">
         <v>100</v>
@@ -7190,8 +7349,11 @@
       <c r="I44" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J44" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
         <v>398</v>
       </c>
@@ -7221,8 +7383,11 @@
       <c r="I45" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J45" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="12" t="s">
         <v>399</v>
       </c>
@@ -7241,7 +7406,7 @@
         <v>401</v>
       </c>
       <c r="F46" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G46" s="8">
         <v>100</v>
@@ -7252,8 +7417,11 @@
       <c r="I46" s="7" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J46" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="12" t="s">
         <v>400</v>
       </c>
@@ -7272,7 +7440,7 @@
         <v>402</v>
       </c>
       <c r="F47" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G47" s="8">
         <v>100</v>
@@ -7280,11 +7448,14 @@
       <c r="H47" s="8" t="s">
         <v>408</v>
       </c>
-      <c r="I47" s="7" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I47" t="s">
+        <v>416</v>
+      </c>
+      <c r="J47" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>405</v>
       </c>

</xml_diff>

<commit_message>
+ Add Inventory and character System. Edit player save game.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="3" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="1" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1371" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1483" uniqueCount="493">
   <si>
     <t>ID</t>
   </si>
@@ -1497,6 +1497,21 @@
   </si>
   <si>
     <t>GoldfishDemon_Main</t>
+  </si>
+  <si>
+    <t>main_stat_type</t>
+  </si>
+  <si>
+    <t>main_stat_valuie</t>
+  </si>
+  <si>
+    <t>random_substat_pool</t>
+  </si>
+  <si>
+    <t>modifier_type</t>
+  </si>
+  <si>
+    <t>hp,100, 1000, Constant|def,50,150, Constant</t>
   </si>
 </sst>
 </file>
@@ -4993,15 +5008,19 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.85546875" customWidth="1"/>
+    <col min="7" max="7" width="40.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5011,8 +5030,20 @@
       <c r="C1" s="18" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" s="18" t="s">
+        <v>488</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>489</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>491</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>212</v>
       </c>
@@ -5022,8 +5053,20 @@
       <c r="C2" s="8" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E2" s="8">
+        <v>10</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>213</v>
       </c>
@@ -5033,8 +5076,20 @@
       <c r="C3" s="8" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E3" s="8">
+        <v>10</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
         <v>214</v>
       </c>
@@ -5044,8 +5099,20 @@
       <c r="C4" s="8" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E4" s="8">
+        <v>10</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
         <v>215</v>
       </c>
@@ -5055,8 +5122,20 @@
       <c r="C5" s="8" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E5" s="8">
+        <v>10</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
         <v>216</v>
       </c>
@@ -5066,8 +5145,20 @@
       <c r="C6" s="8" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D6" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E6" s="8">
+        <v>10</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
         <v>217</v>
       </c>
@@ -5077,8 +5168,20 @@
       <c r="C7" s="8" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D7" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E7" s="8">
+        <v>10</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
         <v>218</v>
       </c>
@@ -5088,8 +5191,20 @@
       <c r="C8" s="8" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D8" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E8" s="8">
+        <v>10</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
         <v>219</v>
       </c>
@@ -5099,8 +5214,20 @@
       <c r="C9" s="8" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E9" s="8">
+        <v>10</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
         <v>220</v>
       </c>
@@ -5110,8 +5237,20 @@
       <c r="C10" s="8" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E10" s="8">
+        <v>10</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
         <v>221</v>
       </c>
@@ -5121,8 +5260,20 @@
       <c r="C11" s="8" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D11" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E11" s="8">
+        <v>10</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
         <v>222</v>
       </c>
@@ -5132,8 +5283,20 @@
       <c r="C12" s="8" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D12" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E12" s="8">
+        <v>10</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
         <v>223</v>
       </c>
@@ -5143,8 +5306,20 @@
       <c r="C13" s="8" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D13" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E13" s="8">
+        <v>10</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
         <v>224</v>
       </c>
@@ -5154,8 +5329,20 @@
       <c r="C14" s="8" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D14" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E14" s="8">
+        <v>10</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
         <v>225</v>
       </c>
@@ -5165,8 +5352,20 @@
       <c r="C15" s="8" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D15" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E15" s="8">
+        <v>10</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
         <v>226</v>
       </c>
@@ -5176,8 +5375,20 @@
       <c r="C16" s="8" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D16" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E16" s="8">
+        <v>10</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
         <v>227</v>
       </c>
@@ -5187,8 +5398,20 @@
       <c r="C17" s="8" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D17" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E17" s="8">
+        <v>10</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
         <v>228</v>
       </c>
@@ -5198,8 +5421,20 @@
       <c r="C18" s="8" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D18" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E18" s="8">
+        <v>10</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
         <v>229</v>
       </c>
@@ -5209,8 +5444,20 @@
       <c r="C19" s="8" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D19" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E19" s="8">
+        <v>10</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
         <v>230</v>
       </c>
@@ -5220,8 +5467,20 @@
       <c r="C20" s="8" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D20" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E20" s="8">
+        <v>10</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
         <v>231</v>
       </c>
@@ -5231,8 +5490,20 @@
       <c r="C21" s="8" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D21" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E21" s="8">
+        <v>10</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
         <v>232</v>
       </c>
@@ -5242,8 +5513,20 @@
       <c r="C22" s="8" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D22" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E22" s="8">
+        <v>10</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
         <v>233</v>
       </c>
@@ -5253,8 +5536,20 @@
       <c r="C23" s="8" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D23" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E23" s="8">
+        <v>10</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
         <v>234</v>
       </c>
@@ -5264,8 +5559,20 @@
       <c r="C24" s="8" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D24" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E24" s="8">
+        <v>10</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
         <v>235</v>
       </c>
@@ -5275,8 +5582,20 @@
       <c r="C25" s="8" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D25" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E25" s="8">
+        <v>10</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
         <v>236</v>
       </c>
@@ -5286,8 +5605,20 @@
       <c r="C26" s="8" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D26" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E26" s="8">
+        <v>10</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="17" t="s">
         <v>237</v>
       </c>
@@ -5297,8 +5628,20 @@
       <c r="C27" s="8" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D27" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E27" s="8">
+        <v>10</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
         <v>238</v>
       </c>
@@ -5308,8 +5651,20 @@
       <c r="C28" s="8" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D28" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E28" s="8">
+        <v>10</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
         <v>239</v>
       </c>
@@ -5319,8 +5674,20 @@
       <c r="C29" s="8" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D29" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E29" s="8">
+        <v>10</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
         <v>240</v>
       </c>
@@ -5330,8 +5697,20 @@
       <c r="C30" s="8" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D30" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E30" s="8">
+        <v>10</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="s">
         <v>241</v>
       </c>
@@ -5341,8 +5720,20 @@
       <c r="C31" s="8" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D31" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E31" s="8">
+        <v>10</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G31" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="17" t="s">
         <v>242</v>
       </c>
@@ -5352,8 +5743,20 @@
       <c r="C32" s="8" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D32" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E32" s="8">
+        <v>10</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="17" t="s">
         <v>243</v>
       </c>
@@ -5363,8 +5766,20 @@
       <c r="C33" s="8" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D33" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E33" s="8">
+        <v>10</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G33" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="17" t="s">
         <v>244</v>
       </c>
@@ -5374,8 +5789,20 @@
       <c r="C34" s="8" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D34" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E34" s="8">
+        <v>10</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="17" t="s">
         <v>245</v>
       </c>
@@ -5385,8 +5812,20 @@
       <c r="C35" s="8" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D35" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E35" s="8">
+        <v>10</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G35" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="17" t="s">
         <v>246</v>
       </c>
@@ -5396,8 +5835,20 @@
       <c r="C36" s="8" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D36" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E36" s="8">
+        <v>10</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="17" t="s">
         <v>247</v>
       </c>
@@ -5407,9 +5858,22 @@
       <c r="C37" s="8" t="s">
         <v>276</v>
       </c>
+      <c r="D37" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E37" s="8">
+        <v>10</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="G37" s="8" t="s">
+        <v>492</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
+ fix bug in character scene.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="1" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="6" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -17,8 +17,10 @@
     <sheet name="CharacterStat" sheetId="6" r:id="rId8"/>
     <sheet name="CharacterAttribute" sheetId="8" r:id="rId9"/>
     <sheet name="CharacterUpgrade" sheetId="7" r:id="rId10"/>
-    <sheet name="BattleConfig" sheetId="9" r:id="rId11"/>
-    <sheet name="StageEnemies" sheetId="10" r:id="rId12"/>
+    <sheet name="ExpCurvesConfig" sheetId="13" r:id="rId11"/>
+    <sheet name="AscensionConfig" sheetId="14" r:id="rId12"/>
+    <sheet name="BattleConfig" sheetId="9" r:id="rId13"/>
+    <sheet name="StageEnemies" sheetId="10" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$111</definedName>
@@ -33,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1483" uniqueCount="493">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1537" uniqueCount="513">
   <si>
     <t>ID</t>
   </si>
@@ -1512,6 +1514,66 @@
   </si>
   <si>
     <t>hp,100, 1000, Constant|def,50,150, Constant</t>
+  </si>
+  <si>
+    <t>Curve_R</t>
+  </si>
+  <si>
+    <t>Curve_SR</t>
+  </si>
+  <si>
+    <t>Curve_SSR</t>
+  </si>
+  <si>
+    <t>Curve_UR</t>
+  </si>
+  <si>
+    <t>exp_base</t>
+  </si>
+  <si>
+    <t>exp_exponent</t>
+  </si>
+  <si>
+    <t>Curve_R_up</t>
+  </si>
+  <si>
+    <t>Curve_SR_up</t>
+  </si>
+  <si>
+    <t>Curve_SSR_up</t>
+  </si>
+  <si>
+    <t>Curve_UR_up</t>
+  </si>
+  <si>
+    <t>Tier</t>
+  </si>
+  <si>
+    <t>Required_Level</t>
+  </si>
+  <si>
+    <t>Unlock_Max_Level</t>
+  </si>
+  <si>
+    <t>Cost_Gold</t>
+  </si>
+  <si>
+    <t>ItemID_01</t>
+  </si>
+  <si>
+    <t>Item_01_Qty</t>
+  </si>
+  <si>
+    <t>ascension_r</t>
+  </si>
+  <si>
+    <t>ascension_sr</t>
+  </si>
+  <si>
+    <t>ascension_ssr</t>
+  </si>
+  <si>
+    <t>ascension_ur</t>
   </si>
 </sst>
 </file>
@@ -4322,6 +4384,4203 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:Q101"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" customWidth="1"/>
+    <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" customWidth="1"/>
+    <col min="10" max="10" width="12.42578125" customWidth="1"/>
+    <col min="11" max="11" width="15.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>493</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>494</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>495</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>496</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>499</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>500</v>
+      </c>
+      <c r="H1" s="18" t="s">
+        <v>501</v>
+      </c>
+      <c r="I1" s="18" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <f>ROUND( $N$3*POWER(A2-1,$N$4), 0)</f>
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <f>ROUND($O$3*POWER(A2 -1,$O$4), 0)</f>
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <f>ROUND($P$3 * POWER(A2 - 1, $P$4), 0)</f>
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <f>ROUND($Q$3 * POWER(A2 - 1, $Q$4), 0)</f>
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="N2" s="18" t="s">
+        <v>493</v>
+      </c>
+      <c r="O2" s="18" t="s">
+        <v>494</v>
+      </c>
+      <c r="P2" s="18" t="s">
+        <v>495</v>
+      </c>
+      <c r="Q2" s="18" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <f>ROUND( $N$3*POWER(A3-1,$N$4), 0)</f>
+        <v>100</v>
+      </c>
+      <c r="C3">
+        <f>ROUND($O$3*POWER(A3 -1,$O$4), 0)</f>
+        <v>150</v>
+      </c>
+      <c r="D3">
+        <f>ROUND($P$3 * POWER(A3 - 1, $P$4), 0)</f>
+        <v>200</v>
+      </c>
+      <c r="E3">
+        <f>ROUND($Q$3 * POWER(A3 - 1, $Q$4), 0)</f>
+        <v>250</v>
+      </c>
+      <c r="F3">
+        <f xml:space="preserve"> B3-B2</f>
+        <v>100</v>
+      </c>
+      <c r="G3">
+        <f>C3-C2</f>
+        <v>150</v>
+      </c>
+      <c r="H3">
+        <f>D3-D2</f>
+        <v>200</v>
+      </c>
+      <c r="I3">
+        <f>E3-E2</f>
+        <v>250</v>
+      </c>
+      <c r="M3" s="12" t="s">
+        <v>497</v>
+      </c>
+      <c r="N3">
+        <v>100</v>
+      </c>
+      <c r="O3">
+        <v>150</v>
+      </c>
+      <c r="P3">
+        <v>200</v>
+      </c>
+      <c r="Q3">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <f>ROUND( $N$3*POWER(A4-1,$N$4), 0)</f>
+        <v>303</v>
+      </c>
+      <c r="C4">
+        <f>ROUND($O$3*POWER(A4 -1,$O$4), 0)</f>
+        <v>487</v>
+      </c>
+      <c r="D4">
+        <f>ROUND($P$3 * POWER(A4 - 1, $P$4), 0)</f>
+        <v>696</v>
+      </c>
+      <c r="E4">
+        <f>ROUND($Q$3 * POWER(A4 - 1, $Q$4), 0)</f>
+        <v>933</v>
+      </c>
+      <c r="F4">
+        <f t="shared" ref="F4:F67" si="0" xml:space="preserve"> B4-B3</f>
+        <v>203</v>
+      </c>
+      <c r="G4">
+        <f t="shared" ref="G4:G67" si="1">C4-C3</f>
+        <v>337</v>
+      </c>
+      <c r="H4">
+        <f t="shared" ref="H4:H67" si="2">D4-D3</f>
+        <v>496</v>
+      </c>
+      <c r="I4">
+        <f t="shared" ref="I4:I67" si="3">E4-E3</f>
+        <v>683</v>
+      </c>
+      <c r="M4" s="12" t="s">
+        <v>498</v>
+      </c>
+      <c r="N4">
+        <v>1.6</v>
+      </c>
+      <c r="O4">
+        <v>1.7</v>
+      </c>
+      <c r="P4">
+        <v>1.8</v>
+      </c>
+      <c r="Q4">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <f>ROUND( $N$3*POWER(A5-1,$N$4), 0)</f>
+        <v>580</v>
+      </c>
+      <c r="C5">
+        <f>ROUND($O$3*POWER(A5 -1,$O$4), 0)</f>
+        <v>971</v>
+      </c>
+      <c r="D5">
+        <f>ROUND($P$3 * POWER(A5 - 1, $P$4), 0)</f>
+        <v>1445</v>
+      </c>
+      <c r="E5">
+        <f>ROUND($Q$3 * POWER(A5 - 1, $Q$4), 0)</f>
+        <v>2016</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>277</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="1"/>
+        <v>484</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="2"/>
+        <v>749</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="3"/>
+        <v>1083</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <f>ROUND( $N$3*POWER(A6-1,$N$4), 0)</f>
+        <v>919</v>
+      </c>
+      <c r="C6">
+        <f>ROUND($O$3*POWER(A6 -1,$O$4), 0)</f>
+        <v>1583</v>
+      </c>
+      <c r="D6">
+        <f>ROUND($P$3 * POWER(A6 - 1, $P$4), 0)</f>
+        <v>2425</v>
+      </c>
+      <c r="E6">
+        <f>ROUND($Q$3 * POWER(A6 - 1, $Q$4), 0)</f>
+        <v>3482</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>339</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="1"/>
+        <v>612</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="2"/>
+        <v>980</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="3"/>
+        <v>1466</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <f>ROUND( $N$3*POWER(A7-1,$N$4), 0)</f>
+        <v>1313</v>
+      </c>
+      <c r="C7">
+        <f>ROUND($O$3*POWER(A7 -1,$O$4), 0)</f>
+        <v>2314</v>
+      </c>
+      <c r="D7">
+        <f>ROUND($P$3 * POWER(A7 - 1, $P$4), 0)</f>
+        <v>3624</v>
+      </c>
+      <c r="E7">
+        <f>ROUND($Q$3 * POWER(A7 - 1, $Q$4), 0)</f>
+        <v>5321</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>394</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="1"/>
+        <v>731</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="2"/>
+        <v>1199</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="3"/>
+        <v>1839</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" s="7">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <f>ROUND( $N$3*POWER(A8-1,$N$4), 0)</f>
+        <v>1758</v>
+      </c>
+      <c r="C8">
+        <f>ROUND($O$3*POWER(A8 -1,$O$4), 0)</f>
+        <v>3155</v>
+      </c>
+      <c r="D8">
+        <f>ROUND($P$3 * POWER(A8 - 1, $P$4), 0)</f>
+        <v>5032</v>
+      </c>
+      <c r="E8">
+        <f>ROUND($Q$3 * POWER(A8 - 1, $Q$4), 0)</f>
+        <v>7524</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>445</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="1"/>
+        <v>841</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="2"/>
+        <v>1408</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="3"/>
+        <v>2203</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <f>ROUND( $N$3*POWER(A9-1,$N$4), 0)</f>
+        <v>2250</v>
+      </c>
+      <c r="C9">
+        <f>ROUND($O$3*POWER(A9 -1,$O$4), 0)</f>
+        <v>4100</v>
+      </c>
+      <c r="D9">
+        <f>ROUND($P$3 * POWER(A9 - 1, $P$4), 0)</f>
+        <v>6641</v>
+      </c>
+      <c r="E9">
+        <f>ROUND($Q$3 * POWER(A9 - 1, $Q$4), 0)</f>
+        <v>10084</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>492</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="1"/>
+        <v>945</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="2"/>
+        <v>1609</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="3"/>
+        <v>2560</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" s="7">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <f>ROUND( $N$3*POWER(A10-1,$N$4), 0)</f>
+        <v>2786</v>
+      </c>
+      <c r="C10">
+        <f>ROUND($O$3*POWER(A10 -1,$O$4), 0)</f>
+        <v>5145</v>
+      </c>
+      <c r="D10">
+        <f>ROUND($P$3 * POWER(A10 - 1, $P$4), 0)</f>
+        <v>8445</v>
+      </c>
+      <c r="E10">
+        <f>ROUND($Q$3 * POWER(A10 - 1, $Q$4), 0)</f>
+        <v>12996</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>536</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="1"/>
+        <v>1045</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="2"/>
+        <v>1804</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="3"/>
+        <v>2912</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <f>ROUND( $N$3*POWER(A11-1,$N$4), 0)</f>
+        <v>3363</v>
+      </c>
+      <c r="C11">
+        <f>ROUND($O$3*POWER(A11 -1,$O$4), 0)</f>
+        <v>6285</v>
+      </c>
+      <c r="D11">
+        <f>ROUND($P$3 * POWER(A11 - 1, $P$4), 0)</f>
+        <v>10439</v>
+      </c>
+      <c r="E11">
+        <f>ROUND($Q$3 * POWER(A11 - 1, $Q$4), 0)</f>
+        <v>16256</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>577</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="1"/>
+        <v>1140</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="2"/>
+        <v>1994</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="3"/>
+        <v>3260</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" s="7">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <f>ROUND( $N$3*POWER(A12-1,$N$4), 0)</f>
+        <v>3981</v>
+      </c>
+      <c r="C12">
+        <f>ROUND($O$3*POWER(A12 -1,$O$4), 0)</f>
+        <v>7518</v>
+      </c>
+      <c r="D12">
+        <f>ROUND($P$3 * POWER(A12 - 1, $P$4), 0)</f>
+        <v>12619</v>
+      </c>
+      <c r="E12">
+        <f>ROUND($Q$3 * POWER(A12 - 1, $Q$4), 0)</f>
+        <v>19858</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>618</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="1"/>
+        <v>1233</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="2"/>
+        <v>2180</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="3"/>
+        <v>3602</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13" s="8">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <f>ROUND( $N$3*POWER(A13-1,$N$4), 0)</f>
+        <v>4637</v>
+      </c>
+      <c r="C13">
+        <f>ROUND($O$3*POWER(A13 -1,$O$4), 0)</f>
+        <v>8840</v>
+      </c>
+      <c r="D13">
+        <f>ROUND($P$3 * POWER(A13 - 1, $P$4), 0)</f>
+        <v>14981</v>
+      </c>
+      <c r="E13">
+        <f>ROUND($Q$3 * POWER(A13 - 1, $Q$4), 0)</f>
+        <v>23801</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>656</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="1"/>
+        <v>1322</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="2"/>
+        <v>2362</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="3"/>
+        <v>3943</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14" s="7">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <f>ROUND( $N$3*POWER(A14-1,$N$4), 0)</f>
+        <v>5330</v>
+      </c>
+      <c r="C14">
+        <f>ROUND($O$3*POWER(A14 -1,$O$4), 0)</f>
+        <v>10249</v>
+      </c>
+      <c r="D14">
+        <f>ROUND($P$3 * POWER(A14 - 1, $P$4), 0)</f>
+        <v>17521</v>
+      </c>
+      <c r="E14">
+        <f>ROUND($Q$3 * POWER(A14 - 1, $Q$4), 0)</f>
+        <v>28079</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="0"/>
+        <v>693</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="1"/>
+        <v>1409</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="2"/>
+        <v>2540</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="3"/>
+        <v>4278</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <f>ROUND( $N$3*POWER(A15-1,$N$4), 0)</f>
+        <v>6058</v>
+      </c>
+      <c r="C15">
+        <f>ROUND($O$3*POWER(A15 -1,$O$4), 0)</f>
+        <v>11743</v>
+      </c>
+      <c r="D15">
+        <f>ROUND($P$3 * POWER(A15 - 1, $P$4), 0)</f>
+        <v>20236</v>
+      </c>
+      <c r="E15">
+        <f>ROUND($Q$3 * POWER(A15 - 1, $Q$4), 0)</f>
+        <v>32691</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="0"/>
+        <v>728</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="1"/>
+        <v>1494</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="2"/>
+        <v>2715</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="3"/>
+        <v>4612</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" s="7">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <f>ROUND( $N$3*POWER(A16-1,$N$4), 0)</f>
+        <v>6820</v>
+      </c>
+      <c r="C16">
+        <f>ROUND($O$3*POWER(A16 -1,$O$4), 0)</f>
+        <v>13320</v>
+      </c>
+      <c r="D16">
+        <f>ROUND($P$3 * POWER(A16 - 1, $P$4), 0)</f>
+        <v>23124</v>
+      </c>
+      <c r="E16">
+        <f>ROUND($Q$3 * POWER(A16 - 1, $Q$4), 0)</f>
+        <v>37634</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="0"/>
+        <v>762</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="1"/>
+        <v>1577</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="2"/>
+        <v>2888</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="3"/>
+        <v>4943</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="8">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <f>ROUND( $N$3*POWER(A17-1,$N$4), 0)</f>
+        <v>7616</v>
+      </c>
+      <c r="C17">
+        <f>ROUND($O$3*POWER(A17 -1,$O$4), 0)</f>
+        <v>14978</v>
+      </c>
+      <c r="D17">
+        <f>ROUND($P$3 * POWER(A17 - 1, $P$4), 0)</f>
+        <v>26181</v>
+      </c>
+      <c r="E17">
+        <f>ROUND($Q$3 * POWER(A17 - 1, $Q$4), 0)</f>
+        <v>42906</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="0"/>
+        <v>796</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="1"/>
+        <v>1658</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="2"/>
+        <v>3057</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="3"/>
+        <v>5272</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="7">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <f>ROUND( $N$3*POWER(A18-1,$N$4), 0)</f>
+        <v>8445</v>
+      </c>
+      <c r="C18">
+        <f>ROUND($O$3*POWER(A18 -1,$O$4), 0)</f>
+        <v>16715</v>
+      </c>
+      <c r="D18">
+        <f>ROUND($P$3 * POWER(A18 - 1, $P$4), 0)</f>
+        <v>29407</v>
+      </c>
+      <c r="E18">
+        <f>ROUND($Q$3 * POWER(A18 - 1, $Q$4), 0)</f>
+        <v>48503</v>
+      </c>
+      <c r="F18">
+        <f t="shared" si="0"/>
+        <v>829</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="1"/>
+        <v>1737</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="2"/>
+        <v>3226</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="3"/>
+        <v>5597</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="8">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <f>ROUND( $N$3*POWER(A19-1,$N$4), 0)</f>
+        <v>9305</v>
+      </c>
+      <c r="C19">
+        <f>ROUND($O$3*POWER(A19 -1,$O$4), 0)</f>
+        <v>18529</v>
+      </c>
+      <c r="D19">
+        <f>ROUND($P$3 * POWER(A19 - 1, $P$4), 0)</f>
+        <v>32797</v>
+      </c>
+      <c r="E19">
+        <f>ROUND($Q$3 * POWER(A19 - 1, $Q$4), 0)</f>
+        <v>54424</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="0"/>
+        <v>860</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="1"/>
+        <v>1814</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="2"/>
+        <v>3390</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="3"/>
+        <v>5921</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="7">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <f>ROUND( $N$3*POWER(A20-1,$N$4), 0)</f>
+        <v>10196</v>
+      </c>
+      <c r="C20">
+        <f>ROUND($O$3*POWER(A20 -1,$O$4), 0)</f>
+        <v>20420</v>
+      </c>
+      <c r="D20">
+        <f>ROUND($P$3 * POWER(A20 - 1, $P$4), 0)</f>
+        <v>36351</v>
+      </c>
+      <c r="E20">
+        <f>ROUND($Q$3 * POWER(A20 - 1, $Q$4), 0)</f>
+        <v>60668</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="0"/>
+        <v>891</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="1"/>
+        <v>1891</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="2"/>
+        <v>3554</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="3"/>
+        <v>6244</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="8">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <f>ROUND( $N$3*POWER(A21-1,$N$4), 0)</f>
+        <v>11117</v>
+      </c>
+      <c r="C21">
+        <f>ROUND($O$3*POWER(A21 -1,$O$4), 0)</f>
+        <v>22386</v>
+      </c>
+      <c r="D21">
+        <f>ROUND($P$3 * POWER(A21 - 1, $P$4), 0)</f>
+        <v>40067</v>
+      </c>
+      <c r="E21">
+        <f>ROUND($Q$3 * POWER(A21 - 1, $Q$4), 0)</f>
+        <v>67231</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="0"/>
+        <v>921</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="1"/>
+        <v>1966</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="2"/>
+        <v>3716</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="3"/>
+        <v>6563</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="7">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <f>ROUND( $N$3*POWER(A22-1,$N$4), 0)</f>
+        <v>12068</v>
+      </c>
+      <c r="C22">
+        <f>ROUND($O$3*POWER(A22 -1,$O$4), 0)</f>
+        <v>24425</v>
+      </c>
+      <c r="D22">
+        <f>ROUND($P$3 * POWER(A22 - 1, $P$4), 0)</f>
+        <v>43942</v>
+      </c>
+      <c r="E22">
+        <f>ROUND($Q$3 * POWER(A22 - 1, $Q$4), 0)</f>
+        <v>74113</v>
+      </c>
+      <c r="F22">
+        <f t="shared" si="0"/>
+        <v>951</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="1"/>
+        <v>2039</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="2"/>
+        <v>3875</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="3"/>
+        <v>6882</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="8">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <f>ROUND( $N$3*POWER(A23-1,$N$4), 0)</f>
+        <v>13048</v>
+      </c>
+      <c r="C23">
+        <f>ROUND($O$3*POWER(A23 -1,$O$4), 0)</f>
+        <v>26538</v>
+      </c>
+      <c r="D23">
+        <f>ROUND($P$3 * POWER(A23 - 1, $P$4), 0)</f>
+        <v>47976</v>
+      </c>
+      <c r="E23">
+        <f>ROUND($Q$3 * POWER(A23 - 1, $Q$4), 0)</f>
+        <v>81312</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="0"/>
+        <v>980</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="1"/>
+        <v>2113</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="2"/>
+        <v>4034</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="3"/>
+        <v>7199</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="7">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <f>ROUND( $N$3*POWER(A24-1,$N$4), 0)</f>
+        <v>14056</v>
+      </c>
+      <c r="C24">
+        <f>ROUND($O$3*POWER(A24 -1,$O$4), 0)</f>
+        <v>28722</v>
+      </c>
+      <c r="D24">
+        <f>ROUND($P$3 * POWER(A24 - 1, $P$4), 0)</f>
+        <v>52166</v>
+      </c>
+      <c r="E24">
+        <f>ROUND($Q$3 * POWER(A24 - 1, $Q$4), 0)</f>
+        <v>88827</v>
+      </c>
+      <c r="F24">
+        <f t="shared" si="0"/>
+        <v>1008</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="1"/>
+        <v>2184</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="2"/>
+        <v>4190</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="3"/>
+        <v>7515</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="8">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <f>ROUND( $N$3*POWER(A25-1,$N$4), 0)</f>
+        <v>15093</v>
+      </c>
+      <c r="C25">
+        <f>ROUND($O$3*POWER(A25 -1,$O$4), 0)</f>
+        <v>30976</v>
+      </c>
+      <c r="D25">
+        <f>ROUND($P$3 * POWER(A25 - 1, $P$4), 0)</f>
+        <v>56512</v>
+      </c>
+      <c r="E25">
+        <f>ROUND($Q$3 * POWER(A25 - 1, $Q$4), 0)</f>
+        <v>96655</v>
+      </c>
+      <c r="F25">
+        <f t="shared" si="0"/>
+        <v>1037</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="1"/>
+        <v>2254</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="2"/>
+        <v>4346</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="3"/>
+        <v>7828</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="7">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <f>ROUND( $N$3*POWER(A26-1,$N$4), 0)</f>
+        <v>16156</v>
+      </c>
+      <c r="C26">
+        <f>ROUND($O$3*POWER(A26 -1,$O$4), 0)</f>
+        <v>33300</v>
+      </c>
+      <c r="D26">
+        <f>ROUND($P$3 * POWER(A26 - 1, $P$4), 0)</f>
+        <v>61011</v>
+      </c>
+      <c r="E26">
+        <f>ROUND($Q$3 * POWER(A26 - 1, $Q$4), 0)</f>
+        <v>104795</v>
+      </c>
+      <c r="F26">
+        <f t="shared" si="0"/>
+        <v>1063</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="1"/>
+        <v>2324</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="2"/>
+        <v>4499</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="3"/>
+        <v>8140</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="8">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <f>ROUND( $N$3*POWER(A27-1,$N$4), 0)</f>
+        <v>17247</v>
+      </c>
+      <c r="C27">
+        <f>ROUND($O$3*POWER(A27 -1,$O$4), 0)</f>
+        <v>35694</v>
+      </c>
+      <c r="D27">
+        <f>ROUND($P$3 * POWER(A27 - 1, $P$4), 0)</f>
+        <v>65663</v>
+      </c>
+      <c r="E27">
+        <f>ROUND($Q$3 * POWER(A27 - 1, $Q$4), 0)</f>
+        <v>113247</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="0"/>
+        <v>1091</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="1"/>
+        <v>2394</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="2"/>
+        <v>4652</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="3"/>
+        <v>8452</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="7">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <f>ROUND( $N$3*POWER(A28-1,$N$4), 0)</f>
+        <v>18364</v>
+      </c>
+      <c r="C28">
+        <f>ROUND($O$3*POWER(A28 -1,$O$4), 0)</f>
+        <v>38155</v>
+      </c>
+      <c r="D28">
+        <f>ROUND($P$3 * POWER(A28 - 1, $P$4), 0)</f>
+        <v>70466</v>
+      </c>
+      <c r="E28">
+        <f>ROUND($Q$3 * POWER(A28 - 1, $Q$4), 0)</f>
+        <v>122008</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="0"/>
+        <v>1117</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="1"/>
+        <v>2461</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="2"/>
+        <v>4803</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="3"/>
+        <v>8761</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="8">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <f>ROUND( $N$3*POWER(A29-1,$N$4), 0)</f>
+        <v>19507</v>
+      </c>
+      <c r="C29">
+        <f>ROUND($O$3*POWER(A29 -1,$O$4), 0)</f>
+        <v>40683</v>
+      </c>
+      <c r="D29">
+        <f>ROUND($P$3 * POWER(A29 - 1, $P$4), 0)</f>
+        <v>75420</v>
+      </c>
+      <c r="E29">
+        <f>ROUND($Q$3 * POWER(A29 - 1, $Q$4), 0)</f>
+        <v>131078</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="0"/>
+        <v>1143</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="1"/>
+        <v>2528</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="2"/>
+        <v>4954</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="3"/>
+        <v>9070</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="7">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <f>ROUND( $N$3*POWER(A30-1,$N$4), 0)</f>
+        <v>20675</v>
+      </c>
+      <c r="C30">
+        <f>ROUND($O$3*POWER(A30 -1,$O$4), 0)</f>
+        <v>43277</v>
+      </c>
+      <c r="D30">
+        <f>ROUND($P$3 * POWER(A30 - 1, $P$4), 0)</f>
+        <v>80522</v>
+      </c>
+      <c r="E30">
+        <f>ROUND($Q$3 * POWER(A30 - 1, $Q$4), 0)</f>
+        <v>140456</v>
+      </c>
+      <c r="F30">
+        <f t="shared" si="0"/>
+        <v>1168</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="1"/>
+        <v>2594</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="2"/>
+        <v>5102</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="3"/>
+        <v>9378</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="8">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <f>ROUND( $N$3*POWER(A31-1,$N$4), 0)</f>
+        <v>21869</v>
+      </c>
+      <c r="C31">
+        <f>ROUND($O$3*POWER(A31 -1,$O$4), 0)</f>
+        <v>45938</v>
+      </c>
+      <c r="D31">
+        <f>ROUND($P$3 * POWER(A31 - 1, $P$4), 0)</f>
+        <v>85772</v>
+      </c>
+      <c r="E31">
+        <f>ROUND($Q$3 * POWER(A31 - 1, $Q$4), 0)</f>
+        <v>150140</v>
+      </c>
+      <c r="F31">
+        <f t="shared" si="0"/>
+        <v>1194</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="1"/>
+        <v>2661</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="2"/>
+        <v>5250</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="3"/>
+        <v>9684</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="7">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <f>ROUND( $N$3*POWER(A32-1,$N$4), 0)</f>
+        <v>23088</v>
+      </c>
+      <c r="C32">
+        <f>ROUND($O$3*POWER(A32 -1,$O$4), 0)</f>
+        <v>48663</v>
+      </c>
+      <c r="D32">
+        <f>ROUND($P$3 * POWER(A32 - 1, $P$4), 0)</f>
+        <v>91169</v>
+      </c>
+      <c r="E32">
+        <f>ROUND($Q$3 * POWER(A32 - 1, $Q$4), 0)</f>
+        <v>160129</v>
+      </c>
+      <c r="F32">
+        <f t="shared" si="0"/>
+        <v>1219</v>
+      </c>
+      <c r="G32">
+        <f t="shared" si="1"/>
+        <v>2725</v>
+      </c>
+      <c r="H32">
+        <f t="shared" si="2"/>
+        <v>5397</v>
+      </c>
+      <c r="I32">
+        <f t="shared" si="3"/>
+        <v>9989</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="8">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <f>ROUND( $N$3*POWER(A33-1,$N$4), 0)</f>
+        <v>24332</v>
+      </c>
+      <c r="C33">
+        <f>ROUND($O$3*POWER(A33 -1,$O$4), 0)</f>
+        <v>51452</v>
+      </c>
+      <c r="D33">
+        <f>ROUND($P$3 * POWER(A33 - 1, $P$4), 0)</f>
+        <v>96712</v>
+      </c>
+      <c r="E33">
+        <f>ROUND($Q$3 * POWER(A33 - 1, $Q$4), 0)</f>
+        <v>170423</v>
+      </c>
+      <c r="F33">
+        <f t="shared" si="0"/>
+        <v>1244</v>
+      </c>
+      <c r="G33">
+        <f t="shared" si="1"/>
+        <v>2789</v>
+      </c>
+      <c r="H33">
+        <f t="shared" si="2"/>
+        <v>5543</v>
+      </c>
+      <c r="I33">
+        <f t="shared" si="3"/>
+        <v>10294</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="7">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <f>ROUND( $N$3*POWER(A34-1,$N$4), 0)</f>
+        <v>25600</v>
+      </c>
+      <c r="C34">
+        <f>ROUND($O$3*POWER(A34 -1,$O$4), 0)</f>
+        <v>54306</v>
+      </c>
+      <c r="D34">
+        <f>ROUND($P$3 * POWER(A34 - 1, $P$4), 0)</f>
+        <v>102400</v>
+      </c>
+      <c r="E34">
+        <f>ROUND($Q$3 * POWER(A34 - 1, $Q$4), 0)</f>
+        <v>181019</v>
+      </c>
+      <c r="F34">
+        <f t="shared" si="0"/>
+        <v>1268</v>
+      </c>
+      <c r="G34">
+        <f t="shared" si="1"/>
+        <v>2854</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="2"/>
+        <v>5688</v>
+      </c>
+      <c r="I34">
+        <f t="shared" si="3"/>
+        <v>10596</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="8">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <f>ROUND( $N$3*POWER(A35-1,$N$4), 0)</f>
+        <v>26892</v>
+      </c>
+      <c r="C35">
+        <f>ROUND($O$3*POWER(A35 -1,$O$4), 0)</f>
+        <v>57222</v>
+      </c>
+      <c r="D35">
+        <f>ROUND($P$3 * POWER(A35 - 1, $P$4), 0)</f>
+        <v>108232</v>
+      </c>
+      <c r="E35">
+        <f>ROUND($Q$3 * POWER(A35 - 1, $Q$4), 0)</f>
+        <v>191918</v>
+      </c>
+      <c r="F35">
+        <f t="shared" si="0"/>
+        <v>1292</v>
+      </c>
+      <c r="G35">
+        <f t="shared" si="1"/>
+        <v>2916</v>
+      </c>
+      <c r="H35">
+        <f t="shared" si="2"/>
+        <v>5832</v>
+      </c>
+      <c r="I35">
+        <f t="shared" si="3"/>
+        <v>10899</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="7">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <f>ROUND( $N$3*POWER(A36-1,$N$4), 0)</f>
+        <v>28208</v>
+      </c>
+      <c r="C36">
+        <f>ROUND($O$3*POWER(A36 -1,$O$4), 0)</f>
+        <v>60201</v>
+      </c>
+      <c r="D36">
+        <f>ROUND($P$3 * POWER(A36 - 1, $P$4), 0)</f>
+        <v>114207</v>
+      </c>
+      <c r="E36">
+        <f>ROUND($Q$3 * POWER(A36 - 1, $Q$4), 0)</f>
+        <v>203119</v>
+      </c>
+      <c r="F36">
+        <f t="shared" si="0"/>
+        <v>1316</v>
+      </c>
+      <c r="G36">
+        <f t="shared" si="1"/>
+        <v>2979</v>
+      </c>
+      <c r="H36">
+        <f t="shared" si="2"/>
+        <v>5975</v>
+      </c>
+      <c r="I36">
+        <f t="shared" si="3"/>
+        <v>11201</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="8">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <f>ROUND( $N$3*POWER(A37-1,$N$4), 0)</f>
+        <v>29547</v>
+      </c>
+      <c r="C37">
+        <f>ROUND($O$3*POWER(A37 -1,$O$4), 0)</f>
+        <v>63242</v>
+      </c>
+      <c r="D37">
+        <f>ROUND($P$3 * POWER(A37 - 1, $P$4), 0)</f>
+        <v>120324</v>
+      </c>
+      <c r="E37">
+        <f>ROUND($Q$3 * POWER(A37 - 1, $Q$4), 0)</f>
+        <v>214620</v>
+      </c>
+      <c r="F37">
+        <f t="shared" si="0"/>
+        <v>1339</v>
+      </c>
+      <c r="G37">
+        <f t="shared" si="1"/>
+        <v>3041</v>
+      </c>
+      <c r="H37">
+        <f t="shared" si="2"/>
+        <v>6117</v>
+      </c>
+      <c r="I37">
+        <f t="shared" si="3"/>
+        <v>11501</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="7">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <f>ROUND( $N$3*POWER(A38-1,$N$4), 0)</f>
+        <v>30909</v>
+      </c>
+      <c r="C38">
+        <f>ROUND($O$3*POWER(A38 -1,$O$4), 0)</f>
+        <v>66345</v>
+      </c>
+      <c r="D38">
+        <f>ROUND($P$3 * POWER(A38 - 1, $P$4), 0)</f>
+        <v>126583</v>
+      </c>
+      <c r="E38">
+        <f>ROUND($Q$3 * POWER(A38 - 1, $Q$4), 0)</f>
+        <v>226420</v>
+      </c>
+      <c r="F38">
+        <f t="shared" si="0"/>
+        <v>1362</v>
+      </c>
+      <c r="G38">
+        <f t="shared" si="1"/>
+        <v>3103</v>
+      </c>
+      <c r="H38">
+        <f t="shared" si="2"/>
+        <v>6259</v>
+      </c>
+      <c r="I38">
+        <f t="shared" si="3"/>
+        <v>11800</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="8">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <f>ROUND( $N$3*POWER(A39-1,$N$4), 0)</f>
+        <v>32294</v>
+      </c>
+      <c r="C39">
+        <f>ROUND($O$3*POWER(A39 -1,$O$4), 0)</f>
+        <v>69508</v>
+      </c>
+      <c r="D39">
+        <f>ROUND($P$3 * POWER(A39 - 1, $P$4), 0)</f>
+        <v>132982</v>
+      </c>
+      <c r="E39">
+        <f>ROUND($Q$3 * POWER(A39 - 1, $Q$4), 0)</f>
+        <v>238519</v>
+      </c>
+      <c r="F39">
+        <f t="shared" si="0"/>
+        <v>1385</v>
+      </c>
+      <c r="G39">
+        <f t="shared" si="1"/>
+        <v>3163</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="2"/>
+        <v>6399</v>
+      </c>
+      <c r="I39">
+        <f t="shared" si="3"/>
+        <v>12099</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="7">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <f>ROUND( $N$3*POWER(A40-1,$N$4), 0)</f>
+        <v>33702</v>
+      </c>
+      <c r="C40">
+        <f>ROUND($O$3*POWER(A40 -1,$O$4), 0)</f>
+        <v>72732</v>
+      </c>
+      <c r="D40">
+        <f>ROUND($P$3 * POWER(A40 - 1, $P$4), 0)</f>
+        <v>139521</v>
+      </c>
+      <c r="E40">
+        <f>ROUND($Q$3 * POWER(A40 - 1, $Q$4), 0)</f>
+        <v>250916</v>
+      </c>
+      <c r="F40">
+        <f t="shared" si="0"/>
+        <v>1408</v>
+      </c>
+      <c r="G40">
+        <f t="shared" si="1"/>
+        <v>3224</v>
+      </c>
+      <c r="H40">
+        <f t="shared" si="2"/>
+        <v>6539</v>
+      </c>
+      <c r="I40">
+        <f t="shared" si="3"/>
+        <v>12397</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="8">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <f>ROUND( $N$3*POWER(A41-1,$N$4), 0)</f>
+        <v>35132</v>
+      </c>
+      <c r="C41">
+        <f>ROUND($O$3*POWER(A41 -1,$O$4), 0)</f>
+        <v>76015</v>
+      </c>
+      <c r="D41">
+        <f>ROUND($P$3 * POWER(A41 - 1, $P$4), 0)</f>
+        <v>146200</v>
+      </c>
+      <c r="E41">
+        <f>ROUND($Q$3 * POWER(A41 - 1, $Q$4), 0)</f>
+        <v>263611</v>
+      </c>
+      <c r="F41">
+        <f t="shared" si="0"/>
+        <v>1430</v>
+      </c>
+      <c r="G41">
+        <f t="shared" si="1"/>
+        <v>3283</v>
+      </c>
+      <c r="H41">
+        <f t="shared" si="2"/>
+        <v>6679</v>
+      </c>
+      <c r="I41">
+        <f t="shared" si="3"/>
+        <v>12695</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="7">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <f>ROUND( $N$3*POWER(A42-1,$N$4), 0)</f>
+        <v>36584</v>
+      </c>
+      <c r="C42">
+        <f>ROUND($O$3*POWER(A42 -1,$O$4), 0)</f>
+        <v>79358</v>
+      </c>
+      <c r="D42">
+        <f>ROUND($P$3 * POWER(A42 - 1, $P$4), 0)</f>
+        <v>153016</v>
+      </c>
+      <c r="E42">
+        <f>ROUND($Q$3 * POWER(A42 - 1, $Q$4), 0)</f>
+        <v>276601</v>
+      </c>
+      <c r="F42">
+        <f t="shared" si="0"/>
+        <v>1452</v>
+      </c>
+      <c r="G42">
+        <f t="shared" si="1"/>
+        <v>3343</v>
+      </c>
+      <c r="H42">
+        <f t="shared" si="2"/>
+        <v>6816</v>
+      </c>
+      <c r="I42">
+        <f t="shared" si="3"/>
+        <v>12990</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="8">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <f>ROUND( $N$3*POWER(A43-1,$N$4), 0)</f>
+        <v>38059</v>
+      </c>
+      <c r="C43">
+        <f>ROUND($O$3*POWER(A43 -1,$O$4), 0)</f>
+        <v>82761</v>
+      </c>
+      <c r="D43">
+        <f>ROUND($P$3 * POWER(A43 - 1, $P$4), 0)</f>
+        <v>159971</v>
+      </c>
+      <c r="E43">
+        <f>ROUND($Q$3 * POWER(A43 - 1, $Q$4), 0)</f>
+        <v>289887</v>
+      </c>
+      <c r="F43">
+        <f t="shared" si="0"/>
+        <v>1475</v>
+      </c>
+      <c r="G43">
+        <f t="shared" si="1"/>
+        <v>3403</v>
+      </c>
+      <c r="H43">
+        <f t="shared" si="2"/>
+        <v>6955</v>
+      </c>
+      <c r="I43">
+        <f t="shared" si="3"/>
+        <v>13286</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="7">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <f>ROUND( $N$3*POWER(A44-1,$N$4), 0)</f>
+        <v>39555</v>
+      </c>
+      <c r="C44">
+        <f>ROUND($O$3*POWER(A44 -1,$O$4), 0)</f>
+        <v>86221</v>
+      </c>
+      <c r="D44">
+        <f>ROUND($P$3 * POWER(A44 - 1, $P$4), 0)</f>
+        <v>167062</v>
+      </c>
+      <c r="E44">
+        <f>ROUND($Q$3 * POWER(A44 - 1, $Q$4), 0)</f>
+        <v>303469</v>
+      </c>
+      <c r="F44">
+        <f t="shared" si="0"/>
+        <v>1496</v>
+      </c>
+      <c r="G44">
+        <f t="shared" si="1"/>
+        <v>3460</v>
+      </c>
+      <c r="H44">
+        <f t="shared" si="2"/>
+        <v>7091</v>
+      </c>
+      <c r="I44">
+        <f t="shared" si="3"/>
+        <v>13582</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="8">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <f>ROUND( $N$3*POWER(A45-1,$N$4), 0)</f>
+        <v>41072</v>
+      </c>
+      <c r="C45">
+        <f>ROUND($O$3*POWER(A45 -1,$O$4), 0)</f>
+        <v>89740</v>
+      </c>
+      <c r="D45">
+        <f>ROUND($P$3 * POWER(A45 - 1, $P$4), 0)</f>
+        <v>174290</v>
+      </c>
+      <c r="E45">
+        <f>ROUND($Q$3 * POWER(A45 - 1, $Q$4), 0)</f>
+        <v>317344</v>
+      </c>
+      <c r="F45">
+        <f t="shared" si="0"/>
+        <v>1517</v>
+      </c>
+      <c r="G45">
+        <f t="shared" si="1"/>
+        <v>3519</v>
+      </c>
+      <c r="H45">
+        <f t="shared" si="2"/>
+        <v>7228</v>
+      </c>
+      <c r="I45">
+        <f t="shared" si="3"/>
+        <v>13875</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="7">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <f>ROUND( $N$3*POWER(A46-1,$N$4), 0)</f>
+        <v>42611</v>
+      </c>
+      <c r="C46">
+        <f>ROUND($O$3*POWER(A46 -1,$O$4), 0)</f>
+        <v>93317</v>
+      </c>
+      <c r="D46">
+        <f>ROUND($P$3 * POWER(A46 - 1, $P$4), 0)</f>
+        <v>181654</v>
+      </c>
+      <c r="E46">
+        <f>ROUND($Q$3 * POWER(A46 - 1, $Q$4), 0)</f>
+        <v>331513</v>
+      </c>
+      <c r="F46">
+        <f t="shared" si="0"/>
+        <v>1539</v>
+      </c>
+      <c r="G46">
+        <f t="shared" si="1"/>
+        <v>3577</v>
+      </c>
+      <c r="H46">
+        <f t="shared" si="2"/>
+        <v>7364</v>
+      </c>
+      <c r="I46">
+        <f t="shared" si="3"/>
+        <v>14169</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="8">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <f>ROUND( $N$3*POWER(A47-1,$N$4), 0)</f>
+        <v>44171</v>
+      </c>
+      <c r="C47">
+        <f>ROUND($O$3*POWER(A47 -1,$O$4), 0)</f>
+        <v>96951</v>
+      </c>
+      <c r="D47">
+        <f>ROUND($P$3 * POWER(A47 - 1, $P$4), 0)</f>
+        <v>189153</v>
+      </c>
+      <c r="E47">
+        <f>ROUND($Q$3 * POWER(A47 - 1, $Q$4), 0)</f>
+        <v>345974</v>
+      </c>
+      <c r="F47">
+        <f t="shared" si="0"/>
+        <v>1560</v>
+      </c>
+      <c r="G47">
+        <f t="shared" si="1"/>
+        <v>3634</v>
+      </c>
+      <c r="H47">
+        <f t="shared" si="2"/>
+        <v>7499</v>
+      </c>
+      <c r="I47">
+        <f t="shared" si="3"/>
+        <v>14461</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="7">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <f>ROUND( $N$3*POWER(A48-1,$N$4), 0)</f>
+        <v>45752</v>
+      </c>
+      <c r="C48">
+        <f>ROUND($O$3*POWER(A48 -1,$O$4), 0)</f>
+        <v>100642</v>
+      </c>
+      <c r="D48">
+        <f>ROUND($P$3 * POWER(A48 - 1, $P$4), 0)</f>
+        <v>196786</v>
+      </c>
+      <c r="E48">
+        <f>ROUND($Q$3 * POWER(A48 - 1, $Q$4), 0)</f>
+        <v>360728</v>
+      </c>
+      <c r="F48">
+        <f t="shared" si="0"/>
+        <v>1581</v>
+      </c>
+      <c r="G48">
+        <f t="shared" si="1"/>
+        <v>3691</v>
+      </c>
+      <c r="H48">
+        <f t="shared" si="2"/>
+        <v>7633</v>
+      </c>
+      <c r="I48">
+        <f t="shared" si="3"/>
+        <v>14754</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" s="8">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <f>ROUND( $N$3*POWER(A49-1,$N$4), 0)</f>
+        <v>47354</v>
+      </c>
+      <c r="C49">
+        <f>ROUND($O$3*POWER(A49 -1,$O$4), 0)</f>
+        <v>104390</v>
+      </c>
+      <c r="D49">
+        <f>ROUND($P$3 * POWER(A49 - 1, $P$4), 0)</f>
+        <v>204553</v>
+      </c>
+      <c r="E49">
+        <f>ROUND($Q$3 * POWER(A49 - 1, $Q$4), 0)</f>
+        <v>375773</v>
+      </c>
+      <c r="F49">
+        <f t="shared" si="0"/>
+        <v>1602</v>
+      </c>
+      <c r="G49">
+        <f t="shared" si="1"/>
+        <v>3748</v>
+      </c>
+      <c r="H49">
+        <f t="shared" si="2"/>
+        <v>7767</v>
+      </c>
+      <c r="I49">
+        <f t="shared" si="3"/>
+        <v>15045</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" s="7">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <f>ROUND( $N$3*POWER(A50-1,$N$4), 0)</f>
+        <v>48976</v>
+      </c>
+      <c r="C50">
+        <f>ROUND($O$3*POWER(A50 -1,$O$4), 0)</f>
+        <v>108194</v>
+      </c>
+      <c r="D50">
+        <f>ROUND($P$3 * POWER(A50 - 1, $P$4), 0)</f>
+        <v>212454</v>
+      </c>
+      <c r="E50">
+        <f>ROUND($Q$3 * POWER(A50 - 1, $Q$4), 0)</f>
+        <v>391109</v>
+      </c>
+      <c r="F50">
+        <f t="shared" si="0"/>
+        <v>1622</v>
+      </c>
+      <c r="G50">
+        <f t="shared" si="1"/>
+        <v>3804</v>
+      </c>
+      <c r="H50">
+        <f t="shared" si="2"/>
+        <v>7901</v>
+      </c>
+      <c r="I50">
+        <f t="shared" si="3"/>
+        <v>15336</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" s="8">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <f>ROUND( $N$3*POWER(A51-1,$N$4), 0)</f>
+        <v>50619</v>
+      </c>
+      <c r="C51">
+        <f>ROUND($O$3*POWER(A51 -1,$O$4), 0)</f>
+        <v>112053</v>
+      </c>
+      <c r="D51">
+        <f>ROUND($P$3 * POWER(A51 - 1, $P$4), 0)</f>
+        <v>220487</v>
+      </c>
+      <c r="E51">
+        <f>ROUND($Q$3 * POWER(A51 - 1, $Q$4), 0)</f>
+        <v>406736</v>
+      </c>
+      <c r="F51">
+        <f t="shared" si="0"/>
+        <v>1643</v>
+      </c>
+      <c r="G51">
+        <f t="shared" si="1"/>
+        <v>3859</v>
+      </c>
+      <c r="H51">
+        <f t="shared" si="2"/>
+        <v>8033</v>
+      </c>
+      <c r="I51">
+        <f t="shared" si="3"/>
+        <v>15627</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" s="7">
+        <v>51</v>
+      </c>
+      <c r="B52">
+        <f>ROUND( $N$3*POWER(A52-1,$N$4), 0)</f>
+        <v>52282</v>
+      </c>
+      <c r="C52">
+        <f>ROUND($O$3*POWER(A52 -1,$O$4), 0)</f>
+        <v>115969</v>
+      </c>
+      <c r="D52">
+        <f>ROUND($P$3 * POWER(A52 - 1, $P$4), 0)</f>
+        <v>228653</v>
+      </c>
+      <c r="E52">
+        <f>ROUND($Q$3 * POWER(A52 - 1, $Q$4), 0)</f>
+        <v>422652</v>
+      </c>
+      <c r="F52">
+        <f t="shared" si="0"/>
+        <v>1663</v>
+      </c>
+      <c r="G52">
+        <f t="shared" si="1"/>
+        <v>3916</v>
+      </c>
+      <c r="H52">
+        <f t="shared" si="2"/>
+        <v>8166</v>
+      </c>
+      <c r="I52">
+        <f t="shared" si="3"/>
+        <v>15916</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" s="8">
+        <v>52</v>
+      </c>
+      <c r="B53">
+        <f>ROUND( $N$3*POWER(A53-1,$N$4), 0)</f>
+        <v>53965</v>
+      </c>
+      <c r="C53">
+        <f>ROUND($O$3*POWER(A53 -1,$O$4), 0)</f>
+        <v>119939</v>
+      </c>
+      <c r="D53">
+        <f>ROUND($P$3 * POWER(A53 - 1, $P$4), 0)</f>
+        <v>236950</v>
+      </c>
+      <c r="E53">
+        <f>ROUND($Q$3 * POWER(A53 - 1, $Q$4), 0)</f>
+        <v>438857</v>
+      </c>
+      <c r="F53">
+        <f t="shared" si="0"/>
+        <v>1683</v>
+      </c>
+      <c r="G53">
+        <f t="shared" si="1"/>
+        <v>3970</v>
+      </c>
+      <c r="H53">
+        <f t="shared" si="2"/>
+        <v>8297</v>
+      </c>
+      <c r="I53">
+        <f t="shared" si="3"/>
+        <v>16205</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="7">
+        <v>53</v>
+      </c>
+      <c r="B54">
+        <f>ROUND( $N$3*POWER(A54-1,$N$4), 0)</f>
+        <v>55668</v>
+      </c>
+      <c r="C54">
+        <f>ROUND($O$3*POWER(A54 -1,$O$4), 0)</f>
+        <v>123964</v>
+      </c>
+      <c r="D54">
+        <f>ROUND($P$3 * POWER(A54 - 1, $P$4), 0)</f>
+        <v>245378</v>
+      </c>
+      <c r="E54">
+        <f>ROUND($Q$3 * POWER(A54 - 1, $Q$4), 0)</f>
+        <v>455351</v>
+      </c>
+      <c r="F54">
+        <f t="shared" si="0"/>
+        <v>1703</v>
+      </c>
+      <c r="G54">
+        <f t="shared" si="1"/>
+        <v>4025</v>
+      </c>
+      <c r="H54">
+        <f t="shared" si="2"/>
+        <v>8428</v>
+      </c>
+      <c r="I54">
+        <f t="shared" si="3"/>
+        <v>16494</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" s="8">
+        <v>54</v>
+      </c>
+      <c r="B55">
+        <f>ROUND( $N$3*POWER(A55-1,$N$4), 0)</f>
+        <v>57391</v>
+      </c>
+      <c r="C55">
+        <f>ROUND($O$3*POWER(A55 -1,$O$4), 0)</f>
+        <v>128044</v>
+      </c>
+      <c r="D55">
+        <f>ROUND($P$3 * POWER(A55 - 1, $P$4), 0)</f>
+        <v>253937</v>
+      </c>
+      <c r="E55">
+        <f>ROUND($Q$3 * POWER(A55 - 1, $Q$4), 0)</f>
+        <v>472133</v>
+      </c>
+      <c r="F55">
+        <f t="shared" si="0"/>
+        <v>1723</v>
+      </c>
+      <c r="G55">
+        <f t="shared" si="1"/>
+        <v>4080</v>
+      </c>
+      <c r="H55">
+        <f t="shared" si="2"/>
+        <v>8559</v>
+      </c>
+      <c r="I55">
+        <f t="shared" si="3"/>
+        <v>16782</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" s="7">
+        <v>55</v>
+      </c>
+      <c r="B56">
+        <f>ROUND( $N$3*POWER(A56-1,$N$4), 0)</f>
+        <v>59133</v>
+      </c>
+      <c r="C56">
+        <f>ROUND($O$3*POWER(A56 -1,$O$4), 0)</f>
+        <v>132178</v>
+      </c>
+      <c r="D56">
+        <f>ROUND($P$3 * POWER(A56 - 1, $P$4), 0)</f>
+        <v>262627</v>
+      </c>
+      <c r="E56">
+        <f>ROUND($Q$3 * POWER(A56 - 1, $Q$4), 0)</f>
+        <v>489202</v>
+      </c>
+      <c r="F56">
+        <f t="shared" si="0"/>
+        <v>1742</v>
+      </c>
+      <c r="G56">
+        <f t="shared" si="1"/>
+        <v>4134</v>
+      </c>
+      <c r="H56">
+        <f t="shared" si="2"/>
+        <v>8690</v>
+      </c>
+      <c r="I56">
+        <f t="shared" si="3"/>
+        <v>17069</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" s="8">
+        <v>56</v>
+      </c>
+      <c r="B57">
+        <f>ROUND( $N$3*POWER(A57-1,$N$4), 0)</f>
+        <v>60895</v>
+      </c>
+      <c r="C57">
+        <f>ROUND($O$3*POWER(A57 -1,$O$4), 0)</f>
+        <v>136367</v>
+      </c>
+      <c r="D57">
+        <f>ROUND($P$3 * POWER(A57 - 1, $P$4), 0)</f>
+        <v>271446</v>
+      </c>
+      <c r="E57">
+        <f>ROUND($Q$3 * POWER(A57 - 1, $Q$4), 0)</f>
+        <v>506558</v>
+      </c>
+      <c r="F57">
+        <f t="shared" si="0"/>
+        <v>1762</v>
+      </c>
+      <c r="G57">
+        <f t="shared" si="1"/>
+        <v>4189</v>
+      </c>
+      <c r="H57">
+        <f t="shared" si="2"/>
+        <v>8819</v>
+      </c>
+      <c r="I57">
+        <f t="shared" si="3"/>
+        <v>17356</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58" s="7">
+        <v>57</v>
+      </c>
+      <c r="B58">
+        <f>ROUND( $N$3*POWER(A58-1,$N$4), 0)</f>
+        <v>62676</v>
+      </c>
+      <c r="C58">
+        <f>ROUND($O$3*POWER(A58 -1,$O$4), 0)</f>
+        <v>140608</v>
+      </c>
+      <c r="D58">
+        <f>ROUND($P$3 * POWER(A58 - 1, $P$4), 0)</f>
+        <v>280394</v>
+      </c>
+      <c r="E58">
+        <f>ROUND($Q$3 * POWER(A58 - 1, $Q$4), 0)</f>
+        <v>524200</v>
+      </c>
+      <c r="F58">
+        <f t="shared" si="0"/>
+        <v>1781</v>
+      </c>
+      <c r="G58">
+        <f t="shared" si="1"/>
+        <v>4241</v>
+      </c>
+      <c r="H58">
+        <f t="shared" si="2"/>
+        <v>8948</v>
+      </c>
+      <c r="I58">
+        <f t="shared" si="3"/>
+        <v>17642</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A59" s="8">
+        <v>58</v>
+      </c>
+      <c r="B59">
+        <f>ROUND( $N$3*POWER(A59-1,$N$4), 0)</f>
+        <v>64476</v>
+      </c>
+      <c r="C59">
+        <f>ROUND($O$3*POWER(A59 -1,$O$4), 0)</f>
+        <v>144903</v>
+      </c>
+      <c r="D59">
+        <f>ROUND($P$3 * POWER(A59 - 1, $P$4), 0)</f>
+        <v>289471</v>
+      </c>
+      <c r="E59">
+        <f>ROUND($Q$3 * POWER(A59 - 1, $Q$4), 0)</f>
+        <v>542128</v>
+      </c>
+      <c r="F59">
+        <f t="shared" si="0"/>
+        <v>1800</v>
+      </c>
+      <c r="G59">
+        <f t="shared" si="1"/>
+        <v>4295</v>
+      </c>
+      <c r="H59">
+        <f t="shared" si="2"/>
+        <v>9077</v>
+      </c>
+      <c r="I59">
+        <f t="shared" si="3"/>
+        <v>17928</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" s="7">
+        <v>59</v>
+      </c>
+      <c r="B60">
+        <f>ROUND( $N$3*POWER(A60-1,$N$4), 0)</f>
+        <v>66296</v>
+      </c>
+      <c r="C60">
+        <f>ROUND($O$3*POWER(A60 -1,$O$4), 0)</f>
+        <v>149252</v>
+      </c>
+      <c r="D60">
+        <f>ROUND($P$3 * POWER(A60 - 1, $P$4), 0)</f>
+        <v>298676</v>
+      </c>
+      <c r="E60">
+        <f>ROUND($Q$3 * POWER(A60 - 1, $Q$4), 0)</f>
+        <v>560342</v>
+      </c>
+      <c r="F60">
+        <f t="shared" si="0"/>
+        <v>1820</v>
+      </c>
+      <c r="G60">
+        <f t="shared" si="1"/>
+        <v>4349</v>
+      </c>
+      <c r="H60">
+        <f t="shared" si="2"/>
+        <v>9205</v>
+      </c>
+      <c r="I60">
+        <f t="shared" si="3"/>
+        <v>18214</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A61" s="8">
+        <v>60</v>
+      </c>
+      <c r="B61">
+        <f>ROUND( $N$3*POWER(A61-1,$N$4), 0)</f>
+        <v>68134</v>
+      </c>
+      <c r="C61">
+        <f>ROUND($O$3*POWER(A61 -1,$O$4), 0)</f>
+        <v>153653</v>
+      </c>
+      <c r="D61">
+        <f>ROUND($P$3 * POWER(A61 - 1, $P$4), 0)</f>
+        <v>308009</v>
+      </c>
+      <c r="E61">
+        <f>ROUND($Q$3 * POWER(A61 - 1, $Q$4), 0)</f>
+        <v>578840</v>
+      </c>
+      <c r="F61">
+        <f t="shared" si="0"/>
+        <v>1838</v>
+      </c>
+      <c r="G61">
+        <f t="shared" si="1"/>
+        <v>4401</v>
+      </c>
+      <c r="H61">
+        <f t="shared" si="2"/>
+        <v>9333</v>
+      </c>
+      <c r="I61">
+        <f t="shared" si="3"/>
+        <v>18498</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A62" s="7">
+        <v>61</v>
+      </c>
+      <c r="B62">
+        <f>ROUND( $N$3*POWER(A62-1,$N$4), 0)</f>
+        <v>69991</v>
+      </c>
+      <c r="C62">
+        <f>ROUND($O$3*POWER(A62 -1,$O$4), 0)</f>
+        <v>158106</v>
+      </c>
+      <c r="D62">
+        <f>ROUND($P$3 * POWER(A62 - 1, $P$4), 0)</f>
+        <v>317470</v>
+      </c>
+      <c r="E62">
+        <f>ROUND($Q$3 * POWER(A62 - 1, $Q$4), 0)</f>
+        <v>597623</v>
+      </c>
+      <c r="F62">
+        <f t="shared" si="0"/>
+        <v>1857</v>
+      </c>
+      <c r="G62">
+        <f t="shared" si="1"/>
+        <v>4453</v>
+      </c>
+      <c r="H62">
+        <f t="shared" si="2"/>
+        <v>9461</v>
+      </c>
+      <c r="I62">
+        <f t="shared" si="3"/>
+        <v>18783</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A63" s="8">
+        <v>62</v>
+      </c>
+      <c r="B63">
+        <f>ROUND( $N$3*POWER(A63-1,$N$4), 0)</f>
+        <v>71867</v>
+      </c>
+      <c r="C63">
+        <f>ROUND($O$3*POWER(A63 -1,$O$4), 0)</f>
+        <v>162612</v>
+      </c>
+      <c r="D63">
+        <f>ROUND($P$3 * POWER(A63 - 1, $P$4), 0)</f>
+        <v>327057</v>
+      </c>
+      <c r="E63">
+        <f>ROUND($Q$3 * POWER(A63 - 1, $Q$4), 0)</f>
+        <v>616690</v>
+      </c>
+      <c r="F63">
+        <f t="shared" si="0"/>
+        <v>1876</v>
+      </c>
+      <c r="G63">
+        <f t="shared" si="1"/>
+        <v>4506</v>
+      </c>
+      <c r="H63">
+        <f t="shared" si="2"/>
+        <v>9587</v>
+      </c>
+      <c r="I63">
+        <f t="shared" si="3"/>
+        <v>19067</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A64" s="7">
+        <v>63</v>
+      </c>
+      <c r="B64">
+        <f>ROUND( $N$3*POWER(A64-1,$N$4), 0)</f>
+        <v>73761</v>
+      </c>
+      <c r="C64">
+        <f>ROUND($O$3*POWER(A64 -1,$O$4), 0)</f>
+        <v>167170</v>
+      </c>
+      <c r="D64">
+        <f>ROUND($P$3 * POWER(A64 - 1, $P$4), 0)</f>
+        <v>336771</v>
+      </c>
+      <c r="E64">
+        <f>ROUND($Q$3 * POWER(A64 - 1, $Q$4), 0)</f>
+        <v>636040</v>
+      </c>
+      <c r="F64">
+        <f t="shared" si="0"/>
+        <v>1894</v>
+      </c>
+      <c r="G64">
+        <f t="shared" si="1"/>
+        <v>4558</v>
+      </c>
+      <c r="H64">
+        <f t="shared" si="2"/>
+        <v>9714</v>
+      </c>
+      <c r="I64">
+        <f t="shared" si="3"/>
+        <v>19350</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65" s="8">
+        <v>64</v>
+      </c>
+      <c r="B65">
+        <f>ROUND( $N$3*POWER(A65-1,$N$4), 0)</f>
+        <v>75674</v>
+      </c>
+      <c r="C65">
+        <f>ROUND($O$3*POWER(A65 -1,$O$4), 0)</f>
+        <v>171779</v>
+      </c>
+      <c r="D65">
+        <f>ROUND($P$3 * POWER(A65 - 1, $P$4), 0)</f>
+        <v>346612</v>
+      </c>
+      <c r="E65">
+        <f>ROUND($Q$3 * POWER(A65 - 1, $Q$4), 0)</f>
+        <v>655673</v>
+      </c>
+      <c r="F65">
+        <f t="shared" si="0"/>
+        <v>1913</v>
+      </c>
+      <c r="G65">
+        <f t="shared" si="1"/>
+        <v>4609</v>
+      </c>
+      <c r="H65">
+        <f t="shared" si="2"/>
+        <v>9841</v>
+      </c>
+      <c r="I65">
+        <f t="shared" si="3"/>
+        <v>19633</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" s="7">
+        <v>65</v>
+      </c>
+      <c r="B66">
+        <f>ROUND( $N$3*POWER(A66-1,$N$4), 0)</f>
+        <v>77605</v>
+      </c>
+      <c r="C66">
+        <f>ROUND($O$3*POWER(A66 -1,$O$4), 0)</f>
+        <v>176440</v>
+      </c>
+      <c r="D66">
+        <f>ROUND($P$3 * POWER(A66 - 1, $P$4), 0)</f>
+        <v>356578</v>
+      </c>
+      <c r="E66">
+        <f>ROUND($Q$3 * POWER(A66 - 1, $Q$4), 0)</f>
+        <v>675588</v>
+      </c>
+      <c r="F66">
+        <f t="shared" si="0"/>
+        <v>1931</v>
+      </c>
+      <c r="G66">
+        <f t="shared" si="1"/>
+        <v>4661</v>
+      </c>
+      <c r="H66">
+        <f t="shared" si="2"/>
+        <v>9966</v>
+      </c>
+      <c r="I66">
+        <f t="shared" si="3"/>
+        <v>19915</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A67" s="8">
+        <v>66</v>
+      </c>
+      <c r="B67">
+        <f>ROUND( $N$3*POWER(A67-1,$N$4), 0)</f>
+        <v>79554</v>
+      </c>
+      <c r="C67">
+        <f>ROUND($O$3*POWER(A67 -1,$O$4), 0)</f>
+        <v>181152</v>
+      </c>
+      <c r="D67">
+        <f>ROUND($P$3 * POWER(A67 - 1, $P$4), 0)</f>
+        <v>366669</v>
+      </c>
+      <c r="E67">
+        <f>ROUND($Q$3 * POWER(A67 - 1, $Q$4), 0)</f>
+        <v>695786</v>
+      </c>
+      <c r="F67">
+        <f t="shared" si="0"/>
+        <v>1949</v>
+      </c>
+      <c r="G67">
+        <f t="shared" si="1"/>
+        <v>4712</v>
+      </c>
+      <c r="H67">
+        <f t="shared" si="2"/>
+        <v>10091</v>
+      </c>
+      <c r="I67">
+        <f t="shared" si="3"/>
+        <v>20198</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A68" s="7">
+        <v>67</v>
+      </c>
+      <c r="B68">
+        <f>ROUND( $N$3*POWER(A68-1,$N$4), 0)</f>
+        <v>81521</v>
+      </c>
+      <c r="C68">
+        <f>ROUND($O$3*POWER(A68 -1,$O$4), 0)</f>
+        <v>185916</v>
+      </c>
+      <c r="D68">
+        <f>ROUND($P$3 * POWER(A68 - 1, $P$4), 0)</f>
+        <v>376885</v>
+      </c>
+      <c r="E68">
+        <f>ROUND($Q$3 * POWER(A68 - 1, $Q$4), 0)</f>
+        <v>716265</v>
+      </c>
+      <c r="F68">
+        <f t="shared" ref="F68:F101" si="4" xml:space="preserve"> B68-B67</f>
+        <v>1967</v>
+      </c>
+      <c r="G68">
+        <f t="shared" ref="G68:G101" si="5">C68-C67</f>
+        <v>4764</v>
+      </c>
+      <c r="H68">
+        <f t="shared" ref="H68:H101" si="6">D68-D67</f>
+        <v>10216</v>
+      </c>
+      <c r="I68">
+        <f t="shared" ref="I68:I101" si="7">E68-E67</f>
+        <v>20479</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A69" s="8">
+        <v>68</v>
+      </c>
+      <c r="B69">
+        <f>ROUND( $N$3*POWER(A69-1,$N$4), 0)</f>
+        <v>83506</v>
+      </c>
+      <c r="C69">
+        <f>ROUND($O$3*POWER(A69 -1,$O$4), 0)</f>
+        <v>190730</v>
+      </c>
+      <c r="D69">
+        <f>ROUND($P$3 * POWER(A69 - 1, $P$4), 0)</f>
+        <v>387226</v>
+      </c>
+      <c r="E69">
+        <f>ROUND($Q$3 * POWER(A69 - 1, $Q$4), 0)</f>
+        <v>737025</v>
+      </c>
+      <c r="F69">
+        <f t="shared" si="4"/>
+        <v>1985</v>
+      </c>
+      <c r="G69">
+        <f t="shared" si="5"/>
+        <v>4814</v>
+      </c>
+      <c r="H69">
+        <f t="shared" si="6"/>
+        <v>10341</v>
+      </c>
+      <c r="I69">
+        <f t="shared" si="7"/>
+        <v>20760</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A70" s="7">
+        <v>69</v>
+      </c>
+      <c r="B70">
+        <f>ROUND( $N$3*POWER(A70-1,$N$4), 0)</f>
+        <v>85509</v>
+      </c>
+      <c r="C70">
+        <f>ROUND($O$3*POWER(A70 -1,$O$4), 0)</f>
+        <v>195594</v>
+      </c>
+      <c r="D70">
+        <f>ROUND($P$3 * POWER(A70 - 1, $P$4), 0)</f>
+        <v>397691</v>
+      </c>
+      <c r="E70">
+        <f>ROUND($Q$3 * POWER(A70 - 1, $Q$4), 0)</f>
+        <v>758066</v>
+      </c>
+      <c r="F70">
+        <f t="shared" si="4"/>
+        <v>2003</v>
+      </c>
+      <c r="G70">
+        <f t="shared" si="5"/>
+        <v>4864</v>
+      </c>
+      <c r="H70">
+        <f t="shared" si="6"/>
+        <v>10465</v>
+      </c>
+      <c r="I70">
+        <f t="shared" si="7"/>
+        <v>21041</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A71" s="8">
+        <v>70</v>
+      </c>
+      <c r="B71">
+        <f>ROUND( $N$3*POWER(A71-1,$N$4), 0)</f>
+        <v>87530</v>
+      </c>
+      <c r="C71">
+        <f>ROUND($O$3*POWER(A71 -1,$O$4), 0)</f>
+        <v>200509</v>
+      </c>
+      <c r="D71">
+        <f>ROUND($P$3 * POWER(A71 - 1, $P$4), 0)</f>
+        <v>408280</v>
+      </c>
+      <c r="E71">
+        <f>ROUND($Q$3 * POWER(A71 - 1, $Q$4), 0)</f>
+        <v>779387</v>
+      </c>
+      <c r="F71">
+        <f t="shared" si="4"/>
+        <v>2021</v>
+      </c>
+      <c r="G71">
+        <f t="shared" si="5"/>
+        <v>4915</v>
+      </c>
+      <c r="H71">
+        <f t="shared" si="6"/>
+        <v>10589</v>
+      </c>
+      <c r="I71">
+        <f t="shared" si="7"/>
+        <v>21321</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A72" s="7">
+        <v>71</v>
+      </c>
+      <c r="B72">
+        <f>ROUND( $N$3*POWER(A72-1,$N$4), 0)</f>
+        <v>89569</v>
+      </c>
+      <c r="C72">
+        <f>ROUND($O$3*POWER(A72 -1,$O$4), 0)</f>
+        <v>205474</v>
+      </c>
+      <c r="D72">
+        <f>ROUND($P$3 * POWER(A72 - 1, $P$4), 0)</f>
+        <v>418993</v>
+      </c>
+      <c r="E72">
+        <f>ROUND($Q$3 * POWER(A72 - 1, $Q$4), 0)</f>
+        <v>800989</v>
+      </c>
+      <c r="F72">
+        <f t="shared" si="4"/>
+        <v>2039</v>
+      </c>
+      <c r="G72">
+        <f t="shared" si="5"/>
+        <v>4965</v>
+      </c>
+      <c r="H72">
+        <f t="shared" si="6"/>
+        <v>10713</v>
+      </c>
+      <c r="I72">
+        <f t="shared" si="7"/>
+        <v>21602</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A73" s="8">
+        <v>72</v>
+      </c>
+      <c r="B73">
+        <f>ROUND( $N$3*POWER(A73-1,$N$4), 0)</f>
+        <v>91625</v>
+      </c>
+      <c r="C73">
+        <f>ROUND($O$3*POWER(A73 -1,$O$4), 0)</f>
+        <v>210490</v>
+      </c>
+      <c r="D73">
+        <f>ROUND($P$3 * POWER(A73 - 1, $P$4), 0)</f>
+        <v>429828</v>
+      </c>
+      <c r="E73">
+        <f>ROUND($Q$3 * POWER(A73 - 1, $Q$4), 0)</f>
+        <v>822869</v>
+      </c>
+      <c r="F73">
+        <f t="shared" si="4"/>
+        <v>2056</v>
+      </c>
+      <c r="G73">
+        <f t="shared" si="5"/>
+        <v>5016</v>
+      </c>
+      <c r="H73">
+        <f t="shared" si="6"/>
+        <v>10835</v>
+      </c>
+      <c r="I73">
+        <f t="shared" si="7"/>
+        <v>21880</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A74" s="7">
+        <v>73</v>
+      </c>
+      <c r="B74">
+        <f>ROUND( $N$3*POWER(A74-1,$N$4), 0)</f>
+        <v>93698</v>
+      </c>
+      <c r="C74">
+        <f>ROUND($O$3*POWER(A74 -1,$O$4), 0)</f>
+        <v>215554</v>
+      </c>
+      <c r="D74">
+        <f>ROUND($P$3 * POWER(A74 - 1, $P$4), 0)</f>
+        <v>440787</v>
+      </c>
+      <c r="E74">
+        <f>ROUND($Q$3 * POWER(A74 - 1, $Q$4), 0)</f>
+        <v>845029</v>
+      </c>
+      <c r="F74">
+        <f t="shared" si="4"/>
+        <v>2073</v>
+      </c>
+      <c r="G74">
+        <f t="shared" si="5"/>
+        <v>5064</v>
+      </c>
+      <c r="H74">
+        <f t="shared" si="6"/>
+        <v>10959</v>
+      </c>
+      <c r="I74">
+        <f t="shared" si="7"/>
+        <v>22160</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A75" s="8">
+        <v>74</v>
+      </c>
+      <c r="B75">
+        <f>ROUND( $N$3*POWER(A75-1,$N$4), 0)</f>
+        <v>95789</v>
+      </c>
+      <c r="C75">
+        <f>ROUND($O$3*POWER(A75 -1,$O$4), 0)</f>
+        <v>220668</v>
+      </c>
+      <c r="D75">
+        <f>ROUND($P$3 * POWER(A75 - 1, $P$4), 0)</f>
+        <v>451868</v>
+      </c>
+      <c r="E75">
+        <f>ROUND($Q$3 * POWER(A75 - 1, $Q$4), 0)</f>
+        <v>867468</v>
+      </c>
+      <c r="F75">
+        <f t="shared" si="4"/>
+        <v>2091</v>
+      </c>
+      <c r="G75">
+        <f t="shared" si="5"/>
+        <v>5114</v>
+      </c>
+      <c r="H75">
+        <f t="shared" si="6"/>
+        <v>11081</v>
+      </c>
+      <c r="I75">
+        <f t="shared" si="7"/>
+        <v>22439</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A76" s="7">
+        <v>75</v>
+      </c>
+      <c r="B76">
+        <f>ROUND( $N$3*POWER(A76-1,$N$4), 0)</f>
+        <v>97897</v>
+      </c>
+      <c r="C76">
+        <f>ROUND($O$3*POWER(A76 -1,$O$4), 0)</f>
+        <v>225832</v>
+      </c>
+      <c r="D76">
+        <f>ROUND($P$3 * POWER(A76 - 1, $P$4), 0)</f>
+        <v>463070</v>
+      </c>
+      <c r="E76">
+        <f>ROUND($Q$3 * POWER(A76 - 1, $Q$4), 0)</f>
+        <v>890185</v>
+      </c>
+      <c r="F76">
+        <f t="shared" si="4"/>
+        <v>2108</v>
+      </c>
+      <c r="G76">
+        <f t="shared" si="5"/>
+        <v>5164</v>
+      </c>
+      <c r="H76">
+        <f t="shared" si="6"/>
+        <v>11202</v>
+      </c>
+      <c r="I76">
+        <f t="shared" si="7"/>
+        <v>22717</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A77" s="8">
+        <v>76</v>
+      </c>
+      <c r="B77">
+        <f>ROUND( $N$3*POWER(A77-1,$N$4), 0)</f>
+        <v>100023</v>
+      </c>
+      <c r="C77">
+        <f>ROUND($O$3*POWER(A77 -1,$O$4), 0)</f>
+        <v>231044</v>
+      </c>
+      <c r="D77">
+        <f>ROUND($P$3 * POWER(A77 - 1, $P$4), 0)</f>
+        <v>474395</v>
+      </c>
+      <c r="E77">
+        <f>ROUND($Q$3 * POWER(A77 - 1, $Q$4), 0)</f>
+        <v>913180</v>
+      </c>
+      <c r="F77">
+        <f t="shared" si="4"/>
+        <v>2126</v>
+      </c>
+      <c r="G77">
+        <f t="shared" si="5"/>
+        <v>5212</v>
+      </c>
+      <c r="H77">
+        <f t="shared" si="6"/>
+        <v>11325</v>
+      </c>
+      <c r="I77">
+        <f t="shared" si="7"/>
+        <v>22995</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A78" s="7">
+        <v>77</v>
+      </c>
+      <c r="B78">
+        <f>ROUND( $N$3*POWER(A78-1,$N$4), 0)</f>
+        <v>102165</v>
+      </c>
+      <c r="C78">
+        <f>ROUND($O$3*POWER(A78 -1,$O$4), 0)</f>
+        <v>236306</v>
+      </c>
+      <c r="D78">
+        <f>ROUND($P$3 * POWER(A78 - 1, $P$4), 0)</f>
+        <v>485841</v>
+      </c>
+      <c r="E78">
+        <f>ROUND($Q$3 * POWER(A78 - 1, $Q$4), 0)</f>
+        <v>936453</v>
+      </c>
+      <c r="F78">
+        <f t="shared" si="4"/>
+        <v>2142</v>
+      </c>
+      <c r="G78">
+        <f t="shared" si="5"/>
+        <v>5262</v>
+      </c>
+      <c r="H78">
+        <f t="shared" si="6"/>
+        <v>11446</v>
+      </c>
+      <c r="I78">
+        <f t="shared" si="7"/>
+        <v>23273</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A79" s="8">
+        <v>78</v>
+      </c>
+      <c r="B79">
+        <f>ROUND( $N$3*POWER(A79-1,$N$4), 0)</f>
+        <v>104324</v>
+      </c>
+      <c r="C79">
+        <f>ROUND($O$3*POWER(A79 -1,$O$4), 0)</f>
+        <v>241616</v>
+      </c>
+      <c r="D79">
+        <f>ROUND($P$3 * POWER(A79 - 1, $P$4), 0)</f>
+        <v>497409</v>
+      </c>
+      <c r="E79">
+        <f>ROUND($Q$3 * POWER(A79 - 1, $Q$4), 0)</f>
+        <v>960003</v>
+      </c>
+      <c r="F79">
+        <f t="shared" si="4"/>
+        <v>2159</v>
+      </c>
+      <c r="G79">
+        <f t="shared" si="5"/>
+        <v>5310</v>
+      </c>
+      <c r="H79">
+        <f t="shared" si="6"/>
+        <v>11568</v>
+      </c>
+      <c r="I79">
+        <f t="shared" si="7"/>
+        <v>23550</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A80" s="7">
+        <v>79</v>
+      </c>
+      <c r="B80">
+        <f>ROUND( $N$3*POWER(A80-1,$N$4), 0)</f>
+        <v>106500</v>
+      </c>
+      <c r="C80">
+        <f>ROUND($O$3*POWER(A80 -1,$O$4), 0)</f>
+        <v>246974</v>
+      </c>
+      <c r="D80">
+        <f>ROUND($P$3 * POWER(A80 - 1, $P$4), 0)</f>
+        <v>509097</v>
+      </c>
+      <c r="E80">
+        <f>ROUND($Q$3 * POWER(A80 - 1, $Q$4), 0)</f>
+        <v>983829</v>
+      </c>
+      <c r="F80">
+        <f t="shared" si="4"/>
+        <v>2176</v>
+      </c>
+      <c r="G80">
+        <f t="shared" si="5"/>
+        <v>5358</v>
+      </c>
+      <c r="H80">
+        <f t="shared" si="6"/>
+        <v>11688</v>
+      </c>
+      <c r="I80">
+        <f t="shared" si="7"/>
+        <v>23826</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A81" s="8">
+        <v>80</v>
+      </c>
+      <c r="B81">
+        <f>ROUND( $N$3*POWER(A81-1,$N$4), 0)</f>
+        <v>108693</v>
+      </c>
+      <c r="C81">
+        <f>ROUND($O$3*POWER(A81 -1,$O$4), 0)</f>
+        <v>252381</v>
+      </c>
+      <c r="D81">
+        <f>ROUND($P$3 * POWER(A81 - 1, $P$4), 0)</f>
+        <v>520905</v>
+      </c>
+      <c r="E81">
+        <f>ROUND($Q$3 * POWER(A81 - 1, $Q$4), 0)</f>
+        <v>1007933</v>
+      </c>
+      <c r="F81">
+        <f t="shared" si="4"/>
+        <v>2193</v>
+      </c>
+      <c r="G81">
+        <f t="shared" si="5"/>
+        <v>5407</v>
+      </c>
+      <c r="H81">
+        <f t="shared" si="6"/>
+        <v>11808</v>
+      </c>
+      <c r="I81">
+        <f t="shared" si="7"/>
+        <v>24104</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A82" s="7">
+        <v>81</v>
+      </c>
+      <c r="B82">
+        <f>ROUND( $N$3*POWER(A82-1,$N$4), 0)</f>
+        <v>110903</v>
+      </c>
+      <c r="C82">
+        <f>ROUND($O$3*POWER(A82 -1,$O$4), 0)</f>
+        <v>257836</v>
+      </c>
+      <c r="D82">
+        <f>ROUND($P$3 * POWER(A82 - 1, $P$4), 0)</f>
+        <v>532834</v>
+      </c>
+      <c r="E82">
+        <f>ROUND($Q$3 * POWER(A82 - 1, $Q$4), 0)</f>
+        <v>1032312</v>
+      </c>
+      <c r="F82">
+        <f t="shared" si="4"/>
+        <v>2210</v>
+      </c>
+      <c r="G82">
+        <f t="shared" si="5"/>
+        <v>5455</v>
+      </c>
+      <c r="H82">
+        <f t="shared" si="6"/>
+        <v>11929</v>
+      </c>
+      <c r="I82">
+        <f t="shared" si="7"/>
+        <v>24379</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A83" s="8">
+        <v>82</v>
+      </c>
+      <c r="B83">
+        <f>ROUND( $N$3*POWER(A83-1,$N$4), 0)</f>
+        <v>113130</v>
+      </c>
+      <c r="C83">
+        <f>ROUND($O$3*POWER(A83 -1,$O$4), 0)</f>
+        <v>263339</v>
+      </c>
+      <c r="D83">
+        <f>ROUND($P$3 * POWER(A83 - 1, $P$4), 0)</f>
+        <v>544883</v>
+      </c>
+      <c r="E83">
+        <f>ROUND($Q$3 * POWER(A83 - 1, $Q$4), 0)</f>
+        <v>1056967</v>
+      </c>
+      <c r="F83">
+        <f t="shared" si="4"/>
+        <v>2227</v>
+      </c>
+      <c r="G83">
+        <f t="shared" si="5"/>
+        <v>5503</v>
+      </c>
+      <c r="H83">
+        <f t="shared" si="6"/>
+        <v>12049</v>
+      </c>
+      <c r="I83">
+        <f t="shared" si="7"/>
+        <v>24655</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A84" s="7">
+        <v>83</v>
+      </c>
+      <c r="B84">
+        <f>ROUND( $N$3*POWER(A84-1,$N$4), 0)</f>
+        <v>115372</v>
+      </c>
+      <c r="C84">
+        <f>ROUND($O$3*POWER(A84 -1,$O$4), 0)</f>
+        <v>268890</v>
+      </c>
+      <c r="D84">
+        <f>ROUND($P$3 * POWER(A84 - 1, $P$4), 0)</f>
+        <v>557051</v>
+      </c>
+      <c r="E84">
+        <f>ROUND($Q$3 * POWER(A84 - 1, $Q$4), 0)</f>
+        <v>1081898</v>
+      </c>
+      <c r="F84">
+        <f t="shared" si="4"/>
+        <v>2242</v>
+      </c>
+      <c r="G84">
+        <f t="shared" si="5"/>
+        <v>5551</v>
+      </c>
+      <c r="H84">
+        <f t="shared" si="6"/>
+        <v>12168</v>
+      </c>
+      <c r="I84">
+        <f t="shared" si="7"/>
+        <v>24931</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A85" s="8">
+        <v>84</v>
+      </c>
+      <c r="B85">
+        <f>ROUND( $N$3*POWER(A85-1,$N$4), 0)</f>
+        <v>117632</v>
+      </c>
+      <c r="C85">
+        <f>ROUND($O$3*POWER(A85 -1,$O$4), 0)</f>
+        <v>274488</v>
+      </c>
+      <c r="D85">
+        <f>ROUND($P$3 * POWER(A85 - 1, $P$4), 0)</f>
+        <v>569339</v>
+      </c>
+      <c r="E85">
+        <f>ROUND($Q$3 * POWER(A85 - 1, $Q$4), 0)</f>
+        <v>1107104</v>
+      </c>
+      <c r="F85">
+        <f t="shared" si="4"/>
+        <v>2260</v>
+      </c>
+      <c r="G85">
+        <f t="shared" si="5"/>
+        <v>5598</v>
+      </c>
+      <c r="H85">
+        <f t="shared" si="6"/>
+        <v>12288</v>
+      </c>
+      <c r="I85">
+        <f t="shared" si="7"/>
+        <v>25206</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A86" s="7">
+        <v>85</v>
+      </c>
+      <c r="B86">
+        <f>ROUND( $N$3*POWER(A86-1,$N$4), 0)</f>
+        <v>119908</v>
+      </c>
+      <c r="C86">
+        <f>ROUND($O$3*POWER(A86 -1,$O$4), 0)</f>
+        <v>280134</v>
+      </c>
+      <c r="D86">
+        <f>ROUND($P$3 * POWER(A86 - 1, $P$4), 0)</f>
+        <v>581745</v>
+      </c>
+      <c r="E86">
+        <f>ROUND($Q$3 * POWER(A86 - 1, $Q$4), 0)</f>
+        <v>1132585</v>
+      </c>
+      <c r="F86">
+        <f t="shared" si="4"/>
+        <v>2276</v>
+      </c>
+      <c r="G86">
+        <f t="shared" si="5"/>
+        <v>5646</v>
+      </c>
+      <c r="H86">
+        <f t="shared" si="6"/>
+        <v>12406</v>
+      </c>
+      <c r="I86">
+        <f t="shared" si="7"/>
+        <v>25481</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A87" s="8">
+        <v>86</v>
+      </c>
+      <c r="B87">
+        <f>ROUND( $N$3*POWER(A87-1,$N$4), 0)</f>
+        <v>122200</v>
+      </c>
+      <c r="C87">
+        <f>ROUND($O$3*POWER(A87 -1,$O$4), 0)</f>
+        <v>285827</v>
+      </c>
+      <c r="D87">
+        <f>ROUND($P$3 * POWER(A87 - 1, $P$4), 0)</f>
+        <v>594270</v>
+      </c>
+      <c r="E87">
+        <f>ROUND($Q$3 * POWER(A87 - 1, $Q$4), 0)</f>
+        <v>1158340</v>
+      </c>
+      <c r="F87">
+        <f t="shared" si="4"/>
+        <v>2292</v>
+      </c>
+      <c r="G87">
+        <f t="shared" si="5"/>
+        <v>5693</v>
+      </c>
+      <c r="H87">
+        <f t="shared" si="6"/>
+        <v>12525</v>
+      </c>
+      <c r="I87">
+        <f t="shared" si="7"/>
+        <v>25755</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A88" s="7">
+        <v>87</v>
+      </c>
+      <c r="B88">
+        <f>ROUND( $N$3*POWER(A88-1,$N$4), 0)</f>
+        <v>124508</v>
+      </c>
+      <c r="C88">
+        <f>ROUND($O$3*POWER(A88 -1,$O$4), 0)</f>
+        <v>291567</v>
+      </c>
+      <c r="D88">
+        <f>ROUND($P$3 * POWER(A88 - 1, $P$4), 0)</f>
+        <v>606914</v>
+      </c>
+      <c r="E88">
+        <f>ROUND($Q$3 * POWER(A88 - 1, $Q$4), 0)</f>
+        <v>1184369</v>
+      </c>
+      <c r="F88">
+        <f t="shared" si="4"/>
+        <v>2308</v>
+      </c>
+      <c r="G88">
+        <f t="shared" si="5"/>
+        <v>5740</v>
+      </c>
+      <c r="H88">
+        <f t="shared" si="6"/>
+        <v>12644</v>
+      </c>
+      <c r="I88">
+        <f t="shared" si="7"/>
+        <v>26029</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A89" s="8">
+        <v>88</v>
+      </c>
+      <c r="B89">
+        <f>ROUND( $N$3*POWER(A89-1,$N$4), 0)</f>
+        <v>126833</v>
+      </c>
+      <c r="C89">
+        <f>ROUND($O$3*POWER(A89 -1,$O$4), 0)</f>
+        <v>297354</v>
+      </c>
+      <c r="D89">
+        <f>ROUND($P$3 * POWER(A89 - 1, $P$4), 0)</f>
+        <v>619676</v>
+      </c>
+      <c r="E89">
+        <f>ROUND($Q$3 * POWER(A89 - 1, $Q$4), 0)</f>
+        <v>1210672</v>
+      </c>
+      <c r="F89">
+        <f t="shared" si="4"/>
+        <v>2325</v>
+      </c>
+      <c r="G89">
+        <f t="shared" si="5"/>
+        <v>5787</v>
+      </c>
+      <c r="H89">
+        <f t="shared" si="6"/>
+        <v>12762</v>
+      </c>
+      <c r="I89">
+        <f t="shared" si="7"/>
+        <v>26303</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A90" s="7">
+        <v>89</v>
+      </c>
+      <c r="B90">
+        <f>ROUND( $N$3*POWER(A90-1,$N$4), 0)</f>
+        <v>129173</v>
+      </c>
+      <c r="C90">
+        <f>ROUND($O$3*POWER(A90 -1,$O$4), 0)</f>
+        <v>303188</v>
+      </c>
+      <c r="D90">
+        <f>ROUND($P$3 * POWER(A90 - 1, $P$4), 0)</f>
+        <v>632556</v>
+      </c>
+      <c r="E90">
+        <f>ROUND($Q$3 * POWER(A90 - 1, $Q$4), 0)</f>
+        <v>1237249</v>
+      </c>
+      <c r="F90">
+        <f t="shared" si="4"/>
+        <v>2340</v>
+      </c>
+      <c r="G90">
+        <f t="shared" si="5"/>
+        <v>5834</v>
+      </c>
+      <c r="H90">
+        <f t="shared" si="6"/>
+        <v>12880</v>
+      </c>
+      <c r="I90">
+        <f t="shared" si="7"/>
+        <v>26577</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A91" s="8">
+        <v>90</v>
+      </c>
+      <c r="B91">
+        <f>ROUND( $N$3*POWER(A91-1,$N$4), 0)</f>
+        <v>131530</v>
+      </c>
+      <c r="C91">
+        <f>ROUND($O$3*POWER(A91 -1,$O$4), 0)</f>
+        <v>309068</v>
+      </c>
+      <c r="D91">
+        <f>ROUND($P$3 * POWER(A91 - 1, $P$4), 0)</f>
+        <v>645553</v>
+      </c>
+      <c r="E91">
+        <f>ROUND($Q$3 * POWER(A91 - 1, $Q$4), 0)</f>
+        <v>1264099</v>
+      </c>
+      <c r="F91">
+        <f t="shared" si="4"/>
+        <v>2357</v>
+      </c>
+      <c r="G91">
+        <f t="shared" si="5"/>
+        <v>5880</v>
+      </c>
+      <c r="H91">
+        <f t="shared" si="6"/>
+        <v>12997</v>
+      </c>
+      <c r="I91">
+        <f t="shared" si="7"/>
+        <v>26850</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A92" s="7">
+        <v>91</v>
+      </c>
+      <c r="B92">
+        <f>ROUND( $N$3*POWER(A92-1,$N$4), 0)</f>
+        <v>133902</v>
+      </c>
+      <c r="C92">
+        <f>ROUND($O$3*POWER(A92 -1,$O$4), 0)</f>
+        <v>314995</v>
+      </c>
+      <c r="D92">
+        <f>ROUND($P$3 * POWER(A92 - 1, $P$4), 0)</f>
+        <v>658668</v>
+      </c>
+      <c r="E92">
+        <f>ROUND($Q$3 * POWER(A92 - 1, $Q$4), 0)</f>
+        <v>1291222</v>
+      </c>
+      <c r="F92">
+        <f t="shared" si="4"/>
+        <v>2372</v>
+      </c>
+      <c r="G92">
+        <f t="shared" si="5"/>
+        <v>5927</v>
+      </c>
+      <c r="H92">
+        <f t="shared" si="6"/>
+        <v>13115</v>
+      </c>
+      <c r="I92">
+        <f t="shared" si="7"/>
+        <v>27123</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A93" s="8">
+        <v>92</v>
+      </c>
+      <c r="B93">
+        <f>ROUND( $N$3*POWER(A93-1,$N$4), 0)</f>
+        <v>136291</v>
+      </c>
+      <c r="C93">
+        <f>ROUND($O$3*POWER(A93 -1,$O$4), 0)</f>
+        <v>320968</v>
+      </c>
+      <c r="D93">
+        <f>ROUND($P$3 * POWER(A93 - 1, $P$4), 0)</f>
+        <v>671900</v>
+      </c>
+      <c r="E93">
+        <f>ROUND($Q$3 * POWER(A93 - 1, $Q$4), 0)</f>
+        <v>1318617</v>
+      </c>
+      <c r="F93">
+        <f t="shared" si="4"/>
+        <v>2389</v>
+      </c>
+      <c r="G93">
+        <f t="shared" si="5"/>
+        <v>5973</v>
+      </c>
+      <c r="H93">
+        <f t="shared" si="6"/>
+        <v>13232</v>
+      </c>
+      <c r="I93">
+        <f t="shared" si="7"/>
+        <v>27395</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A94" s="7">
+        <v>93</v>
+      </c>
+      <c r="B94">
+        <f>ROUND( $N$3*POWER(A94-1,$N$4), 0)</f>
+        <v>138695</v>
+      </c>
+      <c r="C94">
+        <f>ROUND($O$3*POWER(A94 -1,$O$4), 0)</f>
+        <v>326987</v>
+      </c>
+      <c r="D94">
+        <f>ROUND($P$3 * POWER(A94 - 1, $P$4), 0)</f>
+        <v>685248</v>
+      </c>
+      <c r="E94">
+        <f>ROUND($Q$3 * POWER(A94 - 1, $Q$4), 0)</f>
+        <v>1346285</v>
+      </c>
+      <c r="F94">
+        <f t="shared" si="4"/>
+        <v>2404</v>
+      </c>
+      <c r="G94">
+        <f t="shared" si="5"/>
+        <v>6019</v>
+      </c>
+      <c r="H94">
+        <f t="shared" si="6"/>
+        <v>13348</v>
+      </c>
+      <c r="I94">
+        <f t="shared" si="7"/>
+        <v>27668</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A95" s="8">
+        <v>94</v>
+      </c>
+      <c r="B95">
+        <f>ROUND( $N$3*POWER(A95-1,$N$4), 0)</f>
+        <v>141115</v>
+      </c>
+      <c r="C95">
+        <f>ROUND($O$3*POWER(A95 -1,$O$4), 0)</f>
+        <v>333052</v>
+      </c>
+      <c r="D95">
+        <f>ROUND($P$3 * POWER(A95 - 1, $P$4), 0)</f>
+        <v>698714</v>
+      </c>
+      <c r="E95">
+        <f>ROUND($Q$3 * POWER(A95 - 1, $Q$4), 0)</f>
+        <v>1374224</v>
+      </c>
+      <c r="F95">
+        <f t="shared" si="4"/>
+        <v>2420</v>
+      </c>
+      <c r="G95">
+        <f t="shared" si="5"/>
+        <v>6065</v>
+      </c>
+      <c r="H95">
+        <f t="shared" si="6"/>
+        <v>13466</v>
+      </c>
+      <c r="I95">
+        <f t="shared" si="7"/>
+        <v>27939</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A96" s="7">
+        <v>95</v>
+      </c>
+      <c r="B96">
+        <f>ROUND( $N$3*POWER(A96-1,$N$4), 0)</f>
+        <v>143550</v>
+      </c>
+      <c r="C96">
+        <f>ROUND($O$3*POWER(A96 -1,$O$4), 0)</f>
+        <v>339163</v>
+      </c>
+      <c r="D96">
+        <f>ROUND($P$3 * POWER(A96 - 1, $P$4), 0)</f>
+        <v>712295</v>
+      </c>
+      <c r="E96">
+        <f>ROUND($Q$3 * POWER(A96 - 1, $Q$4), 0)</f>
+        <v>1402436</v>
+      </c>
+      <c r="F96">
+        <f t="shared" si="4"/>
+        <v>2435</v>
+      </c>
+      <c r="G96">
+        <f t="shared" si="5"/>
+        <v>6111</v>
+      </c>
+      <c r="H96">
+        <f t="shared" si="6"/>
+        <v>13581</v>
+      </c>
+      <c r="I96">
+        <f t="shared" si="7"/>
+        <v>28212</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A97" s="8">
+        <v>96</v>
+      </c>
+      <c r="B97">
+        <f>ROUND( $N$3*POWER(A97-1,$N$4), 0)</f>
+        <v>146002</v>
+      </c>
+      <c r="C97">
+        <f>ROUND($O$3*POWER(A97 -1,$O$4), 0)</f>
+        <v>345320</v>
+      </c>
+      <c r="D97">
+        <f>ROUND($P$3 * POWER(A97 - 1, $P$4), 0)</f>
+        <v>725993</v>
+      </c>
+      <c r="E97">
+        <f>ROUND($Q$3 * POWER(A97 - 1, $Q$4), 0)</f>
+        <v>1430918</v>
+      </c>
+      <c r="F97">
+        <f t="shared" si="4"/>
+        <v>2452</v>
+      </c>
+      <c r="G97">
+        <f t="shared" si="5"/>
+        <v>6157</v>
+      </c>
+      <c r="H97">
+        <f t="shared" si="6"/>
+        <v>13698</v>
+      </c>
+      <c r="I97">
+        <f t="shared" si="7"/>
+        <v>28482</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A98" s="7">
+        <v>97</v>
+      </c>
+      <c r="B98">
+        <f>ROUND( $N$3*POWER(A98-1,$N$4), 0)</f>
+        <v>148468</v>
+      </c>
+      <c r="C98">
+        <f>ROUND($O$3*POWER(A98 -1,$O$4), 0)</f>
+        <v>351522</v>
+      </c>
+      <c r="D98">
+        <f>ROUND($P$3 * POWER(A98 - 1, $P$4), 0)</f>
+        <v>739807</v>
+      </c>
+      <c r="E98">
+        <f>ROUND($Q$3 * POWER(A98 - 1, $Q$4), 0)</f>
+        <v>1459672</v>
+      </c>
+      <c r="F98">
+        <f t="shared" si="4"/>
+        <v>2466</v>
+      </c>
+      <c r="G98">
+        <f t="shared" si="5"/>
+        <v>6202</v>
+      </c>
+      <c r="H98">
+        <f t="shared" si="6"/>
+        <v>13814</v>
+      </c>
+      <c r="I98">
+        <f t="shared" si="7"/>
+        <v>28754</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A99" s="8">
+        <v>98</v>
+      </c>
+      <c r="B99">
+        <f>ROUND( $N$3*POWER(A99-1,$N$4), 0)</f>
+        <v>150951</v>
+      </c>
+      <c r="C99">
+        <f>ROUND($O$3*POWER(A99 -1,$O$4), 0)</f>
+        <v>357769</v>
+      </c>
+      <c r="D99">
+        <f>ROUND($P$3 * POWER(A99 - 1, $P$4), 0)</f>
+        <v>753736</v>
+      </c>
+      <c r="E99">
+        <f>ROUND($Q$3 * POWER(A99 - 1, $Q$4), 0)</f>
+        <v>1488697</v>
+      </c>
+      <c r="F99">
+        <f t="shared" si="4"/>
+        <v>2483</v>
+      </c>
+      <c r="G99">
+        <f t="shared" si="5"/>
+        <v>6247</v>
+      </c>
+      <c r="H99">
+        <f t="shared" si="6"/>
+        <v>13929</v>
+      </c>
+      <c r="I99">
+        <f t="shared" si="7"/>
+        <v>29025</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A100" s="7">
+        <v>99</v>
+      </c>
+      <c r="B100">
+        <f>ROUND( $N$3*POWER(A100-1,$N$4), 0)</f>
+        <v>153448</v>
+      </c>
+      <c r="C100">
+        <f>ROUND($O$3*POWER(A100 -1,$O$4), 0)</f>
+        <v>364062</v>
+      </c>
+      <c r="D100">
+        <f>ROUND($P$3 * POWER(A100 - 1, $P$4), 0)</f>
+        <v>767780</v>
+      </c>
+      <c r="E100">
+        <f>ROUND($Q$3 * POWER(A100 - 1, $Q$4), 0)</f>
+        <v>1517992</v>
+      </c>
+      <c r="F100">
+        <f t="shared" si="4"/>
+        <v>2497</v>
+      </c>
+      <c r="G100">
+        <f t="shared" si="5"/>
+        <v>6293</v>
+      </c>
+      <c r="H100">
+        <f t="shared" si="6"/>
+        <v>14044</v>
+      </c>
+      <c r="I100">
+        <f t="shared" si="7"/>
+        <v>29295</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A101" s="8">
+        <v>100</v>
+      </c>
+      <c r="B101">
+        <f>ROUND( $N$3*POWER(A101-1,$N$4), 0)</f>
+        <v>155961</v>
+      </c>
+      <c r="C101">
+        <f>ROUND($O$3*POWER(A101 -1,$O$4), 0)</f>
+        <v>370400</v>
+      </c>
+      <c r="D101">
+        <f>ROUND($P$3 * POWER(A101 - 1, $P$4), 0)</f>
+        <v>781940</v>
+      </c>
+      <c r="E101">
+        <f>ROUND($Q$3 * POWER(A101 - 1, $Q$4), 0)</f>
+        <v>1547558</v>
+      </c>
+      <c r="F101">
+        <f t="shared" si="4"/>
+        <v>2513</v>
+      </c>
+      <c r="G101">
+        <f t="shared" si="5"/>
+        <v>6338</v>
+      </c>
+      <c r="H101">
+        <f t="shared" si="6"/>
+        <v>14160</v>
+      </c>
+      <c r="I101">
+        <f t="shared" si="7"/>
+        <v>29566</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>503</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>504</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>505</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>506</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>507</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>509</v>
+      </c>
+      <c r="B2" s="8">
+        <v>1</v>
+      </c>
+      <c r="C2" s="8">
+        <v>20</v>
+      </c>
+      <c r="D2" s="8">
+        <v>40</v>
+      </c>
+      <c r="E2" s="8">
+        <v>10000</v>
+      </c>
+      <c r="F2" t="s">
+        <v>124</v>
+      </c>
+      <c r="G2" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B3" s="8">
+        <v>2</v>
+      </c>
+      <c r="C3" s="8">
+        <v>40</v>
+      </c>
+      <c r="D3" s="8">
+        <v>60</v>
+      </c>
+      <c r="E3" s="8">
+        <v>50000</v>
+      </c>
+      <c r="F3" t="s">
+        <v>124</v>
+      </c>
+      <c r="G3" s="8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>509</v>
+      </c>
+      <c r="B4" s="8">
+        <v>3</v>
+      </c>
+      <c r="C4" s="8">
+        <v>60</v>
+      </c>
+      <c r="D4" s="8">
+        <v>80</v>
+      </c>
+      <c r="E4" s="8">
+        <v>200000</v>
+      </c>
+      <c r="F4" t="s">
+        <v>124</v>
+      </c>
+      <c r="G4" s="8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>509</v>
+      </c>
+      <c r="B5" s="8">
+        <v>4</v>
+      </c>
+      <c r="C5" s="8">
+        <v>80</v>
+      </c>
+      <c r="D5" s="8">
+        <v>100</v>
+      </c>
+      <c r="E5" s="8">
+        <v>500000</v>
+      </c>
+      <c r="F5" t="s">
+        <v>124</v>
+      </c>
+      <c r="G5" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>510</v>
+      </c>
+      <c r="B6" s="8">
+        <v>1</v>
+      </c>
+      <c r="C6" s="8">
+        <v>20</v>
+      </c>
+      <c r="D6" s="8">
+        <v>40</v>
+      </c>
+      <c r="E6" s="8">
+        <v>10000</v>
+      </c>
+      <c r="F6" t="s">
+        <v>124</v>
+      </c>
+      <c r="G6" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>510</v>
+      </c>
+      <c r="B7" s="8">
+        <v>2</v>
+      </c>
+      <c r="C7" s="8">
+        <v>40</v>
+      </c>
+      <c r="D7" s="8">
+        <v>60</v>
+      </c>
+      <c r="E7" s="8">
+        <v>50000</v>
+      </c>
+      <c r="F7" t="s">
+        <v>124</v>
+      </c>
+      <c r="G7" s="8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>510</v>
+      </c>
+      <c r="B8" s="8">
+        <v>3</v>
+      </c>
+      <c r="C8" s="8">
+        <v>60</v>
+      </c>
+      <c r="D8" s="8">
+        <v>80</v>
+      </c>
+      <c r="E8" s="8">
+        <v>200000</v>
+      </c>
+      <c r="F8" t="s">
+        <v>124</v>
+      </c>
+      <c r="G8" s="8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>510</v>
+      </c>
+      <c r="B9" s="8">
+        <v>4</v>
+      </c>
+      <c r="C9" s="8">
+        <v>80</v>
+      </c>
+      <c r="D9" s="8">
+        <v>100</v>
+      </c>
+      <c r="E9" s="8">
+        <v>500000</v>
+      </c>
+      <c r="F9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G9" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>511</v>
+      </c>
+      <c r="B10" s="8">
+        <v>1</v>
+      </c>
+      <c r="C10" s="8">
+        <v>20</v>
+      </c>
+      <c r="D10" s="8">
+        <v>40</v>
+      </c>
+      <c r="E10" s="8">
+        <v>10000</v>
+      </c>
+      <c r="F10" t="s">
+        <v>124</v>
+      </c>
+      <c r="G10" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>511</v>
+      </c>
+      <c r="B11" s="8">
+        <v>2</v>
+      </c>
+      <c r="C11" s="8">
+        <v>40</v>
+      </c>
+      <c r="D11" s="8">
+        <v>60</v>
+      </c>
+      <c r="E11" s="8">
+        <v>50000</v>
+      </c>
+      <c r="F11" t="s">
+        <v>124</v>
+      </c>
+      <c r="G11" s="8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>511</v>
+      </c>
+      <c r="B12" s="8">
+        <v>3</v>
+      </c>
+      <c r="C12" s="8">
+        <v>60</v>
+      </c>
+      <c r="D12" s="8">
+        <v>80</v>
+      </c>
+      <c r="E12" s="8">
+        <v>200000</v>
+      </c>
+      <c r="F12" t="s">
+        <v>124</v>
+      </c>
+      <c r="G12" s="8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>511</v>
+      </c>
+      <c r="B13" s="8">
+        <v>4</v>
+      </c>
+      <c r="C13" s="8">
+        <v>80</v>
+      </c>
+      <c r="D13" s="8">
+        <v>100</v>
+      </c>
+      <c r="E13" s="8">
+        <v>500000</v>
+      </c>
+      <c r="F13" t="s">
+        <v>124</v>
+      </c>
+      <c r="G13" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>512</v>
+      </c>
+      <c r="B14" s="8">
+        <v>1</v>
+      </c>
+      <c r="C14" s="8">
+        <v>20</v>
+      </c>
+      <c r="D14" s="8">
+        <v>40</v>
+      </c>
+      <c r="E14" s="8">
+        <v>10000</v>
+      </c>
+      <c r="F14" t="s">
+        <v>124</v>
+      </c>
+      <c r="G14" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>512</v>
+      </c>
+      <c r="B15" s="8">
+        <v>2</v>
+      </c>
+      <c r="C15" s="8">
+        <v>40</v>
+      </c>
+      <c r="D15" s="8">
+        <v>60</v>
+      </c>
+      <c r="E15" s="8">
+        <v>50000</v>
+      </c>
+      <c r="F15" t="s">
+        <v>124</v>
+      </c>
+      <c r="G15" s="8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>512</v>
+      </c>
+      <c r="B16" s="8">
+        <v>3</v>
+      </c>
+      <c r="C16" s="8">
+        <v>60</v>
+      </c>
+      <c r="D16" s="8">
+        <v>80</v>
+      </c>
+      <c r="E16" s="8">
+        <v>200000</v>
+      </c>
+      <c r="F16" t="s">
+        <v>124</v>
+      </c>
+      <c r="G16" s="8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>512</v>
+      </c>
+      <c r="B17" s="8">
+        <v>4</v>
+      </c>
+      <c r="C17" s="8">
+        <v>80</v>
+      </c>
+      <c r="D17" s="8">
+        <v>100</v>
+      </c>
+      <c r="E17" s="8">
+        <v>500000</v>
+      </c>
+      <c r="F17" t="s">
+        <v>124</v>
+      </c>
+      <c r="G17" s="8">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4379,7 +8638,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
+ Inject runtime data to character in battle.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -10847,7 +10847,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.5703125" customWidth="1"/>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
+ Lazy Loading for UI Framework to prepare for matching VContainer.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -9679,10 +9679,10 @@
         <v>165</v>
       </c>
       <c r="E2" s="10">
-        <v>420</v>
+        <v>42</v>
       </c>
       <c r="F2" s="10">
-        <v>270</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -9699,10 +9699,10 @@
         <v>151</v>
       </c>
       <c r="E3" s="10">
-        <v>435</v>
+        <v>43</v>
       </c>
       <c r="F3" s="10">
-        <v>250</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -9719,10 +9719,10 @@
         <v>236</v>
       </c>
       <c r="E4" s="10">
-        <v>410</v>
+        <v>41</v>
       </c>
       <c r="F4" s="10">
-        <v>290</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -9739,10 +9739,10 @@
         <v>78</v>
       </c>
       <c r="E5" s="10">
-        <v>210</v>
+        <v>21</v>
       </c>
       <c r="F5" s="10">
-        <v>140</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -9759,10 +9759,10 @@
         <v>90</v>
       </c>
       <c r="E6" s="10">
-        <v>450</v>
+        <v>45</v>
       </c>
       <c r="F6" s="10">
-        <v>160</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -9779,10 +9779,10 @@
         <v>74</v>
       </c>
       <c r="E7" s="10">
-        <v>210</v>
+        <v>21</v>
       </c>
       <c r="F7" s="10">
-        <v>136</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -9799,10 +9799,10 @@
         <v>53</v>
       </c>
       <c r="E8" s="10">
-        <v>130</v>
+        <v>13</v>
       </c>
       <c r="F8" s="10">
-        <v>104</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -9819,10 +9819,10 @@
         <v>143</v>
       </c>
       <c r="E9" s="10">
-        <v>360</v>
+        <v>36</v>
       </c>
       <c r="F9" s="10">
-        <v>240</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -9839,10 +9839,10 @@
         <v>64</v>
       </c>
       <c r="E10" s="10">
-        <v>180</v>
+        <v>18</v>
       </c>
       <c r="F10" s="10">
-        <v>124</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -9859,10 +9859,10 @@
         <v>53</v>
       </c>
       <c r="E11" s="10">
-        <v>130</v>
+        <v>13</v>
       </c>
       <c r="F11" s="10">
-        <v>104</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -9879,10 +9879,10 @@
         <v>64</v>
       </c>
       <c r="E12" s="10">
-        <v>190</v>
+        <v>19</v>
       </c>
       <c r="F12" s="10">
-        <v>114</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -9899,10 +9899,10 @@
         <v>134</v>
       </c>
       <c r="E13" s="10">
-        <v>380</v>
+        <v>38</v>
       </c>
       <c r="F13" s="10">
-        <v>230</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -9919,10 +9919,10 @@
         <v>140</v>
       </c>
       <c r="E14" s="10">
-        <v>360</v>
+        <v>36</v>
       </c>
       <c r="F14" s="10">
-        <v>210</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -9939,10 +9939,10 @@
         <v>110</v>
       </c>
       <c r="E15" s="10">
-        <v>395</v>
+        <v>39</v>
       </c>
       <c r="F15" s="10">
-        <v>210</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -9959,10 +9959,10 @@
         <v>165</v>
       </c>
       <c r="E16" s="10">
-        <v>420</v>
+        <v>42</v>
       </c>
       <c r="F16" s="10">
-        <v>270</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Add feature level up for weapon and build passive data.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,25 +4,26 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
     <sheet name="Item_Detail" sheetId="3" r:id="rId2"/>
     <sheet name="Weapon" sheetId="2" r:id="rId3"/>
-    <sheet name="Armor" sheetId="4" r:id="rId4"/>
-    <sheet name="SetBonusConfig" sheetId="16" r:id="rId5"/>
-    <sheet name="Character" sheetId="5" r:id="rId6"/>
-    <sheet name="SkillConfig" sheetId="11" r:id="rId7"/>
-    <sheet name="EffectConfig" sheetId="12" r:id="rId8"/>
-    <sheet name="CharacterStat" sheetId="6" r:id="rId9"/>
-    <sheet name="CharacterAttribute" sheetId="8" r:id="rId10"/>
-    <sheet name="CharacterUpgrade" sheetId="7" r:id="rId11"/>
-    <sheet name="ExpCurvesConfig" sheetId="13" r:id="rId12"/>
-    <sheet name="AscensionConfig" sheetId="14" r:id="rId13"/>
-    <sheet name="StarUp" sheetId="15" r:id="rId14"/>
-    <sheet name="BattleConfig" sheetId="9" r:id="rId15"/>
-    <sheet name="StageEnemies" sheetId="10" r:id="rId16"/>
+    <sheet name="PassiveConfig" sheetId="17" r:id="rId4"/>
+    <sheet name="Armor" sheetId="4" r:id="rId5"/>
+    <sheet name="SetBonusConfig" sheetId="16" r:id="rId6"/>
+    <sheet name="Character" sheetId="5" r:id="rId7"/>
+    <sheet name="SkillConfig" sheetId="11" r:id="rId8"/>
+    <sheet name="EffectConfig" sheetId="12" r:id="rId9"/>
+    <sheet name="CharacterStat" sheetId="6" r:id="rId10"/>
+    <sheet name="CharacterAttribute" sheetId="8" r:id="rId11"/>
+    <sheet name="CharacterUpgrade" sheetId="7" r:id="rId12"/>
+    <sheet name="ExpCurvesConfig" sheetId="13" r:id="rId13"/>
+    <sheet name="AscensionConfig" sheetId="14" r:id="rId14"/>
+    <sheet name="StarUp" sheetId="15" r:id="rId15"/>
+    <sheet name="BattleConfig" sheetId="9" r:id="rId16"/>
+    <sheet name="StageEnemies" sheetId="10" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$111</definedName>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1591" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1679" uniqueCount="578">
   <si>
     <t>ID</t>
   </si>
@@ -1603,19 +1604,193 @@
   </si>
   <si>
     <t>Modifier_Type</t>
+  </si>
+  <si>
+    <t>PassiveID</t>
+  </si>
+  <si>
+    <t>desc_template</t>
+  </si>
+  <si>
+    <t>param0_values</t>
+  </si>
+  <si>
+    <t>param1_values</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Tấn công và phòng thủ tăng {0}%. Sau khi tấn công đơn, nếu đánh bại mục tiêu thì điểm hành động tăng {1}%.</t>
+  </si>
+  <si>
+    <t>ST Bạo kích tăng {0}%. Sau khi thi triển kỹ năng tấn công đơn đánh bại mục tiêu, có {1}% xác suất hiệp hồi chiêu kỹ năng của bản thân -1.</t>
+  </si>
+  <si>
+    <t>ST Bạo Kích tăng {0}%. Sau khi tấn công đơn, nếu mục tiêu vẫn còn sống, có {1}% xác suất thi triển đánh thường để truy kích, mỗi hiệp kích hoạt tối đa 1 lần. Khi Phản Kích, Hỗ Trợ Tấn công se không kích hoạt hiệu ứng này.</t>
+  </si>
+  <si>
+    <t>Hiệu quả chính xác tăng {0}%. Khi bắt đầu hiệp, nếu bản thân có hiệu ứng suy yếu, có 20% xác suất xóa 1 hiệu ứng suy yếu.</t>
+  </si>
+  <si>
+    <t>HP và hiệu quả chính xác tăng {0}% . Khi chịu tấn côn đơn thế. Phòng thủ tăng {1}%, tối đa cộng dồn 6 tầng.</t>
+  </si>
+  <si>
+    <t>Khi bị tấn công phạm vi, điểm hành động của bản thân tăng {0)%.</t>
+  </si>
+  <si>
+    <t>ST tấn công đơn tăng {0}%.</t>
+  </si>
+  <si>
+    <t>Tấn công tăng {0}%. Khi tấn công đơn, có {1}% xác xuất gây Xé Toạc cho mục tiêu tân công, duy trì 2 hiệp.</t>
+  </si>
+  <si>
+    <t>Tỷ lệ bạo kích tăng {0}%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST Bạo Kích tăng {0}%. </t>
+  </si>
+  <si>
+    <t>Phòng thủ tăng {0}%.</t>
+  </si>
+  <si>
+    <t>Tăng {0}% Hiệu quả Chính Xác.Các đòn tấn công đơn mục tiêu có {1}% cơ hội gây hiệu ứng Đánh Dấu lên mục tiêu trong 1 lượt.</t>
+  </si>
+  <si>
+    <t>Kháng hiệu ứng tăng {0}%. Sau khi bị kĩ năng tấn công, nếu bản thân tồn tại hiệu ứng suy yếu, có {1}% xác xuất xóa 2 hiệu ứng suy yếu cảu bản thân, cứ 2 hiệp kích hoạt tối đa 1 lần.</t>
+  </si>
+  <si>
+    <t>psv_nimbus_cudgel</t>
+  </si>
+  <si>
+    <t>psv_triple_edged_blade</t>
+  </si>
+  <si>
+    <t>psv_vanguard_of_volition</t>
+  </si>
+  <si>
+    <t>psv_ninefold_staff</t>
+  </si>
+  <si>
+    <t>psv_nine_toothed_rake</t>
+  </si>
+  <si>
+    <t>psv_nimbus_cloud</t>
+  </si>
+  <si>
+    <t>psv_sunburst_spade</t>
+  </si>
+  <si>
+    <t>psv_reincarnation</t>
+  </si>
+  <si>
+    <t>psv_ennead_spear</t>
+  </si>
+  <si>
+    <t>psv_crescent_axe</t>
+  </si>
+  <si>
+    <t>psv_bronze_hammer</t>
+  </si>
+  <si>
+    <t>psv_moonlit_firefly</t>
+  </si>
+  <si>
+    <t>psv_plantain_fan</t>
+  </si>
+  <si>
+    <t>psv_wings_of_phoenix</t>
+  </si>
+  <si>
+    <t>10, 15, 20, 25, 30</t>
+  </si>
+  <si>
+    <t>10, 15, 20, 25, 31</t>
+  </si>
+  <si>
+    <t>10, 15, 20, 25, 32</t>
+  </si>
+  <si>
+    <t>10, 15, 20, 25, 33</t>
+  </si>
+  <si>
+    <t>10, 15, 20, 25, 34</t>
+  </si>
+  <si>
+    <t>10, 15, 20, 25, 35</t>
+  </si>
+  <si>
+    <t>10, 15, 20, 25, 36</t>
+  </si>
+  <si>
+    <t>10, 15, 20, 25, 37</t>
+  </si>
+  <si>
+    <t>20, 25, 30, 35, 40</t>
+  </si>
+  <si>
+    <t>20, 25, 30, 35, 41</t>
+  </si>
+  <si>
+    <t>20, 25, 30, 35, 42</t>
+  </si>
+  <si>
+    <t>20, 25, 30, 35, 43</t>
+  </si>
+  <si>
+    <t>20, 25, 30, 35, 44</t>
+  </si>
+  <si>
+    <t>20, 25, 30, 35, 45</t>
+  </si>
+  <si>
+    <t>20, 25, 30, 35, 46</t>
+  </si>
+  <si>
+    <t>20, 25, 30, 35, 47</t>
+  </si>
+  <si>
+    <t>10, 15, 20, 25, 38</t>
+  </si>
+  <si>
+    <t>20, 25, 30, 35, 48</t>
+  </si>
+  <si>
+    <t>10, 15, 20, 25, 39</t>
+  </si>
+  <si>
+    <t>20, 25, 30, 35, 49</t>
+  </si>
+  <si>
+    <t>5, 7.5, 10, 12.5, 15</t>
+  </si>
+  <si>
+    <t>5, 7.5, 10, 12.5, 16</t>
+  </si>
+  <si>
+    <t>5, 7.5, 10, 12.5, 17</t>
+  </si>
+  <si>
+    <t>Tấn công và phòng thủ tăng {0}%. Sau khi thi triển kỹ năng không phải tấn công, có {1}% xác suất hiệp hồi chiêu -1.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="18">
@@ -1734,7 +1909,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1807,6 +1982,12 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" readingOrder="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4166,6 +4347,666 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>297</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>298</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>352</v>
+      </c>
+      <c r="H1" s="18" t="s">
+        <v>300</v>
+      </c>
+      <c r="I1" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="J1" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="K1" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="L1" s="18" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="8">
+        <v>3750</v>
+      </c>
+      <c r="E2" s="8">
+        <v>2000</v>
+      </c>
+      <c r="F2" s="8">
+        <v>400</v>
+      </c>
+      <c r="G2" s="8">
+        <v>111</v>
+      </c>
+      <c r="H2" s="8">
+        <v>0</v>
+      </c>
+      <c r="I2" s="8">
+        <v>0</v>
+      </c>
+      <c r="J2" s="8">
+        <v>0</v>
+      </c>
+      <c r="K2" s="8">
+        <v>0</v>
+      </c>
+      <c r="L2" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>284</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>285</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="8">
+        <v>2500</v>
+      </c>
+      <c r="E3" s="8">
+        <v>1650</v>
+      </c>
+      <c r="F3" s="8">
+        <v>280</v>
+      </c>
+      <c r="G3" s="8">
+        <v>90</v>
+      </c>
+      <c r="H3" s="8">
+        <v>0</v>
+      </c>
+      <c r="I3" s="8">
+        <v>0</v>
+      </c>
+      <c r="J3" s="8">
+        <v>0</v>
+      </c>
+      <c r="K3" s="8">
+        <v>0</v>
+      </c>
+      <c r="L3" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>286</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>287</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D4" s="8">
+        <v>3200</v>
+      </c>
+      <c r="E4" s="8">
+        <v>1350</v>
+      </c>
+      <c r="F4" s="8">
+        <v>400</v>
+      </c>
+      <c r="G4" s="8">
+        <v>85</v>
+      </c>
+      <c r="H4" s="8">
+        <v>0</v>
+      </c>
+      <c r="I4" s="8">
+        <v>0</v>
+      </c>
+      <c r="J4" s="8">
+        <v>0</v>
+      </c>
+      <c r="K4" s="8">
+        <v>0</v>
+      </c>
+      <c r="L4" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>288</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="8">
+        <v>3900</v>
+      </c>
+      <c r="E5" s="8">
+        <v>1380</v>
+      </c>
+      <c r="F5" s="8">
+        <v>300</v>
+      </c>
+      <c r="G5" s="8">
+        <v>90</v>
+      </c>
+      <c r="H5" s="8">
+        <v>0</v>
+      </c>
+      <c r="I5" s="8">
+        <v>0</v>
+      </c>
+      <c r="J5" s="8">
+        <v>0</v>
+      </c>
+      <c r="K5" s="8">
+        <v>0</v>
+      </c>
+      <c r="L5" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>290</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" s="8">
+        <v>2930</v>
+      </c>
+      <c r="E6" s="8">
+        <v>1320</v>
+      </c>
+      <c r="F6" s="8">
+        <v>340</v>
+      </c>
+      <c r="G6" s="8">
+        <v>95</v>
+      </c>
+      <c r="H6" s="8">
+        <v>0</v>
+      </c>
+      <c r="I6" s="8">
+        <v>0</v>
+      </c>
+      <c r="J6" s="8">
+        <v>0</v>
+      </c>
+      <c r="K6" s="8">
+        <v>0</v>
+      </c>
+      <c r="L6" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>291</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>287</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="8">
+        <v>2650</v>
+      </c>
+      <c r="E7" s="8">
+        <v>2400</v>
+      </c>
+      <c r="F7" s="8">
+        <v>325</v>
+      </c>
+      <c r="G7" s="8">
+        <v>95</v>
+      </c>
+      <c r="H7" s="8">
+        <v>20</v>
+      </c>
+      <c r="I7" s="8">
+        <v>0</v>
+      </c>
+      <c r="J7" s="8">
+        <v>0</v>
+      </c>
+      <c r="K7" s="8">
+        <v>0</v>
+      </c>
+      <c r="L7" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>292</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="D8" s="8">
+        <v>2750</v>
+      </c>
+      <c r="E8" s="8">
+        <v>1800</v>
+      </c>
+      <c r="F8" s="8">
+        <v>300</v>
+      </c>
+      <c r="G8" s="8">
+        <v>95</v>
+      </c>
+      <c r="H8" s="8">
+        <v>0</v>
+      </c>
+      <c r="I8" s="8">
+        <v>0</v>
+      </c>
+      <c r="J8" s="8">
+        <v>0</v>
+      </c>
+      <c r="K8" s="8">
+        <v>0</v>
+      </c>
+      <c r="L8" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>294</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" s="8">
+        <v>4250</v>
+      </c>
+      <c r="E9" s="8">
+        <v>1500</v>
+      </c>
+      <c r="F9" s="8">
+        <v>420</v>
+      </c>
+      <c r="G9" s="8">
+        <v>95</v>
+      </c>
+      <c r="H9" s="8">
+        <v>0</v>
+      </c>
+      <c r="I9" s="8">
+        <v>0</v>
+      </c>
+      <c r="J9" s="8">
+        <v>0</v>
+      </c>
+      <c r="K9" s="8">
+        <v>0</v>
+      </c>
+      <c r="L9" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>295</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="8">
+        <v>3700</v>
+      </c>
+      <c r="E10" s="8">
+        <v>2100</v>
+      </c>
+      <c r="F10" s="8">
+        <v>350</v>
+      </c>
+      <c r="G10" s="8">
+        <v>95</v>
+      </c>
+      <c r="H10" s="8">
+        <v>0</v>
+      </c>
+      <c r="I10" s="8">
+        <v>0</v>
+      </c>
+      <c r="J10" s="8">
+        <v>0</v>
+      </c>
+      <c r="K10" s="8">
+        <v>0</v>
+      </c>
+      <c r="L10" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>296</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="8">
+        <v>3000</v>
+      </c>
+      <c r="E11" s="8">
+        <v>1950</v>
+      </c>
+      <c r="F11" s="8">
+        <v>330</v>
+      </c>
+      <c r="G11" s="8">
+        <v>95</v>
+      </c>
+      <c r="H11" s="8">
+        <v>0</v>
+      </c>
+      <c r="I11" s="8">
+        <v>0</v>
+      </c>
+      <c r="J11" s="8">
+        <v>0</v>
+      </c>
+      <c r="K11" s="8">
+        <v>0</v>
+      </c>
+      <c r="L11" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="24" t="s">
+        <v>333</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>285</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="8">
+        <v>3500</v>
+      </c>
+      <c r="E12" s="8">
+        <v>2650</v>
+      </c>
+      <c r="F12" s="8">
+        <v>280</v>
+      </c>
+      <c r="G12" s="8">
+        <v>70</v>
+      </c>
+      <c r="H12" s="8">
+        <v>0</v>
+      </c>
+      <c r="I12" s="8">
+        <v>0</v>
+      </c>
+      <c r="J12" s="8">
+        <v>0</v>
+      </c>
+      <c r="K12" s="8">
+        <v>0</v>
+      </c>
+      <c r="L12" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="24" t="s">
+        <v>314</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="8">
+        <v>2650</v>
+      </c>
+      <c r="E13" s="8">
+        <v>2400</v>
+      </c>
+      <c r="F13" s="8">
+        <v>325</v>
+      </c>
+      <c r="G13" s="8">
+        <v>80</v>
+      </c>
+      <c r="H13" s="8">
+        <v>20</v>
+      </c>
+      <c r="I13" s="8">
+        <v>0</v>
+      </c>
+      <c r="J13" s="8">
+        <v>0</v>
+      </c>
+      <c r="K13" s="8">
+        <v>0</v>
+      </c>
+      <c r="L13" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="24" t="s">
+        <v>316</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>287</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" s="8">
+        <v>2650</v>
+      </c>
+      <c r="E14" s="8">
+        <v>2400</v>
+      </c>
+      <c r="F14" s="8">
+        <v>325</v>
+      </c>
+      <c r="G14" s="8">
+        <v>80</v>
+      </c>
+      <c r="H14" s="8">
+        <v>20</v>
+      </c>
+      <c r="I14" s="8">
+        <v>0</v>
+      </c>
+      <c r="J14" s="8">
+        <v>0</v>
+      </c>
+      <c r="K14" s="8">
+        <v>0</v>
+      </c>
+      <c r="L14" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="24" t="s">
+        <v>317</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>287</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" s="8">
+        <v>2650</v>
+      </c>
+      <c r="E15" s="8">
+        <v>2400</v>
+      </c>
+      <c r="F15" s="8">
+        <v>325</v>
+      </c>
+      <c r="G15" s="8">
+        <v>80</v>
+      </c>
+      <c r="H15" s="8">
+        <v>20</v>
+      </c>
+      <c r="I15" s="8">
+        <v>0</v>
+      </c>
+      <c r="J15" s="8">
+        <v>0</v>
+      </c>
+      <c r="K15" s="8">
+        <v>0</v>
+      </c>
+      <c r="L15" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" s="24" t="s">
+        <v>318</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C16" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="8">
+        <v>4900</v>
+      </c>
+      <c r="E16" s="8">
+        <v>2400</v>
+      </c>
+      <c r="F16" s="8">
+        <v>325</v>
+      </c>
+      <c r="G16" s="8">
+        <v>100</v>
+      </c>
+      <c r="H16" s="8">
+        <v>20</v>
+      </c>
+      <c r="I16" s="8">
+        <v>0</v>
+      </c>
+      <c r="J16" s="8">
+        <v>0</v>
+      </c>
+      <c r="K16" s="8">
+        <v>0</v>
+      </c>
+      <c r="L16" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" s="24" t="s">
+        <v>319</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>287</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" s="8">
+        <v>2650</v>
+      </c>
+      <c r="E17" s="8">
+        <v>2400</v>
+      </c>
+      <c r="F17" s="8">
+        <v>325</v>
+      </c>
+      <c r="G17" s="8">
+        <v>80</v>
+      </c>
+      <c r="H17" s="8">
+        <v>20</v>
+      </c>
+      <c r="I17" s="8">
+        <v>0</v>
+      </c>
+      <c r="J17" s="8">
+        <v>0</v>
+      </c>
+      <c r="K17" s="8">
+        <v>0</v>
+      </c>
+      <c r="L17" s="8">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4520,7 +5361,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4774,7 +5615,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8563,7 +9404,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8971,7 +9812,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9284,7 +10125,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9343,7 +10184,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9638,14 +10479,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -9664,8 +10506,11 @@
       <c r="F1" s="1" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="1" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -9684,8 +10529,11 @@
       <c r="F2" s="10">
         <v>27</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="34" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -9704,8 +10552,11 @@
       <c r="F3" s="10">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="34" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -9724,8 +10575,11 @@
       <c r="F4" s="10">
         <v>29</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="34" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -9744,8 +10598,11 @@
       <c r="F5" s="10">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="34" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -9764,8 +10621,11 @@
       <c r="F6" s="10">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="34" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -9784,8 +10644,11 @@
       <c r="F7" s="10">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="34" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -9804,8 +10667,11 @@
       <c r="F8" s="10">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="34" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -9824,8 +10690,11 @@
       <c r="F9" s="10">
         <v>24</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="34" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -9844,8 +10713,11 @@
       <c r="F10" s="10">
         <v>12</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="34" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -9864,8 +10736,11 @@
       <c r="F11" s="10">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="34" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -9884,8 +10759,11 @@
       <c r="F12" s="10">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="34" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -9904,8 +10782,11 @@
       <c r="F13" s="10">
         <v>23</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="34" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -9924,8 +10805,11 @@
       <c r="F14" s="10">
         <v>21</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="34" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -9944,8 +10828,11 @@
       <c r="F15" s="10">
         <v>21</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="34" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>310</v>
       </c>
@@ -9963,6 +10850,9 @@
       </c>
       <c r="F16" s="10">
         <v>27</v>
+      </c>
+      <c r="G16" s="35" t="s">
+        <v>542</v>
       </c>
     </row>
   </sheetData>
@@ -9971,6 +10861,315 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E36"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" customWidth="1"/>
+    <col min="4" max="4" width="21.85546875" customWidth="1"/>
+    <col min="5" max="5" width="105.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>523</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>524</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>525</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="34" t="s">
+        <v>540</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" t="s">
+        <v>554</v>
+      </c>
+      <c r="D2" t="s">
+        <v>562</v>
+      </c>
+      <c r="E2" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="34" t="s">
+        <v>541</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" t="s">
+        <v>555</v>
+      </c>
+      <c r="D3" t="s">
+        <v>563</v>
+      </c>
+      <c r="E3" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="34" t="s">
+        <v>542</v>
+      </c>
+      <c r="B4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" t="s">
+        <v>556</v>
+      </c>
+      <c r="D4" t="s">
+        <v>564</v>
+      </c>
+      <c r="E4" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="34" t="s">
+        <v>543</v>
+      </c>
+      <c r="B5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" t="s">
+        <v>557</v>
+      </c>
+      <c r="D5" t="s">
+        <v>565</v>
+      </c>
+      <c r="E5" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="34" t="s">
+        <v>544</v>
+      </c>
+      <c r="B6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" t="s">
+        <v>558</v>
+      </c>
+      <c r="D6" t="s">
+        <v>566</v>
+      </c>
+      <c r="E6" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="34" t="s">
+        <v>545</v>
+      </c>
+      <c r="B7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" t="s">
+        <v>559</v>
+      </c>
+      <c r="D7" t="s">
+        <v>567</v>
+      </c>
+      <c r="E7" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="34" t="s">
+        <v>546</v>
+      </c>
+      <c r="B8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" t="s">
+        <v>560</v>
+      </c>
+      <c r="D8" t="s">
+        <v>568</v>
+      </c>
+      <c r="E8" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="34" t="s">
+        <v>547</v>
+      </c>
+      <c r="B9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" t="s">
+        <v>561</v>
+      </c>
+      <c r="D9" t="s">
+        <v>569</v>
+      </c>
+      <c r="E9" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="34" t="s">
+        <v>548</v>
+      </c>
+      <c r="B10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" t="s">
+        <v>574</v>
+      </c>
+      <c r="E10" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="34" t="s">
+        <v>549</v>
+      </c>
+      <c r="B11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" t="s">
+        <v>575</v>
+      </c>
+      <c r="E11" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="34" t="s">
+        <v>550</v>
+      </c>
+      <c r="B12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" t="s">
+        <v>576</v>
+      </c>
+      <c r="E12" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="34" t="s">
+        <v>551</v>
+      </c>
+      <c r="B13" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" t="s">
+        <v>561</v>
+      </c>
+      <c r="D13" t="s">
+        <v>569</v>
+      </c>
+      <c r="E13" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="34" t="s">
+        <v>552</v>
+      </c>
+      <c r="B14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" t="s">
+        <v>570</v>
+      </c>
+      <c r="D14" t="s">
+        <v>571</v>
+      </c>
+      <c r="E14" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="34" t="s">
+        <v>553</v>
+      </c>
+      <c r="B15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" t="s">
+        <v>572</v>
+      </c>
+      <c r="D15" t="s">
+        <v>573</v>
+      </c>
+      <c r="E15" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="22" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E22" s="34"/>
+    </row>
+    <row r="23" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E23" s="34"/>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E24" s="34"/>
+    </row>
+    <row r="25" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E25" s="34"/>
+    </row>
+    <row r="26" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E26" s="34"/>
+    </row>
+    <row r="27" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E27" s="34"/>
+    </row>
+    <row r="28" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E28" s="34"/>
+    </row>
+    <row r="29" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E29" s="34"/>
+    </row>
+    <row r="30" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E30" s="34"/>
+    </row>
+    <row r="31" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E31" s="34"/>
+    </row>
+    <row r="32" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E32" s="34"/>
+    </row>
+    <row r="33" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E33" s="34"/>
+    </row>
+    <row r="34" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E34" s="34"/>
+    </row>
+    <row r="35" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E35" s="34"/>
+    </row>
+    <row r="36" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E36" s="34"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10841,7 +12040,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10999,7 +12198,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11455,7 +12654,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13078,7 +14277,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13328,664 +14527,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="C1" s="18" t="s">
-        <v>68</v>
-      </c>
-      <c r="D1" s="18" t="s">
-        <v>297</v>
-      </c>
-      <c r="E1" s="18" t="s">
-        <v>298</v>
-      </c>
-      <c r="F1" s="18" t="s">
-        <v>299</v>
-      </c>
-      <c r="G1" s="18" t="s">
-        <v>352</v>
-      </c>
-      <c r="H1" s="18" t="s">
-        <v>300</v>
-      </c>
-      <c r="I1" s="18" t="s">
-        <v>301</v>
-      </c>
-      <c r="J1" s="18" t="s">
-        <v>302</v>
-      </c>
-      <c r="K1" s="18" t="s">
-        <v>303</v>
-      </c>
-      <c r="L1" s="18" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>282</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="C2" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="D2" s="8">
-        <v>3750</v>
-      </c>
-      <c r="E2" s="8">
-        <v>2000</v>
-      </c>
-      <c r="F2" s="8">
-        <v>400</v>
-      </c>
-      <c r="G2" s="8">
-        <v>111</v>
-      </c>
-      <c r="H2" s="8">
-        <v>0</v>
-      </c>
-      <c r="I2" s="8">
-        <v>0</v>
-      </c>
-      <c r="J2" s="8">
-        <v>0</v>
-      </c>
-      <c r="K2" s="8">
-        <v>0</v>
-      </c>
-      <c r="L2" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>284</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>285</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="D3" s="8">
-        <v>2500</v>
-      </c>
-      <c r="E3" s="8">
-        <v>1650</v>
-      </c>
-      <c r="F3" s="8">
-        <v>280</v>
-      </c>
-      <c r="G3" s="8">
-        <v>90</v>
-      </c>
-      <c r="H3" s="8">
-        <v>0</v>
-      </c>
-      <c r="I3" s="8">
-        <v>0</v>
-      </c>
-      <c r="J3" s="8">
-        <v>0</v>
-      </c>
-      <c r="K3" s="8">
-        <v>0</v>
-      </c>
-      <c r="L3" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>286</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>287</v>
-      </c>
-      <c r="C4" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="D4" s="8">
-        <v>3200</v>
-      </c>
-      <c r="E4" s="8">
-        <v>1350</v>
-      </c>
-      <c r="F4" s="8">
-        <v>400</v>
-      </c>
-      <c r="G4" s="8">
-        <v>85</v>
-      </c>
-      <c r="H4" s="8">
-        <v>0</v>
-      </c>
-      <c r="I4" s="8">
-        <v>0</v>
-      </c>
-      <c r="J4" s="8">
-        <v>0</v>
-      </c>
-      <c r="K4" s="8">
-        <v>0</v>
-      </c>
-      <c r="L4" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>288</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C5" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="D5" s="8">
-        <v>3900</v>
-      </c>
-      <c r="E5" s="8">
-        <v>1380</v>
-      </c>
-      <c r="F5" s="8">
-        <v>300</v>
-      </c>
-      <c r="G5" s="8">
-        <v>90</v>
-      </c>
-      <c r="H5" s="8">
-        <v>0</v>
-      </c>
-      <c r="I5" s="8">
-        <v>0</v>
-      </c>
-      <c r="J5" s="8">
-        <v>0</v>
-      </c>
-      <c r="K5" s="8">
-        <v>0</v>
-      </c>
-      <c r="L5" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>290</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="D6" s="8">
-        <v>2930</v>
-      </c>
-      <c r="E6" s="8">
-        <v>1320</v>
-      </c>
-      <c r="F6" s="8">
-        <v>340</v>
-      </c>
-      <c r="G6" s="8">
-        <v>95</v>
-      </c>
-      <c r="H6" s="8">
-        <v>0</v>
-      </c>
-      <c r="I6" s="8">
-        <v>0</v>
-      </c>
-      <c r="J6" s="8">
-        <v>0</v>
-      </c>
-      <c r="K6" s="8">
-        <v>0</v>
-      </c>
-      <c r="L6" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>291</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>287</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="8">
-        <v>2650</v>
-      </c>
-      <c r="E7" s="8">
-        <v>2400</v>
-      </c>
-      <c r="F7" s="8">
-        <v>325</v>
-      </c>
-      <c r="G7" s="8">
-        <v>95</v>
-      </c>
-      <c r="H7" s="8">
-        <v>20</v>
-      </c>
-      <c r="I7" s="8">
-        <v>0</v>
-      </c>
-      <c r="J7" s="8">
-        <v>0</v>
-      </c>
-      <c r="K7" s="8">
-        <v>0</v>
-      </c>
-      <c r="L7" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>292</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>293</v>
-      </c>
-      <c r="D8" s="8">
-        <v>2750</v>
-      </c>
-      <c r="E8" s="8">
-        <v>1800</v>
-      </c>
-      <c r="F8" s="8">
-        <v>300</v>
-      </c>
-      <c r="G8" s="8">
-        <v>95</v>
-      </c>
-      <c r="H8" s="8">
-        <v>0</v>
-      </c>
-      <c r="I8" s="8">
-        <v>0</v>
-      </c>
-      <c r="J8" s="8">
-        <v>0</v>
-      </c>
-      <c r="K8" s="8">
-        <v>0</v>
-      </c>
-      <c r="L8" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>294</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="D9" s="8">
-        <v>4250</v>
-      </c>
-      <c r="E9" s="8">
-        <v>1500</v>
-      </c>
-      <c r="F9" s="8">
-        <v>420</v>
-      </c>
-      <c r="G9" s="8">
-        <v>95</v>
-      </c>
-      <c r="H9" s="8">
-        <v>0</v>
-      </c>
-      <c r="I9" s="8">
-        <v>0</v>
-      </c>
-      <c r="J9" s="8">
-        <v>0</v>
-      </c>
-      <c r="K9" s="8">
-        <v>0</v>
-      </c>
-      <c r="L9" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>295</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="D10" s="8">
-        <v>3700</v>
-      </c>
-      <c r="E10" s="8">
-        <v>2100</v>
-      </c>
-      <c r="F10" s="8">
-        <v>350</v>
-      </c>
-      <c r="G10" s="8">
-        <v>95</v>
-      </c>
-      <c r="H10" s="8">
-        <v>0</v>
-      </c>
-      <c r="I10" s="8">
-        <v>0</v>
-      </c>
-      <c r="J10" s="8">
-        <v>0</v>
-      </c>
-      <c r="K10" s="8">
-        <v>0</v>
-      </c>
-      <c r="L10" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>296</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="D11" s="8">
-        <v>3000</v>
-      </c>
-      <c r="E11" s="8">
-        <v>1950</v>
-      </c>
-      <c r="F11" s="8">
-        <v>330</v>
-      </c>
-      <c r="G11" s="8">
-        <v>95</v>
-      </c>
-      <c r="H11" s="8">
-        <v>0</v>
-      </c>
-      <c r="I11" s="8">
-        <v>0</v>
-      </c>
-      <c r="J11" s="8">
-        <v>0</v>
-      </c>
-      <c r="K11" s="8">
-        <v>0</v>
-      </c>
-      <c r="L11" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="24" t="s">
-        <v>333</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>285</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="8">
-        <v>3500</v>
-      </c>
-      <c r="E12" s="8">
-        <v>2650</v>
-      </c>
-      <c r="F12" s="8">
-        <v>280</v>
-      </c>
-      <c r="G12" s="8">
-        <v>70</v>
-      </c>
-      <c r="H12" s="8">
-        <v>0</v>
-      </c>
-      <c r="I12" s="8">
-        <v>0</v>
-      </c>
-      <c r="J12" s="8">
-        <v>0</v>
-      </c>
-      <c r="K12" s="8">
-        <v>0</v>
-      </c>
-      <c r="L12" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="24" t="s">
-        <v>314</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="D13" s="8">
-        <v>2650</v>
-      </c>
-      <c r="E13" s="8">
-        <v>2400</v>
-      </c>
-      <c r="F13" s="8">
-        <v>325</v>
-      </c>
-      <c r="G13" s="8">
-        <v>80</v>
-      </c>
-      <c r="H13" s="8">
-        <v>20</v>
-      </c>
-      <c r="I13" s="8">
-        <v>0</v>
-      </c>
-      <c r="J13" s="8">
-        <v>0</v>
-      </c>
-      <c r="K13" s="8">
-        <v>0</v>
-      </c>
-      <c r="L13" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="24" t="s">
-        <v>316</v>
-      </c>
-      <c r="B14" s="16" t="s">
-        <v>287</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="D14" s="8">
-        <v>2650</v>
-      </c>
-      <c r="E14" s="8">
-        <v>2400</v>
-      </c>
-      <c r="F14" s="8">
-        <v>325</v>
-      </c>
-      <c r="G14" s="8">
-        <v>80</v>
-      </c>
-      <c r="H14" s="8">
-        <v>20</v>
-      </c>
-      <c r="I14" s="8">
-        <v>0</v>
-      </c>
-      <c r="J14" s="8">
-        <v>0</v>
-      </c>
-      <c r="K14" s="8">
-        <v>0</v>
-      </c>
-      <c r="L14" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="24" t="s">
-        <v>317</v>
-      </c>
-      <c r="B15" s="16" t="s">
-        <v>287</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="D15" s="8">
-        <v>2650</v>
-      </c>
-      <c r="E15" s="8">
-        <v>2400</v>
-      </c>
-      <c r="F15" s="8">
-        <v>325</v>
-      </c>
-      <c r="G15" s="8">
-        <v>80</v>
-      </c>
-      <c r="H15" s="8">
-        <v>20</v>
-      </c>
-      <c r="I15" s="8">
-        <v>0</v>
-      </c>
-      <c r="J15" s="8">
-        <v>0</v>
-      </c>
-      <c r="K15" s="8">
-        <v>0</v>
-      </c>
-      <c r="L15" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="24" t="s">
-        <v>318</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="D16" s="8">
-        <v>4900</v>
-      </c>
-      <c r="E16" s="8">
-        <v>2400</v>
-      </c>
-      <c r="F16" s="8">
-        <v>325</v>
-      </c>
-      <c r="G16" s="8">
-        <v>100</v>
-      </c>
-      <c r="H16" s="8">
-        <v>20</v>
-      </c>
-      <c r="I16" s="8">
-        <v>0</v>
-      </c>
-      <c r="J16" s="8">
-        <v>0</v>
-      </c>
-      <c r="K16" s="8">
-        <v>0</v>
-      </c>
-      <c r="L16" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" s="24" t="s">
-        <v>319</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>287</v>
-      </c>
-      <c r="C17" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="D17" s="8">
-        <v>2650</v>
-      </c>
-      <c r="E17" s="8">
-        <v>2400</v>
-      </c>
-      <c r="F17" s="8">
-        <v>325</v>
-      </c>
-      <c r="G17" s="8">
-        <v>80</v>
-      </c>
-      <c r="H17" s="8">
-        <v>20</v>
-      </c>
-      <c r="I17" s="8">
-        <v>0</v>
-      </c>
-      <c r="J17" s="8">
-        <v>0</v>
-      </c>
-      <c r="K17" s="8">
-        <v>0</v>
-      </c>
-      <c r="L17" s="8">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
+ Add Upgrade Armor Scene.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="3" activeTab="6"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="4" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -15,18 +15,19 @@
     <sheet name="StaticModifiers" sheetId="19" r:id="rId6"/>
     <sheet name="CombatEvents" sheetId="20" r:id="rId7"/>
     <sheet name="Armor" sheetId="4" r:id="rId8"/>
-    <sheet name="SetBonusConfig" sheetId="16" r:id="rId9"/>
-    <sheet name="Character" sheetId="5" r:id="rId10"/>
-    <sheet name="SkillConfig" sheetId="11" r:id="rId11"/>
-    <sheet name="EffectConfig" sheetId="12" r:id="rId12"/>
-    <sheet name="CharacterStat" sheetId="6" r:id="rId13"/>
-    <sheet name="CharacterAttribute" sheetId="8" r:id="rId14"/>
-    <sheet name="CharacterUpgrade" sheetId="7" r:id="rId15"/>
-    <sheet name="ExpCurvesConfig" sheetId="13" r:id="rId16"/>
-    <sheet name="AscensionConfig" sheetId="14" r:id="rId17"/>
-    <sheet name="StarUp" sheetId="15" r:id="rId18"/>
-    <sheet name="BattleConfig" sheetId="9" r:id="rId19"/>
-    <sheet name="StageEnemies" sheetId="10" r:id="rId20"/>
+    <sheet name="SubstatPool" sheetId="21" r:id="rId9"/>
+    <sheet name="SetBonusConfig" sheetId="16" r:id="rId10"/>
+    <sheet name="Character" sheetId="5" r:id="rId11"/>
+    <sheet name="SkillConfig" sheetId="11" r:id="rId12"/>
+    <sheet name="EffectConfig" sheetId="12" r:id="rId13"/>
+    <sheet name="CharacterStat" sheetId="6" r:id="rId14"/>
+    <sheet name="CharacterAttribute" sheetId="8" r:id="rId15"/>
+    <sheet name="CharacterUpgrade" sheetId="7" r:id="rId16"/>
+    <sheet name="ExpCurvesConfig" sheetId="13" r:id="rId17"/>
+    <sheet name="AscensionConfig" sheetId="14" r:id="rId18"/>
+    <sheet name="StarUp" sheetId="15" r:id="rId19"/>
+    <sheet name="BattleConfig" sheetId="9" r:id="rId20"/>
+    <sheet name="StageEnemies" sheetId="10" r:id="rId21"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$111</definedName>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1925" uniqueCount="630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1954" uniqueCount="635">
   <si>
     <t>ID</t>
   </si>
@@ -1513,15 +1514,9 @@
     <t>main_stat_valuie</t>
   </si>
   <si>
-    <t>random_substat_pool</t>
-  </si>
-  <si>
     <t>modifier_type</t>
   </si>
   <si>
-    <t>hp,100, 1000, Constant|def,50,150, Constant</t>
-  </si>
-  <si>
     <t>Curve_R</t>
   </si>
   <si>
@@ -1931,6 +1926,27 @@
   </si>
   <si>
     <t>40.0, 50.0, 60.0, 70.0, 80.0, 90.0</t>
+  </si>
+  <si>
+    <t>substat_pool_id</t>
+  </si>
+  <si>
+    <t>StatType</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Warrior_Pool</t>
+  </si>
+  <si>
+    <t>PEN</t>
+  </si>
+  <si>
+    <t>CRIT_DMG_RES</t>
   </si>
 </sst>
 </file>
@@ -4518,6 +4534,164 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>516</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>517</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>518</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="B2" t="s">
+        <v>248</v>
+      </c>
+      <c r="C2" s="8">
+        <v>6</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="E2" s="8">
+        <v>15</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>272</v>
+      </c>
+      <c r="B3" t="s">
+        <v>249</v>
+      </c>
+      <c r="C3" s="8">
+        <v>6</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="E3" s="8">
+        <v>15</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B4" t="s">
+        <v>250</v>
+      </c>
+      <c r="C4" s="8">
+        <v>6</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="E4" s="8">
+        <v>15</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="B5" t="s">
+        <v>251</v>
+      </c>
+      <c r="C5" s="8">
+        <v>6</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="E5" s="8">
+        <v>15</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="B6" t="s">
+        <v>252</v>
+      </c>
+      <c r="C6" s="8">
+        <v>6</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="E6" s="8">
+        <v>15</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>276</v>
+      </c>
+      <c r="B7" t="s">
+        <v>253</v>
+      </c>
+      <c r="C7" s="8">
+        <v>6</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="E7" s="8">
+        <v>15</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>446</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4972,7 +5146,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5012,7 +5186,7 @@
         <v>406</v>
       </c>
       <c r="H1" s="18" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="I1" s="18" t="s">
         <v>407</v>
@@ -5049,7 +5223,7 @@
         <v>100</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I2" s="8" t="s">
         <v>408</v>
@@ -5086,7 +5260,7 @@
         <v>100</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I3" s="8" t="s">
         <v>410</v>
@@ -5123,7 +5297,7 @@
         <v>100</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I4" s="8" t="s">
         <v>408</v>
@@ -5160,7 +5334,7 @@
         <v>100</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I5" s="8" t="s">
         <v>408</v>
@@ -5197,7 +5371,7 @@
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>409</v>
@@ -5234,7 +5408,7 @@
         <v>100</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>408</v>
@@ -5271,7 +5445,7 @@
         <v>100</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>408</v>
@@ -5308,7 +5482,7 @@
         <v>100</v>
       </c>
       <c r="H9" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>409</v>
@@ -5345,7 +5519,7 @@
         <v>100</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I10" s="8" t="s">
         <v>408</v>
@@ -5382,7 +5556,7 @@
         <v>100</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>408</v>
@@ -5419,7 +5593,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="I12" s="8" t="s">
         <v>409</v>
@@ -5456,7 +5630,7 @@
         <v>100</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I13" s="8" t="s">
         <v>408</v>
@@ -5493,7 +5667,7 @@
         <v>100</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I14" s="8" t="s">
         <v>408</v>
@@ -5527,7 +5701,7 @@
         <v>100</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I15" s="8" t="s">
         <v>408</v>
@@ -5561,7 +5735,7 @@
         <v>100</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I16" s="8" t="s">
         <v>408</v>
@@ -5595,7 +5769,7 @@
         <v>100</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I17" s="8" t="s">
         <v>408</v>
@@ -5632,7 +5806,7 @@
         <v>100</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I18" s="8" t="s">
         <v>408</v>
@@ -5669,7 +5843,7 @@
         <v>100</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I19" s="8" t="s">
         <v>408</v>
@@ -5706,7 +5880,7 @@
         <v>100</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I20" s="8" t="s">
         <v>408</v>
@@ -5743,7 +5917,7 @@
         <v>100</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I21" s="8" t="s">
         <v>408</v>
@@ -5780,7 +5954,7 @@
         <v>100</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>408</v>
@@ -5817,7 +5991,7 @@
         <v>100</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I23" s="8" t="s">
         <v>408</v>
@@ -5854,7 +6028,7 @@
         <v>0</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I24" s="8" t="s">
         <v>409</v>
@@ -5891,7 +6065,7 @@
         <v>100</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>408</v>
@@ -5928,7 +6102,7 @@
         <v>100</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I26" s="8" t="s">
         <v>408</v>
@@ -5962,7 +6136,7 @@
         <v>100</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I27" s="8" t="s">
         <v>408</v>
@@ -5996,7 +6170,7 @@
         <v>100</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I28" s="8" t="s">
         <v>408</v>
@@ -6030,7 +6204,7 @@
         <v>100</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>408</v>
@@ -6064,7 +6238,7 @@
         <v>100</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I30" s="8" t="s">
         <v>408</v>
@@ -6098,7 +6272,7 @@
         <v>100</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I31" s="8" t="s">
         <v>408</v>
@@ -6132,7 +6306,7 @@
         <v>100</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I32" s="8" t="s">
         <v>408</v>
@@ -6169,7 +6343,7 @@
         <v>100</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I33" s="8" t="s">
         <v>408</v>
@@ -6206,7 +6380,7 @@
         <v>100</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I34" s="8" t="s">
         <v>408</v>
@@ -6243,7 +6417,7 @@
         <v>100</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I35" s="8" t="s">
         <v>408</v>
@@ -6280,7 +6454,7 @@
         <v>100</v>
       </c>
       <c r="H36" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I36" s="8" t="s">
         <v>408</v>
@@ -6317,7 +6491,7 @@
         <v>100</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I37" s="8" t="s">
         <v>408</v>
@@ -6354,7 +6528,7 @@
         <v>100</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I38" s="8" t="s">
         <v>408</v>
@@ -6391,7 +6565,7 @@
         <v>100</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>408</v>
@@ -6428,7 +6602,7 @@
         <v>100</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I40" s="8" t="s">
         <v>408</v>
@@ -6465,7 +6639,7 @@
         <v>100</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I41" s="8" t="s">
         <v>408</v>
@@ -6502,7 +6676,7 @@
         <v>100</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I42" s="8" t="s">
         <v>408</v>
@@ -6539,7 +6713,7 @@
         <v>1000</v>
       </c>
       <c r="H43" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I43" s="8" t="s">
         <v>408</v>
@@ -6576,7 +6750,7 @@
         <v>100</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I44" s="8" t="s">
         <v>408</v>
@@ -6613,7 +6787,7 @@
         <v>100</v>
       </c>
       <c r="H45" s="8" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I45" s="8" t="s">
         <v>408</v>
@@ -6650,7 +6824,7 @@
         <v>100</v>
       </c>
       <c r="H46" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I46" s="8" t="s">
         <v>408</v>
@@ -6687,7 +6861,7 @@
         <v>100</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I47" s="8" t="s">
         <v>408</v>
@@ -6724,7 +6898,7 @@
         <v>100</v>
       </c>
       <c r="H48" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="I48" s="8" t="s">
         <v>408</v>
@@ -6739,7 +6913,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6991,7 +7165,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7651,7 +7825,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8007,7 +8181,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8261,7 +8435,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8283,28 +8457,28 @@
         <v>332</v>
       </c>
       <c r="B1" s="18" t="s">
+        <v>491</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>492</v>
+      </c>
+      <c r="D1" s="18" t="s">
         <v>493</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="E1" s="18" t="s">
         <v>494</v>
       </c>
-      <c r="D1" s="18" t="s">
-        <v>495</v>
-      </c>
-      <c r="E1" s="18" t="s">
-        <v>496</v>
-      </c>
       <c r="F1" s="18" t="s">
+        <v>497</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>498</v>
+      </c>
+      <c r="H1" s="18" t="s">
         <v>499</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="I1" s="18" t="s">
         <v>500</v>
-      </c>
-      <c r="H1" s="18" t="s">
-        <v>501</v>
-      </c>
-      <c r="I1" s="18" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -8340,16 +8514,16 @@
         <v>0</v>
       </c>
       <c r="N2" s="18" t="s">
+        <v>491</v>
+      </c>
+      <c r="O2" s="18" t="s">
+        <v>492</v>
+      </c>
+      <c r="P2" s="18" t="s">
         <v>493</v>
       </c>
-      <c r="O2" s="18" t="s">
+      <c r="Q2" s="18" t="s">
         <v>494</v>
-      </c>
-      <c r="P2" s="18" t="s">
-        <v>495</v>
-      </c>
-      <c r="Q2" s="18" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -8389,7 +8563,7 @@
         <v>250</v>
       </c>
       <c r="M3" s="12" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="N3">
         <v>100</v>
@@ -8441,7 +8615,7 @@
         <v>683</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="N4">
         <v>1.6</v>
@@ -12050,7 +12224,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -12067,27 +12241,27 @@
         <v>0</v>
       </c>
       <c r="B1" s="18" t="s">
+        <v>501</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>502</v>
+      </c>
+      <c r="D1" s="18" t="s">
         <v>503</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="E1" s="18" t="s">
+        <v>510</v>
+      </c>
+      <c r="F1" s="18" t="s">
         <v>504</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="G1" s="18" t="s">
         <v>505</v>
-      </c>
-      <c r="E1" s="18" t="s">
-        <v>512</v>
-      </c>
-      <c r="F1" s="18" t="s">
-        <v>506</v>
-      </c>
-      <c r="G1" s="18" t="s">
-        <v>507</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="B2" s="8">
         <v>1</v>
@@ -12110,7 +12284,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="B3" s="8">
         <v>2</v>
@@ -12133,7 +12307,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="B4" s="8">
         <v>3</v>
@@ -12156,7 +12330,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="B5" s="8">
         <v>4</v>
@@ -12179,7 +12353,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="B6" s="8">
         <v>1</v>
@@ -12202,7 +12376,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="B7" s="8">
         <v>2</v>
@@ -12225,7 +12399,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="B8" s="8">
         <v>3</v>
@@ -12248,7 +12422,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="B9" s="8">
         <v>4</v>
@@ -12271,7 +12445,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="B10" s="8">
         <v>1</v>
@@ -12294,7 +12468,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="B11" s="8">
         <v>2</v>
@@ -12317,7 +12491,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="B12" s="8">
         <v>3</v>
@@ -12340,7 +12514,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="B13" s="8">
         <v>4</v>
@@ -12363,7 +12537,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="B14" s="8">
         <v>1</v>
@@ -12386,7 +12560,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="B15" s="8">
         <v>2</v>
@@ -12409,7 +12583,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="B16" s="8">
         <v>3</v>
@@ -12432,7 +12606,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="B17" s="8">
         <v>4</v>
@@ -12458,7 +12632,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -12477,18 +12651,18 @@
         <v>0</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="B2" s="7">
         <v>2</v>
@@ -12502,7 +12676,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="B3" s="7">
         <v>3</v>
@@ -12516,7 +12690,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="B4" s="7">
         <v>4</v>
@@ -12530,7 +12704,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="B5" s="7">
         <v>5</v>
@@ -12544,7 +12718,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="B6" s="7">
         <v>6</v>
@@ -12558,7 +12732,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="B7" s="7">
         <v>2</v>
@@ -12572,7 +12746,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="B8" s="7">
         <v>3</v>
@@ -12586,7 +12760,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="B9" s="7">
         <v>4</v>
@@ -12600,7 +12774,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="B10" s="7">
         <v>5</v>
@@ -12614,7 +12788,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="B11" s="7">
         <v>6</v>
@@ -12628,7 +12802,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="33" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="B12" s="7">
         <v>2</v>
@@ -12642,7 +12816,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="33" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="B13" s="7">
         <v>3</v>
@@ -12656,7 +12830,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="33" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="B14" s="7">
         <v>4</v>
@@ -12670,7 +12844,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="33" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="B15" s="7">
         <v>5</v>
@@ -12684,7 +12858,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="33" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="B16" s="7">
         <v>6</v>
@@ -12698,7 +12872,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="B17" s="7">
         <v>2</v>
@@ -12712,7 +12886,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="B18" s="7">
         <v>3</v>
@@ -12726,7 +12900,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="B19" s="7">
         <v>4</v>
@@ -12740,7 +12914,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="B20" s="7">
         <v>5</v>
@@ -12754,7 +12928,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="B21" s="7">
         <v>6</v>
@@ -12764,65 +12938,6 @@
       </c>
       <c r="D21">
         <v>300</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" customWidth="1"/>
-    <col min="3" max="3" width="21.28515625" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" customWidth="1"/>
-    <col min="5" max="5" width="23.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="18" t="s">
-        <v>444</v>
-      </c>
-      <c r="D1" s="18" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>324</v>
-      </c>
-      <c r="B2" t="s">
-        <v>326</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>325</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>462</v>
-      </c>
-      <c r="B3" t="s">
-        <v>326</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>325</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>328</v>
       </c>
     </row>
   </sheetData>
@@ -12888,6 +13003,65 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>444</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="B2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="B3" t="s">
+        <v>326</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>328</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13153,7 +13327,7 @@
         <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -13176,7 +13350,7 @@
         <v>27</v>
       </c>
       <c r="G2" s="34" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -13199,7 +13373,7 @@
         <v>25</v>
       </c>
       <c r="G3" s="34" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -13222,7 +13396,7 @@
         <v>29</v>
       </c>
       <c r="G4" s="34" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -13245,7 +13419,7 @@
         <v>14</v>
       </c>
       <c r="G5" s="34" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -13268,7 +13442,7 @@
         <v>16</v>
       </c>
       <c r="G6" s="34" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -13291,7 +13465,7 @@
         <v>13</v>
       </c>
       <c r="G7" s="34" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -13314,7 +13488,7 @@
         <v>10</v>
       </c>
       <c r="G8" s="34" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -13337,7 +13511,7 @@
         <v>24</v>
       </c>
       <c r="G9" s="34" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -13360,7 +13534,7 @@
         <v>12</v>
       </c>
       <c r="G10" s="34" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -13383,7 +13557,7 @@
         <v>10</v>
       </c>
       <c r="G11" s="34" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -13406,7 +13580,7 @@
         <v>11</v>
       </c>
       <c r="G12" s="34" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -13429,7 +13603,7 @@
         <v>23</v>
       </c>
       <c r="G13" s="34" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -13452,7 +13626,7 @@
         <v>21</v>
       </c>
       <c r="G14" s="34" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -13475,7 +13649,7 @@
         <v>21</v>
       </c>
       <c r="G15" s="34" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -13498,7 +13672,7 @@
         <v>27</v>
       </c>
       <c r="G16" s="35" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
     </row>
   </sheetData>
@@ -13523,242 +13697,242 @@
         <v>0</v>
       </c>
       <c r="B1" s="18" t="s">
+        <v>521</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>522</v>
+      </c>
+      <c r="D1" s="18" t="s">
         <v>523</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="E1" s="18" t="s">
         <v>524</v>
-      </c>
-      <c r="D1" s="18" t="s">
-        <v>525</v>
-      </c>
-      <c r="E1" s="18" t="s">
-        <v>526</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="34" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="B2" t="s">
         <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="D2" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="E2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="34" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B3" t="s">
         <v>49</v>
       </c>
       <c r="C3" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="D3" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="E3" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="34" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="B4" t="s">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="D4" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="E4" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="34" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="B5" t="s">
         <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="D5" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="E5" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="B6" t="s">
         <v>52</v>
       </c>
       <c r="C6" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="D6" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="E6" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="34" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="B7" t="s">
         <v>53</v>
       </c>
       <c r="C7" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="E7" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="B8" t="s">
         <v>54</v>
       </c>
       <c r="C8" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="D8" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="E8" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="34" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="B9" t="s">
         <v>55</v>
       </c>
       <c r="C9" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="D9" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="E9" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="34" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="B10" t="s">
         <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="E10" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="34" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="B11" t="s">
         <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="E11" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="34" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="B12" t="s">
         <v>58</v>
       </c>
       <c r="C12" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="E12" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="34" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="B13" t="s">
         <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="D13" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="E13" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="34" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="B14" t="s">
         <v>60</v>
       </c>
       <c r="C14" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="D14" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="E14" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="34" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="B15" t="s">
         <v>61</v>
       </c>
       <c r="C15" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="D15" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="E15" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
     <row r="22" spans="5:5" x14ac:dyDescent="0.25">
@@ -13827,164 +14001,164 @@
         <v>0</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="34" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="B2" t="s">
         <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="34" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B3" t="s">
         <v>49</v>
       </c>
       <c r="C3" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="34" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="B4" t="s">
         <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="34" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="B5" t="s">
         <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="B6" t="s">
         <v>52</v>
       </c>
       <c r="C6" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="34" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="B7" t="s">
         <v>53</v>
       </c>
       <c r="C7" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="B8" t="s">
         <v>54</v>
       </c>
       <c r="C8" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="34" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="B9" t="s">
         <v>55</v>
       </c>
       <c r="C9" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="34" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="B10" t="s">
         <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="34" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="B11" t="s">
         <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="34" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="B12" t="s">
         <v>58</v>
       </c>
       <c r="C12" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="34" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="B13" t="s">
         <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="34" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="B14" t="s">
         <v>60</v>
       </c>
       <c r="C14" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="34" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="B15" t="s">
         <v>61</v>
       </c>
       <c r="C15" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
   </sheetData>
@@ -14006,24 +14180,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
+        <v>575</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>576</v>
+      </c>
+      <c r="C1" s="18" t="s">
         <v>577</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="D1" s="18" t="s">
         <v>578</v>
       </c>
-      <c r="C1" s="18" t="s">
-        <v>579</v>
-      </c>
-      <c r="D1" s="18" t="s">
-        <v>580</v>
-      </c>
       <c r="E1" s="18" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="36" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>70</v>
@@ -14032,15 +14206,15 @@
         <v>446</v>
       </c>
       <c r="D2" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="E2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="36" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>421</v>
@@ -14049,66 +14223,66 @@
         <v>446</v>
       </c>
       <c r="D3" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="E3" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="34" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>446</v>
       </c>
       <c r="D4" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="E4" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="34" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>446</v>
       </c>
       <c r="D5" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="E5" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>446</v>
       </c>
       <c r="D6" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="E6" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="36" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>69</v>
@@ -14117,32 +14291,32 @@
         <v>446</v>
       </c>
       <c r="D7" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E7" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="36" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>446</v>
       </c>
       <c r="D8" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E8" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="34" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>70</v>
@@ -14151,49 +14325,49 @@
         <v>446</v>
       </c>
       <c r="D9" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="E9" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="34" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>446</v>
       </c>
       <c r="D10" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E10" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="34" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>446</v>
       </c>
       <c r="D11" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="E11" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="34" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>422</v>
@@ -14202,15 +14376,15 @@
         <v>446</v>
       </c>
       <c r="D12" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="E12" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="36" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>421</v>
@@ -14219,15 +14393,15 @@
         <v>446</v>
       </c>
       <c r="D13" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="E13" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="36" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>70</v>
@@ -14236,44 +14410,44 @@
         <v>446</v>
       </c>
       <c r="D14" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="E14" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="34" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>446</v>
       </c>
       <c r="D15" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="E15" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="34" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>446</v>
       </c>
       <c r="D16" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="E16" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
   </sheetData>
@@ -14302,69 +14476,69 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="F1" s="18" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="H1" s="18" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="34" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="B2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="D2" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="E2" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="F2" s="8">
         <v>0</v>
       </c>
       <c r="G2" s="8"/>
       <c r="H2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="34" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B3" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C3" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="D3" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="E3" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="F3" s="8">
         <v>1</v>
@@ -14373,48 +14547,48 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="38" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="B4" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C4" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="D4" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="E4" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="F4" s="8"/>
       <c r="G4" s="8">
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="34" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="B5" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="C5" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="D5" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="E5" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="F5" s="8">
         <v>1</v>
@@ -14423,24 +14597,24 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="B6" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="C6" t="s">
+        <v>592</v>
+      </c>
+      <c r="D6" t="s">
+        <v>626</v>
+      </c>
+      <c r="E6" s="37" t="s">
         <v>594</v>
-      </c>
-      <c r="D6" t="s">
-        <v>628</v>
-      </c>
-      <c r="E6" s="37" t="s">
-        <v>596</v>
       </c>
       <c r="F6" s="8">
         <v>6</v>
@@ -14449,24 +14623,24 @@
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="34" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="B7" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="C7" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="D7" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="E7" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="F7" s="8">
         <v>0</v>
@@ -14475,48 +14649,48 @@
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="B8" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="C8" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="D8" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="E8" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="F8" s="8">
         <v>2</v>
       </c>
       <c r="G8" s="8"/>
       <c r="H8" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="34" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="B9" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="C9" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="D9" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="E9" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="F9" s="8">
         <v>1</v>
@@ -14525,24 +14699,24 @@
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="34" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="B10" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="C10" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="D10" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="E10" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="F10" s="8">
         <v>1</v>
@@ -14551,24 +14725,24 @@
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="38" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="B11" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="C11" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="D11" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="E11" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="F11" s="8">
         <v>2</v>
@@ -14577,24 +14751,24 @@
         <v>2</v>
       </c>
       <c r="H11" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="B12" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="C12" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="D12" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="E12" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="F12" s="8">
         <v>0</v>
@@ -14603,7 +14777,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
     </row>
   </sheetData>
@@ -14613,7 +14787,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
@@ -14622,10 +14796,11 @@
     <col min="4" max="4" width="17.85546875" customWidth="1"/>
     <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.85546875" customWidth="1"/>
-    <col min="7" max="7" width="40.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" customWidth="1"/>
+    <col min="9" max="9" width="73.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -14642,13 +14817,13 @@
         <v>489</v>
       </c>
       <c r="F1" s="18" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>212</v>
       </c>
@@ -14667,11 +14842,12 @@
       <c r="F2" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G2" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G2" t="s">
+        <v>632</v>
+      </c>
+      <c r="I2" s="8"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>213</v>
       </c>
@@ -14690,11 +14866,11 @@
       <c r="F3" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G3" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
         <v>214</v>
       </c>
@@ -14713,11 +14889,11 @@
       <c r="F4" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G4" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
         <v>215</v>
       </c>
@@ -14736,11 +14912,11 @@
       <c r="F5" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G5" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
         <v>216</v>
       </c>
@@ -14759,11 +14935,11 @@
       <c r="F6" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G6" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G6" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
         <v>217</v>
       </c>
@@ -14782,11 +14958,11 @@
       <c r="F7" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G7" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
         <v>218</v>
       </c>
@@ -14805,11 +14981,11 @@
       <c r="F8" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G8" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G8" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
         <v>219</v>
       </c>
@@ -14828,11 +15004,11 @@
       <c r="F9" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G9" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G9" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
         <v>220</v>
       </c>
@@ -14851,11 +15027,11 @@
       <c r="F10" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G10" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G10" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
         <v>221</v>
       </c>
@@ -14874,11 +15050,11 @@
       <c r="F11" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G11" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G11" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
         <v>222</v>
       </c>
@@ -14897,11 +15073,11 @@
       <c r="F12" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G12" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G12" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
         <v>223</v>
       </c>
@@ -14920,11 +15096,11 @@
       <c r="F13" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G13" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G13" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
         <v>224</v>
       </c>
@@ -14943,11 +15119,11 @@
       <c r="F14" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G14" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G14" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
         <v>225</v>
       </c>
@@ -14966,11 +15142,11 @@
       <c r="F15" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G15" s="8" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G15" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
         <v>226</v>
       </c>
@@ -14989,8 +15165,8 @@
       <c r="F16" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G16" s="8" t="s">
-        <v>492</v>
+      <c r="G16" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -15012,8 +15188,8 @@
       <c r="F17" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G17" s="8" t="s">
-        <v>492</v>
+      <c r="G17" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -15035,8 +15211,8 @@
       <c r="F18" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G18" s="8" t="s">
-        <v>492</v>
+      <c r="G18" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -15058,8 +15234,8 @@
       <c r="F19" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G19" s="8" t="s">
-        <v>492</v>
+      <c r="G19" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -15081,8 +15257,8 @@
       <c r="F20" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G20" s="8" t="s">
-        <v>492</v>
+      <c r="G20" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -15104,8 +15280,8 @@
       <c r="F21" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G21" s="8" t="s">
-        <v>492</v>
+      <c r="G21" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -15127,8 +15303,8 @@
       <c r="F22" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G22" s="8" t="s">
-        <v>492</v>
+      <c r="G22" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -15150,8 +15326,8 @@
       <c r="F23" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G23" s="8" t="s">
-        <v>492</v>
+      <c r="G23" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -15173,8 +15349,8 @@
       <c r="F24" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G24" s="8" t="s">
-        <v>492</v>
+      <c r="G24" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -15196,8 +15372,8 @@
       <c r="F25" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G25" s="8" t="s">
-        <v>492</v>
+      <c r="G25" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -15219,8 +15395,8 @@
       <c r="F26" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G26" s="8" t="s">
-        <v>492</v>
+      <c r="G26" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -15242,8 +15418,8 @@
       <c r="F27" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G27" s="8" t="s">
-        <v>492</v>
+      <c r="G27" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -15265,8 +15441,8 @@
       <c r="F28" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G28" s="8" t="s">
-        <v>492</v>
+      <c r="G28" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -15288,8 +15464,8 @@
       <c r="F29" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G29" s="8" t="s">
-        <v>492</v>
+      <c r="G29" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -15311,8 +15487,8 @@
       <c r="F30" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G30" s="8" t="s">
-        <v>492</v>
+      <c r="G30" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -15334,8 +15510,8 @@
       <c r="F31" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G31" s="8" t="s">
-        <v>492</v>
+      <c r="G31" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -15357,8 +15533,8 @@
       <c r="F32" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G32" s="8" t="s">
-        <v>492</v>
+      <c r="G32" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -15380,8 +15556,8 @@
       <c r="F33" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G33" s="8" t="s">
-        <v>492</v>
+      <c r="G33" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -15403,8 +15579,8 @@
       <c r="F34" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G34" s="8" t="s">
-        <v>492</v>
+      <c r="G34" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -15426,8 +15602,8 @@
       <c r="F35" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G35" s="8" t="s">
-        <v>492</v>
+      <c r="G35" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -15449,8 +15625,8 @@
       <c r="F36" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G36" s="8" t="s">
-        <v>492</v>
+      <c r="G36" t="s">
+        <v>632</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -15472,8 +15648,8 @@
       <c r="F37" s="8" t="s">
         <v>447</v>
       </c>
-      <c r="G37" s="8" t="s">
-        <v>492</v>
+      <c r="G37" t="s">
+        <v>632</v>
       </c>
     </row>
   </sheetData>
@@ -15484,158 +15660,182 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>1</v>
+        <v>629</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>518</v>
+        <v>630</v>
       </c>
       <c r="D1" s="18" t="s">
+        <v>631</v>
+      </c>
+      <c r="E1" s="18" t="s">
         <v>519</v>
       </c>
-      <c r="E1" s="18" t="s">
-        <v>520</v>
-      </c>
-      <c r="F1" s="18" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>271</v>
-      </c>
-      <c r="B2" t="s">
-        <v>248</v>
-      </c>
-      <c r="C2" s="8">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>632</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="7">
+        <v>100</v>
+      </c>
+      <c r="D2" s="7">
+        <v>2000</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>632</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="7">
+        <v>100</v>
+      </c>
+      <c r="D3" s="7">
+        <v>1000</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>632</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>421</v>
+      </c>
+      <c r="C4" s="7">
+        <v>100</v>
+      </c>
+      <c r="D4" s="7">
+        <v>300</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>632</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>422</v>
+      </c>
+      <c r="C5" s="7">
+        <v>2</v>
+      </c>
+      <c r="D5" s="7">
+        <v>5</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>632</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>580</v>
+      </c>
+      <c r="C6" s="7">
+        <v>3</v>
+      </c>
+      <c r="D6" s="7">
         <v>6</v>
       </c>
-      <c r="D2" s="8" t="s">
-        <v>298</v>
-      </c>
-      <c r="E2" s="8">
-        <v>15</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>272</v>
-      </c>
-      <c r="B3" t="s">
-        <v>249</v>
-      </c>
-      <c r="C3" s="8">
-        <v>6</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>298</v>
-      </c>
-      <c r="E3" s="8">
-        <v>15</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
-        <v>273</v>
-      </c>
-      <c r="B4" t="s">
-        <v>250</v>
-      </c>
-      <c r="C4" s="8">
-        <v>6</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>298</v>
-      </c>
-      <c r="E4" s="8">
-        <v>15</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>274</v>
-      </c>
-      <c r="B5" t="s">
-        <v>251</v>
-      </c>
-      <c r="C5" s="8">
-        <v>6</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>298</v>
-      </c>
-      <c r="E5" s="8">
-        <v>15</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>275</v>
-      </c>
-      <c r="B6" t="s">
-        <v>252</v>
-      </c>
-      <c r="C6" s="8">
-        <v>6</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>298</v>
-      </c>
-      <c r="E6" s="8">
-        <v>15</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>276</v>
-      </c>
-      <c r="B7" t="s">
-        <v>253</v>
-      </c>
-      <c r="C7" s="8">
-        <v>6</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>298</v>
-      </c>
-      <c r="E7" s="8">
-        <v>15</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>446</v>
-      </c>
+      <c r="E6" s="7" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>632</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>579</v>
+      </c>
+      <c r="C7" s="7">
+        <v>10</v>
+      </c>
+      <c r="D7" s="7">
+        <v>20</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>632</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>633</v>
+      </c>
+      <c r="C8" s="7">
+        <v>10</v>
+      </c>
+      <c r="D8" s="7">
+        <v>20</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>632</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>634</v>
+      </c>
+      <c r="C9" s="7">
+        <v>10</v>
+      </c>
+      <c r="D9" s="7">
+        <v>20</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E10" s="7"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E11" s="7"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B9">
+      <formula1>"HP, ATK, DEF, SPEED, DEF_SHRED, CRIT_RATE, CRIT_DMG, PEN, CRIT_DMG_RES, SHIELD, EHR,  RES,  None"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
+ Fix bug UI in the character scene, upgrade armor and upgrade weapon scene.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="4" activeTab="8"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="11" activeTab="17"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1954" uniqueCount="635">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1962" uniqueCount="635">
   <si>
     <t>ID</t>
   </si>
@@ -1968,7 +1968,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2071,6 +2071,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -2084,7 +2090,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2175,6 +2181,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12226,7 +12236,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -12352,26 +12362,26 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>507</v>
-      </c>
-      <c r="B6" s="8">
-        <v>1</v>
-      </c>
-      <c r="C6" s="8">
+      <c r="A6" t="s">
+        <v>506</v>
+      </c>
+      <c r="B6" s="40">
+        <v>5</v>
+      </c>
+      <c r="C6" s="40">
+        <v>100</v>
+      </c>
+      <c r="D6" s="40">
+        <v>100</v>
+      </c>
+      <c r="E6" s="40">
+        <v>500000</v>
+      </c>
+      <c r="F6" s="41" t="s">
+        <v>124</v>
+      </c>
+      <c r="G6" s="40">
         <v>20</v>
-      </c>
-      <c r="D6" s="8">
-        <v>40</v>
-      </c>
-      <c r="E6" s="8">
-        <v>10000</v>
-      </c>
-      <c r="F6" t="s">
-        <v>124</v>
-      </c>
-      <c r="G6" s="8">
-        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -12379,22 +12389,22 @@
         <v>507</v>
       </c>
       <c r="B7" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="8">
+        <v>20</v>
+      </c>
+      <c r="D7" s="8">
         <v>40</v>
       </c>
-      <c r="D7" s="8">
-        <v>60</v>
-      </c>
       <c r="E7" s="8">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c r="F7" t="s">
         <v>124</v>
       </c>
       <c r="G7" s="8">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -12402,22 +12412,22 @@
         <v>507</v>
       </c>
       <c r="B8" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C8" s="8">
+        <v>40</v>
+      </c>
+      <c r="D8" s="8">
         <v>60</v>
       </c>
-      <c r="D8" s="8">
-        <v>80</v>
-      </c>
       <c r="E8" s="8">
-        <v>200000</v>
+        <v>50000</v>
       </c>
       <c r="F8" t="s">
         <v>124</v>
       </c>
       <c r="G8" s="8">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -12425,68 +12435,68 @@
         <v>507</v>
       </c>
       <c r="B9" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9" s="8">
+        <v>60</v>
+      </c>
+      <c r="D9" s="8">
         <v>80</v>
       </c>
-      <c r="D9" s="8">
-        <v>100</v>
-      </c>
       <c r="E9" s="8">
-        <v>500000</v>
+        <v>200000</v>
       </c>
       <c r="F9" t="s">
         <v>124</v>
       </c>
       <c r="G9" s="8">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>508</v>
+      <c r="A10" s="12" t="s">
+        <v>507</v>
       </c>
       <c r="B10" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C10" s="8">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="D10" s="8">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="E10" s="8">
-        <v>10000</v>
+        <v>500000</v>
       </c>
       <c r="F10" t="s">
         <v>124</v>
       </c>
       <c r="G10" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>507</v>
+      </c>
+      <c r="B11" s="40">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>508</v>
-      </c>
-      <c r="B11" s="8">
-        <v>2</v>
-      </c>
-      <c r="C11" s="8">
-        <v>40</v>
-      </c>
-      <c r="D11" s="8">
-        <v>60</v>
-      </c>
-      <c r="E11" s="8">
-        <v>50000</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="C11" s="40">
+        <v>100</v>
+      </c>
+      <c r="D11" s="40">
+        <v>100</v>
+      </c>
+      <c r="E11" s="40">
+        <v>500000</v>
+      </c>
+      <c r="F11" s="41" t="s">
         <v>124</v>
       </c>
-      <c r="G11" s="8">
-        <v>10</v>
+      <c r="G11" s="40">
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -12494,22 +12504,22 @@
         <v>508</v>
       </c>
       <c r="B12" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C12" s="8">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="D12" s="8">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="E12" s="8">
-        <v>200000</v>
+        <v>10000</v>
       </c>
       <c r="F12" t="s">
         <v>124</v>
       </c>
       <c r="G12" s="8">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -12517,91 +12527,91 @@
         <v>508</v>
       </c>
       <c r="B13" s="8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C13" s="8">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="D13" s="8">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="E13" s="8">
-        <v>500000</v>
+        <v>50000</v>
       </c>
       <c r="F13" t="s">
         <v>124</v>
       </c>
       <c r="G13" s="8">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
-        <v>509</v>
+      <c r="A14" t="s">
+        <v>508</v>
       </c>
       <c r="B14" s="8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C14" s="8">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="D14" s="8">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="E14" s="8">
-        <v>10000</v>
+        <v>200000</v>
       </c>
       <c r="F14" t="s">
         <v>124</v>
       </c>
       <c r="G14" s="8">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
-        <v>509</v>
+      <c r="A15" t="s">
+        <v>508</v>
       </c>
       <c r="B15" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C15" s="8">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="D15" s="8">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="E15" s="8">
-        <v>50000</v>
+        <v>500000</v>
       </c>
       <c r="F15" t="s">
         <v>124</v>
       </c>
       <c r="G15" s="8">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
-        <v>509</v>
-      </c>
-      <c r="B16" s="8">
-        <v>3</v>
-      </c>
-      <c r="C16" s="8">
-        <v>60</v>
-      </c>
-      <c r="D16" s="8">
-        <v>80</v>
-      </c>
-      <c r="E16" s="8">
-        <v>200000</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="A16" t="s">
+        <v>508</v>
+      </c>
+      <c r="B16" s="40">
+        <v>5</v>
+      </c>
+      <c r="C16" s="40">
+        <v>100</v>
+      </c>
+      <c r="D16" s="40">
+        <v>100</v>
+      </c>
+      <c r="E16" s="40">
+        <v>500000</v>
+      </c>
+      <c r="F16" s="41" t="s">
         <v>124</v>
       </c>
-      <c r="G16" s="8">
-        <v>15</v>
+      <c r="G16" s="40">
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -12609,21 +12619,113 @@
         <v>509</v>
       </c>
       <c r="B17" s="8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C17" s="8">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="D17" s="8">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E17" s="8">
-        <v>500000</v>
+        <v>10000</v>
       </c>
       <c r="F17" t="s">
         <v>124</v>
       </c>
       <c r="G17" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>509</v>
+      </c>
+      <c r="B18" s="8">
+        <v>2</v>
+      </c>
+      <c r="C18" s="8">
+        <v>40</v>
+      </c>
+      <c r="D18" s="8">
+        <v>60</v>
+      </c>
+      <c r="E18" s="8">
+        <v>50000</v>
+      </c>
+      <c r="F18" t="s">
+        <v>124</v>
+      </c>
+      <c r="G18" s="8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>509</v>
+      </c>
+      <c r="B19" s="8">
+        <v>3</v>
+      </c>
+      <c r="C19" s="8">
+        <v>60</v>
+      </c>
+      <c r="D19" s="8">
+        <v>80</v>
+      </c>
+      <c r="E19" s="8">
+        <v>200000</v>
+      </c>
+      <c r="F19" t="s">
+        <v>124</v>
+      </c>
+      <c r="G19" s="8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>509</v>
+      </c>
+      <c r="B20" s="8">
+        <v>4</v>
+      </c>
+      <c r="C20" s="8">
+        <v>80</v>
+      </c>
+      <c r="D20" s="8">
+        <v>100</v>
+      </c>
+      <c r="E20" s="8">
+        <v>500000</v>
+      </c>
+      <c r="F20" t="s">
+        <v>124</v>
+      </c>
+      <c r="G20" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>509</v>
+      </c>
+      <c r="B21" s="40">
+        <v>5</v>
+      </c>
+      <c r="C21" s="40">
+        <v>100</v>
+      </c>
+      <c r="D21" s="40">
+        <v>100</v>
+      </c>
+      <c r="E21" s="40">
+        <v>500000</v>
+      </c>
+      <c r="F21" s="41" t="s">
+        <v>124</v>
+      </c>
+      <c r="G21" s="40">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
+ Make skill tooltips in character scene.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="2" activeTab="10"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="9" activeTab="17"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1979" uniqueCount="620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2024" uniqueCount="624">
   <si>
     <t>ID</t>
   </si>
@@ -1720,30 +1720,15 @@
     <t>effect_id</t>
   </si>
   <si>
-    <t>Action_Point_Boost</t>
-  </si>
-  <si>
-    <t>Reduce_Cooldown</t>
-  </si>
-  <si>
     <t>OnAfterAttack</t>
   </si>
   <si>
-    <t>FollowUp_BasicAttack</t>
-  </si>
-  <si>
     <t>OnTurnStart</t>
   </si>
   <si>
-    <t>Dispel_Debuff</t>
-  </si>
-  <si>
     <t>OnTakeDamage</t>
   </si>
   <si>
-    <t>Stackable_DEF_Buff</t>
-  </si>
-  <si>
     <t>condition_filter</t>
   </si>
   <si>
@@ -1771,33 +1756,18 @@
     <t>OnHit</t>
   </si>
   <si>
-    <t>Lacerate_Debuff</t>
-  </si>
-  <si>
     <t>OnSkillCast</t>
   </si>
   <si>
     <t>NonAttackSkill</t>
   </si>
   <si>
-    <t>Apply_Mark_Debuff</t>
-  </si>
-  <si>
-    <t>Dispel_Self_Debuff</t>
-  </si>
-  <si>
-    <t>80.0IsSkill, HasDebuff</t>
-  </si>
-  <si>
     <t>internal_cooldown</t>
   </si>
   <si>
     <t>OnBeforeAttack</t>
   </si>
   <si>
-    <t>Damage_Multiplier_Boost</t>
-  </si>
-  <si>
     <t>SkillType</t>
   </si>
   <si>
@@ -1870,21 +1840,6 @@
     <t>CRIT_DMG_RES</t>
   </si>
   <si>
-    <t>0, 0</t>
-  </si>
-  <si>
-    <t>1, 1.2</t>
-  </si>
-  <si>
-    <t>1, 1.5</t>
-  </si>
-  <si>
-    <t>1.5, 1.8</t>
-  </si>
-  <si>
-    <t>1, 1</t>
-  </si>
-  <si>
     <t>psv_sunwukong_main</t>
   </si>
   <si>
@@ -1901,6 +1856,63 @@
   </si>
   <si>
     <t>Gây {0}% ST Tấn Công cho kẻ định, kèm thêm Giảm Phòng Thù cho mục tiêu, duy trì 2 hiệp.</t>
+  </si>
+  <si>
+    <t>Eff_Action_Point_Boost</t>
+  </si>
+  <si>
+    <t>Eff_Reduce_Cooldown</t>
+  </si>
+  <si>
+    <t>Eff_FollowUp_BasicAttack</t>
+  </si>
+  <si>
+    <t>Eff_Dispel_Debuff</t>
+  </si>
+  <si>
+    <t>Eff_Stackable_DEF_Buff</t>
+  </si>
+  <si>
+    <t>Eff_Lacerate_Debuff</t>
+  </si>
+  <si>
+    <t>Eff_Apply_Mark_Debuff</t>
+  </si>
+  <si>
+    <t>Eff_Dispel_Self_Debuff</t>
+  </si>
+  <si>
+    <t>Eff_Damage_Multiplier_Boost</t>
+  </si>
+  <si>
+    <t>Eff_Heal_By_Attack</t>
+  </si>
+  <si>
+    <t>20, 30</t>
+  </si>
+  <si>
+    <t>Eff_Reduce_Def</t>
+  </si>
+  <si>
+    <t>0.8, 1, 1.2</t>
+  </si>
+  <si>
+    <t>1, 1.5, 1.5</t>
+  </si>
+  <si>
+    <t>4.0, 4.0, 3.0</t>
+  </si>
+  <si>
+    <t>1.5, 1.8, 1.8</t>
+  </si>
+  <si>
+    <t>5.0, 5.0, 4.0</t>
+  </si>
+  <si>
+    <t>0, 0, 0</t>
+  </si>
+  <si>
+    <t>1, 1, 1</t>
   </si>
 </sst>
 </file>
@@ -4993,7 +5005,7 @@
         <v>404</v>
       </c>
       <c r="H1" s="18" t="s">
-        <v>585</v>
+        <v>575</v>
       </c>
       <c r="I1" s="18" t="s">
         <v>405</v>
@@ -5024,16 +5036,16 @@
         <v>335</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G2" s="8">
         <v>100</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I2" s="8" t="s">
         <v>406</v>
@@ -5064,16 +5076,16 @@
         <v>337</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F3" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G3" s="8">
         <v>100</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I3" s="8" t="s">
         <v>408</v>
@@ -5085,7 +5097,7 @@
         <v>453</v>
       </c>
       <c r="L3" s="34" t="s">
-        <v>614</v>
+        <v>599</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -5104,16 +5116,16 @@
         <v>343</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F4" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G4" s="8">
         <v>100</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I4" s="8" t="s">
         <v>406</v>
@@ -5125,7 +5137,7 @@
         <v>452</v>
       </c>
       <c r="L4" s="34" t="s">
-        <v>615</v>
+        <v>600</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -5144,16 +5156,16 @@
         <v>336</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G5" s="8">
         <v>100</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I5" s="8" t="s">
         <v>406</v>
@@ -5184,16 +5196,16 @@
         <v>338</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F6" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G6" s="8">
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>407</v>
@@ -5224,16 +5236,16 @@
         <v>343</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F7" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G7" s="8">
         <v>100</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>406</v>
@@ -5264,16 +5276,16 @@
         <v>335</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G8" s="8">
         <v>100</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>406</v>
@@ -5304,16 +5316,16 @@
         <v>338</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F9" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G9" s="8">
         <v>100</v>
       </c>
       <c r="H9" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>407</v>
@@ -5344,16 +5356,16 @@
         <v>343</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F10" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G10" s="8">
         <v>100</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I10" s="8" t="s">
         <v>406</v>
@@ -5384,16 +5396,16 @@
         <v>335</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G11" s="8">
         <v>100</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>406</v>
@@ -5424,16 +5436,16 @@
         <v>339</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F12" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G12" s="8">
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="I12" s="8" t="s">
         <v>407</v>
@@ -5464,16 +5476,16 @@
         <v>343</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F13" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G13" s="8">
         <v>100</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I13" s="8" t="s">
         <v>406</v>
@@ -5504,16 +5516,16 @@
         <v>335</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G14" s="8">
         <v>100</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I14" s="8" t="s">
         <v>406</v>
@@ -5541,16 +5553,16 @@
         <v>350</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F15" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G15" s="8">
         <v>100</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I15" s="8" t="s">
         <v>406</v>
@@ -5578,16 +5590,16 @@
         <v>350</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F16" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G16" s="8">
         <v>100</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I16" s="8" t="s">
         <v>406</v>
@@ -5615,16 +5627,16 @@
         <v>335</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G17" s="8">
         <v>100</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I17" s="8" t="s">
         <v>406</v>
@@ -5655,16 +5667,16 @@
         <v>341</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F18" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G18" s="8">
         <v>100</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I18" s="8" t="s">
         <v>406</v>
@@ -5695,16 +5707,16 @@
         <v>343</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F19" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G19" s="8">
         <v>100</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I19" s="8" t="s">
         <v>406</v>
@@ -5735,16 +5747,16 @@
         <v>335</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G20" s="8">
         <v>100</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I20" s="8" t="s">
         <v>406</v>
@@ -5775,16 +5787,16 @@
         <v>340</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F21" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G21" s="8">
         <v>100</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I21" s="8" t="s">
         <v>406</v>
@@ -5815,16 +5827,16 @@
         <v>343</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F22" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G22" s="8">
         <v>100</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>406</v>
@@ -5855,16 +5867,16 @@
         <v>335</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G23" s="8">
         <v>100</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I23" s="8" t="s">
         <v>406</v>
@@ -5895,16 +5907,16 @@
         <v>447</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F24" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G24" s="8">
         <v>0</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I24" s="8" t="s">
         <v>407</v>
@@ -5935,16 +5947,16 @@
         <v>446</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F25" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G25" s="8">
         <v>100</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>406</v>
@@ -5975,16 +5987,16 @@
         <v>335</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G26" s="8">
         <v>100</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I26" s="8" t="s">
         <v>406</v>
@@ -6012,16 +6024,16 @@
         <v>350</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F27" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G27" s="8">
         <v>100</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I27" s="8" t="s">
         <v>406</v>
@@ -6049,16 +6061,16 @@
         <v>350</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F28" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G28" s="8">
         <v>100</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I28" s="8" t="s">
         <v>406</v>
@@ -6086,16 +6098,16 @@
         <v>336</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G29" s="8">
         <v>100</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>406</v>
@@ -6123,16 +6135,16 @@
         <v>350</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F30" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G30" s="8">
         <v>100</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I30" s="8" t="s">
         <v>406</v>
@@ -6160,16 +6172,16 @@
         <v>350</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F31" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G31" s="8">
         <v>100</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I31" s="8" t="s">
         <v>406</v>
@@ -6197,16 +6209,16 @@
         <v>335</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>613</v>
-      </c>
-      <c r="F32" s="8">
-        <v>0</v>
+        <v>623</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>622</v>
       </c>
       <c r="G32" s="8">
         <v>100</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I32" s="8" t="s">
         <v>406</v>
@@ -6237,16 +6249,16 @@
         <v>335</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G33" s="8">
         <v>100</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I33" s="8" t="s">
         <v>406</v>
@@ -6277,16 +6289,16 @@
         <v>342</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F34" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G34" s="8">
         <v>100</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I34" s="8" t="s">
         <v>406</v>
@@ -6317,16 +6329,16 @@
         <v>343</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F35" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G35" s="8">
         <v>100</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I35" s="8" t="s">
         <v>406</v>
@@ -6357,16 +6369,16 @@
         <v>335</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G36" s="8">
         <v>100</v>
       </c>
       <c r="H36" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I36" s="8" t="s">
         <v>406</v>
@@ -6397,16 +6409,16 @@
         <v>351</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F37" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G37" s="8">
         <v>100</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I37" s="8" t="s">
         <v>406</v>
@@ -6437,16 +6449,16 @@
         <v>343</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F38" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G38" s="8">
         <v>100</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I38" s="8" t="s">
         <v>406</v>
@@ -6477,16 +6489,16 @@
         <v>335</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G39" s="8">
         <v>100</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>406</v>
@@ -6517,16 +6529,16 @@
         <v>344</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F40" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G40" s="8">
         <v>100</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I40" s="8" t="s">
         <v>406</v>
@@ -6557,16 +6569,16 @@
         <v>343</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F41" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G41" s="8">
         <v>100</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I41" s="8" t="s">
         <v>406</v>
@@ -6597,16 +6609,16 @@
         <v>335</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G42" s="8">
         <v>100</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I42" s="8" t="s">
         <v>406</v>
@@ -6637,16 +6649,16 @@
         <v>345</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F43" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F43" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G43" s="8">
         <v>1000</v>
       </c>
       <c r="H43" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I43" s="8" t="s">
         <v>406</v>
@@ -6677,16 +6689,16 @@
         <v>346</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F44" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G44" s="8">
         <v>100</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I44" s="8" t="s">
         <v>406</v>
@@ -6717,16 +6729,16 @@
         <v>335</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G45" s="8">
         <v>100</v>
       </c>
       <c r="H45" s="8" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="I45" s="8" t="s">
         <v>406</v>
@@ -6757,16 +6769,16 @@
         <v>351</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F46" s="8">
-        <v>4.3</v>
+        <v>618</v>
+      </c>
+      <c r="F46" s="8" t="s">
+        <v>619</v>
       </c>
       <c r="G46" s="8">
         <v>100</v>
       </c>
       <c r="H46" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I46" s="8" t="s">
         <v>406</v>
@@ -6797,16 +6809,16 @@
         <v>343</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F47" s="8">
-        <v>5.4</v>
+        <v>620</v>
+      </c>
+      <c r="F47" s="8" t="s">
+        <v>621</v>
       </c>
       <c r="G47" s="8">
         <v>100</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="I47" s="8" t="s">
         <v>406</v>
@@ -6837,16 +6849,16 @@
         <v>350</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G48" s="8">
         <v>100</v>
       </c>
       <c r="H48" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="I48" s="8" t="s">
         <v>406</v>
@@ -12677,7 +12689,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" customWidth="1"/>
@@ -12708,7 +12720,7 @@
         <v>510</v>
       </c>
       <c r="B2" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2">
         <v>10000</v>
@@ -12722,7 +12734,7 @@
         <v>510</v>
       </c>
       <c r="B3" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3">
         <v>20000</v>
@@ -12736,7 +12748,7 @@
         <v>510</v>
       </c>
       <c r="B4" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4">
         <v>50000</v>
@@ -12750,7 +12762,7 @@
         <v>510</v>
       </c>
       <c r="B5" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5">
         <v>100000</v>
@@ -12764,7 +12776,7 @@
         <v>510</v>
       </c>
       <c r="B6" s="7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6">
         <v>250000</v>
@@ -12774,17 +12786,17 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
-        <v>511</v>
+      <c r="A7" t="s">
+        <v>510</v>
       </c>
       <c r="B7" s="7">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C7">
-        <v>10000</v>
+        <v>500000</v>
       </c>
       <c r="D7">
-        <v>60</v>
+        <v>600</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -12792,13 +12804,13 @@
         <v>511</v>
       </c>
       <c r="B8" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C8">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="D8">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -12806,13 +12818,13 @@
         <v>511</v>
       </c>
       <c r="B9" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C9">
-        <v>50000</v>
+        <v>20000</v>
       </c>
       <c r="D9">
-        <v>240</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -12820,13 +12832,13 @@
         <v>511</v>
       </c>
       <c r="B10" s="7">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C10">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="D10">
-        <v>360</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -12834,41 +12846,41 @@
         <v>511</v>
       </c>
       <c r="B11" s="7">
+        <v>4</v>
+      </c>
+      <c r="C11">
+        <v>100000</v>
+      </c>
+      <c r="D11">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>511</v>
+      </c>
+      <c r="B12" s="7">
+        <v>5</v>
+      </c>
+      <c r="C12">
+        <v>250000</v>
+      </c>
+      <c r="D12">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>511</v>
+      </c>
+      <c r="B13" s="7">
         <v>6</v>
       </c>
-      <c r="C11">
-        <v>250000</v>
-      </c>
-      <c r="D11">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="33" t="s">
-        <v>512</v>
-      </c>
-      <c r="B12" s="7">
-        <v>2</v>
-      </c>
-      <c r="C12">
-        <v>10000</v>
-      </c>
-      <c r="D12">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="33" t="s">
-        <v>512</v>
-      </c>
-      <c r="B13" s="7">
-        <v>3</v>
-      </c>
       <c r="C13">
-        <v>20000</v>
+        <v>500000</v>
       </c>
       <c r="D13">
-        <v>120</v>
+        <v>480</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -12876,13 +12888,13 @@
         <v>512</v>
       </c>
       <c r="B14" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C14">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c r="D14">
-        <v>240</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -12890,13 +12902,13 @@
         <v>512</v>
       </c>
       <c r="B15" s="7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C15">
-        <v>100000</v>
+        <v>20000</v>
       </c>
       <c r="D15">
-        <v>300</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -12904,55 +12916,55 @@
         <v>512</v>
       </c>
       <c r="B16" s="7">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>50000</v>
+      </c>
+      <c r="D16">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="33" t="s">
+        <v>512</v>
+      </c>
+      <c r="B17" s="7">
+        <v>4</v>
+      </c>
+      <c r="C17">
+        <v>100000</v>
+      </c>
+      <c r="D17">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="33" t="s">
+        <v>512</v>
+      </c>
+      <c r="B18" s="7">
+        <v>5</v>
+      </c>
+      <c r="C18">
+        <v>250000</v>
+      </c>
+      <c r="D18">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="33" t="s">
+        <v>512</v>
+      </c>
+      <c r="B19" s="7">
         <v>6</v>
       </c>
-      <c r="C16">
-        <v>250000</v>
-      </c>
-      <c r="D16">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
-        <v>513</v>
-      </c>
-      <c r="B17" s="7">
-        <v>2</v>
-      </c>
-      <c r="C17">
-        <v>10000</v>
-      </c>
-      <c r="D17">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
-        <v>513</v>
-      </c>
-      <c r="B18" s="7">
-        <v>3</v>
-      </c>
-      <c r="C18">
-        <v>20000</v>
-      </c>
-      <c r="D18">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
-        <v>513</v>
-      </c>
-      <c r="B19" s="7">
-        <v>4</v>
-      </c>
       <c r="C19">
-        <v>50000</v>
+        <v>500000</v>
       </c>
       <c r="D19">
-        <v>180</v>
+        <v>420</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -12960,13 +12972,13 @@
         <v>513</v>
       </c>
       <c r="B20" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C20">
-        <v>100000</v>
+        <v>10000</v>
       </c>
       <c r="D20">
-        <v>240</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -12974,13 +12986,69 @@
         <v>513</v>
       </c>
       <c r="B21" s="7">
+        <v>2</v>
+      </c>
+      <c r="C21">
+        <v>20000</v>
+      </c>
+      <c r="D21">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>513</v>
+      </c>
+      <c r="B22" s="7">
+        <v>3</v>
+      </c>
+      <c r="C22">
+        <v>50000</v>
+      </c>
+      <c r="D22">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>513</v>
+      </c>
+      <c r="B23" s="7">
+        <v>4</v>
+      </c>
+      <c r="C23">
+        <v>100000</v>
+      </c>
+      <c r="D23">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
+        <v>513</v>
+      </c>
+      <c r="B24" s="7">
+        <v>5</v>
+      </c>
+      <c r="C24">
+        <v>250000</v>
+      </c>
+      <c r="D24">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
+        <v>513</v>
+      </c>
+      <c r="B25" s="7">
         <v>6</v>
       </c>
-      <c r="C21">
-        <v>250000</v>
-      </c>
-      <c r="D21">
-        <v>300</v>
+      <c r="C25">
+        <v>500000</v>
+      </c>
+      <c r="D25">
+        <v>360</v>
       </c>
     </row>
   </sheetData>
@@ -13900,24 +13968,24 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="34" t="s">
-        <v>614</v>
+        <v>599</v>
       </c>
       <c r="B16" t="s">
-        <v>616</v>
+        <v>601</v>
       </c>
       <c r="C16" t="s">
-        <v>618</v>
+        <v>603</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="34" t="s">
-        <v>615</v>
+        <v>600</v>
       </c>
       <c r="B17" t="s">
-        <v>617</v>
+        <v>602</v>
       </c>
       <c r="C17" t="s">
-        <v>619</v>
+        <v>604</v>
       </c>
     </row>
   </sheetData>
@@ -13965,7 +14033,7 @@
         <v>444</v>
       </c>
       <c r="D2" t="s">
-        <v>588</v>
+        <v>578</v>
       </c>
       <c r="E2" t="s">
         <v>521</v>
@@ -13982,7 +14050,7 @@
         <v>444</v>
       </c>
       <c r="D3" t="s">
-        <v>588</v>
+        <v>578</v>
       </c>
       <c r="E3" t="s">
         <v>521</v>
@@ -13999,7 +14067,7 @@
         <v>444</v>
       </c>
       <c r="D4" t="s">
-        <v>589</v>
+        <v>579</v>
       </c>
       <c r="E4" t="s">
         <v>522</v>
@@ -14016,7 +14084,7 @@
         <v>444</v>
       </c>
       <c r="D5" t="s">
-        <v>589</v>
+        <v>579</v>
       </c>
       <c r="E5" t="s">
         <v>523</v>
@@ -14033,7 +14101,7 @@
         <v>444</v>
       </c>
       <c r="D6" t="s">
-        <v>589</v>
+        <v>579</v>
       </c>
       <c r="E6" t="s">
         <v>548</v>
@@ -14050,7 +14118,7 @@
         <v>444</v>
       </c>
       <c r="D7" t="s">
-        <v>590</v>
+        <v>580</v>
       </c>
       <c r="E7" t="s">
         <v>524</v>
@@ -14067,7 +14135,7 @@
         <v>444</v>
       </c>
       <c r="D8" t="s">
-        <v>590</v>
+        <v>580</v>
       </c>
       <c r="E8" t="s">
         <v>524</v>
@@ -14084,7 +14152,7 @@
         <v>444</v>
       </c>
       <c r="D9" t="s">
-        <v>591</v>
+        <v>581</v>
       </c>
       <c r="E9" t="s">
         <v>527</v>
@@ -14101,7 +14169,7 @@
         <v>444</v>
       </c>
       <c r="D10" t="s">
-        <v>590</v>
+        <v>580</v>
       </c>
       <c r="E10" t="s">
         <v>528</v>
@@ -14118,7 +14186,7 @@
         <v>444</v>
       </c>
       <c r="D11" t="s">
-        <v>592</v>
+        <v>582</v>
       </c>
       <c r="E11" t="s">
         <v>529</v>
@@ -14135,7 +14203,7 @@
         <v>444</v>
       </c>
       <c r="D12" t="s">
-        <v>593</v>
+        <v>583</v>
       </c>
       <c r="E12" t="s">
         <v>530</v>
@@ -14152,7 +14220,7 @@
         <v>444</v>
       </c>
       <c r="D13" t="s">
-        <v>594</v>
+        <v>584</v>
       </c>
       <c r="E13" t="s">
         <v>547</v>
@@ -14169,7 +14237,7 @@
         <v>444</v>
       </c>
       <c r="D14" t="s">
-        <v>595</v>
+        <v>585</v>
       </c>
       <c r="E14" t="s">
         <v>547</v>
@@ -14186,7 +14254,7 @@
         <v>444</v>
       </c>
       <c r="D15" t="s">
-        <v>596</v>
+        <v>586</v>
       </c>
       <c r="E15" t="s">
         <v>531</v>
@@ -14203,7 +14271,7 @@
         <v>444</v>
       </c>
       <c r="D16" t="s">
-        <v>597</v>
+        <v>587</v>
       </c>
       <c r="E16" t="s">
         <v>532</v>
@@ -14221,7 +14289,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
@@ -14247,13 +14315,13 @@
         <v>552</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>567</v>
+        <v>562</v>
       </c>
       <c r="F1" s="18" t="s">
-        <v>571</v>
+        <v>566</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>582</v>
+        <v>573</v>
       </c>
       <c r="H1" s="18" t="s">
         <v>520</v>
@@ -14264,16 +14332,16 @@
         <v>533</v>
       </c>
       <c r="B2" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="C2" t="s">
-        <v>559</v>
+        <v>605</v>
       </c>
       <c r="D2" t="s">
-        <v>598</v>
+        <v>588</v>
       </c>
       <c r="E2" t="s">
-        <v>572</v>
+        <v>567</v>
       </c>
       <c r="F2" s="8">
         <v>0</v>
@@ -14288,16 +14356,16 @@
         <v>534</v>
       </c>
       <c r="B3" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="C3" t="s">
-        <v>560</v>
+        <v>606</v>
       </c>
       <c r="D3" t="s">
-        <v>599</v>
+        <v>589</v>
       </c>
       <c r="E3" t="s">
-        <v>573</v>
+        <v>568</v>
       </c>
       <c r="F3" s="8">
         <v>1</v>
@@ -14314,16 +14382,16 @@
         <v>535</v>
       </c>
       <c r="B4" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="C4" t="s">
-        <v>562</v>
+        <v>607</v>
       </c>
       <c r="D4" t="s">
-        <v>599</v>
+        <v>589</v>
       </c>
       <c r="E4" t="s">
-        <v>569</v>
+        <v>564</v>
       </c>
       <c r="F4" s="8"/>
       <c r="G4" s="8">
@@ -14338,16 +14406,16 @@
         <v>536</v>
       </c>
       <c r="B5" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="C5" t="s">
-        <v>564</v>
+        <v>608</v>
       </c>
       <c r="D5" t="s">
-        <v>599</v>
+        <v>589</v>
       </c>
       <c r="E5" t="s">
-        <v>570</v>
+        <v>565</v>
       </c>
       <c r="F5" s="8">
         <v>1</v>
@@ -14364,16 +14432,16 @@
         <v>537</v>
       </c>
       <c r="B6" t="s">
-        <v>565</v>
+        <v>561</v>
       </c>
       <c r="C6" t="s">
-        <v>566</v>
+        <v>609</v>
       </c>
       <c r="D6" t="s">
-        <v>600</v>
+        <v>590</v>
       </c>
       <c r="E6" s="37" t="s">
-        <v>568</v>
+        <v>563</v>
       </c>
       <c r="F6" s="8">
         <v>6</v>
@@ -14390,16 +14458,16 @@
         <v>538</v>
       </c>
       <c r="B7" t="s">
-        <v>565</v>
+        <v>561</v>
       </c>
       <c r="C7" t="s">
-        <v>559</v>
+        <v>605</v>
       </c>
       <c r="D7" t="s">
-        <v>598</v>
+        <v>588</v>
       </c>
       <c r="E7" t="s">
-        <v>574</v>
+        <v>569</v>
       </c>
       <c r="F7" s="8">
         <v>0</v>
@@ -14416,16 +14484,16 @@
         <v>540</v>
       </c>
       <c r="B8" t="s">
-        <v>575</v>
+        <v>570</v>
       </c>
       <c r="C8" t="s">
-        <v>576</v>
+        <v>610</v>
       </c>
       <c r="D8" t="s">
-        <v>599</v>
+        <v>589</v>
       </c>
       <c r="E8" t="s">
-        <v>568</v>
+        <v>563</v>
       </c>
       <c r="F8" s="8">
         <v>2</v>
@@ -14440,16 +14508,16 @@
         <v>544</v>
       </c>
       <c r="B9" t="s">
-        <v>577</v>
+        <v>571</v>
       </c>
       <c r="C9" t="s">
-        <v>560</v>
+        <v>606</v>
       </c>
       <c r="D9" t="s">
-        <v>599</v>
+        <v>589</v>
       </c>
       <c r="E9" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="F9" s="8">
         <v>1</v>
@@ -14466,16 +14534,16 @@
         <v>545</v>
       </c>
       <c r="B10" t="s">
-        <v>575</v>
+        <v>570</v>
       </c>
       <c r="C10" t="s">
-        <v>579</v>
+        <v>611</v>
       </c>
       <c r="D10" t="s">
-        <v>601</v>
+        <v>591</v>
       </c>
       <c r="E10" t="s">
-        <v>568</v>
+        <v>563</v>
       </c>
       <c r="F10" s="8">
         <v>1</v>
@@ -14492,16 +14560,16 @@
         <v>546</v>
       </c>
       <c r="B11" t="s">
+        <v>561</v>
+      </c>
+      <c r="C11" t="s">
+        <v>612</v>
+      </c>
+      <c r="D11" t="s">
+        <v>591</v>
+      </c>
+      <c r="E11" t="s">
         <v>565</v>
-      </c>
-      <c r="C11" t="s">
-        <v>580</v>
-      </c>
-      <c r="D11" t="s">
-        <v>601</v>
-      </c>
-      <c r="E11" t="s">
-        <v>581</v>
       </c>
       <c r="F11" s="8">
         <v>2</v>
@@ -14518,16 +14586,16 @@
         <v>539</v>
       </c>
       <c r="B12" t="s">
-        <v>583</v>
+        <v>574</v>
       </c>
       <c r="C12" t="s">
-        <v>584</v>
+        <v>613</v>
       </c>
       <c r="D12" t="s">
-        <v>598</v>
+        <v>588</v>
       </c>
       <c r="E12" t="s">
-        <v>568</v>
+        <v>563</v>
       </c>
       <c r="F12" s="8">
         <v>0</v>
@@ -14537,6 +14605,40 @@
       </c>
       <c r="H12" t="s">
         <v>526</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="34" t="s">
+        <v>599</v>
+      </c>
+      <c r="B13" t="s">
+        <v>559</v>
+      </c>
+      <c r="C13" t="s">
+        <v>614</v>
+      </c>
+      <c r="D13" t="s">
+        <v>615</v>
+      </c>
+      <c r="E13" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="34" t="s">
+        <v>600</v>
+      </c>
+      <c r="B14" t="s">
+        <v>559</v>
+      </c>
+      <c r="C14" t="s">
+        <v>616</v>
+      </c>
+      <c r="D14" t="s">
+        <v>615</v>
+      </c>
+      <c r="E14" t="s">
+        <v>563</v>
       </c>
     </row>
   </sheetData>
@@ -14579,7 +14681,7 @@
         <v>488</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>602</v>
+        <v>592</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -14602,7 +14704,7 @@
         <v>445</v>
       </c>
       <c r="G2" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="I2" s="8"/>
     </row>
@@ -14626,7 +14728,7 @@
         <v>445</v>
       </c>
       <c r="G3" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -14649,7 +14751,7 @@
         <v>445</v>
       </c>
       <c r="G4" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -14672,7 +14774,7 @@
         <v>445</v>
       </c>
       <c r="G5" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -14695,7 +14797,7 @@
         <v>445</v>
       </c>
       <c r="G6" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -14718,7 +14820,7 @@
         <v>445</v>
       </c>
       <c r="G7" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -14741,7 +14843,7 @@
         <v>445</v>
       </c>
       <c r="G8" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -14764,7 +14866,7 @@
         <v>445</v>
       </c>
       <c r="G9" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -14787,7 +14889,7 @@
         <v>445</v>
       </c>
       <c r="G10" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -14810,7 +14912,7 @@
         <v>445</v>
       </c>
       <c r="G11" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -14833,7 +14935,7 @@
         <v>445</v>
       </c>
       <c r="G12" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -14856,7 +14958,7 @@
         <v>445</v>
       </c>
       <c r="G13" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -14879,7 +14981,7 @@
         <v>445</v>
       </c>
       <c r="G14" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -14902,7 +15004,7 @@
         <v>445</v>
       </c>
       <c r="G15" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -14925,7 +15027,7 @@
         <v>445</v>
       </c>
       <c r="G16" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -14948,7 +15050,7 @@
         <v>445</v>
       </c>
       <c r="G17" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -14971,7 +15073,7 @@
         <v>445</v>
       </c>
       <c r="G18" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -14994,7 +15096,7 @@
         <v>445</v>
       </c>
       <c r="G19" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -15017,7 +15119,7 @@
         <v>445</v>
       </c>
       <c r="G20" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -15040,7 +15142,7 @@
         <v>445</v>
       </c>
       <c r="G21" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -15063,7 +15165,7 @@
         <v>445</v>
       </c>
       <c r="G22" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -15086,7 +15188,7 @@
         <v>445</v>
       </c>
       <c r="G23" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -15109,7 +15211,7 @@
         <v>445</v>
       </c>
       <c r="G24" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -15132,7 +15234,7 @@
         <v>445</v>
       </c>
       <c r="G25" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -15155,7 +15257,7 @@
         <v>445</v>
       </c>
       <c r="G26" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -15178,7 +15280,7 @@
         <v>445</v>
       </c>
       <c r="G27" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -15201,7 +15303,7 @@
         <v>445</v>
       </c>
       <c r="G28" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -15224,7 +15326,7 @@
         <v>445</v>
       </c>
       <c r="G29" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -15247,7 +15349,7 @@
         <v>445</v>
       </c>
       <c r="G30" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -15270,7 +15372,7 @@
         <v>445</v>
       </c>
       <c r="G31" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -15293,7 +15395,7 @@
         <v>445</v>
       </c>
       <c r="G32" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -15316,7 +15418,7 @@
         <v>445</v>
       </c>
       <c r="G33" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -15339,7 +15441,7 @@
         <v>445</v>
       </c>
       <c r="G34" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -15362,7 +15464,7 @@
         <v>445</v>
       </c>
       <c r="G35" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -15385,7 +15487,7 @@
         <v>445</v>
       </c>
       <c r="G36" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -15408,7 +15510,7 @@
         <v>445</v>
       </c>
       <c r="G37" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
   </sheetData>
@@ -15434,13 +15536,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>603</v>
+        <v>593</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>604</v>
+        <v>594</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>605</v>
+        <v>595</v>
       </c>
       <c r="E1" s="18" t="s">
         <v>517</v>
@@ -15448,7 +15550,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>69</v>
@@ -15465,7 +15567,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>70</v>
@@ -15482,7 +15584,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>419</v>
@@ -15499,7 +15601,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>420</v>
@@ -15516,7 +15618,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>554</v>
@@ -15533,7 +15635,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>553</v>
@@ -15550,10 +15652,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>607</v>
+        <v>597</v>
       </c>
       <c r="C8" s="7">
         <v>10</v>
@@ -15567,10 +15669,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>608</v>
+        <v>598</v>
       </c>
       <c r="C9" s="7">
         <v>10</v>

</xml_diff>

<commit_message>
+ Make passive system for battle in game.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="9" activeTab="17"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="3" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2024" uniqueCount="624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2040" uniqueCount="630">
   <si>
     <t>ID</t>
   </si>
@@ -1720,12 +1720,6 @@
     <t>effect_id</t>
   </si>
   <si>
-    <t>OnAfterAttack</t>
-  </si>
-  <si>
-    <t>OnTurnStart</t>
-  </si>
-  <si>
     <t>OnTakeDamage</t>
   </si>
   <si>
@@ -1753,21 +1747,12 @@
     <t>AoEAttack</t>
   </si>
   <si>
-    <t>OnHit</t>
-  </si>
-  <si>
-    <t>OnSkillCast</t>
-  </si>
-  <si>
     <t>NonAttackSkill</t>
   </si>
   <si>
     <t>internal_cooldown</t>
   </si>
   <si>
-    <t>OnBeforeAttack</t>
-  </si>
-  <si>
     <t>SkillType</t>
   </si>
   <si>
@@ -1840,9 +1825,6 @@
     <t>CRIT_DMG_RES</t>
   </si>
   <si>
-    <t>psv_sunwukong_main</t>
-  </si>
-  <si>
     <t>psv_sunwukong_ultiamte</t>
   </si>
   <si>
@@ -1867,9 +1849,6 @@
     <t>Eff_FollowUp_BasicAttack</t>
   </si>
   <si>
-    <t>Eff_Dispel_Debuff</t>
-  </si>
-  <si>
     <t>Eff_Stackable_DEF_Buff</t>
   </si>
   <si>
@@ -1882,18 +1861,9 @@
     <t>Eff_Dispel_Self_Debuff</t>
   </si>
   <si>
-    <t>Eff_Damage_Multiplier_Boost</t>
-  </si>
-  <si>
-    <t>Eff_Heal_By_Attack</t>
-  </si>
-  <si>
     <t>20, 30</t>
   </si>
   <si>
-    <t>Eff_Reduce_Def</t>
-  </si>
-  <si>
     <t>0.8, 1, 1.2</t>
   </si>
   <si>
@@ -1913,6 +1883,54 @@
   </si>
   <si>
     <t>1, 1, 1</t>
+  </si>
+  <si>
+    <t>UltimateSkill</t>
+  </si>
+  <si>
+    <t>MajorSkill</t>
+  </si>
+  <si>
+    <t>psv_sunwukong_major</t>
+  </si>
+  <si>
+    <t>OnAfterSkillExcute</t>
+  </si>
+  <si>
+    <t>OnSkillStart</t>
+  </si>
+  <si>
+    <t>OnAfterTakeDamage</t>
+  </si>
+  <si>
+    <t>OnAfterDealDamage</t>
+  </si>
+  <si>
+    <t>OnBeforeDealDamage</t>
+  </si>
+  <si>
+    <t>OnAfterSkillExecute</t>
+  </si>
+  <si>
+    <t>target</t>
+  </si>
+  <si>
+    <t>self</t>
+  </si>
+  <si>
+    <t>enemy</t>
+  </si>
+  <si>
+    <t>Eff_ReduceDefense</t>
+  </si>
+  <si>
+    <t>Eff_Cleanse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eff_IncreaseAttack </t>
+  </si>
+  <si>
+    <t>Eff_Lifesteal</t>
   </si>
 </sst>
 </file>
@@ -4978,7 +4996,7 @@
     <col min="7" max="8" width="16.85546875" customWidth="1"/>
     <col min="9" max="9" width="16.5703125" customWidth="1"/>
     <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="26.42578125" customWidth="1"/>
     <col min="12" max="12" width="24.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5005,7 +5023,7 @@
         <v>404</v>
       </c>
       <c r="H1" s="18" t="s">
-        <v>575</v>
+        <v>570</v>
       </c>
       <c r="I1" s="18" t="s">
         <v>405</v>
@@ -5036,16 +5054,16 @@
         <v>335</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G2" s="8">
         <v>100</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I2" s="8" t="s">
         <v>406</v>
@@ -5076,16 +5094,16 @@
         <v>337</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G3" s="8">
         <v>100</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I3" s="8" t="s">
         <v>408</v>
@@ -5097,7 +5115,7 @@
         <v>453</v>
       </c>
       <c r="L3" s="34" t="s">
-        <v>599</v>
+        <v>616</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -5116,16 +5134,16 @@
         <v>343</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G4" s="8">
         <v>100</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I4" s="8" t="s">
         <v>406</v>
@@ -5137,7 +5155,7 @@
         <v>452</v>
       </c>
       <c r="L4" s="34" t="s">
-        <v>600</v>
+        <v>594</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -5156,16 +5174,16 @@
         <v>336</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G5" s="8">
         <v>100</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I5" s="8" t="s">
         <v>406</v>
@@ -5196,16 +5214,16 @@
         <v>338</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G6" s="8">
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>572</v>
+        <v>568</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>407</v>
@@ -5236,16 +5254,16 @@
         <v>343</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G7" s="8">
         <v>100</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>406</v>
@@ -5276,16 +5294,16 @@
         <v>335</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G8" s="8">
         <v>100</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>406</v>
@@ -5316,16 +5334,16 @@
         <v>338</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G9" s="8">
         <v>100</v>
       </c>
       <c r="H9" t="s">
-        <v>572</v>
+        <v>568</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>407</v>
@@ -5356,16 +5374,16 @@
         <v>343</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G10" s="8">
         <v>100</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I10" s="8" t="s">
         <v>406</v>
@@ -5396,16 +5414,16 @@
         <v>335</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G11" s="8">
         <v>100</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>406</v>
@@ -5436,16 +5454,16 @@
         <v>339</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G12" s="8">
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>572</v>
+        <v>568</v>
       </c>
       <c r="I12" s="8" t="s">
         <v>407</v>
@@ -5476,16 +5494,16 @@
         <v>343</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G13" s="8">
         <v>100</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I13" s="8" t="s">
         <v>406</v>
@@ -5516,16 +5534,16 @@
         <v>335</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G14" s="8">
         <v>100</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I14" s="8" t="s">
         <v>406</v>
@@ -5553,16 +5571,16 @@
         <v>350</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G15" s="8">
         <v>100</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I15" s="8" t="s">
         <v>406</v>
@@ -5590,16 +5608,16 @@
         <v>350</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G16" s="8">
         <v>100</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I16" s="8" t="s">
         <v>406</v>
@@ -5627,16 +5645,16 @@
         <v>335</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G17" s="8">
         <v>100</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I17" s="8" t="s">
         <v>406</v>
@@ -5667,16 +5685,16 @@
         <v>341</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G18" s="8">
         <v>100</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I18" s="8" t="s">
         <v>406</v>
@@ -5707,16 +5725,16 @@
         <v>343</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G19" s="8">
         <v>100</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I19" s="8" t="s">
         <v>406</v>
@@ -5747,16 +5765,16 @@
         <v>335</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G20" s="8">
         <v>100</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I20" s="8" t="s">
         <v>406</v>
@@ -5787,16 +5805,16 @@
         <v>340</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G21" s="8">
         <v>100</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I21" s="8" t="s">
         <v>406</v>
@@ -5827,16 +5845,16 @@
         <v>343</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G22" s="8">
         <v>100</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>406</v>
@@ -5867,16 +5885,16 @@
         <v>335</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G23" s="8">
         <v>100</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I23" s="8" t="s">
         <v>406</v>
@@ -5907,16 +5925,16 @@
         <v>447</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G24" s="8">
         <v>0</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I24" s="8" t="s">
         <v>407</v>
@@ -5947,16 +5965,16 @@
         <v>446</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G25" s="8">
         <v>100</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>406</v>
@@ -5987,16 +6005,16 @@
         <v>335</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G26" s="8">
         <v>100</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I26" s="8" t="s">
         <v>406</v>
@@ -6024,16 +6042,16 @@
         <v>350</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G27" s="8">
         <v>100</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I27" s="8" t="s">
         <v>406</v>
@@ -6061,16 +6079,16 @@
         <v>350</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G28" s="8">
         <v>100</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I28" s="8" t="s">
         <v>406</v>
@@ -6098,16 +6116,16 @@
         <v>336</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G29" s="8">
         <v>100</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>406</v>
@@ -6135,16 +6153,16 @@
         <v>350</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G30" s="8">
         <v>100</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I30" s="8" t="s">
         <v>406</v>
@@ -6172,16 +6190,16 @@
         <v>350</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G31" s="8">
         <v>100</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I31" s="8" t="s">
         <v>406</v>
@@ -6209,16 +6227,16 @@
         <v>335</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>623</v>
+        <v>613</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G32" s="8">
         <v>100</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I32" s="8" t="s">
         <v>406</v>
@@ -6249,16 +6267,16 @@
         <v>335</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G33" s="8">
         <v>100</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I33" s="8" t="s">
         <v>406</v>
@@ -6289,16 +6307,16 @@
         <v>342</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G34" s="8">
         <v>100</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I34" s="8" t="s">
         <v>406</v>
@@ -6329,16 +6347,16 @@
         <v>343</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G35" s="8">
         <v>100</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I35" s="8" t="s">
         <v>406</v>
@@ -6369,16 +6387,16 @@
         <v>335</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G36" s="8">
         <v>100</v>
       </c>
       <c r="H36" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I36" s="8" t="s">
         <v>406</v>
@@ -6409,16 +6427,16 @@
         <v>351</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G37" s="8">
         <v>100</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I37" s="8" t="s">
         <v>406</v>
@@ -6449,16 +6467,16 @@
         <v>343</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G38" s="8">
         <v>100</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I38" s="8" t="s">
         <v>406</v>
@@ -6489,16 +6507,16 @@
         <v>335</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G39" s="8">
         <v>100</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>406</v>
@@ -6529,16 +6547,16 @@
         <v>344</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G40" s="8">
         <v>100</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I40" s="8" t="s">
         <v>406</v>
@@ -6569,16 +6587,16 @@
         <v>343</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G41" s="8">
         <v>100</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I41" s="8" t="s">
         <v>406</v>
@@ -6609,16 +6627,16 @@
         <v>335</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G42" s="8">
         <v>100</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I42" s="8" t="s">
         <v>406</v>
@@ -6649,16 +6667,16 @@
         <v>345</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G43" s="8">
         <v>1000</v>
       </c>
       <c r="H43" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I43" s="8" t="s">
         <v>406</v>
@@ -6689,16 +6707,16 @@
         <v>346</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G44" s="8">
         <v>100</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I44" s="8" t="s">
         <v>406</v>
@@ -6729,16 +6747,16 @@
         <v>335</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G45" s="8">
         <v>100</v>
       </c>
       <c r="H45" s="8" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="I45" s="8" t="s">
         <v>406</v>
@@ -6769,16 +6787,16 @@
         <v>351</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F46" s="8" t="s">
-        <v>619</v>
+        <v>609</v>
       </c>
       <c r="G46" s="8">
         <v>100</v>
       </c>
       <c r="H46" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I46" s="8" t="s">
         <v>406</v>
@@ -6809,16 +6827,16 @@
         <v>343</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>620</v>
+        <v>610</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>621</v>
+        <v>611</v>
       </c>
       <c r="G47" s="8">
         <v>100</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="I47" s="8" t="s">
         <v>406</v>
@@ -6849,16 +6867,16 @@
         <v>350</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="G48" s="8">
         <v>100</v>
       </c>
       <c r="H48" t="s">
-        <v>572</v>
+        <v>568</v>
       </c>
       <c r="I48" s="8" t="s">
         <v>406</v>
@@ -13968,24 +13986,24 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="34" t="s">
-        <v>599</v>
+        <v>616</v>
       </c>
       <c r="B16" t="s">
-        <v>601</v>
+        <v>595</v>
       </c>
       <c r="C16" t="s">
-        <v>603</v>
+        <v>597</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="34" t="s">
-        <v>600</v>
+        <v>594</v>
       </c>
       <c r="B17" t="s">
-        <v>602</v>
+        <v>596</v>
       </c>
       <c r="C17" t="s">
-        <v>604</v>
+        <v>598</v>
       </c>
     </row>
   </sheetData>
@@ -14033,7 +14051,7 @@
         <v>444</v>
       </c>
       <c r="D2" t="s">
-        <v>578</v>
+        <v>573</v>
       </c>
       <c r="E2" t="s">
         <v>521</v>
@@ -14050,7 +14068,7 @@
         <v>444</v>
       </c>
       <c r="D3" t="s">
-        <v>578</v>
+        <v>573</v>
       </c>
       <c r="E3" t="s">
         <v>521</v>
@@ -14067,7 +14085,7 @@
         <v>444</v>
       </c>
       <c r="D4" t="s">
-        <v>579</v>
+        <v>574</v>
       </c>
       <c r="E4" t="s">
         <v>522</v>
@@ -14084,7 +14102,7 @@
         <v>444</v>
       </c>
       <c r="D5" t="s">
-        <v>579</v>
+        <v>574</v>
       </c>
       <c r="E5" t="s">
         <v>523</v>
@@ -14101,7 +14119,7 @@
         <v>444</v>
       </c>
       <c r="D6" t="s">
-        <v>579</v>
+        <v>574</v>
       </c>
       <c r="E6" t="s">
         <v>548</v>
@@ -14118,7 +14136,7 @@
         <v>444</v>
       </c>
       <c r="D7" t="s">
-        <v>580</v>
+        <v>575</v>
       </c>
       <c r="E7" t="s">
         <v>524</v>
@@ -14135,7 +14153,7 @@
         <v>444</v>
       </c>
       <c r="D8" t="s">
-        <v>580</v>
+        <v>575</v>
       </c>
       <c r="E8" t="s">
         <v>524</v>
@@ -14152,7 +14170,7 @@
         <v>444</v>
       </c>
       <c r="D9" t="s">
-        <v>581</v>
+        <v>576</v>
       </c>
       <c r="E9" t="s">
         <v>527</v>
@@ -14169,7 +14187,7 @@
         <v>444</v>
       </c>
       <c r="D10" t="s">
-        <v>580</v>
+        <v>575</v>
       </c>
       <c r="E10" t="s">
         <v>528</v>
@@ -14186,7 +14204,7 @@
         <v>444</v>
       </c>
       <c r="D11" t="s">
-        <v>582</v>
+        <v>577</v>
       </c>
       <c r="E11" t="s">
         <v>529</v>
@@ -14203,7 +14221,7 @@
         <v>444</v>
       </c>
       <c r="D12" t="s">
-        <v>583</v>
+        <v>578</v>
       </c>
       <c r="E12" t="s">
         <v>530</v>
@@ -14220,7 +14238,7 @@
         <v>444</v>
       </c>
       <c r="D13" t="s">
-        <v>584</v>
+        <v>579</v>
       </c>
       <c r="E13" t="s">
         <v>547</v>
@@ -14237,7 +14255,7 @@
         <v>444</v>
       </c>
       <c r="D14" t="s">
-        <v>585</v>
+        <v>580</v>
       </c>
       <c r="E14" t="s">
         <v>547</v>
@@ -14254,7 +14272,7 @@
         <v>444</v>
       </c>
       <c r="D15" t="s">
-        <v>586</v>
+        <v>581</v>
       </c>
       <c r="E15" t="s">
         <v>531</v>
@@ -14271,7 +14289,7 @@
         <v>444</v>
       </c>
       <c r="D16" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="E16" t="s">
         <v>532</v>
@@ -14289,19 +14307,19 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.5703125" customWidth="1"/>
     <col min="4" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="30" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="23.28515625" customWidth="1"/>
-    <col min="8" max="8" width="67.42578125" customWidth="1"/>
+    <col min="6" max="8" width="23.28515625" customWidth="1"/>
+    <col min="9" max="9" width="67.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
         <v>549</v>
       </c>
@@ -14315,57 +14333,63 @@
         <v>552</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="F1" s="18" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>573</v>
+        <v>569</v>
       </c>
       <c r="H1" s="18" t="s">
+        <v>623</v>
+      </c>
+      <c r="I1" s="18" t="s">
         <v>520</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="34" t="s">
         <v>533</v>
       </c>
       <c r="B2" t="s">
-        <v>559</v>
+        <v>617</v>
       </c>
       <c r="C2" t="s">
-        <v>605</v>
+        <v>599</v>
       </c>
       <c r="D2" t="s">
-        <v>588</v>
+        <v>583</v>
       </c>
       <c r="E2" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="F2" s="8">
         <v>0</v>
       </c>
       <c r="G2" s="8"/>
-      <c r="H2" t="s">
+      <c r="H2" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="I2" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="34" t="s">
         <v>534</v>
       </c>
       <c r="B3" t="s">
-        <v>559</v>
+        <v>617</v>
       </c>
       <c r="C3" t="s">
-        <v>606</v>
+        <v>600</v>
       </c>
       <c r="D3" t="s">
-        <v>589</v>
+        <v>584</v>
       </c>
       <c r="E3" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="F3" s="8">
         <v>1</v>
@@ -14373,49 +14397,55 @@
       <c r="G3" s="8">
         <v>0</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="I3" t="s">
         <v>522</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="38" t="s">
         <v>535</v>
       </c>
       <c r="B4" t="s">
-        <v>559</v>
+        <v>617</v>
       </c>
       <c r="C4" t="s">
-        <v>607</v>
+        <v>601</v>
       </c>
       <c r="D4" t="s">
-        <v>589</v>
+        <v>584</v>
       </c>
       <c r="E4" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="F4" s="8"/>
       <c r="G4" s="8">
         <v>1</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="I4" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="34" t="s">
         <v>536</v>
       </c>
       <c r="B5" t="s">
-        <v>560</v>
+        <v>618</v>
       </c>
       <c r="C5" t="s">
-        <v>608</v>
+        <v>627</v>
       </c>
       <c r="D5" t="s">
-        <v>589</v>
+        <v>584</v>
       </c>
       <c r="E5" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="F5" s="8">
         <v>1</v>
@@ -14423,25 +14453,28 @@
       <c r="G5" s="8">
         <v>0</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="I5" t="s">
         <v>548</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
         <v>537</v>
       </c>
       <c r="B6" t="s">
+        <v>559</v>
+      </c>
+      <c r="C6" t="s">
+        <v>602</v>
+      </c>
+      <c r="D6" t="s">
+        <v>585</v>
+      </c>
+      <c r="E6" s="37" t="s">
         <v>561</v>
-      </c>
-      <c r="C6" t="s">
-        <v>609</v>
-      </c>
-      <c r="D6" t="s">
-        <v>590</v>
-      </c>
-      <c r="E6" s="37" t="s">
-        <v>563</v>
       </c>
       <c r="F6" s="8">
         <v>6</v>
@@ -14449,25 +14482,28 @@
       <c r="G6" s="8">
         <v>0</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="I6" t="s">
         <v>524</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="34" t="s">
         <v>538</v>
       </c>
       <c r="B7" t="s">
-        <v>561</v>
+        <v>619</v>
       </c>
       <c r="C7" t="s">
-        <v>605</v>
+        <v>599</v>
       </c>
       <c r="D7" t="s">
-        <v>588</v>
+        <v>583</v>
       </c>
       <c r="E7" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="F7" s="8">
         <v>0</v>
@@ -14475,49 +14511,55 @@
       <c r="G7" s="8">
         <v>0</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="I7" t="s">
         <v>525</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
         <v>540</v>
       </c>
       <c r="B8" t="s">
-        <v>570</v>
+        <v>619</v>
       </c>
       <c r="C8" t="s">
-        <v>610</v>
+        <v>603</v>
       </c>
       <c r="D8" t="s">
-        <v>589</v>
+        <v>584</v>
       </c>
       <c r="E8" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="F8" s="8">
         <v>2</v>
       </c>
       <c r="G8" s="8"/>
-      <c r="H8" t="s">
+      <c r="H8" s="8" t="s">
+        <v>625</v>
+      </c>
+      <c r="I8" t="s">
         <v>527</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="34" t="s">
         <v>544</v>
       </c>
       <c r="B9" t="s">
-        <v>571</v>
+        <v>622</v>
       </c>
       <c r="C9" t="s">
-        <v>606</v>
+        <v>600</v>
       </c>
       <c r="D9" t="s">
-        <v>589</v>
+        <v>584</v>
       </c>
       <c r="E9" t="s">
-        <v>572</v>
+        <v>568</v>
       </c>
       <c r="F9" s="8">
         <v>1</v>
@@ -14525,25 +14567,28 @@
       <c r="G9" s="8">
         <v>0</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="I9" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="34" t="s">
         <v>545</v>
       </c>
       <c r="B10" t="s">
-        <v>570</v>
+        <v>622</v>
       </c>
       <c r="C10" t="s">
-        <v>611</v>
+        <v>604</v>
       </c>
       <c r="D10" t="s">
-        <v>591</v>
+        <v>586</v>
       </c>
       <c r="E10" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="F10" s="8">
         <v>1</v>
@@ -14551,25 +14596,28 @@
       <c r="G10" s="8">
         <v>0</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="8" t="s">
+        <v>625</v>
+      </c>
+      <c r="I10" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="38" t="s">
         <v>546</v>
       </c>
       <c r="B11" t="s">
-        <v>561</v>
+        <v>617</v>
       </c>
       <c r="C11" t="s">
-        <v>612</v>
+        <v>605</v>
       </c>
       <c r="D11" t="s">
-        <v>591</v>
+        <v>586</v>
       </c>
       <c r="E11" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="F11" s="8">
         <v>2</v>
@@ -14577,25 +14625,28 @@
       <c r="G11" s="8">
         <v>2</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="I11" t="s">
         <v>532</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
         <v>539</v>
       </c>
       <c r="B12" t="s">
-        <v>574</v>
+        <v>621</v>
       </c>
       <c r="C12" t="s">
-        <v>613</v>
+        <v>628</v>
       </c>
       <c r="D12" t="s">
-        <v>588</v>
+        <v>583</v>
       </c>
       <c r="E12" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="F12" s="8">
         <v>0</v>
@@ -14603,46 +14654,62 @@
       <c r="G12" s="8">
         <v>0</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="I12" t="s">
         <v>526</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="34" t="s">
-        <v>599</v>
+        <v>616</v>
       </c>
       <c r="B13" t="s">
-        <v>559</v>
+        <v>620</v>
       </c>
       <c r="C13" t="s">
+        <v>629</v>
+      </c>
+      <c r="D13" t="s">
+        <v>606</v>
+      </c>
+      <c r="E13" t="s">
+        <v>615</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>624</v>
+      </c>
+      <c r="I13" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="34" t="s">
+        <v>594</v>
+      </c>
+      <c r="B14" t="s">
+        <v>620</v>
+      </c>
+      <c r="C14" t="s">
+        <v>626</v>
+      </c>
+      <c r="D14" t="s">
+        <v>606</v>
+      </c>
+      <c r="E14" t="s">
         <v>614</v>
       </c>
-      <c r="D13" t="s">
-        <v>615</v>
-      </c>
-      <c r="E13" t="s">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="34" t="s">
-        <v>600</v>
-      </c>
-      <c r="B14" t="s">
-        <v>559</v>
-      </c>
-      <c r="C14" t="s">
-        <v>616</v>
-      </c>
-      <c r="D14" t="s">
-        <v>615</v>
-      </c>
-      <c r="E14" t="s">
-        <v>563</v>
+      <c r="H14" s="8" t="s">
+        <v>625</v>
+      </c>
+      <c r="I14" t="s">
+        <v>598</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -14681,7 +14748,7 @@
         <v>488</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>592</v>
+        <v>587</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -14704,7 +14771,7 @@
         <v>445</v>
       </c>
       <c r="G2" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="I2" s="8"/>
     </row>
@@ -14728,7 +14795,7 @@
         <v>445</v>
       </c>
       <c r="G3" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -14751,7 +14818,7 @@
         <v>445</v>
       </c>
       <c r="G4" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -14774,7 +14841,7 @@
         <v>445</v>
       </c>
       <c r="G5" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -14797,7 +14864,7 @@
         <v>445</v>
       </c>
       <c r="G6" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -14820,7 +14887,7 @@
         <v>445</v>
       </c>
       <c r="G7" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -14843,7 +14910,7 @@
         <v>445</v>
       </c>
       <c r="G8" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -14866,7 +14933,7 @@
         <v>445</v>
       </c>
       <c r="G9" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -14889,7 +14956,7 @@
         <v>445</v>
       </c>
       <c r="G10" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -14912,7 +14979,7 @@
         <v>445</v>
       </c>
       <c r="G11" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -14935,7 +15002,7 @@
         <v>445</v>
       </c>
       <c r="G12" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -14958,7 +15025,7 @@
         <v>445</v>
       </c>
       <c r="G13" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -14981,7 +15048,7 @@
         <v>445</v>
       </c>
       <c r="G14" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -15004,7 +15071,7 @@
         <v>445</v>
       </c>
       <c r="G15" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -15027,7 +15094,7 @@
         <v>445</v>
       </c>
       <c r="G16" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -15050,7 +15117,7 @@
         <v>445</v>
       </c>
       <c r="G17" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -15073,7 +15140,7 @@
         <v>445</v>
       </c>
       <c r="G18" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -15096,7 +15163,7 @@
         <v>445</v>
       </c>
       <c r="G19" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -15119,7 +15186,7 @@
         <v>445</v>
       </c>
       <c r="G20" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -15142,7 +15209,7 @@
         <v>445</v>
       </c>
       <c r="G21" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -15165,7 +15232,7 @@
         <v>445</v>
       </c>
       <c r="G22" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -15188,7 +15255,7 @@
         <v>445</v>
       </c>
       <c r="G23" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -15211,7 +15278,7 @@
         <v>445</v>
       </c>
       <c r="G24" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -15234,7 +15301,7 @@
         <v>445</v>
       </c>
       <c r="G25" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -15257,7 +15324,7 @@
         <v>445</v>
       </c>
       <c r="G26" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -15280,7 +15347,7 @@
         <v>445</v>
       </c>
       <c r="G27" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -15303,7 +15370,7 @@
         <v>445</v>
       </c>
       <c r="G28" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -15326,7 +15393,7 @@
         <v>445</v>
       </c>
       <c r="G29" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -15349,7 +15416,7 @@
         <v>445</v>
       </c>
       <c r="G30" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -15372,7 +15439,7 @@
         <v>445</v>
       </c>
       <c r="G31" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -15395,7 +15462,7 @@
         <v>445</v>
       </c>
       <c r="G32" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -15418,7 +15485,7 @@
         <v>445</v>
       </c>
       <c r="G33" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -15441,7 +15508,7 @@
         <v>445</v>
       </c>
       <c r="G34" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -15464,7 +15531,7 @@
         <v>445</v>
       </c>
       <c r="G35" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -15487,7 +15554,7 @@
         <v>445</v>
       </c>
       <c r="G36" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -15510,7 +15577,7 @@
         <v>445</v>
       </c>
       <c r="G37" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
   </sheetData>
@@ -15536,13 +15603,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>593</v>
+        <v>588</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>594</v>
+        <v>589</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>595</v>
+        <v>590</v>
       </c>
       <c r="E1" s="18" t="s">
         <v>517</v>
@@ -15550,7 +15617,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>69</v>
@@ -15567,7 +15634,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>70</v>
@@ -15584,7 +15651,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>419</v>
@@ -15601,7 +15668,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>420</v>
@@ -15618,7 +15685,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>554</v>
@@ -15635,7 +15702,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>553</v>
@@ -15652,10 +15719,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>597</v>
+        <v>592</v>
       </c>
       <c r="C8" s="7">
         <v>10</v>
@@ -15669,10 +15736,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>598</v>
+        <v>593</v>
       </c>
       <c r="C9" s="7">
         <v>10</v>

</xml_diff>

<commit_message>
+ Make popup to buy the item in the Shop.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -3939,8 +3939,8 @@
       <c r="E76" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F76" s="13" t="s">
-        <v>38</v>
+      <c r="F76" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -4023,8 +4023,8 @@
       <c r="E82" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F82" s="13" t="s">
-        <v>38</v>
+      <c r="F82" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
@@ -4107,8 +4107,8 @@
       <c r="E88" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F88" s="13" t="s">
-        <v>38</v>
+      <c r="F88" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -4275,8 +4275,8 @@
       <c r="E100" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F100" s="13" t="s">
-        <v>38</v>
+      <c r="F100" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -4359,8 +4359,8 @@
       <c r="E106" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F106" s="13" t="s">
-        <v>38</v>
+      <c r="F106" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
+ Make Battle Result Scene.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="13" activeTab="18"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -32,6 +32,7 @@
     <sheet name="StarUp" sheetId="18" r:id="rId18"/>
     <sheet name="BattleConfig" sheetId="19" r:id="rId19"/>
     <sheet name="StageEnemies" sheetId="20" r:id="rId20"/>
+    <sheet name="RewardConfig" sheetId="21" r:id="rId21"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$111</definedName>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2067" uniqueCount="636">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2081" uniqueCount="646">
   <si>
     <t>ID</t>
   </si>
@@ -1949,6 +1950,36 @@
   </si>
   <si>
     <t xml:space="preserve">Constant </t>
+  </si>
+  <si>
+    <t>reward_id</t>
+  </si>
+  <si>
+    <t>item_01</t>
+  </si>
+  <si>
+    <t>amount_01</t>
+  </si>
+  <si>
+    <t>item_02</t>
+  </si>
+  <si>
+    <t>amount_02</t>
+  </si>
+  <si>
+    <t>item_03</t>
+  </si>
+  <si>
+    <t>amount_03</t>
+  </si>
+  <si>
+    <t>item_04</t>
+  </si>
+  <si>
+    <t>amount_04</t>
+  </si>
+  <si>
+    <t>ExpReward</t>
   </si>
 </sst>
 </file>
@@ -13098,10 +13129,10 @@
     <col min="2" max="2" width="21.140625" style="27" customWidth="1"/>
     <col min="3" max="3" width="21.28515625" style="27" customWidth="1"/>
     <col min="4" max="4" width="15.5703125" style="27" customWidth="1"/>
-    <col min="5" max="5" width="23.85546875" style="27" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" style="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -13114,8 +13145,11 @@
       <c r="D1" s="17" t="s">
         <v>625</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="17" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>626</v>
       </c>
@@ -13128,8 +13162,11 @@
       <c r="D2" s="7" t="s">
         <v>629</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" s="27">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>630</v>
       </c>
@@ -13141,6 +13178,9 @@
       </c>
       <c r="D3" s="7" t="s">
         <v>629</v>
+      </c>
+      <c r="E3" s="27">
+        <v>600</v>
       </c>
     </row>
   </sheetData>
@@ -13572,6 +13612,79 @@
       </c>
       <c r="E13" t="b">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="28"/>
+    <col min="3" max="3" width="10.85546875" style="28" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="28"/>
+    <col min="5" max="5" width="10.85546875" style="28" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" style="28" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" style="28" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" style="28"/>
+    <col min="9" max="9" width="10.85546875" style="28" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>636</v>
+      </c>
+      <c r="B1" s="28" t="s">
+        <v>637</v>
+      </c>
+      <c r="C1" s="28" t="s">
+        <v>638</v>
+      </c>
+      <c r="D1" s="28" t="s">
+        <v>639</v>
+      </c>
+      <c r="E1" s="28" t="s">
+        <v>640</v>
+      </c>
+      <c r="F1" s="28" t="s">
+        <v>641</v>
+      </c>
+      <c r="G1" s="28" t="s">
+        <v>642</v>
+      </c>
+      <c r="H1" s="28" t="s">
+        <v>643</v>
+      </c>
+      <c r="I1" s="28" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>629</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="28">
+        <v>100</v>
+      </c>
+      <c r="D2" s="28" t="s">
+        <v>101</v>
+      </c>
+      <c r="E2" s="28">
+        <v>10000</v>
+      </c>
+      <c r="F2" s="28" t="s">
+        <v>183</v>
+      </c>
+      <c r="G2" s="28">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Added some items that can be picked up in the game (peach, slime, meat, and lotus).
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="13" activeTab="20"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -35,14 +35,14 @@
     <sheet name="RewardConfig" sheetId="21" r:id="rId21"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_Master!$A$1:$A$114</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2121" uniqueCount="650">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2145" uniqueCount="667">
   <si>
     <t>ID</t>
   </si>
@@ -1992,6 +1992,57 @@
   </si>
   <si>
     <t>ascension_legend</t>
+  </si>
+  <si>
+    <t>Meat</t>
+  </si>
+  <si>
+    <t>STR_MEAT_NAME</t>
+  </si>
+  <si>
+    <t>Slime</t>
+  </si>
+  <si>
+    <t>STR_SLIME_NAME</t>
+  </si>
+  <si>
+    <t>Lotus</t>
+  </si>
+  <si>
+    <t>STR_LOTUS_NAME</t>
+  </si>
+  <si>
+    <t>STR_MEAT_DES</t>
+  </si>
+  <si>
+    <t>STR_SLIME_DES</t>
+  </si>
+  <si>
+    <t>STR_LOTUS_DES</t>
+  </si>
+  <si>
+    <t>STR_MEAT_USEFUL</t>
+  </si>
+  <si>
+    <t>STR_SLIME_USEFUL</t>
+  </si>
+  <si>
+    <t>STR_LOTUS_USEFUL</t>
+  </si>
+  <si>
+    <t>Material</t>
+  </si>
+  <si>
+    <t>Peach</t>
+  </si>
+  <si>
+    <t>STR_PEACH_DES</t>
+  </si>
+  <si>
+    <t>STR_PEACH_USEFUL</t>
+  </si>
+  <si>
+    <t>STR_PEACH_NAME</t>
   </si>
 </sst>
 </file>
@@ -2507,7 +2558,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G121"/>
+  <dimension ref="A1:G124"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="27" bestFit="1" customWidth="1"/>
@@ -2960,17 +3011,17 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="27" t="s">
         <v>98</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="27" t="s">
         <v>99</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="27" t="s">
         <v>100</v>
       </c>
       <c r="E23" s="7" t="s">
@@ -2980,78 +3031,78 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>101</v>
-      </c>
-      <c r="B24" t="s">
-        <v>102</v>
-      </c>
-      <c r="C24" t="s">
-        <v>103</v>
-      </c>
-      <c r="D24" t="s">
-        <v>104</v>
+    <row r="24" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="B24" s="27" t="s">
+        <v>651</v>
+      </c>
+      <c r="C24" s="27" t="s">
+        <v>656</v>
+      </c>
+      <c r="D24" s="27" t="s">
+        <v>659</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>12</v>
+        <v>77</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>106</v>
-      </c>
-      <c r="B25" t="s">
-        <v>107</v>
-      </c>
-      <c r="C25" t="s">
-        <v>108</v>
-      </c>
-      <c r="D25" t="s">
-        <v>109</v>
+      <c r="A25" s="10" t="s">
+        <v>663</v>
+      </c>
+      <c r="B25" s="27" t="s">
+        <v>666</v>
+      </c>
+      <c r="C25" s="27" t="s">
+        <v>664</v>
+      </c>
+      <c r="D25" s="27" t="s">
+        <v>665</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>12</v>
+        <v>77</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>110</v>
+      <c r="A26" s="10" t="s">
+        <v>654</v>
       </c>
       <c r="B26" t="s">
-        <v>111</v>
-      </c>
-      <c r="C26" t="s">
-        <v>112</v>
-      </c>
-      <c r="D26" t="s">
-        <v>113</v>
+        <v>655</v>
+      </c>
+      <c r="C26" s="27" t="s">
+        <v>658</v>
+      </c>
+      <c r="D26" s="27" t="s">
+        <v>661</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>12</v>
+        <v>77</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="B27" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="C27" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
       <c r="D27" t="s">
-        <v>117</v>
+        <v>104</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>105</v>
@@ -3061,60 +3112,60 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="12" t="s">
-        <v>118</v>
+      <c r="A28" t="s">
+        <v>106</v>
       </c>
       <c r="B28" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C28" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="D28" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="12" t="s">
-        <v>123</v>
+      <c r="A29" t="s">
+        <v>110</v>
       </c>
       <c r="B29" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="C29" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="D29" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="12" t="s">
-        <v>126</v>
+      <c r="A30" t="s">
+        <v>114</v>
       </c>
       <c r="B30" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C30" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="D30" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>12</v>
@@ -3122,13 +3173,13 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="B31" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="C31" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="D31" t="s">
         <v>121</v>
@@ -3142,13 +3193,13 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="B32" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="C32" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="D32" t="s">
         <v>121</v>
@@ -3162,13 +3213,13 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="B33" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="C33" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="D33" t="s">
         <v>121</v>
@@ -3182,13 +3233,13 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="B34" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="C34" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="D34" t="s">
         <v>121</v>
@@ -3202,13 +3253,13 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="B35" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="C35" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="D35" t="s">
         <v>121</v>
@@ -3216,19 +3267,19 @@
       <c r="E35" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="F35" s="5" t="s">
-        <v>43</v>
+      <c r="F35" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="12" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="B36" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="C36" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="D36" t="s">
         <v>121</v>
@@ -3236,19 +3287,19 @@
       <c r="E36" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="F36" s="5" t="s">
-        <v>43</v>
+      <c r="F36" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="B37" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="C37" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="D37" t="s">
         <v>121</v>
@@ -3256,19 +3307,19 @@
       <c r="E37" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="F37" s="5" t="s">
-        <v>43</v>
+      <c r="F37" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B38" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C38" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="D38" t="s">
         <v>121</v>
@@ -3282,13 +3333,13 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="B39" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C39" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="D39" t="s">
         <v>121</v>
@@ -3302,13 +3353,13 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B40" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C40" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="D40" t="s">
         <v>121</v>
@@ -3322,13 +3373,13 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="B41" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C41" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="D41" t="s">
         <v>121</v>
@@ -3342,13 +3393,13 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="12" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="B42" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C42" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="D42" t="s">
         <v>121</v>
@@ -3356,19 +3407,19 @@
       <c r="E42" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="F42" s="3" t="s">
-        <v>25</v>
+      <c r="F42" s="5" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="12" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B43" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="C43" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="D43" t="s">
         <v>121</v>
@@ -3376,19 +3427,19 @@
       <c r="E43" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="F43" s="3" t="s">
-        <v>25</v>
+      <c r="F43" s="5" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="12" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="B44" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C44" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="D44" t="s">
         <v>121</v>
@@ -3396,19 +3447,19 @@
       <c r="E44" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="F44" s="3" t="s">
-        <v>25</v>
+      <c r="F44" s="5" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B45" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C45" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="D45" t="s">
         <v>121</v>
@@ -3422,13 +3473,13 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="12" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B46" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C46" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="D46" t="s">
         <v>121</v>
@@ -3442,13 +3493,13 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="12" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="B47" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C47" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="D47" t="s">
         <v>121</v>
@@ -3462,13 +3513,13 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="12" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B48" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C48" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="D48" t="s">
         <v>121</v>
@@ -3482,13 +3533,13 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="12" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="B49" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C49" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="D49" t="s">
         <v>121</v>
@@ -3496,19 +3547,19 @@
       <c r="E49" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="F49" s="6" t="s">
-        <v>48</v>
+      <c r="F49" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="12" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B50" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C50" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="D50" t="s">
         <v>121</v>
@@ -3516,19 +3567,19 @@
       <c r="E50" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="F50" s="6" t="s">
-        <v>48</v>
+      <c r="F50" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="12" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B51" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C51" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="D51" t="s">
         <v>121</v>
@@ -3536,19 +3587,19 @@
       <c r="E51" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="F51" s="6" t="s">
-        <v>48</v>
+      <c r="F51" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B52" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C52" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="D52" t="s">
         <v>121</v>
@@ -3562,13 +3613,13 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="B53" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="C53" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="D53" t="s">
         <v>121</v>
@@ -3582,13 +3633,13 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="12" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B54" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C54" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="D54" t="s">
         <v>121</v>
@@ -3602,13 +3653,13 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="12" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="B55" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C55" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="D55" t="s">
         <v>121</v>
@@ -3621,71 +3672,71 @@
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="14" t="s">
-        <v>183</v>
+      <c r="A56" s="12" t="s">
+        <v>177</v>
       </c>
       <c r="B56" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C56" t="s">
-        <v>185</v>
+        <v>134</v>
       </c>
       <c r="D56" t="s">
-        <v>186</v>
+        <v>121</v>
       </c>
       <c r="E56" s="7" t="s">
-        <v>187</v>
+        <v>122</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="14" t="s">
-        <v>188</v>
+      <c r="A57" s="12" t="s">
+        <v>179</v>
       </c>
       <c r="B57" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="C57" t="s">
-        <v>185</v>
+        <v>137</v>
       </c>
       <c r="D57" t="s">
-        <v>186</v>
+        <v>121</v>
       </c>
       <c r="E57" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>25</v>
+        <v>122</v>
+      </c>
+      <c r="F57" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="14" t="s">
-        <v>190</v>
+      <c r="A58" s="12" t="s">
+        <v>181</v>
       </c>
       <c r="B58" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="C58" t="s">
-        <v>185</v>
+        <v>140</v>
       </c>
       <c r="D58" t="s">
-        <v>186</v>
+        <v>121</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="F58" s="5" t="s">
-        <v>43</v>
+        <v>122</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="B59" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="C59" t="s">
         <v>185</v>
@@ -3696,67 +3747,76 @@
       <c r="E59" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="F59" s="2" t="s">
+      <c r="F59" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="B60" t="s">
+        <v>189</v>
+      </c>
+      <c r="C60" t="s">
+        <v>185</v>
+      </c>
+      <c r="D60" t="s">
+        <v>186</v>
+      </c>
+      <c r="E60" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="F60" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="B61" t="s">
+        <v>191</v>
+      </c>
+      <c r="C61" t="s">
+        <v>185</v>
+      </c>
+      <c r="D61" t="s">
+        <v>186</v>
+      </c>
+      <c r="E61" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="F61" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="B62" t="s">
+        <v>193</v>
+      </c>
+      <c r="C62" t="s">
+        <v>185</v>
+      </c>
+      <c r="D62" t="s">
+        <v>186</v>
+      </c>
+      <c r="E62" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="F62" s="2" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="11" t="s">
-        <v>194</v>
-      </c>
-      <c r="B60" t="s">
-        <v>195</v>
-      </c>
-      <c r="C60" t="s">
-        <v>196</v>
-      </c>
-      <c r="E60" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="B61" t="s">
-        <v>199</v>
-      </c>
-      <c r="C61" t="s">
-        <v>196</v>
-      </c>
-      <c r="E61" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="F61" s="10" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="11" t="s">
-        <v>200</v>
-      </c>
-      <c r="B62" t="s">
-        <v>201</v>
-      </c>
-      <c r="C62" t="s">
-        <v>196</v>
-      </c>
-      <c r="E62" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="F62" s="15" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="B63" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="C63" t="s">
         <v>196</v>
@@ -3764,16 +3824,16 @@
       <c r="E63" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="F63" s="3" t="s">
-        <v>25</v>
+      <c r="F63" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="B64" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="C64" t="s">
         <v>196</v>
@@ -3781,16 +3841,16 @@
       <c r="E64" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="F64" s="3" t="s">
-        <v>25</v>
+      <c r="F64" s="10" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B65" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="C65" t="s">
         <v>196</v>
@@ -3798,16 +3858,16 @@
       <c r="E65" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="F65" s="2" t="s">
-        <v>12</v>
+      <c r="F65" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="B66" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="C66" t="s">
         <v>196</v>
@@ -3815,16 +3875,16 @@
       <c r="E66" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="F66" s="13" t="s">
-        <v>38</v>
+      <c r="F66" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="B67" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="C67" t="s">
         <v>196</v>
@@ -3832,16 +3892,16 @@
       <c r="E67" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="F67" s="2" t="s">
-        <v>12</v>
+      <c r="F67" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="B68" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="C68" t="s">
         <v>196</v>
@@ -3855,10 +3915,10 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="B69" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="C69" t="s">
         <v>196</v>
@@ -3866,16 +3926,16 @@
       <c r="E69" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="F69" s="2" t="s">
-        <v>12</v>
+      <c r="F69" s="13" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" s="23" t="s">
-        <v>216</v>
+      <c r="A70" s="11" t="s">
+        <v>210</v>
       </c>
       <c r="B70" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C70" t="s">
         <v>196</v>
@@ -3883,16 +3943,16 @@
       <c r="E70" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="F70" s="13" t="s">
-        <v>38</v>
+      <c r="F70" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" s="23" t="s">
-        <v>218</v>
+      <c r="A71" s="11" t="s">
+        <v>212</v>
       </c>
       <c r="B71" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="C71" t="s">
         <v>196</v>
@@ -3905,11 +3965,11 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" s="23" t="s">
-        <v>220</v>
+      <c r="A72" s="11" t="s">
+        <v>214</v>
       </c>
       <c r="B72" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="C72" t="s">
         <v>196</v>
@@ -3917,16 +3977,16 @@
       <c r="E72" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="F72" s="15" t="s">
-        <v>43</v>
+      <c r="F72" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="23" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="B73" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="C73" t="s">
         <v>196</v>
@@ -3934,16 +3994,16 @@
       <c r="E73" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="F73" s="15" t="s">
-        <v>43</v>
+      <c r="F73" s="13" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="23" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="B74" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C74" t="s">
         <v>196</v>
@@ -3957,10 +4017,10 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="B75" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C75" t="s">
         <v>196</v>
@@ -3973,67 +4033,76 @@
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A76" s="16" t="s">
-        <v>228</v>
+      <c r="A76" s="23" t="s">
+        <v>222</v>
       </c>
       <c r="B76" t="s">
-        <v>229</v>
+        <v>223</v>
+      </c>
+      <c r="C76" t="s">
+        <v>196</v>
       </c>
       <c r="E76" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="F76" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F76" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="23" t="s">
+        <v>224</v>
+      </c>
+      <c r="B77" t="s">
+        <v>225</v>
+      </c>
+      <c r="C77" t="s">
+        <v>196</v>
+      </c>
+      <c r="E77" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="F77" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A77" s="16" t="s">
-        <v>231</v>
-      </c>
-      <c r="B77" t="s">
-        <v>232</v>
-      </c>
-      <c r="E77" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="F77" s="13" t="s">
-        <v>38</v>
-      </c>
-    </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A78" s="16" t="s">
-        <v>233</v>
+      <c r="A78" s="23" t="s">
+        <v>226</v>
       </c>
       <c r="B78" t="s">
-        <v>234</v>
+        <v>227</v>
+      </c>
+      <c r="C78" t="s">
+        <v>196</v>
       </c>
       <c r="E78" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="F78" s="13" t="s">
-        <v>38</v>
+        <v>197</v>
+      </c>
+      <c r="F78" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="16" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="B79" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="E79" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F79" s="13" t="s">
-        <v>38</v>
+      <c r="F79" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="16" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="B80" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="E80" s="7" t="s">
         <v>230</v>
@@ -4044,10 +4113,10 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="16" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="B81" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E81" s="7" t="s">
         <v>230</v>
@@ -4058,24 +4127,24 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="16" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B82" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="E82" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F82" s="2" t="s">
-        <v>12</v>
+      <c r="F82" s="13" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="16" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="B83" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="E83" s="7" t="s">
         <v>230</v>
@@ -4086,10 +4155,10 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="16" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="B84" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="E84" s="7" t="s">
         <v>230</v>
@@ -4100,24 +4169,24 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="16" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B85" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="E85" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F85" s="13" t="s">
-        <v>38</v>
+      <c r="F85" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="16" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B86" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="E86" s="7" t="s">
         <v>230</v>
@@ -4128,10 +4197,10 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="16" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B87" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E87" s="7" t="s">
         <v>230</v>
@@ -4142,24 +4211,24 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="16" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B88" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="E88" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F88" s="2" t="s">
-        <v>12</v>
+      <c r="F88" s="13" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="16" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="B89" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="E89" s="7" t="s">
         <v>230</v>
@@ -4170,10 +4239,10 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="16" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B90" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="E90" s="7" t="s">
         <v>230</v>
@@ -4184,24 +4253,24 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="16" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B91" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="E91" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F91" s="13" t="s">
-        <v>38</v>
+      <c r="F91" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="16" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="B92" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="E92" s="7" t="s">
         <v>230</v>
@@ -4212,10 +4281,10 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="16" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B93" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E93" s="7" t="s">
         <v>230</v>
@@ -4226,10 +4295,10 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="16" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B94" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="E94" s="7" t="s">
         <v>230</v>
@@ -4240,10 +4309,10 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="16" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="B95" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="E95" s="7" t="s">
         <v>230</v>
@@ -4254,10 +4323,10 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="16" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B96" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="E96" s="7" t="s">
         <v>230</v>
@@ -4268,10 +4337,10 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="16" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B97" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="E97" s="7" t="s">
         <v>230</v>
@@ -4282,10 +4351,10 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="16" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B98" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="E98" s="7" t="s">
         <v>230</v>
@@ -4296,10 +4365,10 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="16" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B99" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E99" s="7" t="s">
         <v>230</v>
@@ -4310,24 +4379,24 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="16" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B100" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="E100" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F100" s="2" t="s">
-        <v>12</v>
+      <c r="F100" s="13" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="16" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B101" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="E101" s="7" t="s">
         <v>230</v>
@@ -4338,10 +4407,10 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="16" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="B102" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="E102" s="7" t="s">
         <v>230</v>
@@ -4352,24 +4421,24 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="16" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B103" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="E103" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F103" s="13" t="s">
-        <v>38</v>
+      <c r="F103" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="16" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="B104" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="E104" s="7" t="s">
         <v>230</v>
@@ -4380,10 +4449,10 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="16" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="B105" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E105" s="7" t="s">
         <v>230</v>
@@ -4394,24 +4463,24 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="16" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B106" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="E106" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F106" s="2" t="s">
-        <v>12</v>
+      <c r="F106" s="13" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="16" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B107" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="E107" s="7" t="s">
         <v>230</v>
@@ -4422,10 +4491,10 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="16" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B108" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="E108" s="7" t="s">
         <v>230</v>
@@ -4436,24 +4505,24 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="16" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="B109" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="E109" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="F109" s="13" t="s">
-        <v>38</v>
+      <c r="F109" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="16" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B110" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="E110" s="7" t="s">
         <v>230</v>
@@ -4464,10 +4533,10 @@
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="16" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B111" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E111" s="7" t="s">
         <v>230</v>
@@ -4477,33 +4546,42 @@
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A112" s="10" t="s">
-        <v>271</v>
+      <c r="A112" s="16" t="s">
+        <v>268</v>
+      </c>
+      <c r="B112" t="s">
+        <v>236</v>
       </c>
       <c r="E112" s="7" t="s">
-        <v>272</v>
+        <v>230</v>
       </c>
       <c r="F112" s="13" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A113" s="10" t="s">
-        <v>273</v>
+      <c r="A113" s="16" t="s">
+        <v>269</v>
+      </c>
+      <c r="B113" t="s">
+        <v>238</v>
       </c>
       <c r="E113" s="7" t="s">
-        <v>272</v>
+        <v>230</v>
       </c>
       <c r="F113" s="13" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A114" s="10" t="s">
-        <v>274</v>
+      <c r="A114" s="16" t="s">
+        <v>270</v>
+      </c>
+      <c r="B114" t="s">
+        <v>240</v>
       </c>
       <c r="E114" s="7" t="s">
-        <v>272</v>
+        <v>230</v>
       </c>
       <c r="F114" s="13" t="s">
         <v>38</v>
@@ -4511,7 +4589,7 @@
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="10" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="E115" s="7" t="s">
         <v>272</v>
@@ -4522,7 +4600,7 @@
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="10" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="E116" s="7" t="s">
         <v>272</v>
@@ -4533,7 +4611,7 @@
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" s="10" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="E117" s="7" t="s">
         <v>272</v>
@@ -4544,7 +4622,7 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="10" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="E118" s="7" t="s">
         <v>272</v>
@@ -4555,7 +4633,7 @@
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="10" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="E119" s="7" t="s">
         <v>272</v>
@@ -4566,7 +4644,7 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="10" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="E120" s="7" t="s">
         <v>272</v>
@@ -4576,10 +4654,60 @@
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E121" s="7"/>
+      <c r="A121" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="E121" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="F121" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="E122" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="F122" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="E123" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="F123" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="10" t="s">
+        <v>652</v>
+      </c>
+      <c r="B124" s="27" t="s">
+        <v>653</v>
+      </c>
+      <c r="C124" s="27" t="s">
+        <v>657</v>
+      </c>
+      <c r="D124" s="27" t="s">
+        <v>660</v>
+      </c>
+      <c r="E124" s="7" t="s">
+        <v>662</v>
+      </c>
+      <c r="F124" s="4" t="s">
+        <v>38</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A111"/>
+  <autoFilter ref="A1:A114"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
+ Improve UI in the Battle and fixed some bugs about restart battle (sync and null reference)
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="4" activeTab="12"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -7405,10 +7405,10 @@
         <v>0</v>
       </c>
       <c r="I2" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J2" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K2" s="28">
         <v>0</v>
@@ -7443,7 +7443,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J3" s="28">
         <v>0</v>
@@ -7481,7 +7481,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J4" s="28">
         <v>0</v>
@@ -7519,7 +7519,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J5" s="28">
         <v>0</v>
@@ -7557,7 +7557,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J6" s="28">
         <v>0</v>
@@ -7595,7 +7595,7 @@
         <v>20</v>
       </c>
       <c r="I7" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J7" s="28">
         <v>0</v>
@@ -7633,7 +7633,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J8" s="28">
         <v>0</v>
@@ -7671,7 +7671,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J9" s="28">
         <v>0</v>
@@ -7709,7 +7709,7 @@
         <v>0</v>
       </c>
       <c r="I10" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J10" s="28">
         <v>0</v>
@@ -7747,7 +7747,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J11" s="28">
         <v>0</v>
@@ -7785,7 +7785,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J12" s="28">
         <v>0</v>
@@ -7823,7 +7823,7 @@
         <v>20</v>
       </c>
       <c r="I13" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J13" s="28">
         <v>0</v>
@@ -7861,7 +7861,7 @@
         <v>20</v>
       </c>
       <c r="I14" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J14" s="28">
         <v>0</v>
@@ -7899,7 +7899,7 @@
         <v>20</v>
       </c>
       <c r="I15" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J15" s="28">
         <v>0</v>
@@ -7937,7 +7937,7 @@
         <v>20</v>
       </c>
       <c r="I16" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J16" s="28">
         <v>0</v>
@@ -7975,7 +7975,7 @@
         <v>20</v>
       </c>
       <c r="I17" s="28">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J17" s="28">
         <v>0</v>

</xml_diff>

<commit_message>
+ Add Daily Quest and Main Quest System
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="4" activeTab="12"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="13" activeTab="20"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -14237,31 +14237,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="12" t="s">
         <v>636</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="29" t="s">
         <v>637</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="29" t="s">
         <v>638</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="29" t="s">
         <v>639</v>
       </c>
-      <c r="E1" s="28" t="s">
+      <c r="E1" s="29" t="s">
         <v>640</v>
       </c>
-      <c r="F1" s="28" t="s">
+      <c r="F1" s="29" t="s">
         <v>641</v>
       </c>
-      <c r="G1" s="28" t="s">
+      <c r="G1" s="29" t="s">
         <v>642</v>
       </c>
-      <c r="H1" s="28" t="s">
+      <c r="H1" s="29" t="s">
         <v>643</v>
       </c>
-      <c r="I1" s="28" t="s">
+      <c r="I1" s="29" t="s">
         <v>644</v>
       </c>
     </row>

</xml_diff>

<commit_message>
+ Add Li Jing vs Erlang Shen Character
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="6" activeTab="10"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="9" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2394" uniqueCount="698">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2397" uniqueCount="703">
   <si>
     <t>ID</t>
   </si>
@@ -2136,6 +2136,21 @@
   </si>
   <si>
     <t>MoonBlade</t>
+  </si>
+  <si>
+    <t>ErlangShen_Major</t>
+  </si>
+  <si>
+    <t>ErlangShen_Ultimate</t>
+  </si>
+  <si>
+    <t>LiJing_Attack</t>
+  </si>
+  <si>
+    <t>LiJing_Major</t>
+  </si>
+  <si>
+    <t>LiJing_Ultimate</t>
   </si>
 </sst>
 </file>
@@ -2279,7 +2294,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2378,6 +2393,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5608,7 +5624,7 @@
         <f t="shared" si="0"/>
         <v>DragonKing_B_Name</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C14" s="24" t="str">
         <f t="shared" si="1"/>
         <v>DragonKing_B_Des</v>
       </c>
@@ -5645,7 +5661,7 @@
         <f t="shared" si="0"/>
         <v>DragonKing_M_Name</v>
       </c>
-      <c r="C15" t="str">
+      <c r="C15" s="24" t="str">
         <f t="shared" si="1"/>
         <v>DragonKing_M_Des</v>
       </c>
@@ -5682,7 +5698,7 @@
         <f t="shared" si="0"/>
         <v>DragonKing_U_Name</v>
       </c>
-      <c r="C16" t="str">
+      <c r="C16" s="24" t="str">
         <f t="shared" si="1"/>
         <v>DragonKing_U_Des</v>
       </c>
@@ -6072,14 +6088,14 @@
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A26" s="24" t="s">
+      <c r="A26" s="44" t="s">
         <v>517</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
         <v>ErlangShen_B_Name</v>
       </c>
-      <c r="C26" t="str">
+      <c r="C26" s="44" t="str">
         <f t="shared" si="1"/>
         <v>ErlangShen_B_Des</v>
       </c>
@@ -6104,19 +6120,22 @@
       <c r="J26" s="7" t="s">
         <v>452</v>
       </c>
+      <c r="K26" s="28" t="s">
+        <v>494</v>
+      </c>
       <c r="L26" s="28" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27" s="24" t="s">
+      <c r="A27" s="44" t="s">
         <v>518</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="0"/>
         <v>ErlangShen_M_Name</v>
       </c>
-      <c r="C27" t="str">
+      <c r="C27" s="44" t="str">
         <f t="shared" si="1"/>
         <v>ErlangShen_M_Des</v>
       </c>
@@ -6141,19 +6160,22 @@
       <c r="J27" s="7" t="s">
         <v>452</v>
       </c>
+      <c r="K27" s="28" t="s">
+        <v>698</v>
+      </c>
       <c r="L27" s="28" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="44" t="s">
         <v>519</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="0"/>
         <v>ErlangShen_U_Name</v>
       </c>
-      <c r="C28" t="str">
+      <c r="C28" s="44" t="str">
         <f t="shared" si="1"/>
         <v>ErlangShen_U_Des</v>
       </c>
@@ -6177,6 +6199,9 @@
       </c>
       <c r="J28" s="7" t="s">
         <v>452</v>
+      </c>
+      <c r="K28" s="28" t="s">
+        <v>699</v>
       </c>
       <c r="L28" s="28" t="s">
         <v>452</v>
@@ -7291,111 +7316,111 @@
       </c>
     </row>
     <row r="57" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="27" t="s">
-        <v>694</v>
+      <c r="A57" s="44" t="s">
+        <v>696</v>
       </c>
       <c r="B57" s="27" t="str">
         <f t="shared" si="10"/>
-        <v>LiJing_M_Name</v>
-      </c>
-      <c r="C57" s="27" t="str">
+        <v>LiJing_B_Name</v>
+      </c>
+      <c r="C57" s="44" t="str">
         <f>A57&amp;"_Des"</f>
-        <v>LiJing_M_Des</v>
-      </c>
-      <c r="D57" s="28" t="s">
-        <v>470</v>
+        <v>LiJing_B_Des</v>
+      </c>
+      <c r="D57" s="8" t="s">
+        <v>447</v>
       </c>
       <c r="E57" s="28" t="s">
-        <v>456</v>
+        <v>448</v>
       </c>
       <c r="F57" s="28" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
       <c r="G57" s="28">
         <v>100</v>
       </c>
-      <c r="H57" s="27" t="s">
-        <v>385</v>
+      <c r="H57" s="28" t="s">
+        <v>450</v>
       </c>
       <c r="I57" s="28" t="s">
-        <v>471</v>
+        <v>451</v>
       </c>
       <c r="J57" s="7" t="s">
         <v>452</v>
       </c>
       <c r="K57" s="31" t="s">
-        <v>479</v>
+        <v>700</v>
       </c>
       <c r="L57" s="28" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="58" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="27" t="s">
-        <v>695</v>
+      <c r="A58" s="44" t="s">
+        <v>694</v>
       </c>
       <c r="B58" s="27" t="str">
         <f t="shared" si="10"/>
+        <v>LiJing_M_Name</v>
+      </c>
+      <c r="C58" s="44" t="str">
+        <f t="shared" si="11"/>
+        <v>LiJing_M_Des</v>
+      </c>
+      <c r="D58" s="8" t="s">
+        <v>470</v>
+      </c>
+      <c r="E58" s="28" t="s">
+        <v>456</v>
+      </c>
+      <c r="F58" s="28" t="s">
+        <v>457</v>
+      </c>
+      <c r="G58" s="28">
+        <v>0</v>
+      </c>
+      <c r="H58" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="I58" s="28" t="s">
+        <v>471</v>
+      </c>
+      <c r="J58" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="K58" s="31" t="s">
+        <v>701</v>
+      </c>
+      <c r="L58" s="28" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="44" t="s">
+        <v>695</v>
+      </c>
+      <c r="B59" s="27" t="str">
+        <f t="shared" si="10"/>
         <v>LiJing_U_Name</v>
       </c>
-      <c r="C58" s="27" t="str">
+      <c r="C59" s="44" t="str">
         <f t="shared" si="11"/>
         <v>LiJing_U_Des</v>
       </c>
-      <c r="D58" s="7" t="s">
+      <c r="D59" s="7" t="s">
         <v>462</v>
       </c>
-      <c r="E58" s="28" t="s">
+      <c r="E59" s="28" t="s">
         <v>463</v>
       </c>
-      <c r="F58" s="28" t="s">
+      <c r="F59" s="28" t="s">
         <v>464</v>
-      </c>
-      <c r="G58" s="28">
-        <v>100</v>
-      </c>
-      <c r="H58" s="28" t="s">
-        <v>458</v>
-      </c>
-      <c r="I58" s="28" t="s">
-        <v>451</v>
-      </c>
-      <c r="J58" s="7" t="s">
-        <v>452</v>
-      </c>
-      <c r="K58" s="31" t="s">
-        <v>481</v>
-      </c>
-      <c r="L58" s="28" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="11" t="s">
-        <v>696</v>
-      </c>
-      <c r="B59" s="27" t="str">
-        <f t="shared" si="10"/>
-        <v>LiJing_B_Name</v>
-      </c>
-      <c r="C59" s="27" t="str">
-        <f t="shared" si="11"/>
-        <v>LiJing_B_Des</v>
-      </c>
-      <c r="D59" s="8" t="s">
-        <v>447</v>
-      </c>
-      <c r="E59" s="28" t="s">
-        <v>448</v>
-      </c>
-      <c r="F59" s="28" t="s">
-        <v>449</v>
       </c>
       <c r="G59" s="28">
         <v>100</v>
       </c>
       <c r="H59" s="28" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="I59" s="28" t="s">
         <v>451</v>
@@ -7404,7 +7429,7 @@
         <v>452</v>
       </c>
       <c r="K59" s="31" t="s">
-        <v>483</v>
+        <v>702</v>
       </c>
       <c r="L59" s="28" t="s">
         <v>452</v>

</xml_diff>

<commit_message>
+ Make some boss in game.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="9" activeTab="10"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="11" activeTab="11"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2397" uniqueCount="703">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2506" uniqueCount="712">
   <si>
     <t>ID</t>
   </si>
@@ -2151,6 +2151,33 @@
   </si>
   <si>
     <t>LiJing_Ultimate</t>
+  </si>
+  <si>
+    <t>MarshalTianpeng</t>
+  </si>
+  <si>
+    <t>STR_MARSHAL_TIANPENG</t>
+  </si>
+  <si>
+    <t>MarshalTianpeng_B</t>
+  </si>
+  <si>
+    <t>MarshalTianpeng_M</t>
+  </si>
+  <si>
+    <t>MarshalTianpeng_U</t>
+  </si>
+  <si>
+    <t>ThirdPrinceNezha_Boss</t>
+  </si>
+  <si>
+    <t>BullDemonKing_Boss</t>
+  </si>
+  <si>
+    <t>ErlangShen_Boss</t>
+  </si>
+  <si>
+    <t>LiJing_Boss</t>
   </si>
 </sst>
 </file>
@@ -5082,7 +5109,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" style="27" customWidth="1"/>
@@ -5760,7 +5787,7 @@
       <c r="J17" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K17" t="s">
+      <c r="K17" s="27" t="s">
         <v>494</v>
       </c>
       <c r="L17" s="28" t="s">
@@ -5800,7 +5827,7 @@
       <c r="J18" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K18" t="s">
+      <c r="K18" s="27" t="s">
         <v>497</v>
       </c>
       <c r="L18" s="28" t="s">
@@ -5840,7 +5867,7 @@
       <c r="J19" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K19" t="s">
+      <c r="K19" s="27" t="s">
         <v>499</v>
       </c>
       <c r="L19" s="28" t="s">
@@ -5880,7 +5907,7 @@
       <c r="J20" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K20" t="s">
+      <c r="K20" s="27" t="s">
         <v>501</v>
       </c>
       <c r="L20" s="28" t="s">
@@ -5920,7 +5947,7 @@
       <c r="J21" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K21" t="s">
+      <c r="K21" s="27" t="s">
         <v>504</v>
       </c>
       <c r="L21" s="28" t="s">
@@ -5960,7 +5987,7 @@
       <c r="J22" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K22" t="s">
+      <c r="K22" s="27" t="s">
         <v>506</v>
       </c>
       <c r="L22" s="28" t="s">
@@ -6000,7 +6027,7 @@
       <c r="J23" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K23" t="s">
+      <c r="K23" s="27" t="s">
         <v>508</v>
       </c>
       <c r="L23" s="28" t="s">
@@ -6351,7 +6378,7 @@
       <c r="J32" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K32" t="s">
+      <c r="K32" s="27" t="s">
         <v>508</v>
       </c>
       <c r="L32" s="28" t="s">
@@ -6391,7 +6418,7 @@
       <c r="J33" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K33" t="s">
+      <c r="K33" s="27" t="s">
         <v>526</v>
       </c>
       <c r="L33" s="28" t="s">
@@ -6431,7 +6458,7 @@
       <c r="J34" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K34" t="s">
+      <c r="K34" s="27" t="s">
         <v>529</v>
       </c>
       <c r="L34" s="28" t="s">
@@ -6471,7 +6498,7 @@
       <c r="J35" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K35" t="s">
+      <c r="K35" s="27" t="s">
         <v>531</v>
       </c>
       <c r="L35" s="28" t="s">
@@ -6511,7 +6538,7 @@
       <c r="J36" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K36" t="s">
+      <c r="K36" s="27" t="s">
         <v>533</v>
       </c>
       <c r="L36" s="28" t="s">
@@ -6551,7 +6578,7 @@
       <c r="J37" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K37" t="s">
+      <c r="K37" s="27" t="s">
         <v>536</v>
       </c>
       <c r="L37" s="28" t="s">
@@ -6591,7 +6618,7 @@
       <c r="J38" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K38" t="s">
+      <c r="K38" s="27" t="s">
         <v>538</v>
       </c>
       <c r="L38" s="28" t="s">
@@ -6631,7 +6658,7 @@
       <c r="J39" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K39" t="s">
+      <c r="K39" s="27" t="s">
         <v>540</v>
       </c>
       <c r="L39" s="28" t="s">
@@ -6671,7 +6698,7 @@
       <c r="J40" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K40" t="s">
+      <c r="K40" s="27" t="s">
         <v>543</v>
       </c>
       <c r="L40" s="28" t="s">
@@ -6711,7 +6738,7 @@
       <c r="J41" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K41" t="s">
+      <c r="K41" s="27" t="s">
         <v>538</v>
       </c>
       <c r="L41" s="28" t="s">
@@ -6751,7 +6778,7 @@
       <c r="J42" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K42" t="s">
+      <c r="K42" s="27" t="s">
         <v>546</v>
       </c>
       <c r="L42" s="28" t="s">
@@ -6791,7 +6818,7 @@
       <c r="J43" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K43" t="s">
+      <c r="K43" s="27" t="s">
         <v>549</v>
       </c>
       <c r="L43" s="28" t="s">
@@ -6831,7 +6858,7 @@
       <c r="J44" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K44" t="s">
+      <c r="K44" s="27" t="s">
         <v>552</v>
       </c>
       <c r="L44" s="28" t="s">
@@ -6871,7 +6898,7 @@
       <c r="J45" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K45" t="s">
+      <c r="K45" s="27" t="s">
         <v>554</v>
       </c>
       <c r="L45" s="28" t="s">
@@ -6911,7 +6938,7 @@
       <c r="J46" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="K46" t="s">
+      <c r="K46" s="27" t="s">
         <v>556</v>
       </c>
       <c r="L46" s="28" t="s">
@@ -6951,7 +6978,7 @@
       <c r="J47" t="s">
         <v>474</v>
       </c>
-      <c r="K47" t="s">
+      <c r="K47" s="27" t="s">
         <v>558</v>
       </c>
       <c r="L47" s="28" t="s">
@@ -7200,7 +7227,7 @@
         <v>683</v>
       </c>
       <c r="B54" s="27" t="str">
-        <f t="shared" ref="B54:B59" si="10">A54&amp;"_Name"</f>
+        <f t="shared" ref="B54:B62" si="10">A54&amp;"_Name"</f>
         <v>SquidSolider_B_Name</v>
       </c>
       <c r="C54" s="27" t="str">
@@ -7244,7 +7271,7 @@
         <v>Benborba_B_Name</v>
       </c>
       <c r="C55" s="27" t="str">
-        <f t="shared" ref="C55:C59" si="11">A55&amp;"_Des"</f>
+        <f t="shared" ref="C55:C62" si="11">A55&amp;"_Des"</f>
         <v>Benborba_B_Des</v>
       </c>
       <c r="D55" s="29" t="s">
@@ -7432,6 +7459,126 @@
         <v>702</v>
       </c>
       <c r="L59" s="28" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="27" t="s">
+        <v>705</v>
+      </c>
+      <c r="B60" s="27" t="str">
+        <f t="shared" si="10"/>
+        <v>MarshalTianpeng_B_Name</v>
+      </c>
+      <c r="C60" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>MarshalTianpeng_B_Des</v>
+      </c>
+      <c r="D60" s="28" t="s">
+        <v>447</v>
+      </c>
+      <c r="E60" s="28" t="s">
+        <v>448</v>
+      </c>
+      <c r="F60" s="28" t="s">
+        <v>449</v>
+      </c>
+      <c r="G60" s="28">
+        <v>100</v>
+      </c>
+      <c r="H60" s="28" t="s">
+        <v>450</v>
+      </c>
+      <c r="I60" s="28" t="s">
+        <v>451</v>
+      </c>
+      <c r="J60" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="K60" s="31" t="s">
+        <v>477</v>
+      </c>
+      <c r="L60" s="28" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="27" t="s">
+        <v>706</v>
+      </c>
+      <c r="B61" s="27" t="str">
+        <f t="shared" si="10"/>
+        <v>MarshalTianpeng_M_Name</v>
+      </c>
+      <c r="C61" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>MarshalTianpeng_M_Des</v>
+      </c>
+      <c r="D61" s="28" t="s">
+        <v>470</v>
+      </c>
+      <c r="E61" s="28" t="s">
+        <v>456</v>
+      </c>
+      <c r="F61" s="28" t="s">
+        <v>457</v>
+      </c>
+      <c r="G61" s="28">
+        <v>100</v>
+      </c>
+      <c r="H61" s="27" t="s">
+        <v>385</v>
+      </c>
+      <c r="I61" s="28" t="s">
+        <v>471</v>
+      </c>
+      <c r="J61" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="K61" s="31" t="s">
+        <v>479</v>
+      </c>
+      <c r="L61" s="28" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="27" t="s">
+        <v>707</v>
+      </c>
+      <c r="B62" s="27" t="str">
+        <f t="shared" si="10"/>
+        <v>MarshalTianpeng_U_Name</v>
+      </c>
+      <c r="C62" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>MarshalTianpeng_U_Des</v>
+      </c>
+      <c r="D62" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="E62" s="28" t="s">
+        <v>463</v>
+      </c>
+      <c r="F62" s="28" t="s">
+        <v>464</v>
+      </c>
+      <c r="G62" s="28">
+        <v>100</v>
+      </c>
+      <c r="H62" s="28" t="s">
+        <v>458</v>
+      </c>
+      <c r="I62" s="28" t="s">
+        <v>451</v>
+      </c>
+      <c r="J62" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="K62" s="31" t="s">
+        <v>481</v>
+      </c>
+      <c r="L62" s="28" t="s">
         <v>452</v>
       </c>
     </row>
@@ -7443,7 +7590,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" style="27" bestFit="1" customWidth="1"/>
@@ -8074,7 +8221,7 @@
         <v>295</v>
       </c>
       <c r="E25" s="28" t="str">
-        <f t="shared" ref="E25:E26" si="7">A25&amp;"_B"</f>
+        <f t="shared" ref="E25:E28" si="7">A25&amp;"_B"</f>
         <v>Baborben_B</v>
       </c>
       <c r="F25" s="28" t="s">
@@ -8102,25 +8249,144 @@
         <v>LiJing_B</v>
       </c>
       <c r="F26" s="28" t="str">
-        <f t="shared" ref="F26" si="8">A26&amp;"_M"</f>
+        <f t="shared" ref="F26:F28" si="8">A26&amp;"_M"</f>
         <v>LiJing_M</v>
       </c>
       <c r="G26" s="28" t="str">
-        <f t="shared" ref="G26" si="9">A26&amp;"_U"</f>
+        <f t="shared" ref="G26:G28" si="9">A26&amp;"_U"</f>
         <v>LiJing_U</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="27" t="s">
+        <v>703</v>
+      </c>
+      <c r="B27" s="27" t="s">
+        <v>704</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="D27" s="28" t="s">
+        <v>302</v>
+      </c>
+      <c r="E27" s="28" t="str">
+        <f t="shared" si="7"/>
+        <v>MarshalTianpeng_B</v>
+      </c>
+      <c r="F27" s="28" t="str">
+        <f t="shared" si="8"/>
+        <v>MarshalTianpeng_M</v>
+      </c>
+      <c r="G27" s="28" t="str">
+        <f t="shared" si="9"/>
+        <v>MarshalTianpeng_U</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="27" t="s">
+        <v>708</v>
+      </c>
+      <c r="B28" s="27" t="s">
+        <v>207</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="D28" s="28" t="s">
+        <v>298</v>
+      </c>
+      <c r="E28" s="28" t="s">
+        <v>493</v>
+      </c>
+      <c r="F28" s="28" t="s">
+        <v>495</v>
+      </c>
+      <c r="G28" s="28" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="27" t="s">
+        <v>709</v>
+      </c>
+      <c r="B29" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="D29" s="28" t="s">
+        <v>302</v>
+      </c>
+      <c r="E29" s="28" t="s">
+        <v>507</v>
+      </c>
+      <c r="F29" s="28" t="s">
+        <v>509</v>
+      </c>
+      <c r="G29" s="28" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" s="41" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="41" t="s">
+        <v>710</v>
+      </c>
+      <c r="B30" s="41" t="s">
+        <v>213</v>
+      </c>
+      <c r="C30" s="42" t="s">
+        <v>431</v>
+      </c>
+      <c r="D30" s="43" t="s">
+        <v>295</v>
+      </c>
+      <c r="E30" s="43" t="s">
+        <v>517</v>
+      </c>
+      <c r="F30" s="43" t="s">
+        <v>518</v>
+      </c>
+      <c r="G30" s="43" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="41" t="s">
+        <v>711</v>
+      </c>
+      <c r="B31" s="27" t="s">
+        <v>693</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="D31" s="28" t="s">
+        <v>302</v>
+      </c>
+      <c r="E31" s="28" t="s">
+        <v>696</v>
+      </c>
+      <c r="F31" s="28" t="s">
+        <v>694</v>
+      </c>
+      <c r="G31" s="28" t="s">
+        <v>695</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19" style="27" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.140625" style="27" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.28515625" style="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9109,6 +9375,196 @@
         <v>0</v>
       </c>
       <c r="L26" s="28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="27" t="s">
+        <v>703</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="C27" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="D27" s="28">
+        <v>3200</v>
+      </c>
+      <c r="E27" s="28">
+        <v>1350</v>
+      </c>
+      <c r="F27" s="28">
+        <v>400</v>
+      </c>
+      <c r="G27" s="28">
+        <v>85</v>
+      </c>
+      <c r="H27" s="28">
+        <v>0</v>
+      </c>
+      <c r="I27" s="28">
+        <v>50</v>
+      </c>
+      <c r="J27" s="28">
+        <v>0</v>
+      </c>
+      <c r="K27" s="28">
+        <v>0</v>
+      </c>
+      <c r="L27" s="28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A28" s="27" t="s">
+        <v>708</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="C28" s="22" t="s">
+        <v>298</v>
+      </c>
+      <c r="D28" s="28">
+        <v>2650</v>
+      </c>
+      <c r="E28" s="28">
+        <v>2400</v>
+      </c>
+      <c r="F28" s="28">
+        <v>325</v>
+      </c>
+      <c r="G28" s="28">
+        <v>95</v>
+      </c>
+      <c r="H28" s="28">
+        <v>20</v>
+      </c>
+      <c r="I28" s="28">
+        <v>50</v>
+      </c>
+      <c r="J28" s="28">
+        <v>0</v>
+      </c>
+      <c r="K28" s="28">
+        <v>0</v>
+      </c>
+      <c r="L28" s="28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="27" t="s">
+        <v>709</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="D29" s="28">
+        <v>4250</v>
+      </c>
+      <c r="E29" s="28">
+        <v>1500</v>
+      </c>
+      <c r="F29" s="28">
+        <v>420</v>
+      </c>
+      <c r="G29" s="28">
+        <v>95</v>
+      </c>
+      <c r="H29" s="28">
+        <v>0</v>
+      </c>
+      <c r="I29" s="28">
+        <v>50</v>
+      </c>
+      <c r="J29" s="28">
+        <v>0</v>
+      </c>
+      <c r="K29" s="28">
+        <v>0</v>
+      </c>
+      <c r="L29" s="28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30" s="41" t="s">
+        <v>710</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="D30" s="28">
+        <v>3700</v>
+      </c>
+      <c r="E30" s="28">
+        <v>2100</v>
+      </c>
+      <c r="F30" s="28">
+        <v>350</v>
+      </c>
+      <c r="G30" s="28">
+        <v>95</v>
+      </c>
+      <c r="H30" s="28">
+        <v>0</v>
+      </c>
+      <c r="I30" s="28">
+        <v>50</v>
+      </c>
+      <c r="J30" s="28">
+        <v>0</v>
+      </c>
+      <c r="K30" s="28">
+        <v>0</v>
+      </c>
+      <c r="L30" s="28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A31" s="41" t="s">
+        <v>711</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="D31" s="28">
+        <v>3200</v>
+      </c>
+      <c r="E31" s="28">
+        <v>1350</v>
+      </c>
+      <c r="F31" s="28">
+        <v>400</v>
+      </c>
+      <c r="G31" s="28">
+        <v>85</v>
+      </c>
+      <c r="H31" s="28">
+        <v>0</v>
+      </c>
+      <c r="I31" s="28">
+        <v>50</v>
+      </c>
+      <c r="J31" s="28">
+        <v>0</v>
+      </c>
+      <c r="K31" s="28">
+        <v>0</v>
+      </c>
+      <c r="L31" s="28">
         <v>0</v>
       </c>
     </row>
@@ -9119,10 +9575,10 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19" style="27" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.140625" style="27" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.5703125" style="27" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.140625" style="27" customWidth="1"/>
   </cols>
@@ -9644,6 +10100,106 @@
         <v>291</v>
       </c>
       <c r="F26" s="7" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="27" t="s">
+        <v>703</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="C27" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>586</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="27" t="s">
+        <v>708</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="C28" s="22" t="s">
+        <v>298</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>586</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="27" t="s">
+        <v>709</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>586</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="41" t="s">
+        <v>710</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>586</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="41" t="s">
+        <v>711</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>586</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="F31" s="7" t="s">
         <v>596</v>
       </c>
     </row>
@@ -9655,10 +10211,10 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19" style="27" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.140625" style="27" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" style="27" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" style="27" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.85546875" style="27" bestFit="1" customWidth="1"/>
@@ -9913,6 +10469,76 @@
         <v>121</v>
       </c>
       <c r="D18" s="28">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="27" t="s">
+        <v>703</v>
+      </c>
+      <c r="B19" s="28">
+        <v>350</v>
+      </c>
+      <c r="C19" s="28">
+        <v>121</v>
+      </c>
+      <c r="D19" s="28">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="27" t="s">
+        <v>708</v>
+      </c>
+      <c r="B20" s="28">
+        <v>238</v>
+      </c>
+      <c r="C20" s="28">
+        <v>216</v>
+      </c>
+      <c r="D20" s="28">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="27" t="s">
+        <v>709</v>
+      </c>
+      <c r="B21" s="28">
+        <v>425</v>
+      </c>
+      <c r="C21" s="28">
+        <v>150</v>
+      </c>
+      <c r="D21" s="28">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="41" t="s">
+        <v>710</v>
+      </c>
+      <c r="B22" s="28">
+        <v>370</v>
+      </c>
+      <c r="C22" s="28">
+        <v>210</v>
+      </c>
+      <c r="D22" s="28">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="41" t="s">
+        <v>711</v>
+      </c>
+      <c r="B23" s="28">
+        <v>350</v>
+      </c>
+      <c r="C23" s="28">
+        <v>121</v>
+      </c>
+      <c r="D23" s="28">
         <v>36</v>
       </c>
     </row>
@@ -15559,7 +16185,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>686</v>
+        <v>668</v>
       </c>
       <c r="D14" s="7">
         <v>5</v>
@@ -15576,7 +16202,7 @@
         <v>2</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>686</v>
+        <v>668</v>
       </c>
       <c r="D15" s="7">
         <v>5</v>
@@ -15593,7 +16219,7 @@
         <v>3</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>686</v>
+        <v>668</v>
       </c>
       <c r="D16" s="7">
         <v>5</v>
@@ -15610,7 +16236,7 @@
         <v>4</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>687</v>
+        <v>668</v>
       </c>
       <c r="D17" s="7">
         <v>5</v>
@@ -15626,11 +16252,11 @@
       <c r="B18" s="7">
         <v>5</v>
       </c>
-      <c r="C18" s="23" t="s">
-        <v>224</v>
+      <c r="C18" s="41" t="s">
+        <v>711</v>
       </c>
       <c r="D18" s="7">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E18" s="27" t="b">
         <v>1</v>
@@ -15644,7 +16270,7 @@
         <v>6</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>687</v>
+        <v>668</v>
       </c>
       <c r="D19" s="7">
         <v>5</v>

</xml_diff>

<commit_message>
+ Add Third Dragon Prince character.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="9" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2514" uniqueCount="713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2555" uniqueCount="721">
   <si>
     <t>ID</t>
   </si>
@@ -2181,6 +2181,30 @@
   </si>
   <si>
     <t>STR_WINDFIRE_WHEEL_SKILL</t>
+  </si>
+  <si>
+    <t>ThirdDragonPrince</t>
+  </si>
+  <si>
+    <t>STR_THIRD_DRAGON_PRINCE</t>
+  </si>
+  <si>
+    <t>ThirdDragonPrince_B</t>
+  </si>
+  <si>
+    <t>ThirdDragonPrince_M</t>
+  </si>
+  <si>
+    <t>ThirdDragonPrince_U</t>
+  </si>
+  <si>
+    <t>FrozenBall</t>
+  </si>
+  <si>
+    <t>ThirdDragonPrince_Ultimate</t>
+  </si>
+  <si>
+    <t>ThirdDragonPrince_Major</t>
   </si>
 </sst>
 </file>
@@ -5132,7 +5156,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" style="27" customWidth="1"/>
@@ -7250,7 +7274,7 @@
         <v>679</v>
       </c>
       <c r="B54" s="27" t="str">
-        <f t="shared" ref="B54:B62" si="10">A54&amp;"_Name"</f>
+        <f t="shared" ref="B54:B65" si="10">A54&amp;"_Name"</f>
         <v>SquidSolider_B_Name</v>
       </c>
       <c r="C54" s="27" t="str">
@@ -7294,7 +7318,7 @@
         <v>Benborba_B_Name</v>
       </c>
       <c r="C55" s="27" t="str">
-        <f t="shared" ref="C55:C62" si="11">A55&amp;"_Des"</f>
+        <f t="shared" ref="C55:C65" si="11">A55&amp;"_Des"</f>
         <v>Benborba_B_Des</v>
       </c>
       <c r="D55" s="29" t="s">
@@ -7602,6 +7626,126 @@
         <v>477</v>
       </c>
       <c r="L62" s="28" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="B63" s="27" t="str">
+        <f t="shared" si="10"/>
+        <v>ThirdDragonPrince_B_Name</v>
+      </c>
+      <c r="C63" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>ThirdDragonPrince_B_Des</v>
+      </c>
+      <c r="D63" s="28" t="s">
+        <v>443</v>
+      </c>
+      <c r="E63" s="28" t="s">
+        <v>444</v>
+      </c>
+      <c r="F63" s="28" t="s">
+        <v>445</v>
+      </c>
+      <c r="G63" s="28">
+        <v>100</v>
+      </c>
+      <c r="H63" s="28" t="s">
+        <v>446</v>
+      </c>
+      <c r="I63" s="28" t="s">
+        <v>447</v>
+      </c>
+      <c r="J63" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="K63" s="31" t="s">
+        <v>550</v>
+      </c>
+      <c r="L63" s="28" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="11" t="s">
+        <v>716</v>
+      </c>
+      <c r="B64" s="27" t="str">
+        <f t="shared" si="10"/>
+        <v>ThirdDragonPrince_M_Name</v>
+      </c>
+      <c r="C64" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>ThirdDragonPrince_M_Des</v>
+      </c>
+      <c r="D64" s="28" t="s">
+        <v>718</v>
+      </c>
+      <c r="E64" s="28" t="s">
+        <v>452</v>
+      </c>
+      <c r="F64" s="28" t="s">
+        <v>453</v>
+      </c>
+      <c r="G64" s="28">
+        <v>0</v>
+      </c>
+      <c r="H64" s="28" t="s">
+        <v>454</v>
+      </c>
+      <c r="I64" s="28" t="s">
+        <v>447</v>
+      </c>
+      <c r="J64" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="K64" s="31" t="s">
+        <v>720</v>
+      </c>
+      <c r="L64" s="28" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="11" t="s">
+        <v>717</v>
+      </c>
+      <c r="B65" s="27" t="str">
+        <f t="shared" si="10"/>
+        <v>ThirdDragonPrince_U_Name</v>
+      </c>
+      <c r="C65" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>ThirdDragonPrince_U_Des</v>
+      </c>
+      <c r="D65" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="E65" s="28" t="s">
+        <v>459</v>
+      </c>
+      <c r="F65" s="28" t="s">
+        <v>460</v>
+      </c>
+      <c r="G65" s="28">
+        <v>100</v>
+      </c>
+      <c r="H65" s="28" t="s">
+        <v>454</v>
+      </c>
+      <c r="I65" s="28" t="s">
+        <v>447</v>
+      </c>
+      <c r="J65" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="K65" s="27" t="s">
+        <v>719</v>
+      </c>
+      <c r="L65" s="28" t="s">
         <v>448</v>
       </c>
     </row>
@@ -7613,7 +7757,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" style="27" bestFit="1" customWidth="1"/>
@@ -8398,6 +8542,32 @@
         <v>691</v>
       </c>
     </row>
+    <row r="32" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="27" t="s">
+        <v>713</v>
+      </c>
+      <c r="B32" s="27" t="s">
+        <v>714</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="D32" s="28" t="s">
+        <v>291</v>
+      </c>
+      <c r="E32" s="28" t="str">
+        <f t="shared" ref="E32" si="10">A32&amp;"_B"</f>
+        <v>ThirdDragonPrince_B</v>
+      </c>
+      <c r="F32" s="28" t="str">
+        <f t="shared" ref="F32" si="11">A32&amp;"_M"</f>
+        <v>ThirdDragonPrince_M</v>
+      </c>
+      <c r="G32" s="28" t="str">
+        <f t="shared" ref="G32" si="12">A32&amp;"_U"</f>
+        <v>ThirdDragonPrince_U</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -8406,7 +8576,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.140625" style="27" bestFit="1" customWidth="1"/>
@@ -9591,6 +9761,44 @@
         <v>0</v>
       </c>
     </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A32" s="27" t="s">
+        <v>713</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>291</v>
+      </c>
+      <c r="D32" s="28">
+        <v>3750</v>
+      </c>
+      <c r="E32" s="28">
+        <v>2000</v>
+      </c>
+      <c r="F32" s="28">
+        <v>400</v>
+      </c>
+      <c r="G32" s="28">
+        <v>111</v>
+      </c>
+      <c r="H32" s="28">
+        <v>0</v>
+      </c>
+      <c r="I32" s="28">
+        <v>50</v>
+      </c>
+      <c r="J32" s="28">
+        <v>50</v>
+      </c>
+      <c r="K32" s="28">
+        <v>0</v>
+      </c>
+      <c r="L32" s="28">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9598,7 +9806,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.140625" style="27" bestFit="1" customWidth="1"/>
@@ -10226,6 +10434,26 @@
         <v>592</v>
       </c>
     </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="27" t="s">
+        <v>713</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>291</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>582</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>592</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -10234,7 +10462,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.140625" style="27" bestFit="1" customWidth="1"/>
@@ -10563,6 +10791,20 @@
       </c>
       <c r="D23" s="28">
         <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="27" t="s">
+        <v>713</v>
+      </c>
+      <c r="B24" s="28">
+        <v>375</v>
+      </c>
+      <c r="C24" s="28">
+        <v>200</v>
+      </c>
+      <c r="D24" s="28">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -16275,8 +16517,8 @@
       <c r="B18" s="7">
         <v>5</v>
       </c>
-      <c r="C18" s="41" t="s">
-        <v>707</v>
+      <c r="C18" s="27" t="s">
+        <v>713</v>
       </c>
       <c r="D18" s="7">
         <v>10</v>

</xml_diff>

<commit_message>
+ Add the frozen effect and fix collision of character
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="9" activeTab="10"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="9" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2555" uniqueCount="721">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2561" uniqueCount="725">
   <si>
     <t>ID</t>
   </si>
@@ -2205,6 +2205,18 @@
   </si>
   <si>
     <t>ThirdDragonPrince_Major</t>
+  </si>
+  <si>
+    <t>EFF_Frozen_def</t>
+  </si>
+  <si>
+    <t>DEBUFF_FRONZEN_NAME</t>
+  </si>
+  <si>
+    <t>DEBUFF_FRONZEN_DES</t>
+  </si>
+  <si>
+    <t>Frozen</t>
   </si>
 </sst>
 </file>
@@ -4904,7 +4916,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" style="27" customWidth="1"/>
@@ -5146,6 +5158,35 @@
         <v>0</v>
       </c>
       <c r="I8" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="27" t="s">
+        <v>721</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>722</v>
+      </c>
+      <c r="C9" s="27" t="s">
+        <v>723</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>724</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="G9" s="7">
+        <v>2</v>
+      </c>
+      <c r="H9" s="7">
+        <v>100</v>
+      </c>
+      <c r="I9" s="7">
         <v>1</v>
       </c>
     </row>
@@ -7740,7 +7781,7 @@
         <v>447</v>
       </c>
       <c r="J65" s="7" t="s">
-        <v>448</v>
+        <v>721</v>
       </c>
       <c r="K65" s="27" t="s">
         <v>719</v>

</xml_diff>

<commit_message>
+ Config battle and fix a lot of bugs.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="9" activeTab="9"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="13" activeTab="19"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2561" uniqueCount="725">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2651" uniqueCount="733">
   <si>
     <t>ID</t>
   </si>
@@ -1922,9 +1922,6 @@
     <t>Default_01</t>
   </si>
   <si>
-    <t>Battle_Test</t>
-  </si>
-  <si>
     <t>BattleID</t>
   </si>
   <si>
@@ -2039,9 +2036,6 @@
     <t>HeavenlySoddier</t>
   </si>
   <si>
-    <t>Battle_Solo</t>
-  </si>
-  <si>
     <t>HeavenlySoddier_B</t>
   </si>
   <si>
@@ -2217,6 +2211,36 @@
   </si>
   <si>
     <t>Frozen</t>
+  </si>
+  <si>
+    <t>Battle_ThirdDragonPrince</t>
+  </si>
+  <si>
+    <t>Battle_GoldfishDemon</t>
+  </si>
+  <si>
+    <t>Battle_TheBoySage</t>
+  </si>
+  <si>
+    <t>Battle_BullDemonKing</t>
+  </si>
+  <si>
+    <t>Battle_YellowWindMonster</t>
+  </si>
+  <si>
+    <t>Battle_GoldHornKing</t>
+  </si>
+  <si>
+    <t>Battle_MarshalTianpeng</t>
+  </si>
+  <si>
+    <t>Battle_ThirdPrinceNezha</t>
+  </si>
+  <si>
+    <t>Battle_LiJing_Boss</t>
+  </si>
+  <si>
+    <t>Battle_ErlangShen_Boss</t>
   </si>
 </sst>
 </file>
@@ -3055,7 +3079,7 @@
     </row>
     <row r="16" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="B16" s="27" t="s">
         <v>50</v>
@@ -3075,16 +3099,16 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
+        <v>707</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>708</v>
+      </c>
+      <c r="C17" s="27" t="s">
         <v>709</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="D17" s="27" t="s">
         <v>710</v>
-      </c>
-      <c r="C17" s="27" t="s">
-        <v>711</v>
-      </c>
-      <c r="D17" s="27" t="s">
-        <v>712</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>11</v>
@@ -3235,16 +3259,16 @@
     </row>
     <row r="25" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
+        <v>645</v>
+      </c>
+      <c r="B25" s="27" t="s">
         <v>646</v>
       </c>
-      <c r="B25" s="27" t="s">
-        <v>647</v>
-      </c>
       <c r="C25" s="27" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D25" s="27" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>73</v>
@@ -3255,16 +3279,16 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
+        <v>658</v>
+      </c>
+      <c r="B26" s="27" t="s">
+        <v>661</v>
+      </c>
+      <c r="C26" s="27" t="s">
         <v>659</v>
       </c>
-      <c r="B26" s="27" t="s">
-        <v>662</v>
-      </c>
-      <c r="C26" s="27" t="s">
+      <c r="D26" s="27" t="s">
         <v>660</v>
-      </c>
-      <c r="D26" s="27" t="s">
-        <v>661</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>73</v>
@@ -3275,16 +3299,16 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
+        <v>649</v>
+      </c>
+      <c r="B27" t="s">
         <v>650</v>
       </c>
-      <c r="B27" t="s">
-        <v>651</v>
-      </c>
       <c r="C27" s="27" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D27" s="27" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>73</v>
@@ -4168,10 +4192,10 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B73" s="27" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="C73" t="s">
         <v>192</v>
@@ -4890,19 +4914,19 @@
     </row>
     <row r="125" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="10" t="s">
+        <v>647</v>
+      </c>
+      <c r="B125" s="27" t="s">
         <v>648</v>
       </c>
-      <c r="B125" s="27" t="s">
-        <v>649</v>
-      </c>
       <c r="C125" s="27" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="D125" s="27" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="E125" s="7" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="F125" s="4" t="s">
         <v>38</v>
@@ -5163,16 +5187,16 @@
     </row>
     <row r="9" spans="1:9" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
+        <v>719</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>720</v>
+      </c>
+      <c r="C9" s="27" t="s">
         <v>721</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="D9" s="7" t="s">
         <v>722</v>
-      </c>
-      <c r="C9" s="27" t="s">
-        <v>723</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>724</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>448</v>
@@ -6276,7 +6300,7 @@
         <v>448</v>
       </c>
       <c r="K27" s="28" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="L27" s="28" t="s">
         <v>448</v>
@@ -6295,7 +6319,7 @@
         <v>ErlangShen_U_Des</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="E28" s="28" t="s">
         <v>459</v>
@@ -6316,7 +6340,7 @@
         <v>448</v>
       </c>
       <c r="K28" s="28" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="L28" s="28" t="s">
         <v>448</v>
@@ -7112,7 +7136,7 @@
     </row>
     <row r="49" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="12" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="B49" s="27" t="str">
         <f t="shared" ref="B49" si="2">A49&amp;"_Name"</f>
@@ -7152,7 +7176,7 @@
     </row>
     <row r="50" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="12" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="B50" s="27" t="str">
         <f t="shared" ref="B50" si="4">A50&amp;"_Name"</f>
@@ -7192,7 +7216,7 @@
     </row>
     <row r="51" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="12" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="B51" s="27" t="str">
         <f t="shared" ref="B51" si="6">A51&amp;"_Name"</f>
@@ -7232,7 +7256,7 @@
     </row>
     <row r="52" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="B52" s="27" t="str">
         <f t="shared" ref="B52:B53" si="8">A52&amp;"_Name"</f>
@@ -7272,7 +7296,7 @@
     </row>
     <row r="53" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="B53" s="27" t="str">
         <f t="shared" si="8"/>
@@ -7312,7 +7336,7 @@
     </row>
     <row r="54" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="12" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="B54" s="27" t="str">
         <f t="shared" ref="B54:B65" si="10">A54&amp;"_Name"</f>
@@ -7352,7 +7376,7 @@
     </row>
     <row r="55" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="12" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="B55" s="27" t="str">
         <f t="shared" si="10"/>
@@ -7392,7 +7416,7 @@
     </row>
     <row r="56" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="12" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="B56" s="27" t="str">
         <f t="shared" si="10"/>
@@ -7432,7 +7456,7 @@
     </row>
     <row r="57" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="44" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="B57" s="27" t="str">
         <f t="shared" si="10"/>
@@ -7464,7 +7488,7 @@
         <v>448</v>
       </c>
       <c r="K57" s="31" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="L57" s="28" t="s">
         <v>448</v>
@@ -7472,7 +7496,7 @@
     </row>
     <row r="58" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="44" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="B58" s="27" t="str">
         <f t="shared" si="10"/>
@@ -7504,7 +7528,7 @@
         <v>448</v>
       </c>
       <c r="K58" s="31" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="L58" s="28" t="s">
         <v>448</v>
@@ -7512,7 +7536,7 @@
     </row>
     <row r="59" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="44" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="B59" s="27" t="str">
         <f t="shared" si="10"/>
@@ -7544,7 +7568,7 @@
         <v>448</v>
       </c>
       <c r="K59" s="31" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="L59" s="28" t="s">
         <v>448</v>
@@ -7552,7 +7576,7 @@
     </row>
     <row r="60" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="27" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="B60" s="27" t="str">
         <f t="shared" si="10"/>
@@ -7592,7 +7616,7 @@
     </row>
     <row r="61" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="27" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="B61" s="27" t="str">
         <f t="shared" si="10"/>
@@ -7632,7 +7656,7 @@
     </row>
     <row r="62" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="27" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="B62" s="27" t="str">
         <f t="shared" si="10"/>
@@ -7672,7 +7696,7 @@
     </row>
     <row r="63" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="B63" s="27" t="str">
         <f t="shared" si="10"/>
@@ -7712,7 +7736,7 @@
     </row>
     <row r="64" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="B64" s="27" t="str">
         <f t="shared" si="10"/>
@@ -7723,7 +7747,7 @@
         <v>ThirdDragonPrince_M_Des</v>
       </c>
       <c r="D64" s="28" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="E64" s="28" t="s">
         <v>452</v>
@@ -7744,7 +7768,7 @@
         <v>448</v>
       </c>
       <c r="K64" s="31" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="L64" s="28" t="s">
         <v>448</v>
@@ -7752,7 +7776,7 @@
     </row>
     <row r="65" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="B65" s="27" t="str">
         <f t="shared" si="10"/>
@@ -7781,10 +7805,10 @@
         <v>447</v>
       </c>
       <c r="J65" s="7" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="K65" s="27" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="L65" s="28" t="s">
         <v>448</v>
@@ -8249,10 +8273,10 @@
     </row>
     <row r="18" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="C18" s="18" t="s">
         <v>428</v>
@@ -8273,10 +8297,10 @@
     </row>
     <row r="19" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="C19" s="18" t="s">
         <v>428</v>
@@ -8297,10 +8321,10 @@
     </row>
     <row r="20" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="B20" s="27" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="C20" s="18" t="s">
         <v>428</v>
@@ -8321,10 +8345,10 @@
     </row>
     <row r="21" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="C21" s="18" t="s">
         <v>428</v>
@@ -8345,10 +8369,10 @@
     </row>
     <row r="22" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="B22" s="27" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="C22" s="18" t="s">
         <v>428</v>
@@ -8369,10 +8393,10 @@
     </row>
     <row r="23" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="B23" s="27" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="C23" s="18" t="s">
         <v>428</v>
@@ -8393,10 +8417,10 @@
     </row>
     <row r="24" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
+        <v>680</v>
+      </c>
+      <c r="B24" s="27" t="s">
         <v>682</v>
-      </c>
-      <c r="B24" s="27" t="s">
-        <v>684</v>
       </c>
       <c r="C24" s="18" t="s">
         <v>428</v>
@@ -8417,10 +8441,10 @@
     </row>
     <row r="25" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
+        <v>681</v>
+      </c>
+      <c r="B25" s="27" t="s">
         <v>683</v>
-      </c>
-      <c r="B25" s="27" t="s">
-        <v>685</v>
       </c>
       <c r="C25" s="18" t="s">
         <v>428</v>
@@ -8441,10 +8465,10 @@
     </row>
     <row r="26" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="41" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B26" s="27" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="C26" s="15" t="s">
         <v>429</v>
@@ -8467,10 +8491,10 @@
     </row>
     <row r="27" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="27" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="B27" s="27" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>429</v>
@@ -8493,7 +8517,7 @@
     </row>
     <row r="28" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="27" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="B28" s="27" t="s">
         <v>203</v>
@@ -8516,7 +8540,7 @@
     </row>
     <row r="29" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="27" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="B29" s="27" t="s">
         <v>207</v>
@@ -8539,7 +8563,7 @@
     </row>
     <row r="30" spans="1:7" s="41" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="41" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B30" s="41" t="s">
         <v>209</v>
@@ -8562,10 +8586,10 @@
     </row>
     <row r="31" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="41" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="B31" s="27" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="C31" s="15" t="s">
         <v>429</v>
@@ -8574,21 +8598,21 @@
         <v>298</v>
       </c>
       <c r="E31" s="28" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="F31" s="28" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="G31" s="28" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
     </row>
     <row r="32" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="27" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B32" s="27" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>427</v>
@@ -9272,7 +9296,7 @@
     </row>
     <row r="18" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="23" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B18" s="18" t="s">
         <v>428</v>
@@ -9310,7 +9334,7 @@
     </row>
     <row r="19" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="23" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="B19" s="18" t="s">
         <v>428</v>
@@ -9348,7 +9372,7 @@
     </row>
     <row r="20" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="23" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="B20" s="18" t="s">
         <v>428</v>
@@ -9386,7 +9410,7 @@
     </row>
     <row r="21" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="23" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B21" s="18" t="s">
         <v>428</v>
@@ -9424,7 +9448,7 @@
     </row>
     <row r="22" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="23" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="B22" s="18" t="s">
         <v>428</v>
@@ -9462,7 +9486,7 @@
     </row>
     <row r="23" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="23" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="B23" s="18" t="s">
         <v>428</v>
@@ -9500,7 +9524,7 @@
     </row>
     <row r="24" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="23" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="B24" s="18" t="s">
         <v>428</v>
@@ -9538,7 +9562,7 @@
     </row>
     <row r="25" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="23" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="B25" s="18" t="s">
         <v>428</v>
@@ -9576,7 +9600,7 @@
     </row>
     <row r="26" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="41" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>429</v>
@@ -9614,7 +9638,7 @@
     </row>
     <row r="27" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="27" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="B27" s="15" t="s">
         <v>429</v>
@@ -9652,7 +9676,7 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="27" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>429</v>
@@ -9690,7 +9714,7 @@
     </row>
     <row r="29" spans="1:12" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="27" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>427</v>
@@ -9728,7 +9752,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="41" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>427</v>
@@ -9766,7 +9790,7 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="41" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>429</v>
@@ -9804,7 +9828,7 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="27" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>427</v>
@@ -10197,7 +10221,7 @@
     </row>
     <row r="18" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="23" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B18" s="18" t="s">
         <v>428</v>
@@ -10217,7 +10241,7 @@
     </row>
     <row r="19" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="23" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="B19" s="18" t="s">
         <v>428</v>
@@ -10237,7 +10261,7 @@
     </row>
     <row r="20" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="23" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="B20" s="18" t="s">
         <v>428</v>
@@ -10257,7 +10281,7 @@
     </row>
     <row r="21" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="23" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B21" s="18" t="s">
         <v>428</v>
@@ -10277,7 +10301,7 @@
     </row>
     <row r="22" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="23" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="B22" s="18" t="s">
         <v>428</v>
@@ -10297,7 +10321,7 @@
     </row>
     <row r="23" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="23" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="B23" s="18" t="s">
         <v>428</v>
@@ -10317,7 +10341,7 @@
     </row>
     <row r="24" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="23" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="B24" s="18" t="s">
         <v>428</v>
@@ -10337,7 +10361,7 @@
     </row>
     <row r="25" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="23" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="B25" s="18" t="s">
         <v>428</v>
@@ -10357,7 +10381,7 @@
     </row>
     <row r="26" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="41" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>429</v>
@@ -10377,7 +10401,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="27" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="B27" s="15" t="s">
         <v>429</v>
@@ -10397,7 +10421,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="27" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>429</v>
@@ -10417,7 +10441,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="27" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>427</v>
@@ -10437,7 +10461,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="41" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>427</v>
@@ -10457,7 +10481,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="41" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>429</v>
@@ -10477,7 +10501,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="27" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>427</v>
@@ -10752,7 +10776,7 @@
     </row>
     <row r="18" spans="1:4" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="41" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B18" s="28">
         <v>350</v>
@@ -10766,7 +10790,7 @@
     </row>
     <row r="19" spans="1:4" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="B19" s="28">
         <v>350</v>
@@ -10780,7 +10804,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="B20" s="28">
         <v>238</v>
@@ -10794,7 +10818,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="B21" s="28">
         <v>425</v>
@@ -10808,7 +10832,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="41" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B22" s="28">
         <v>370</v>
@@ -10822,7 +10846,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="41" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="B23" s="28">
         <v>350</v>
@@ -10836,7 +10860,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B24" s="28">
         <v>375</v>
@@ -15139,7 +15163,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="27" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B22" s="28">
         <v>1</v>
@@ -15162,7 +15186,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="27" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B23" s="28">
         <v>2</v>
@@ -15185,7 +15209,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B24" s="28">
         <v>3</v>
@@ -15209,7 +15233,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="27" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B25" s="28">
         <v>4</v>
@@ -15232,7 +15256,7 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="27" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B26" s="38">
         <v>5</v>
@@ -15255,7 +15279,7 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B27" s="28">
         <v>1</v>
@@ -15278,7 +15302,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B28" s="28">
         <v>2</v>
@@ -15301,7 +15325,7 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B29" s="28">
         <v>3</v>
@@ -15324,7 +15348,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B30" s="28">
         <v>4</v>
@@ -15347,7 +15371,7 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B31" s="38">
         <v>5</v>
@@ -15370,7 +15394,7 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="27" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B32" s="28">
         <v>1</v>
@@ -15393,7 +15417,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="27" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B33" s="28">
         <v>2</v>
@@ -15416,7 +15440,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="27" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B34" s="28">
         <v>3</v>
@@ -15439,7 +15463,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="27" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B35" s="28">
         <v>4</v>
@@ -15462,7 +15486,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="27" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B36" s="38">
         <v>5</v>
@@ -15485,7 +15509,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B37" s="28">
         <v>1</v>
@@ -15508,7 +15532,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B38" s="28">
         <v>2</v>
@@ -15531,7 +15555,7 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B39" s="28">
         <v>3</v>
@@ -15554,7 +15578,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B40" s="28">
         <v>4</v>
@@ -15577,7 +15601,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B41" s="38">
         <v>5</v>
@@ -15974,11 +15998,11 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" style="27" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" style="27" customWidth="1"/>
+    <col min="1" max="1" width="26" style="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" style="27" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.28515625" style="27" customWidth="1"/>
     <col min="4" max="4" width="15.5703125" style="27" customWidth="1"/>
     <col min="5" max="5" width="10.85546875" style="27" customWidth="1"/>
@@ -15998,7 +16022,7 @@
         <v>621</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -16020,10 +16044,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>626</v>
-      </c>
-      <c r="B3" t="s">
-        <v>623</v>
+        <v>723</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>712</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>624</v>
@@ -16037,10 +16061,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>665</v>
+        <v>724</v>
       </c>
       <c r="B4" s="27" t="s">
-        <v>623</v>
+        <v>223</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>624</v>
@@ -16049,6 +16073,142 @@
         <v>625</v>
       </c>
       <c r="E4" s="27">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>725</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="E5" s="27">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>726</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>207</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="E6" s="27">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>727</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>221</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="E7" s="27">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>728</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>217</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="E8" s="27">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>729</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>698</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="E9" s="27">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>730</v>
+      </c>
+      <c r="B10" s="27" t="s">
+        <v>203</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="E10" s="27">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>731</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>687</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="E11" s="27">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>732</v>
+      </c>
+      <c r="B12" s="41" t="s">
+        <v>209</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="E12" s="27">
         <v>600</v>
       </c>
     </row>
@@ -16134,7 +16294,7 @@
         <v>344</v>
       </c>
       <c r="E6" s="27" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="F6" s="27">
         <v>10</v>
@@ -16154,7 +16314,7 @@
         <v>419</v>
       </c>
       <c r="E7" s="27" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="F7" s="27">
         <v>10</v>
@@ -16174,7 +16334,7 @@
         <v>283</v>
       </c>
       <c r="E8" s="27" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="F8" s="27">
         <v>10</v>
@@ -16194,7 +16354,7 @@
         <v>287</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="F9" s="27">
         <v>5</v>
@@ -16214,7 +16374,7 @@
         <v>338</v>
       </c>
       <c r="E10" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="F10">
         <v>5</v>
@@ -16254,33 +16414,33 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.5703125" style="27" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26" style="27" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" style="27" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" style="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" style="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1" s="17" t="s">
         <v>627</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="C1" s="17" t="s">
         <v>628</v>
-      </c>
-      <c r="C1" s="17" t="s">
-        <v>629</v>
       </c>
       <c r="D1" s="17" t="s">
         <v>594</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="2" t="s">
         <v>622</v>
       </c>
       <c r="B2" s="7">
@@ -16297,7 +16457,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="2" t="s">
         <v>622</v>
       </c>
       <c r="B3" s="7">
@@ -16314,7 +16474,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="2" t="s">
         <v>622</v>
       </c>
       <c r="B4" s="7">
@@ -16332,50 +16492,50 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>622</v>
+        <v>724</v>
       </c>
       <c r="B5" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>216</v>
+        <v>680</v>
       </c>
       <c r="D5" s="7">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>622</v>
-      </c>
-      <c r="B6" s="5">
-        <v>5</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="D6" s="5">
-        <v>5</v>
+      <c r="A6" s="7" t="s">
+        <v>724</v>
+      </c>
+      <c r="B6" s="7">
+        <v>2</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>681</v>
+      </c>
+      <c r="D6" s="7">
+        <v>15</v>
       </c>
       <c r="E6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>622</v>
+        <v>724</v>
       </c>
       <c r="B7" s="7">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>218</v>
+        <v>680</v>
       </c>
       <c r="D7" s="7">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -16383,206 +16543,699 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>626</v>
+        <v>724</v>
       </c>
       <c r="B8" s="7">
+        <v>5</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>222</v>
+      </c>
+      <c r="D8" s="7">
+        <v>10</v>
+      </c>
+      <c r="E8" t="b">
         <v>1</v>
       </c>
-      <c r="C8" s="23" t="s">
-        <v>664</v>
-      </c>
-      <c r="D8" s="7">
-        <v>5</v>
-      </c>
-      <c r="E8" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>626</v>
+      <c r="A9" s="2" t="s">
+        <v>723</v>
       </c>
       <c r="B9" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>214</v>
+        <v>675</v>
       </c>
       <c r="D9" s="7">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>626</v>
+      <c r="A10" s="2" t="s">
+        <v>723</v>
       </c>
       <c r="B10" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>222</v>
+        <v>678</v>
       </c>
       <c r="D10" s="7">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>626</v>
+      <c r="A11" s="2" t="s">
+        <v>723</v>
       </c>
       <c r="B11" s="7">
+        <v>3</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>675</v>
+      </c>
+      <c r="D11" s="7">
+        <v>15</v>
+      </c>
+      <c r="E11" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>723</v>
+      </c>
+      <c r="B12" s="7">
         <v>5</v>
       </c>
-      <c r="C11" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="D11" s="7">
-        <v>5</v>
-      </c>
-      <c r="E11" t="b">
+      <c r="C12" s="22" t="s">
+        <v>711</v>
+      </c>
+      <c r="D12" s="7">
+        <v>20</v>
+      </c>
+      <c r="E12" s="27" t="b">
         <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>626</v>
-      </c>
-      <c r="B12" s="7">
-        <v>4</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>216</v>
-      </c>
-      <c r="D12" s="7">
-        <v>5</v>
-      </c>
-      <c r="E12" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>626</v>
+        <v>725</v>
       </c>
       <c r="B13" s="7">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>218</v>
+        <v>665</v>
       </c>
       <c r="D13" s="7">
-        <v>5</v>
-      </c>
-      <c r="E13" t="b">
+        <v>15</v>
+      </c>
+      <c r="E13" s="27" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
+        <v>725</v>
+      </c>
+      <c r="B14" s="7">
+        <v>2</v>
+      </c>
+      <c r="C14" s="23" t="s">
         <v>665</v>
       </c>
-      <c r="B14" s="7">
-        <v>1</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>664</v>
-      </c>
       <c r="D14" s="7">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E14" s="27" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
+        <v>725</v>
+      </c>
+      <c r="B15" s="7">
+        <v>3</v>
+      </c>
+      <c r="C15" s="23" t="s">
         <v>665</v>
       </c>
-      <c r="B15" s="7">
-        <v>2</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>664</v>
-      </c>
       <c r="D15" s="7">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E15" s="27" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
+        <v>725</v>
+      </c>
+      <c r="B16" s="7">
+        <v>5</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>214</v>
+      </c>
+      <c r="D16" s="7">
+        <v>25</v>
+      </c>
+      <c r="E16" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="B17" s="7">
+        <v>1</v>
+      </c>
+      <c r="C17" s="23" t="s">
         <v>665</v>
       </c>
-      <c r="B16" s="7">
-        <v>3</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>664</v>
-      </c>
-      <c r="D16" s="7">
-        <v>5</v>
-      </c>
-      <c r="E16" s="27" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
-        <v>665</v>
-      </c>
-      <c r="B17" s="7">
-        <v>4</v>
-      </c>
-      <c r="C17" s="23" t="s">
-        <v>664</v>
-      </c>
       <c r="D17" s="7">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E17" s="27" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="B18" s="7">
+        <v>2</v>
+      </c>
+      <c r="C18" s="23" t="s">
         <v>665</v>
       </c>
-      <c r="B18" s="7">
-        <v>5</v>
-      </c>
-      <c r="C18" s="27" t="s">
-        <v>713</v>
-      </c>
       <c r="D18" s="7">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E18" s="27" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="B19" s="7">
+        <v>3</v>
+      </c>
+      <c r="C19" s="23" t="s">
         <v>665</v>
       </c>
-      <c r="B19" s="7">
-        <v>6</v>
-      </c>
-      <c r="C19" s="23" t="s">
-        <v>664</v>
-      </c>
       <c r="D19" s="7">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E19" s="27" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="B20" s="7">
+        <v>5</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>206</v>
+      </c>
+      <c r="D20" s="7">
+        <v>30</v>
+      </c>
+      <c r="E20" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="B21" s="7">
+        <v>4</v>
+      </c>
+      <c r="C21" s="23" t="s">
+        <v>214</v>
+      </c>
+      <c r="D21" s="7">
+        <v>15</v>
+      </c>
+      <c r="E21" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>727</v>
+      </c>
+      <c r="B22" s="7">
+        <v>1</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>212</v>
+      </c>
+      <c r="D22" s="7">
+        <v>15</v>
+      </c>
+      <c r="E22" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
+        <v>727</v>
+      </c>
+      <c r="B23" s="7">
+        <v>2</v>
+      </c>
+      <c r="C23" s="23" t="s">
+        <v>671</v>
+      </c>
+      <c r="D23" s="7">
+        <v>15</v>
+      </c>
+      <c r="E23" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>727</v>
+      </c>
+      <c r="B24" s="7">
+        <v>3</v>
+      </c>
+      <c r="C24" s="23" t="s">
+        <v>212</v>
+      </c>
+      <c r="D24" s="7">
+        <v>15</v>
+      </c>
+      <c r="E24" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>727</v>
+      </c>
+      <c r="B25" s="7">
+        <v>5</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>220</v>
+      </c>
+      <c r="D25" s="7">
+        <v>20</v>
+      </c>
+      <c r="E25" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="B26" s="7">
+        <v>1</v>
+      </c>
+      <c r="C26" s="23" t="s">
+        <v>668</v>
+      </c>
+      <c r="D26" s="7">
+        <v>15</v>
+      </c>
+      <c r="E26" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="B27" s="7">
+        <v>2</v>
+      </c>
+      <c r="C27" s="23" t="s">
+        <v>668</v>
+      </c>
+      <c r="D27" s="7">
+        <v>15</v>
+      </c>
+      <c r="E27" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="B28" s="7">
+        <v>3</v>
+      </c>
+      <c r="C28" s="23" t="s">
+        <v>668</v>
+      </c>
+      <c r="D28" s="7">
+        <v>15</v>
+      </c>
+      <c r="E28" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="B29" s="7">
+        <v>5</v>
+      </c>
+      <c r="C29" s="22" t="s">
+        <v>216</v>
+      </c>
+      <c r="D29" s="7">
+        <v>25</v>
+      </c>
+      <c r="E29" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="B30" s="7">
+        <v>4</v>
+      </c>
+      <c r="C30" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="D30" s="7">
+        <v>15</v>
+      </c>
+      <c r="E30" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
+        <v>729</v>
+      </c>
+      <c r="B31" s="7">
+        <v>1</v>
+      </c>
+      <c r="C31" s="23" t="s">
+        <v>663</v>
+      </c>
+      <c r="D31" s="7">
+        <v>15</v>
+      </c>
+      <c r="E31" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
+        <v>729</v>
+      </c>
+      <c r="B32" s="7">
+        <v>2</v>
+      </c>
+      <c r="C32" s="23" t="s">
+        <v>663</v>
+      </c>
+      <c r="D32" s="7">
+        <v>15</v>
+      </c>
+      <c r="E32" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>729</v>
+      </c>
+      <c r="B33" s="7">
+        <v>3</v>
+      </c>
+      <c r="C33" s="23" t="s">
+        <v>663</v>
+      </c>
+      <c r="D33" s="7">
+        <v>15</v>
+      </c>
+      <c r="E33" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="7" t="s">
+        <v>729</v>
+      </c>
+      <c r="B34" s="7">
+        <v>5</v>
+      </c>
+      <c r="C34" s="22" t="s">
+        <v>697</v>
+      </c>
+      <c r="D34" s="7">
+        <v>30</v>
+      </c>
+      <c r="E34" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>730</v>
+      </c>
+      <c r="B35" s="7">
+        <v>1</v>
+      </c>
+      <c r="C35" s="23" t="s">
+        <v>663</v>
+      </c>
+      <c r="D35" s="7">
+        <v>15</v>
+      </c>
+      <c r="E35" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>730</v>
+      </c>
+      <c r="B36" s="7">
+        <v>2</v>
+      </c>
+      <c r="C36" s="23" t="s">
+        <v>663</v>
+      </c>
+      <c r="D36" s="7">
+        <v>15</v>
+      </c>
+      <c r="E36" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>730</v>
+      </c>
+      <c r="B37" s="7">
+        <v>3</v>
+      </c>
+      <c r="C37" s="23" t="s">
+        <v>663</v>
+      </c>
+      <c r="D37" s="7">
+        <v>15</v>
+      </c>
+      <c r="E37" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>730</v>
+      </c>
+      <c r="B38" s="7">
+        <v>5</v>
+      </c>
+      <c r="C38" s="22" t="s">
+        <v>702</v>
+      </c>
+      <c r="D38" s="7">
+        <v>20</v>
+      </c>
+      <c r="E38" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="7" t="s">
+        <v>731</v>
+      </c>
+      <c r="B39" s="7">
+        <v>1</v>
+      </c>
+      <c r="C39" s="23" t="s">
+        <v>663</v>
+      </c>
+      <c r="D39" s="7">
+        <v>15</v>
+      </c>
+      <c r="E39" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="7" t="s">
+        <v>731</v>
+      </c>
+      <c r="B40" s="7">
+        <v>2</v>
+      </c>
+      <c r="C40" s="23" t="s">
+        <v>663</v>
+      </c>
+      <c r="D40" s="7">
+        <v>15</v>
+      </c>
+      <c r="E40" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="7" t="s">
+        <v>731</v>
+      </c>
+      <c r="B41" s="7">
+        <v>3</v>
+      </c>
+      <c r="C41" s="23" t="s">
+        <v>663</v>
+      </c>
+      <c r="D41" s="7">
+        <v>15</v>
+      </c>
+      <c r="E41" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="7" t="s">
+        <v>731</v>
+      </c>
+      <c r="B42" s="7">
+        <v>5</v>
+      </c>
+      <c r="C42" s="22" t="s">
+        <v>705</v>
+      </c>
+      <c r="D42" s="7">
+        <v>25</v>
+      </c>
+      <c r="E42" s="27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="7" t="s">
+        <v>731</v>
+      </c>
+      <c r="B43" s="7">
+        <v>4</v>
+      </c>
+      <c r="C43" s="23" t="s">
+        <v>702</v>
+      </c>
+      <c r="D43" s="7">
+        <v>15</v>
+      </c>
+      <c r="E43" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="7" t="s">
+        <v>731</v>
+      </c>
+      <c r="B44" s="7">
+        <v>6</v>
+      </c>
+      <c r="C44" s="23" t="s">
+        <v>697</v>
+      </c>
+      <c r="D44" s="7">
+        <v>15</v>
+      </c>
+      <c r="E44" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="B45" s="7">
+        <v>1</v>
+      </c>
+      <c r="C45" s="23" t="s">
+        <v>663</v>
+      </c>
+      <c r="D45" s="7">
+        <v>15</v>
+      </c>
+      <c r="E45" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="B46" s="7">
+        <v>2</v>
+      </c>
+      <c r="C46" s="23" t="s">
+        <v>663</v>
+      </c>
+      <c r="D46" s="7">
+        <v>15</v>
+      </c>
+      <c r="E46" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="B47" s="7">
+        <v>3</v>
+      </c>
+      <c r="C47" s="23" t="s">
+        <v>663</v>
+      </c>
+      <c r="D47" s="7">
+        <v>15</v>
+      </c>
+      <c r="E47" s="27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="B48" s="7">
+        <v>5</v>
+      </c>
+      <c r="C48" s="22" t="s">
+        <v>704</v>
+      </c>
+      <c r="D48" s="7">
+        <v>30</v>
+      </c>
+      <c r="E48" s="27" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -16608,31 +17261,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
+        <v>631</v>
+      </c>
+      <c r="B1" s="29" t="s">
         <v>632</v>
       </c>
-      <c r="B1" s="29" t="s">
+      <c r="C1" s="29" t="s">
         <v>633</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="D1" s="29" t="s">
         <v>634</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="E1" s="29" t="s">
         <v>635</v>
       </c>
-      <c r="E1" s="29" t="s">
+      <c r="F1" s="29" t="s">
         <v>636</v>
       </c>
-      <c r="F1" s="29" t="s">
+      <c r="G1" s="29" t="s">
         <v>637</v>
       </c>
-      <c r="G1" s="29" t="s">
+      <c r="H1" s="29" t="s">
         <v>638</v>
       </c>
-      <c r="H1" s="29" t="s">
+      <c r="I1" s="29" t="s">
         <v>639</v>
-      </c>
-      <c r="I1" s="29" t="s">
-        <v>640</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -17020,7 +17673,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="B16" s="28" t="s">
         <v>291</v>
@@ -17043,7 +17696,7 @@
     </row>
     <row r="17" spans="1:6" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="B17" s="28" t="s">
         <v>301</v>

</xml_diff>

<commit_message>
+ Add Battle view Scene and edit InteractionManager
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="13" activeTab="19"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="13" activeTab="18"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2651" uniqueCount="733">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2637" uniqueCount="731">
   <si>
     <t>ID</t>
   </si>
@@ -2229,12 +2229,6 @@
   </si>
   <si>
     <t>Battle_GoldHornKing</t>
-  </si>
-  <si>
-    <t>Battle_MarshalTianpeng</t>
-  </si>
-  <si>
-    <t>Battle_ThirdPrinceNezha</t>
   </si>
   <si>
     <t>Battle_LiJing_Boss</t>
@@ -4190,7 +4184,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
         <v>686</v>
       </c>
@@ -4333,8 +4327,8 @@
       <c r="E81" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F81" s="13" t="s">
-        <v>38</v>
+      <c r="F81" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
@@ -4347,8 +4341,8 @@
       <c r="E82" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F82" s="13" t="s">
-        <v>38</v>
+      <c r="F82" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
@@ -4361,8 +4355,8 @@
       <c r="E83" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F83" s="13" t="s">
-        <v>38</v>
+      <c r="F83" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
@@ -4389,8 +4383,8 @@
       <c r="E85" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F85" s="13" t="s">
-        <v>38</v>
+      <c r="F85" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
@@ -4417,8 +4411,8 @@
       <c r="E87" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F87" s="13" t="s">
-        <v>38</v>
+      <c r="F87" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
@@ -4431,8 +4425,8 @@
       <c r="E88" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F88" s="13" t="s">
-        <v>38</v>
+      <c r="F88" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -4445,8 +4439,8 @@
       <c r="E89" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F89" s="13" t="s">
-        <v>38</v>
+      <c r="F89" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
@@ -4473,8 +4467,8 @@
       <c r="E91" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F91" s="13" t="s">
-        <v>38</v>
+      <c r="F91" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
@@ -4501,8 +4495,8 @@
       <c r="E93" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F93" s="13" t="s">
-        <v>38</v>
+      <c r="F93" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
@@ -4515,8 +4509,8 @@
       <c r="E94" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F94" s="13" t="s">
-        <v>38</v>
+      <c r="F94" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
@@ -4529,8 +4523,8 @@
       <c r="E95" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F95" s="13" t="s">
-        <v>38</v>
+      <c r="F95" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
@@ -4557,8 +4551,8 @@
       <c r="E97" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F97" s="13" t="s">
-        <v>38</v>
+      <c r="F97" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -4571,8 +4565,8 @@
       <c r="E98" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F98" s="13" t="s">
-        <v>38</v>
+      <c r="F98" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -4585,8 +4579,8 @@
       <c r="E99" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F99" s="13" t="s">
-        <v>38</v>
+      <c r="F99" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
@@ -4599,8 +4593,8 @@
       <c r="E100" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F100" s="13" t="s">
-        <v>38</v>
+      <c r="F100" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -4613,8 +4607,8 @@
       <c r="E101" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F101" s="13" t="s">
-        <v>38</v>
+      <c r="F101" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -4641,8 +4635,8 @@
       <c r="E103" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F103" s="13" t="s">
-        <v>38</v>
+      <c r="F103" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
@@ -4669,8 +4663,8 @@
       <c r="E105" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F105" s="13" t="s">
-        <v>38</v>
+      <c r="F105" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
@@ -4683,8 +4677,8 @@
       <c r="E106" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F106" s="13" t="s">
-        <v>38</v>
+      <c r="F106" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
@@ -4697,8 +4691,8 @@
       <c r="E107" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F107" s="13" t="s">
-        <v>38</v>
+      <c r="F107" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
@@ -4725,8 +4719,8 @@
       <c r="E109" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F109" s="13" t="s">
-        <v>38</v>
+      <c r="F109" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
@@ -4753,8 +4747,8 @@
       <c r="E111" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F111" s="13" t="s">
-        <v>38</v>
+      <c r="F111" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
@@ -4767,8 +4761,8 @@
       <c r="E112" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F112" s="13" t="s">
-        <v>38</v>
+      <c r="F112" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
@@ -4781,8 +4775,8 @@
       <c r="E113" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F113" s="13" t="s">
-        <v>38</v>
+      <c r="F113" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
@@ -4809,8 +4803,8 @@
       <c r="E115" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="F115" s="13" t="s">
-        <v>38</v>
+      <c r="F115" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
@@ -7916,8 +7910,8 @@
       <c r="B4" t="s">
         <v>197</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>429</v>
+      <c r="C4" s="3" t="s">
+        <v>430</v>
       </c>
       <c r="D4" s="28" t="s">
         <v>298</v>
@@ -15998,17 +15992,17 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.28515625" style="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.28515625" style="27" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" style="27" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" style="27" customWidth="1"/>
+    <col min="2" max="3" width="27.28515625" style="27" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.28515625" style="27" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" style="27" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" style="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -16016,199 +16010,195 @@
         <v>1</v>
       </c>
       <c r="C1" s="17" t="s">
+        <v>434</v>
+      </c>
+      <c r="D1" s="17" t="s">
         <v>620</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="E1" s="17" t="s">
         <v>621</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="F1" s="17" t="s">
         <v>640</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>622</v>
       </c>
       <c r="B2" t="s">
         <v>623</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="27" t="s">
+        <v>623</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>624</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>625</v>
       </c>
-      <c r="E2" s="27">
+      <c r="F2" s="27">
         <v>600</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>723</v>
       </c>
       <c r="B3" s="27" t="s">
         <v>712</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="27" t="s">
+        <v>712</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>624</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>625</v>
       </c>
-      <c r="E3" s="27">
+      <c r="F3" s="27">
         <v>600</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>724</v>
       </c>
       <c r="B4" s="27" t="s">
         <v>223</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="27" t="s">
+        <v>223</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>624</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>625</v>
       </c>
-      <c r="E4" s="27">
+      <c r="F4" s="27">
         <v>600</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>725</v>
       </c>
       <c r="B5" s="27" t="s">
         <v>215</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>624</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="E5" s="7" t="s">
         <v>625</v>
       </c>
-      <c r="E5" s="27">
+      <c r="F5" s="27">
         <v>600</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>726</v>
       </c>
       <c r="B6" s="27" t="s">
         <v>207</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="27" t="s">
+        <v>207</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>624</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>625</v>
       </c>
-      <c r="E6" s="27">
+      <c r="F6" s="27">
         <v>600</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>727</v>
       </c>
       <c r="B7" s="27" t="s">
         <v>221</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="27" t="s">
+        <v>221</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>624</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="E7" s="7" t="s">
         <v>625</v>
       </c>
-      <c r="E7" s="27">
+      <c r="F7" s="27">
         <v>600</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>728</v>
       </c>
       <c r="B8" s="27" t="s">
         <v>217</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="27" t="s">
+        <v>217</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>624</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="E8" s="7" t="s">
         <v>625</v>
       </c>
-      <c r="E8" s="27">
+      <c r="F8" s="27">
         <v>600</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>729</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>698</v>
-      </c>
-      <c r="C9" s="7" t="s">
+        <v>687</v>
+      </c>
+      <c r="C9" s="27" t="s">
+        <v>687</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>624</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="E9" s="7" t="s">
         <v>625</v>
       </c>
-      <c r="E9" s="27">
+      <c r="F9" s="27">
         <v>600</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>730</v>
       </c>
-      <c r="B10" s="27" t="s">
-        <v>203</v>
-      </c>
-      <c r="C10" s="7" t="s">
+      <c r="B10" s="41" t="s">
+        <v>209</v>
+      </c>
+      <c r="C10" s="41" t="s">
+        <v>209</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>624</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="7" t="s">
         <v>625</v>
       </c>
-      <c r="E10" s="27">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>731</v>
-      </c>
-      <c r="B11" s="27" t="s">
-        <v>687</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>624</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>625</v>
-      </c>
-      <c r="E11" s="27">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>732</v>
-      </c>
-      <c r="B12" s="41" t="s">
-        <v>209</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>624</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>625</v>
-      </c>
-      <c r="E12" s="27">
+      <c r="F10" s="27">
         <v>600</v>
       </c>
     </row>
@@ -16414,7 +16404,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="27" bestFit="1" customWidth="1"/>
@@ -16991,24 +16981,24 @@
         <v>5</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>697</v>
+        <v>705</v>
       </c>
       <c r="D34" s="7">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E34" s="27" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
-        <v>730</v>
+      <c r="A35" s="7" t="s">
+        <v>729</v>
       </c>
       <c r="B35" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>663</v>
+        <v>702</v>
       </c>
       <c r="D35" s="7">
         <v>15</v>
@@ -17018,14 +17008,14 @@
       </c>
     </row>
     <row r="36" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
-        <v>730</v>
+      <c r="A36" s="7" t="s">
+        <v>729</v>
       </c>
       <c r="B36" s="7">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>663</v>
+        <v>697</v>
       </c>
       <c r="D36" s="7">
         <v>15</v>
@@ -17039,7 +17029,7 @@
         <v>730</v>
       </c>
       <c r="B37" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C37" s="23" t="s">
         <v>663</v>
@@ -17056,24 +17046,24 @@
         <v>730</v>
       </c>
       <c r="B38" s="7">
-        <v>5</v>
-      </c>
-      <c r="C38" s="22" t="s">
-        <v>702</v>
+        <v>2</v>
+      </c>
+      <c r="C38" s="23" t="s">
+        <v>663</v>
       </c>
       <c r="D38" s="7">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E38" s="27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="7" t="s">
-        <v>731</v>
+      <c r="A39" s="2" t="s">
+        <v>730</v>
       </c>
       <c r="B39" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C39" s="23" t="s">
         <v>663</v>
@@ -17086,155 +17076,19 @@
       </c>
     </row>
     <row r="40" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="7" t="s">
-        <v>731</v>
+      <c r="A40" s="2" t="s">
+        <v>730</v>
       </c>
       <c r="B40" s="7">
-        <v>2</v>
-      </c>
-      <c r="C40" s="23" t="s">
-        <v>663</v>
+        <v>5</v>
+      </c>
+      <c r="C40" s="22" t="s">
+        <v>704</v>
       </c>
       <c r="D40" s="7">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="E40" s="27" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="7" t="s">
-        <v>731</v>
-      </c>
-      <c r="B41" s="7">
-        <v>3</v>
-      </c>
-      <c r="C41" s="23" t="s">
-        <v>663</v>
-      </c>
-      <c r="D41" s="7">
-        <v>15</v>
-      </c>
-      <c r="E41" s="27" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="7" t="s">
-        <v>731</v>
-      </c>
-      <c r="B42" s="7">
-        <v>5</v>
-      </c>
-      <c r="C42" s="22" t="s">
-        <v>705</v>
-      </c>
-      <c r="D42" s="7">
-        <v>25</v>
-      </c>
-      <c r="E42" s="27" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="7" t="s">
-        <v>731</v>
-      </c>
-      <c r="B43" s="7">
-        <v>4</v>
-      </c>
-      <c r="C43" s="23" t="s">
-        <v>702</v>
-      </c>
-      <c r="D43" s="7">
-        <v>15</v>
-      </c>
-      <c r="E43" s="27" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="7" t="s">
-        <v>731</v>
-      </c>
-      <c r="B44" s="7">
-        <v>6</v>
-      </c>
-      <c r="C44" s="23" t="s">
-        <v>697</v>
-      </c>
-      <c r="D44" s="7">
-        <v>15</v>
-      </c>
-      <c r="E44" s="27" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
-        <v>732</v>
-      </c>
-      <c r="B45" s="7">
-        <v>1</v>
-      </c>
-      <c r="C45" s="23" t="s">
-        <v>663</v>
-      </c>
-      <c r="D45" s="7">
-        <v>15</v>
-      </c>
-      <c r="E45" s="27" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="2" t="s">
-        <v>732</v>
-      </c>
-      <c r="B46" s="7">
-        <v>2</v>
-      </c>
-      <c r="C46" s="23" t="s">
-        <v>663</v>
-      </c>
-      <c r="D46" s="7">
-        <v>15</v>
-      </c>
-      <c r="E46" s="27" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="2" t="s">
-        <v>732</v>
-      </c>
-      <c r="B47" s="7">
-        <v>3</v>
-      </c>
-      <c r="C47" s="23" t="s">
-        <v>663</v>
-      </c>
-      <c r="D47" s="7">
-        <v>15</v>
-      </c>
-      <c r="E47" s="27" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="2" t="s">
-        <v>732</v>
-      </c>
-      <c r="B48" s="7">
-        <v>5</v>
-      </c>
-      <c r="C48" s="22" t="s">
-        <v>704</v>
-      </c>
-      <c r="D48" s="7">
-        <v>30</v>
-      </c>
-      <c r="E48" s="27" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
+ Add content for Battle View Scene.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2637" uniqueCount="731">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2637" uniqueCount="748">
   <si>
     <t>ID</t>
   </si>
@@ -2235,6 +2235,57 @@
   </si>
   <si>
     <t>Battle_ErlangShen_Boss</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_TUTORIAL_DES</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_THIRD_DRAGON_PRINCE</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_THIRD_DRAGON_PRINCE_DES</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_GOLD_FISH_DEMON</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_GOLD_FISH_DEMON_DES</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_THE_BOY_SAGE</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_THE_BOY_SAGE_DES</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_BULL_DEMON_KING</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_BULL_DEMON_KING_DES</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_YELLOW_WIND_MONSTER</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_YELLOW_WIND_MONSTER_DES</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_GOLD_HORN_KING</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_GOLD_HORN_KING_DES</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_LI_JING_BOSS</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_LI_JING_BOSS_DES</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_ERLANG_SHEN_BOSS</t>
+  </si>
+  <si>
+    <t>STR_BATTLE_ERLANG_SHEN_BOSS_DES</t>
   </si>
 </sst>
 </file>
@@ -2378,7 +2429,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2478,6 +2529,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15996,7 +16050,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" style="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="27.28515625" style="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.140625" style="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.28515625" style="27" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.28515625" style="27" customWidth="1"/>
     <col min="5" max="5" width="15.5703125" style="27" customWidth="1"/>
     <col min="6" max="6" width="10.85546875" style="27" customWidth="1"/>
@@ -16023,14 +16078,14 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="45" t="s">
         <v>622</v>
       </c>
       <c r="B2" t="s">
         <v>623</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>623</v>
+        <v>731</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>624</v>
@@ -16043,14 +16098,14 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="45" t="s">
         <v>723</v>
       </c>
       <c r="B3" s="27" t="s">
-        <v>712</v>
+        <v>732</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>712</v>
+        <v>733</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>624</v>
@@ -16063,14 +16118,14 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="45" t="s">
         <v>724</v>
       </c>
       <c r="B4" s="27" t="s">
-        <v>223</v>
+        <v>734</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>223</v>
+        <v>735</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>624</v>
@@ -16083,14 +16138,14 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="45" t="s">
         <v>725</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>215</v>
+        <v>736</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>215</v>
+        <v>737</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>624</v>
@@ -16103,14 +16158,14 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="45" t="s">
         <v>726</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>207</v>
+        <v>738</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>207</v>
+        <v>739</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>624</v>
@@ -16123,14 +16178,14 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="45" t="s">
         <v>727</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>221</v>
+        <v>740</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>221</v>
+        <v>741</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>624</v>
@@ -16143,14 +16198,14 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="45" t="s">
         <v>728</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>217</v>
+        <v>742</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>217</v>
+        <v>743</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>624</v>
@@ -16163,14 +16218,14 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="45" t="s">
         <v>729</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>687</v>
+        <v>744</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>687</v>
+        <v>745</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>624</v>
@@ -16183,14 +16238,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="45" t="s">
         <v>730</v>
       </c>
-      <c r="B10" s="41" t="s">
-        <v>209</v>
-      </c>
-      <c r="C10" s="41" t="s">
-        <v>209</v>
+      <c r="B10" s="27" t="s">
+        <v>746</v>
+      </c>
+      <c r="C10" s="27" t="s">
+        <v>747</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>624</v>

</xml_diff>

<commit_message>
+ Balance skill and weapon of Na Zha
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" state="visible" r:id="rId1"/>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Legendary</t>
+          <t>Epic</t>
         </is>
       </c>
     </row>
@@ -8604,7 +8604,7 @@
           <t>ThirdPrinceNezha_B_Name</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>ThirdPrinceNezha_B_Des</t>
         </is>
@@ -8661,7 +8661,7 @@
           <t>ThirdPrinceNezha_M_Name</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>ThirdPrinceNezha_M_Des</t>
         </is>
@@ -8673,7 +8673,7 @@
       </c>
       <c r="E18" s="37" t="inlineStr">
         <is>
-          <t>1, 1.5, 1.5</t>
+          <t>0.4, 0.5, 0.6</t>
         </is>
       </c>
       <c r="F18" s="37" t="inlineStr">
@@ -8718,19 +8718,19 @@
           <t>ThirdPrinceNezha_U_Name</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>ThirdPrinceNezha_U_Des</t>
         </is>
       </c>
       <c r="D19" s="36" t="inlineStr">
         <is>
-          <t>EmpowerAttack</t>
+          <t>NezhaExecution</t>
         </is>
       </c>
       <c r="E19" s="37" t="inlineStr">
         <is>
-          <t>1.5, 1.8, 1.8</t>
+          <t>1.4, 1.6, 1.8</t>
         </is>
       </c>
       <c r="F19" s="37" t="inlineStr">
@@ -8760,7 +8760,7 @@
       </c>
       <c r="K19" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>psv_nezha_ultimate</t>
         </is>
       </c>
     </row>
@@ -21417,24 +21417,24 @@
       </c>
       <c r="C16" s="37" t="inlineStr">
         <is>
-          <t>Fighter</t>
+          <t>Assassin</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1375</v>
+        <v>578</v>
       </c>
       <c r="E16" t="n">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="F16" t="n">
-        <v>138</v>
+        <v>58</v>
       </c>
       <c r="G16" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H16" s="30" t="inlineStr">
         <is>
-          <t>psv_vanguard_of_volition</t>
+          <t>psv_windfire_wheel</t>
         </is>
       </c>
     </row>
@@ -21546,7 +21546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.7109375" bestFit="1" customWidth="1" style="35" min="1" max="1"/>
@@ -21964,6 +21964,40 @@
       <c r="C24" t="inlineStr">
         <is>
           <t>Tăng {0}% Tấn Công và {0}% Phòng Thủ. Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng. Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu tương đương 16% tổng sát thương gây ra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>psv_nezha_ultimate</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>STR_NEZHA_ULT_PASSIVE</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Khi kết liễu kẻ địch bằng chiêu cuối, kích hoạt hiệu ứng [Càn Quét] tấn công 1 kẻ địch khác với 120% ATK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>psv_windfire_wheel</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>STR_WINDFIRE_WHEEL_SKILL</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {0}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
         </is>
       </c>
     </row>
@@ -21978,7 +22012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.7109375" bestFit="1" customWidth="1" style="35" min="1" max="1"/>
@@ -22498,6 +22532,60 @@
       <c r="E19" t="inlineStr">
         <is>
           <t>Tăng {0}% Tấn Công và {0}% Phòng Thủ. Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng. Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu tương đương 16% tổng sát thương gây ra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>psv_windfire_wheel</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CRIT_DMG</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>8, 10, 12, 14, 17, 20</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {0}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>psv_windfire_wheel</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ATK</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>8, 10, 12, 14, 17, 20</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {0}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
         </is>
       </c>
     </row>
@@ -22517,7 +22605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26.7109375" customWidth="1" style="35" min="1" max="1"/>
@@ -23424,6 +23512,92 @@
       <c r="I21" t="inlineStr">
         <is>
           <t>Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>psv_nezha_ultimate</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>OnAfterDealDamage</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Eff_FollowUp_BasicAttack</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>100, 120, 150, 200, 200, 200</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>UltimateSkill, TargetDead</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Khi kết liễu kẻ địch bằng chiêu cuối, kích hoạt hiệu ứng [Càn Quét] tấn công 1 kẻ địch khác với 120% ATK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>psv_windfire_wheel</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>OnAfterDealDamage</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Eff_Action_Point_Boost</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>10, 12, 14, 16, 18, 20</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>IsCritical</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
+ Balance skill and weapon for Tang San Zang.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" tabRatio="600" firstSheet="5" activeTab="12" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Item_Master" sheetId="1" state="visible" r:id="rId1"/>
@@ -7999,12 +7999,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>BuffShield</t>
+          <t>StatModifier</t>
         </is>
       </c>
       <c r="E6" s="37" t="inlineStr">
         <is>
-          <t>1, 1.5, 1.5</t>
+          <t>0, 0, 0</t>
         </is>
       </c>
       <c r="F6" s="37" t="inlineStr">
@@ -8019,12 +8019,12 @@
       </c>
       <c r="H6" s="37" t="inlineStr">
         <is>
-          <t>Self</t>
+          <t>SameRowAllies</t>
         </is>
       </c>
       <c r="I6" s="36" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>EFF_Tang_Buff_ATK</t>
         </is>
       </c>
       <c r="J6" s="28" t="inlineStr">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="I21" s="36" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>EFF_Dragon_Speed</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -20883,6 +20883,8 @@
     <col width="21" bestFit="1" customWidth="1" style="35" min="1" max="1"/>
     <col width="11.140625" bestFit="1" customWidth="1" style="35" min="2" max="2"/>
     <col width="8.42578125" bestFit="1" customWidth="1" style="35" min="3" max="3"/>
+    <col width="10" bestFit="1" customWidth="1" style="35" min="6" max="6"/>
+    <col width="11" bestFit="1" customWidth="1" style="35" min="7" max="7"/>
     <col width="24.7109375" bestFit="1" customWidth="1" style="35" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -20944,16 +20946,16 @@
           <t>Fighter</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="36" t="n">
         <v>1375</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="36" t="n">
         <v>225</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="36" t="n">
         <v>138</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="36" t="n">
         <v>23</v>
       </c>
       <c r="H2" s="31" t="inlineStr">
@@ -20978,16 +20980,16 @@
           <t>Fighter</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="36" t="n">
         <v>1375</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="36" t="n">
         <v>225</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="36" t="n">
         <v>138</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="36" t="n">
         <v>23</v>
       </c>
       <c r="H3" s="31" t="inlineStr">
@@ -21012,16 +21014,16 @@
           <t>Assassin</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="36" t="n">
         <v>875</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="36" t="n">
         <v>325</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="36" t="n">
         <v>88</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="36" t="n">
         <v>33</v>
       </c>
       <c r="H4" s="31" t="inlineStr">
@@ -21043,19 +21045,19 @@
       </c>
       <c r="C5" s="37" t="inlineStr">
         <is>
-          <t>Mage</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D5" s="36" t="n">
         <v>495</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="36" t="n">
         <v>121</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="36" t="n">
         <v>50</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="36" t="n">
         <v>12</v>
       </c>
       <c r="H5" s="31" t="inlineStr">
@@ -21080,16 +21082,16 @@
           <t>Tanker</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="36" t="n">
         <v>2000</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="36" t="n">
         <v>100</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="36" t="n">
         <v>200</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="36" t="n">
         <v>10</v>
       </c>
       <c r="H6" s="31" t="inlineStr">
@@ -21114,16 +21116,16 @@
           <t>Mage</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="36" t="n">
         <v>495</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="36" t="n">
         <v>121</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="36" t="n">
         <v>50</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="36" t="n">
         <v>12</v>
       </c>
       <c r="H7" s="31" t="inlineStr">
@@ -21148,16 +21150,16 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="36" t="n">
         <v>300</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="36" t="n">
         <v>40</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="36" t="n">
         <v>30</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="36" t="n">
         <v>4</v>
       </c>
       <c r="H8" s="31" t="inlineStr">
@@ -21179,19 +21181,19 @@
       </c>
       <c r="C9" s="37" t="inlineStr">
         <is>
-          <t>Assassin</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
+          <t>ADCarry</t>
+        </is>
+      </c>
+      <c r="D9" s="36" t="n">
         <v>578</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="36" t="n">
         <v>214</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="36" t="n">
         <v>58</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="36" t="n">
         <v>21</v>
       </c>
       <c r="H9" s="31" t="inlineStr">
@@ -21216,16 +21218,16 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="36" t="n">
         <v>450</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="36" t="n">
         <v>60</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="36" t="n">
         <v>45</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="36" t="n">
         <v>6</v>
       </c>
       <c r="H10" s="31" t="inlineStr">
@@ -21250,16 +21252,16 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="36" t="n">
         <v>300</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="36" t="n">
         <v>40</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="36" t="n">
         <v>30</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="36" t="n">
         <v>4</v>
       </c>
       <c r="H11" s="31" t="inlineStr">
@@ -21284,16 +21286,16 @@
           <t>Tanker</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="36" t="n">
         <v>600</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="36" t="n">
         <v>30</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="36" t="n">
         <v>60</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" s="36" t="n">
         <v>3</v>
       </c>
       <c r="H12" s="31" t="inlineStr">
@@ -21318,16 +21320,16 @@
           <t>Mage</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="36" t="n">
         <v>1125</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="36" t="n">
         <v>275</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="36" t="n">
         <v>113</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" s="36" t="n">
         <v>28</v>
       </c>
       <c r="H13" s="31" t="inlineStr">
@@ -21352,16 +21354,16 @@
           <t>Mage</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="36" t="n">
         <v>742</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="36" t="n">
         <v>182</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="36" t="n">
         <v>74</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" s="36" t="n">
         <v>18</v>
       </c>
       <c r="H14" s="31" t="inlineStr">
@@ -21386,16 +21388,16 @@
           <t>Support</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="36" t="n">
         <v>1750</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="36" t="n">
         <v>150</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="36" t="n">
         <v>175</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" s="36" t="n">
         <v>15</v>
       </c>
       <c r="H15" s="31" t="inlineStr">
@@ -21420,16 +21422,16 @@
           <t>Assassin</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" s="36" t="n">
         <v>578</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="36" t="n">
         <v>214</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" s="36" t="n">
         <v>58</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16" s="36" t="n">
         <v>21</v>
       </c>
       <c r="H16" s="30" t="inlineStr">
@@ -21454,16 +21456,16 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="36" t="n">
         <v>300</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="36" t="n">
         <v>40</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="36" t="n">
         <v>30</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17" s="36" t="n">
         <v>4</v>
       </c>
     </row>
@@ -21478,21 +21480,21 @@
           <t>Legendary</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="36" t="inlineStr">
         <is>
           <t>Tanker</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D18" s="36" t="n">
         <v>2200</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="36" t="n">
         <v>120</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="36" t="n">
         <v>220</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G18" s="36" t="n">
         <v>12</v>
       </c>
       <c r="H18" t="inlineStr">
@@ -21517,16 +21519,16 @@
           <t>Fighter</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D19" s="36" t="n">
         <v>1375</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="36" t="n">
         <v>225</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="36" t="n">
         <v>138</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" s="36" t="n">
         <v>23</v>
       </c>
       <c r="H19" s="31" t="inlineStr">
@@ -21635,7 +21637,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hiệu quả chính xác tăng {0}%. Khi bắt đầu hiệp, nếu bản thân có hiệu ứng suy yếu, có {1}% xác suất xóa 1 hiệu ứng suy yếu.</t>
+          <t>Tăng {0}% Tốc độ. Tăng thêm {1}% hiệu quả cho các kỹ năng Cường Hóa và Buff.</t>
         </is>
       </c>
     </row>
@@ -21686,7 +21688,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ST tấn công đơn tăng {0}%.</t>
+          <t>Tấn công tăng {0}%.</t>
         </is>
       </c>
     </row>
@@ -21703,7 +21705,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tấn công tăng {0}%. Khi tấn công đơn, có {1}% xác xuất gây Xé Toạc cho mục tiêu tân công, duy trì 2 hiệp.</t>
+          <t>Tấn công tăng {0}%. Đòn tấn công đơn mục tiêu gây thêm {1}% Sát thương.</t>
         </is>
       </c>
     </row>
@@ -22012,7 +22014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.7109375" bestFit="1" customWidth="1" style="35" min="1" max="1"/>
@@ -22165,7 +22167,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EHR</t>
+          <t>SPEED</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -22175,12 +22177,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10, 15, 20, 25, 31, 34</t>
+          <t>6, 8, 10, 12, 15, 20</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Hiệu quả chính xác tăng {0}%. Khi bắt đầu hiệp, nếu bản thân có hiệu ứng suy yếu, có {1}% xác suất xóa 1 hiệu ứng suy yếu.</t>
+          <t>Tăng {0}% Tốc độ. Tăng thêm {1}% hiệu quả cho các kỹ năng Cường Hóa và Buff.</t>
         </is>
       </c>
     </row>
@@ -22202,12 +22204,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10, 15, 20, 25, 35, 40</t>
+          <t>8, 11, 14, 17, 20, 25</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Tấn công tăng {0}%. Khi tấn công đơn, có {1}% xác xuất gây Xé Toạc cho mục tiêu tân công, duy trì 2 hiệp.</t>
+          <t>Tấn công tăng {0}%. Đòn tấn công đơn mục tiêu gây thêm {1}% Sát thương.</t>
         </is>
       </c>
     </row>
@@ -22273,7 +22275,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SPEED</t>
+          <t>DEF</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -22283,7 +22285,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>5, 7.5, 10, 12.5, 17,, 22</t>
+          <t>5, 7.5, 10, 12.5, 16, 20</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -22586,6 +22588,33 @@
       <c r="E21" t="inlineStr">
         <is>
           <t>Tăng {0}% HP và {0}% Phòng Thủ. Mỗi khi chịu sát thương, Phòng Thủ tăng thêm {1}%, tối đa cộng dồn 5 tầng. Khi đạt 5 tầng, hồi phục 10% HP Tối Đa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>psv_sunburst_spade</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ATK</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>5, 7.5, 10, 12.5, 15, 20</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Tấn công tăng {0}%.</t>
         </is>
       </c>
     </row>
@@ -22605,7 +22634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26.7109375" customWidth="1" style="35" min="1" max="1"/>
@@ -22800,21 +22829,21 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Eff_Cleanse</t>
+          <t>Eff_Buff_Enhance</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>30.0, 40.0, 50.0, 60.0, 70.0, 80.0</t>
+          <t>30.0, 35.0, 40.0, 45.0, 50.0, 60.0</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>HasDebuff</t>
+          <t>None</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -22826,7 +22855,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Hiệu quả chính xác tăng {0}%. Khi bắt đầu hiệp, nếu bản thân có hiệu ứng suy yếu, có {1}% xác suất xóa 1 hiệu ứng suy yếu.</t>
+          <t>Tăng {0}% Tốc độ. Tăng thêm {1}% hiệu quả cho các kỹ năng Cường Hóa và Buff.</t>
         </is>
       </c>
     </row>
@@ -22881,17 +22910,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OnAfterTakeDamage</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eff_Lacerate_Debuff</t>
+          <t>Eff_IncreaseAttack</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>30.0, 40.0, 50.0, 60.0, 70.0, 80.0</t>
+          <t>10.0, 13.0, 16.0, 19.0, 22.0, 25.0</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -22900,16 +22929,19 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>self</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Tấn công tăng {0}%. Khi tấn công đơn, có {1}% xác xuất gây Xé Toạc cho mục tiêu tân công, duy trì 2 hiệp.</t>
+          <t>Tấn công tăng {0}%. Đòn tấn công đơn mục tiêu gây thêm {1}% Sát thương.</t>
         </is>
       </c>
     </row>
@@ -23045,27 +23077,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>psv_sunburst_spade</t>
+          <t>psv_sunwukong_major</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>OnBeforeDealDamage</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eff_IncreaseAttack </t>
+          <t>Eff_Lifesteal</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.0, 15.0, 20.0, 25.0, 30.0, 40.0</t>
+          <t>20, 25, 30, 30, 30, 30</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SingleTarget</t>
+          <t>MajorSkill</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -23081,29 +23113,29 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ST tấn công đơn tăng {0}%.</t>
+          <t>Kỹ năng Major hút máu 25%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>psv_sunwukong_major</t>
+          <t>psv_erlangshen_major</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>OnAfterDealDamage</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Eff_Lifesteal</t>
+          <t>Eff_IncreaseCritDmg</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>20, 25, 30, 30, 30, 30</t>
+          <t>60, 80, 100, 100, 100, 100</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -23124,38 +23156,38 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Kỹ năng Major hút máu 25%</t>
+          <t>Kỹ năng Major tăng 100% Crit DMG</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>psv_erlangshen_major</t>
+          <t>psv_lijing_base</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>OnBeforeDealDamage</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Eff_IncreaseCritDmg</t>
+          <t>Eff_AddShield</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>60, 80, 100, 100, 100, 100</t>
+          <t>5, 5, 5, 5, 5, 5</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MajorSkill</t>
+          <t>BasicAttack</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -23167,38 +23199,38 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Kỹ năng Major tăng 100% Crit DMG</t>
+          <t>Đánh thường nhận khiên 5% Max HP (max 5 tầng)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>psv_lijing_base</t>
+          <t>psv_lijing_ultimate</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OnAfterDealDamage</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eff_AddShield</t>
+          <t>Eff_HPScalingDamage</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>5, 5, 5, 5, 5, 5</t>
+          <t>30, 30, 30, 30, 30, 30</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BasicAttack</t>
+          <t>UltimateSkill</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -23210,14 +23242,14 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Đánh thường nhận khiên 5% Max HP (max 5 tầng)</t>
+          <t>Tuyệt kỹ nộ tăng 30% Max HP vào Base Damage</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>psv_lijing_ultimate</t>
+          <t>psv_erlangshen_ultimate</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -23227,7 +23259,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Eff_HPScalingDamage</t>
+          <t>Eff_ArmorPenetration</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -23253,29 +23285,29 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Tuyệt kỹ nộ tăng 30% Max HP vào Base Damage</t>
+          <t>Tuyệt kỹ tăng 30% Xuyên Giáp</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>psv_erlangshen_ultimate</t>
+          <t>psv_sunwukong_ultiamte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>OnBeforeDealDamage</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Eff_ArmorPenetration</t>
+          <t>Eff_ReduceDefense</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>30, 30, 30, 30, 30, 30</t>
+          <t>15, 20, 25, 25, 25, 25</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -23291,43 +23323,43 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>enemy</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Tuyệt kỹ tăng 30% Xuyên Giáp</t>
+          <t>Tuyệt kỹ giảm 25% DEF mục tiêu</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>psv_sunwukong_ultiamte</t>
+          <t>psv_bulldemonking_counter</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>OnAfterDealDamage</t>
+          <t>OnTakeDamage</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Eff_ReduceDefense</t>
+          <t>Eff_CounterAttack</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>15, 20, 25, 25, 25, 25</t>
+          <t>50, 75, 100, 100, 100, 100</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>UltimateSkill</t>
+          <t>BasicAttack</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -23339,50 +23371,50 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Tuyệt kỹ giảm 25% DEF mục tiêu</t>
+          <t>Có 50%, 75%, 100% cơ hội phản kích khi bị đánh thường, gây 100% ATK</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>psv_bulldemonking_counter</t>
+          <t>psv_ferrous_chaos</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>OnTakeDamage</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Eff_CounterAttack</t>
+          <t>Eff_IncreaseAttack</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>50, 75, 100, 100, 100, 100</t>
+          <t>16, 16, 16, 16, 16, 16</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BasicAttack</t>
+          <t>IsSkill, HP_Above_50</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>self</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Có 50%, 75%, 100% cơ hội phản kích khi bị đánh thường, gây 100% ATK</t>
+          <t>Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng</t>
         </is>
       </c>
     </row>
@@ -23394,12 +23426,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>OnBeforeDealDamage</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Eff_IncreaseAttack</t>
+          <t>Eff_Lifesteal</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -23409,7 +23441,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>IsSkill, HP_Above_50</t>
+          <t>HP_BelowOrEqual_50</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -23425,14 +23457,14 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng</t>
+          <t>Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>psv_ferrous_chaos</t>
+          <t>psv_nezha_ultimate</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -23442,17 +23474,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Eff_Lifesteal</t>
+          <t>Eff_FollowUp_BasicAttack</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>16, 16, 16, 16, 16, 16</t>
+          <t>100, 120, 150, 200, 200, 200</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>HP_BelowOrEqual_50</t>
+          <t>UltimateSkill, TargetDead</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -23468,14 +23500,14 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu</t>
+          <t>Khi kết liễu kẻ địch bằng chiêu cuối, kích hoạt hiệu ứng [Càn Quét] tấn công 1 kẻ địch khác với 120% ATK.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>psv_nezha_ultimate</t>
+          <t>psv_windfire_wheel</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -23485,17 +23517,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Eff_FollowUp_BasicAttack</t>
+          <t>Eff_Action_Point_Boost</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>100, 120, 150, 200, 200, 200</t>
+          <t>10, 12, 14, 16, 18, 20</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>UltimateSkill, TargetDead</t>
+          <t>IsCritical</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -23511,38 +23543,38 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Khi kết liễu kẻ địch bằng chiêu cuối, kích hoạt hiệu ứng [Càn Quét] tấn công 1 kẻ địch khác với 120% ATK.</t>
+          <t>Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>psv_windfire_wheel</t>
+          <t>psv_nine_toothed_rake</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>OnAfterDealDamage</t>
+          <t>OnTakeDamage</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Eff_Action_Point_Boost</t>
+          <t>Eff_Stackable_DEF_Buff</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10, 12, 14, 16, 18, 20</t>
+          <t>4.0, 5.0, 6.0, 7.0, 8.0, 10.0</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>IsCritical</t>
+          <t>None</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -23553,49 +23585,6 @@
         </is>
       </c>
       <c r="I22" t="inlineStr">
-        <is>
-          <t>Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>psv_nine_toothed_rake</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>OnTakeDamage</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Eff_Stackable_DEF_Buff</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>4.0, 5.0, 6.0, 7.0, 8.0, 10.0</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
         <is>
           <t>Mỗi khi chịu sát thương, Phòng Thủ tăng thêm {1}%, tối đa cộng dồn 5 tầng. Khi đạt 5 tầng, hồi phục 10% HP Tối Đa.</t>
         </is>
@@ -23613,7 +23602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.140625" customWidth="1" style="35" min="1" max="1"/>
@@ -24162,6 +24151,88 @@
         <v>25</v>
       </c>
       <c r="I13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>EFF_Dragon_Speed</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>BUFF_SPEED_NAME</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>BUFF_SPEED_DES</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>StatBuff</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SPEED</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" t="n">
+        <v>30</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>EFF_Tang_Buff_ATK</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BUFF_ATTACK_NAME</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BUFF_ATTACK_DES</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>StatBuff</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ATK</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" t="n">
+        <v>20</v>
+      </c>
+      <c r="I15" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
+ Balance for Vanguard Of Volition (Tùy Tâm Thiết Canh Binh)
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -21620,7 +21620,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ST Bạo Kích tăng {0}%. Sau khi tấn công đơn, nếu mục tiêu vẫn còn sống, có {1}% xác suất thi triển đánh thường để truy kích, mỗi hiệp kích hoạt tối đa 1 lần. Khi Phản Kích, Hỗ Trợ Tấn công se không kích hoạt hiệu ứng này.</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {2}% Điểm Hành Động của bản thân. Sau khi tấn công đơn mục tiêu, nếu mục tiêu còn sống, có {3}% xác suất lập tức tung đòn Đánh Thường để truy kích.</t>
         </is>
       </c>
     </row>
@@ -22014,7 +22014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.7109375" bestFit="1" customWidth="1" style="35" min="1" max="1"/>
@@ -22135,12 +22135,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>psv_vanguard_of_volition</t>
+          <t>psv_ninefold_staff</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CRIT_DMG</t>
+          <t>SPEED</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -22150,24 +22150,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10, 15, 20, 25, 31, 34</t>
+          <t>6, 8, 10, 12, 15, 20</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ST Bạo Kích tăng {0}%. Sau khi tấn công đơn, nếu mục tiêu vẫn còn sống, có {1}% xác suất thi triển đánh thường để truy kích, mỗi hiệp kích hoạt tối đa 1 lần. Khi Phản Kích, Hỗ Trợ Tấn công se không kích hoạt hiệu ứng này.</t>
+          <t>Tăng {0}% Tốc độ. Tăng thêm {1}% hiệu quả cho các kỹ năng Cường Hóa và Buff.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>psv_ninefold_staff</t>
+          <t>psv_reincarnation</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SPEED</t>
+          <t>ATK</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -22177,24 +22177,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6, 8, 10, 12, 15, 20</t>
+          <t>8, 11, 14, 17, 20, 25</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Tăng {0}% Tốc độ. Tăng thêm {1}% hiệu quả cho các kỹ năng Cường Hóa và Buff.</t>
+          <t>Tấn công tăng {0}%. Đòn tấn công đơn mục tiêu gây thêm {1}% Sát thương.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>psv_reincarnation</t>
+          <t>psv_ennead_spear</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ATK</t>
+          <t>CRIT_RATE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -22204,24 +22204,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>8, 11, 14, 17, 20, 25</t>
+          <t>5, 7.5, 10, 12.5, 16, 20</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Tấn công tăng {0}%. Đòn tấn công đơn mục tiêu gây thêm {1}% Sát thương.</t>
+          <t>Tỷ lệ bạo kích tăng {0}%.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>psv_ennead_spear</t>
+          <t>psv_crescent_axe</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CRIT_RATE</t>
+          <t>CRIT_DMG</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -22231,24 +22231,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5, 7.5, 10, 12.5, 16, 20</t>
+          <t>5, 7.5, 10, 12.5, 17,, 21</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Tỷ lệ bạo kích tăng {0}%.</t>
+          <t xml:space="preserve">ST Bạo Kích tăng {0}%. </t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>psv_crescent_axe</t>
+          <t>psv_bronze_hammer</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CRIT_DMG</t>
+          <t>DEF</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -22258,19 +22258,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>5, 7.5, 10, 12.5, 17,, 21</t>
+          <t>5, 7.5, 10, 12.5, 16, 20</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ST Bạo Kích tăng {0}%. </t>
+          <t>Phòng thủ tăng {0}%.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>psv_bronze_hammer</t>
+          <t>psv_moonlit_firefly</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -22285,12 +22285,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>5, 7.5, 10, 12.5, 16, 20</t>
+          <t>5, 7.5, 10, 12.5, 17,, 23</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Phòng thủ tăng {0}%.</t>
+          <t>Tấn công và phòng thủ tăng {0}%. Sau khi thi triển kỹ năng không phải tấn công, có {1}% xác suất hiệp hồi chiêu -1.</t>
         </is>
       </c>
     </row>
@@ -22302,7 +22302,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>ATK</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -22312,7 +22312,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5, 7.5, 10, 12.5, 17,, 23</t>
+          <t>5, 7.5, 10, 12.5, 17,, 24</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -22324,12 +22324,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>psv_moonlit_firefly</t>
+          <t>psv_plantain_fan</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ATK</t>
+          <t>EHR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -22339,24 +22339,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5, 7.5, 10, 12.5, 17,, 24</t>
+          <t>10, 15, 20, 25, 34, 40</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Tấn công và phòng thủ tăng {0}%. Sau khi thi triển kỹ năng không phải tấn công, có {1}% xác suất hiệp hồi chiêu -1.</t>
+          <t>Tăng {0}% Hiệu quả Chính Xác.Các đòn tấn công đơn mục tiêu có {1}% cơ hội gây hiệu ứng Đánh Dấu lên mục tiêu trong 1 lượt.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>psv_plantain_fan</t>
+          <t>psv_wings_of_phoenix</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EHR</t>
+          <t>RES</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -22366,24 +22366,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10, 15, 20, 25, 34, 40</t>
+          <t>10, 15, 20, 25, 34, 41</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Tăng {0}% Hiệu quả Chính Xác.Các đòn tấn công đơn mục tiêu có {1}% cơ hội gây hiệu ứng Đánh Dấu lên mục tiêu trong 1 lượt.</t>
+          <t>Kháng hiệu ứng tăng {0}%. Sau khi bị kĩ năng tấn công, nếu bản thân tồn tại hiệu ứng suy yếu, có {1}% xác xuất xóa 2 hiệu ứng suy yếu cảu bản thân, cứ 2 hiệp kích hoạt tối đa 1 lần.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>psv_wings_of_phoenix</t>
+          <t>psv_linglong_pagoda</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RES</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -22393,24 +22393,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10, 15, 20, 25, 34, 41</t>
+          <t>15, 20, 25, 30, 35, 40</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kháng hiệu ứng tăng {0}%. Sau khi bị kĩ năng tấn công, nếu bản thân tồn tại hiệu ứng suy yếu, có {1}% xác xuất xóa 2 hiệu ứng suy yếu cảu bản thân, cứ 2 hiệp kích hoạt tối đa 1 lần.</t>
+          <t>HP tối đa tăng {0}%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>psv_linglong_pagoda</t>
+          <t>psv_ferrous_chaos</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ATK</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -22420,12 +22420,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>15, 20, 25, 30, 35, 40</t>
+          <t>10, 15, 20, 25, 30, 35</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>HP tối đa tăng {0}%</t>
+          <t>Tăng {0}% Tấn Công và {0}% Phòng Thủ. Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng. Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu tương đương 16% tổng sát thương gây ra.</t>
         </is>
       </c>
     </row>
@@ -22437,7 +22437,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ATK</t>
+          <t>DEF</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -22459,12 +22459,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>psv_ferrous_chaos</t>
+          <t>psv_windfire_wheel</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>CRIT_DMG</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -22474,12 +22474,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10, 15, 20, 25, 30, 35</t>
+          <t>8, 10, 12, 14, 17, 20</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Tăng {0}% Tấn Công và {0}% Phòng Thủ. Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng. Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu tương đương 16% tổng sát thương gây ra.</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {0}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
         </is>
       </c>
     </row>
@@ -22491,7 +22491,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CRIT_DMG</t>
+          <t>ATK</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -22513,12 +22513,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>psv_windfire_wheel</t>
+          <t>psv_nine_toothed_rake</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ATK</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -22528,12 +22528,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>8, 10, 12, 14, 17, 20</t>
+          <t>10, 14, 18, 22, 26, 32</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Tăng {0}% Sát Thương Bạo Kích và {0}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
+          <t>Tăng {0}% HP và {0}% Phòng Thủ. Mỗi khi chịu sát thương, Phòng Thủ tăng thêm {1}%, tối đa cộng dồn 5 tầng. Khi đạt 5 tầng, hồi phục 10% HP Tối Đa.</t>
         </is>
       </c>
     </row>
@@ -22545,7 +22545,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>DEF</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -22567,12 +22567,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>psv_nine_toothed_rake</t>
+          <t>psv_sunburst_spade</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>ATK</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -22582,39 +22582,66 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10, 14, 18, 22, 26, 32</t>
+          <t>5, 7.5, 10, 12.5, 15, 20</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Tăng {0}% HP và {0}% Phòng Thủ. Mỗi khi chịu sát thương, Phòng Thủ tăng thêm {1}%, tối đa cộng dồn 5 tầng. Khi đạt 5 tầng, hồi phục 10% HP Tối Đa.</t>
+          <t>Tấn công tăng {0}%.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>psv_sunburst_spade</t>
+          <t>psv_vanguard_of_volition</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>CRIT_DMG</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>20, 25, 30, 35, 40, 50</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {2}% Điểm Hành Động của bản thân. Sau khi tấn công đơn mục tiêu, nếu mục tiêu còn sống, có {3}% xác suất lập tức tung đòn Đánh Thường để truy kích.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>psv_vanguard_of_volition</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>ATK</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Percent</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>5, 7.5, 10, 12.5, 15, 20</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Tấn công tăng {0}%.</t>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>10, 12, 14, 17, 20, 25</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {2}% Điểm Hành Động của bản thân. Sau khi tấn công đơn mục tiêu, nếu mục tiêu còn sống, có {3}% xác suất lập tức tung đòn Đánh Thường để truy kích.</t>
         </is>
       </c>
     </row>
@@ -22634,7 +22661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26.7109375" customWidth="1" style="35" min="1" max="1"/>
@@ -22779,31 +22806,34 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>psv_vanguard_of_volition</t>
+          <t>psv_ninefold_staff</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>OnAfterSkillExcute</t>
+          <t>OnSkillStart</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Eff_FollowUp_BasicAttack</t>
+          <t>Eff_Buff_Enhance</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>30.0, 40.0, 50.0, 60.0, 70.0, 80.0</t>
+          <t>30.0, 35.0, 40.0, 45.0, 50.0, 60.0</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SingleTarget, TargetAlive</t>
-        </is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -22812,34 +22842,34 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ST Bạo Kích tăng {0}%. Sau khi tấn công đơn, nếu mục tiêu vẫn còn sống, có {1}% xác suất thi triển đánh thường để truy kích, mỗi hiệp kích hoạt tối đa 1 lần. Khi Phản Kích, Hỗ Trợ Tấn công se không kích hoạt hiệu ứng này.</t>
+          <t>Tăng {0}% Tốc độ. Tăng thêm {1}% hiệu quả cho các kỹ năng Cường Hóa và Buff.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>psv_ninefold_staff</t>
+          <t>psv_nimbus_cloud</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OnSkillStart</t>
+          <t>OnAfterTakeDamage</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Eff_Buff_Enhance</t>
+          <t>Eff_Action_Point_Boost</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>30.0, 35.0, 40.0, 45.0, 50.0, 60.0</t>
+          <t>10.0, 15.0, 20.0, 25.0, 30.0, 40.0</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>AoEAttack</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -22855,34 +22885,34 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Tăng {0}% Tốc độ. Tăng thêm {1}% hiệu quả cho các kỹ năng Cường Hóa và Buff.</t>
+          <t>Khi bị tấn công phạm vi, điểm hành động của bản thân tăng {0)%.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>psv_nimbus_cloud</t>
+          <t>psv_reincarnation</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>OnAfterTakeDamage</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Eff_Action_Point_Boost</t>
+          <t>Eff_IncreaseAttack</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.0, 15.0, 20.0, 25.0, 30.0, 40.0</t>
+          <t>10.0, 13.0, 16.0, 19.0, 22.0, 25.0</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AoEAttack</t>
+          <t>SingleTarget</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -22898,38 +22928,38 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Khi bị tấn công phạm vi, điểm hành động của bản thân tăng {0)%.</t>
+          <t>Tấn công tăng {0}%. Đòn tấn công đơn mục tiêu gây thêm {1}% Sát thương.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>psv_reincarnation</t>
+          <t>psv_moonlit_firefly</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OnBeforeDealDamage</t>
+          <t>OnAfterSkillExecute</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eff_IncreaseAttack</t>
+          <t>Eff_Reduce_Cooldown</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10.0, 13.0, 16.0, 19.0, 22.0, 25.0</t>
+          <t>30.0, 40.0, 50.0, 60.0, 70.0, 80.0</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SingleTarget</t>
+          <t>NonAttackSkill</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -22941,14 +22971,14 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Tấn công tăng {0}%. Đòn tấn công đơn mục tiêu gây thêm {1}% Sát thương.</t>
+          <t>Tấn công và phòng thủ tăng {0}%. Sau khi thi triển kỹ năng không phải tấn công, có {1}% xác suất hiệp hồi chiêu -1.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>psv_moonlit_firefly</t>
+          <t>psv_plantain_fan</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -22958,17 +22988,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Eff_Reduce_Cooldown</t>
+          <t>Eff_Apply_Mark_Debuff</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>30.0, 40.0, 50.0, 60.0, 70.0, 80.0</t>
+          <t>40.0, 50.0, 60.0, 70.0, 80.0, 90.0</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>NonAttackSkill</t>
+          <t>SingleTarget</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -22979,19 +23009,19 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>enemy</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Tấn công và phòng thủ tăng {0}%. Sau khi thi triển kỹ năng không phải tấn công, có {1}% xác suất hiệp hồi chiêu -1.</t>
+          <t>Tăng {0}% Hiệu quả Chính Xác.Các đòn tấn công đơn mục tiêu có {1}% cơ hội gây hiệu ứng Đánh Dấu lên mục tiêu trong 1 lượt.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>psv_plantain_fan</t>
+          <t>psv_wings_of_phoenix</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -23001,7 +23031,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Eff_Apply_Mark_Debuff</t>
+          <t>Eff_Dispel_Self_Debuff</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -23011,57 +23041,57 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SingleTarget</t>
+          <t>HasDebuff</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>self</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Tăng {0}% Hiệu quả Chính Xác.Các đòn tấn công đơn mục tiêu có {1}% cơ hội gây hiệu ứng Đánh Dấu lên mục tiêu trong 1 lượt.</t>
+          <t>Kháng hiệu ứng tăng {0}%. Sau khi bị kĩ năng tấn công, nếu bản thân tồn tại hiệu ứng suy yếu, có {1}% xác xuất xóa 2 hiệu ứng suy yếu cảu bản thân, cứ 2 hiệp kích hoạt tối đa 1 lần.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>psv_wings_of_phoenix</t>
+          <t>psv_sunwukong_major</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>OnAfterSkillExcute</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Eff_Dispel_Self_Debuff</t>
+          <t>Eff_Lifesteal</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>40.0, 50.0, 60.0, 70.0, 80.0, 90.0</t>
+          <t>20, 25, 30, 30, 30, 30</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>HasDebuff</t>
+          <t>MajorSkill</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -23070,29 +23100,29 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Kháng hiệu ứng tăng {0}%. Sau khi bị kĩ năng tấn công, nếu bản thân tồn tại hiệu ứng suy yếu, có {1}% xác xuất xóa 2 hiệu ứng suy yếu cảu bản thân, cứ 2 hiệp kích hoạt tối đa 1 lần.</t>
+          <t>Kỹ năng Major hút máu 25%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>psv_sunwukong_major</t>
+          <t>psv_erlangshen_major</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>OnAfterDealDamage</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Eff_Lifesteal</t>
+          <t>Eff_IncreaseCritDmg</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>20, 25, 30, 30, 30, 30</t>
+          <t>60, 80, 100, 100, 100, 100</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -23113,38 +23143,38 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Kỹ năng Major hút máu 25%</t>
+          <t>Kỹ năng Major tăng 100% Crit DMG</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>psv_erlangshen_major</t>
+          <t>psv_lijing_base</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>OnBeforeDealDamage</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Eff_IncreaseCritDmg</t>
+          <t>Eff_AddShield</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>60, 80, 100, 100, 100, 100</t>
+          <t>5, 5, 5, 5, 5, 5</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MajorSkill</t>
+          <t>BasicAttack</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -23156,38 +23186,38 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Kỹ năng Major tăng 100% Crit DMG</t>
+          <t>Đánh thường nhận khiên 5% Max HP (max 5 tầng)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>psv_lijing_base</t>
+          <t>psv_lijing_ultimate</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>OnAfterDealDamage</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Eff_AddShield</t>
+          <t>Eff_HPScalingDamage</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5, 5, 5, 5, 5, 5</t>
+          <t>30, 30, 30, 30, 30, 30</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BasicAttack</t>
+          <t>UltimateSkill</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -23199,14 +23229,14 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Đánh thường nhận khiên 5% Max HP (max 5 tầng)</t>
+          <t>Tuyệt kỹ nộ tăng 30% Max HP vào Base Damage</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>psv_lijing_ultimate</t>
+          <t>psv_erlangshen_ultimate</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -23216,7 +23246,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eff_HPScalingDamage</t>
+          <t>Eff_ArmorPenetration</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -23242,29 +23272,29 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Tuyệt kỹ nộ tăng 30% Max HP vào Base Damage</t>
+          <t>Tuyệt kỹ tăng 30% Xuyên Giáp</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>psv_erlangshen_ultimate</t>
+          <t>psv_sunwukong_ultiamte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>OnBeforeDealDamage</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Eff_ArmorPenetration</t>
+          <t>Eff_ReduceDefense</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>30, 30, 30, 30, 30, 30</t>
+          <t>15, 20, 25, 25, 25, 25</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -23280,43 +23310,43 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>enemy</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Tuyệt kỹ tăng 30% Xuyên Giáp</t>
+          <t>Tuyệt kỹ giảm 25% DEF mục tiêu</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>psv_sunwukong_ultiamte</t>
+          <t>psv_bulldemonking_counter</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>OnAfterDealDamage</t>
+          <t>OnTakeDamage</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Eff_ReduceDefense</t>
+          <t>Eff_CounterAttack</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>15, 20, 25, 25, 25, 25</t>
+          <t>50, 75, 100, 100, 100, 100</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>UltimateSkill</t>
+          <t>BasicAttack</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -23328,50 +23358,50 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Tuyệt kỹ giảm 25% DEF mục tiêu</t>
+          <t>Có 50%, 75%, 100% cơ hội phản kích khi bị đánh thường, gây 100% ATK</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>psv_bulldemonking_counter</t>
+          <t>psv_ferrous_chaos</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>OnTakeDamage</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Eff_CounterAttack</t>
+          <t>Eff_IncreaseAttack</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>50, 75, 100, 100, 100, 100</t>
+          <t>16, 16, 16, 16, 16, 16</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BasicAttack</t>
+          <t>IsSkill, HP_Above_50</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>self</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Có 50%, 75%, 100% cơ hội phản kích khi bị đánh thường, gây 100% ATK</t>
+          <t>Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng</t>
         </is>
       </c>
     </row>
@@ -23383,12 +23413,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>OnBeforeDealDamage</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Eff_IncreaseAttack</t>
+          <t>Eff_Lifesteal</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -23398,7 +23428,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>IsSkill, HP_Above_50</t>
+          <t>HP_BelowOrEqual_50</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -23414,14 +23444,14 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng</t>
+          <t>Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>psv_ferrous_chaos</t>
+          <t>psv_nezha_ultimate</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -23431,17 +23461,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Eff_Lifesteal</t>
+          <t>Eff_FollowUp_BasicAttack</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>16, 16, 16, 16, 16, 16</t>
+          <t>100, 120, 150, 200, 200, 200</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HP_BelowOrEqual_50</t>
+          <t>UltimateSkill, TargetDead</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -23457,14 +23487,14 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu</t>
+          <t>Khi kết liễu kẻ địch bằng chiêu cuối, kích hoạt hiệu ứng [Càn Quét] tấn công 1 kẻ địch khác với 120% ATK.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>psv_nezha_ultimate</t>
+          <t>psv_windfire_wheel</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -23474,17 +23504,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Eff_FollowUp_BasicAttack</t>
+          <t>Eff_Action_Point_Boost</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>100, 120, 150, 200, 200, 200</t>
+          <t>10, 12, 14, 16, 18, 20</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>UltimateSkill, TargetDead</t>
+          <t>IsCritical</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -23500,38 +23530,38 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Khi kết liễu kẻ địch bằng chiêu cuối, kích hoạt hiệu ứng [Càn Quét] tấn công 1 kẻ địch khác với 120% ATK.</t>
+          <t>Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>psv_windfire_wheel</t>
+          <t>psv_nine_toothed_rake</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>OnAfterDealDamage</t>
+          <t>OnTakeDamage</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Eff_Action_Point_Boost</t>
+          <t>Eff_Stackable_DEF_Buff</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10, 12, 14, 16, 18, 20</t>
+          <t>4.0, 5.0, 6.0, 7.0, 8.0, 10.0</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>IsCritical</t>
+          <t>None</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -23543,38 +23573,38 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
+          <t>Mỗi khi chịu sát thương, Phòng Thủ tăng thêm {1}%, tối đa cộng dồn 5 tầng. Khi đạt 5 tầng, hồi phục 10% HP Tối Đa.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>psv_nine_toothed_rake</t>
+          <t>psv_vanguard_of_volition</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>OnTakeDamage</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Eff_Stackable_DEF_Buff</t>
+          <t>Eff_Action_Point_Boost</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>4.0, 5.0, 6.0, 7.0, 8.0, 10.0</t>
+          <t>15.0, 18.0, 21.0, 24.0, 27.0, 30.0</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>IsCritical</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -23586,7 +23616,50 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Mỗi khi chịu sát thương, Phòng Thủ tăng thêm {1}%, tối đa cộng dồn 5 tầng. Khi đạt 5 tầng, hồi phục 10% HP Tối Đa.</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {2}% Điểm Hành Động của bản thân. Sau khi tấn công đơn mục tiêu, nếu mục tiêu còn sống, có {3}% xác suất lập tức tung đòn Đánh Thường để truy kích.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>psv_vanguard_of_volition</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>OnAfterSkillExecute</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Eff_FollowUp_BasicAttack</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>50.0, 60.0, 70.0, 80.0, 90.0, 100.0</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SingleTarget, TargetAlive</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {2}% Điểm Hành Động của bản thân. Sau khi tấn công đơn mục tiêu, nếu mục tiêu còn sống, có {3}% xác suất lập tức tung đòn Đánh Thường để truy kích.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
+ Balance all weapon done.
</commit_message>
<xml_diff>
--- a/Tool/data/GameConfig.xlsx
+++ b/Tool/data/GameConfig.xlsx
@@ -1078,9 +1078,9 @@
           <t>Weapon</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Legendary</t>
         </is>
       </c>
     </row>
@@ -1110,9 +1110,9 @@
           <t>Weapon</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Legendary</t>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
     </row>
@@ -21344,9 +21344,9 @@
           <t>Plantain_Fan</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Epic</t>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Legendary</t>
         </is>
       </c>
       <c r="C14" s="37" t="inlineStr">
@@ -21378,9 +21378,9 @@
           <t>Wings_of_Phoenix</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Legendary</t>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Epic</t>
         </is>
       </c>
       <c r="C15" s="37" t="inlineStr">
@@ -21603,7 +21603,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ST Bạo kích tăng {0}%. Sau khi thi triển kỹ năng tấn công đơn đánh bại mục tiêu, có {1}% xác suất hiệp hồi chiêu kỹ năng của bản thân -1.</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Sau khi thi triển kỹ năng tấn công đơn đánh bại mục tiêu, có {2}% xác suất hiệp hồi chiêu kỹ năng của bản thân -1.</t>
         </is>
       </c>
     </row>
@@ -21637,7 +21637,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tăng {0}% Tốc độ. Tăng thêm {1}% hiệu quả cho các kỹ năng Cường Hóa và Buff.</t>
+          <t>Tăng {0}% Tốc Độ. Tăng thêm {1}% hiệu quả cho các kỹ năng Cường Hóa và Hỗ Trợ.</t>
         </is>
       </c>
     </row>
@@ -21671,7 +21671,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Khi bị tấn công phạm vi, điểm hành động của bản thân tăng {0)%.</t>
+          <t>Tăng {0}% Tốc Độ và {1}% Tấn Công. Khi bắt đầu lượt, tăng {2}% Điểm Hành Động của bản thân.</t>
         </is>
       </c>
     </row>
@@ -21773,7 +21773,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tấn công và phòng thủ tăng {0}%. Sau khi thi triển kỹ năng không phải tấn công, có {1}% xác suất hiệp hồi chiêu -1.</t>
+          <t>Tăng {0}% Tốc Độ và {1}% Tấn Công. Tăng thêm {2}% hiệu quả cho các kỹ năng Cường Hóa và Hỗ Trợ.</t>
         </is>
       </c>
     </row>
@@ -21790,7 +21790,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tăng {0}% Hiệu quả Chính Xác.Các đòn tấn công đơn mục tiêu có {1}% cơ hội gây hiệu ứng Đánh Dấu lên mục tiêu trong 1 lượt.</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Đòn tấn công kỹ năng có 60% xác suất giảm {2}% Phòng Thủ của mục tiêu trong 2 hiệp và gây thêm {3}% Sát Thương lên kẻ địch đang chịu hiệu ứng bất lợi.</t>
         </is>
       </c>
     </row>
@@ -21807,7 +21807,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Kháng hiệu ứng tăng {0}%. Sau khi bị kĩ năng tấn công, nếu bản thân tồn tại hiệu ứng suy yếu, có {1}% xác xuất xóa 2 hiệu ứng suy yếu cảu bản thân, cứ 2 hiệp kích hoạt tối đa 1 lần.</t>
+          <t>Tăng {0}% HP và {1}% Phòng Thủ. Tăng thêm {2}% hiệu quả cho các kỹ năng Hồi Máu.</t>
         </is>
       </c>
     </row>
@@ -22014,7 +22014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.7109375" bestFit="1" customWidth="1" style="35" min="1" max="1"/>
@@ -22108,12 +22108,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>psv_triple_edged_blade</t>
+          <t>psv_ninefold_staff</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CRIT_DMG</t>
+          <t>SPEED</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -22123,24 +22123,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>30, 36, 42, 48, 54, 60</t>
+          <t>6, 8, 10, 12, 15, 20</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ST Bạo kích tăng {0}%. Sau khi thi triển kỹ năng tấn công đơn đánh bại mục tiêu, có {1}% xác suất hiệp hồi chiêu kỹ năng của bản thân -1.</t>
+          <t>Tăng {0}% Tốc Độ. Tăng thêm {1}% hiệu quả cho các kỹ năng Cường Hóa và Hỗ Trợ.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>psv_ninefold_staff</t>
+          <t>psv_reincarnation</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SPEED</t>
+          <t>ATK</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -22150,24 +22150,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6, 8, 10, 12, 15, 20</t>
+          <t>8, 11, 14, 17, 20, 25</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Tăng {0}% Tốc độ. Tăng thêm {1}% hiệu quả cho các kỹ năng Cường Hóa và Buff.</t>
+          <t>Tấn công tăng {0}%. Đòn tấn công đơn mục tiêu gây thêm {1}% Sát thương.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>psv_reincarnation</t>
+          <t>psv_ennead_spear</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ATK</t>
+          <t>CRIT_RATE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -22177,24 +22177,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8, 11, 14, 17, 20, 25</t>
+          <t>5, 7.5, 10, 12.5, 16, 20</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Tấn công tăng {0}%. Đòn tấn công đơn mục tiêu gây thêm {1}% Sát thương.</t>
+          <t>Tỷ lệ bạo kích tăng {0}%.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>psv_ennead_spear</t>
+          <t>psv_crescent_axe</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CRIT_RATE</t>
+          <t>CRIT_DMG</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -22204,24 +22204,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5, 7.5, 10, 12.5, 16, 20</t>
+          <t>5, 7.5, 10, 12.5, 17,, 21</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Tỷ lệ bạo kích tăng {0}%.</t>
+          <t xml:space="preserve">ST Bạo Kích tăng {0}%. </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>psv_crescent_axe</t>
+          <t>psv_bronze_hammer</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CRIT_DMG</t>
+          <t>DEF</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -22231,24 +22231,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5, 7.5, 10, 12.5, 17,, 21</t>
+          <t>5, 7.5, 10, 12.5, 16, 20</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ST Bạo Kích tăng {0}%. </t>
+          <t>Phòng thủ tăng {0}%.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>psv_bronze_hammer</t>
+          <t>psv_linglong_pagoda</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -22258,24 +22258,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>5, 7.5, 10, 12.5, 16, 20</t>
+          <t>15, 20, 25, 30, 35, 40</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Phòng thủ tăng {0}%.</t>
+          <t>HP tối đa tăng {0}%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>psv_moonlit_firefly</t>
+          <t>psv_ferrous_chaos</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>ATK</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -22285,24 +22285,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>5, 7.5, 10, 12.5, 17,, 23</t>
+          <t>10, 15, 20, 25, 30, 35</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Tấn công và phòng thủ tăng {0}%. Sau khi thi triển kỹ năng không phải tấn công, có {1}% xác suất hiệp hồi chiêu -1.</t>
+          <t>Tăng {0}% Tấn Công và {0}% Phòng Thủ. Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng. Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu tương đương 16% tổng sát thương gây ra.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>psv_moonlit_firefly</t>
+          <t>psv_ferrous_chaos</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ATK</t>
+          <t>DEF</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -22312,24 +22312,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5, 7.5, 10, 12.5, 17,, 24</t>
+          <t>10, 15, 20, 25, 30, 35</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Tấn công và phòng thủ tăng {0}%. Sau khi thi triển kỹ năng không phải tấn công, có {1}% xác suất hiệp hồi chiêu -1.</t>
+          <t>Tăng {0}% Tấn Công và {0}% Phòng Thủ. Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng. Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu tương đương 16% tổng sát thương gây ra.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>psv_plantain_fan</t>
+          <t>psv_windfire_wheel</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EHR</t>
+          <t>CRIT_DMG</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -22339,24 +22339,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10, 15, 20, 25, 34, 40</t>
+          <t>8, 10, 12, 14, 17, 20</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Tăng {0}% Hiệu quả Chính Xác.Các đòn tấn công đơn mục tiêu có {1}% cơ hội gây hiệu ứng Đánh Dấu lên mục tiêu trong 1 lượt.</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {0}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>psv_wings_of_phoenix</t>
+          <t>psv_windfire_wheel</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RES</t>
+          <t>ATK</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -22366,19 +22366,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10, 15, 20, 25, 34, 41</t>
+          <t>8, 10, 12, 14, 17, 20</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Kháng hiệu ứng tăng {0}%. Sau khi bị kĩ năng tấn công, nếu bản thân tồn tại hiệu ứng suy yếu, có {1}% xác xuất xóa 2 hiệu ứng suy yếu cảu bản thân, cứ 2 hiệp kích hoạt tối đa 1 lần.</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {0}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>psv_linglong_pagoda</t>
+          <t>psv_nine_toothed_rake</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -22393,24 +22393,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>15, 20, 25, 30, 35, 40</t>
+          <t>10, 14, 18, 22, 26, 32</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>HP tối đa tăng {0}%</t>
+          <t>Tăng {0}% HP và {0}% Phòng Thủ. Mỗi khi chịu sát thương, Phòng Thủ tăng thêm {1}%, tối đa cộng dồn 5 tầng. Khi đạt 5 tầng, hồi phục 10% HP Tối Đa.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>psv_ferrous_chaos</t>
+          <t>psv_nine_toothed_rake</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ATK</t>
+          <t>DEF</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -22420,24 +22420,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10, 15, 20, 25, 30, 35</t>
+          <t>10, 14, 18, 22, 26, 32</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Tăng {0}% Tấn Công và {0}% Phòng Thủ. Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng. Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu tương đương 16% tổng sát thương gây ra.</t>
+          <t>Tăng {0}% HP và {0}% Phòng Thủ. Mỗi khi chịu sát thương, Phòng Thủ tăng thêm {1}%, tối đa cộng dồn 5 tầng. Khi đạt 5 tầng, hồi phục 10% HP Tối Đa.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>psv_ferrous_chaos</t>
+          <t>psv_sunburst_spade</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>ATK</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -22447,19 +22447,19 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>10, 15, 20, 25, 30, 35</t>
+          <t>5, 7.5, 10, 12.5, 15, 20</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Tăng {0}% Tấn Công và {0}% Phòng Thủ. Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng. Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu tương đương 16% tổng sát thương gây ra.</t>
+          <t>Tấn công tăng {0}%.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>psv_windfire_wheel</t>
+          <t>psv_vanguard_of_volition</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -22474,19 +22474,19 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>8, 10, 12, 14, 17, 20</t>
+          <t>20, 25, 30, 35, 40, 50</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Tăng {0}% Sát Thương Bạo Kích và {0}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {2}% Điểm Hành Động của bản thân. Sau khi tấn công đơn mục tiêu, nếu mục tiêu còn sống, có {3}% xác suất lập tức tung đòn Đánh Thường để truy kích.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>psv_windfire_wheel</t>
+          <t>psv_vanguard_of_volition</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -22501,24 +22501,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>8, 10, 12, 14, 17, 20</t>
+          <t>10, 12, 14, 17, 20, 25</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Tăng {0}% Sát Thương Bạo Kích và {0}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {2}% Điểm Hành Động của bản thân. Sau khi tấn công đơn mục tiêu, nếu mục tiêu còn sống, có {3}% xác suất lập tức tung đòn Đánh Thường để truy kích.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>psv_nine_toothed_rake</t>
+          <t>psv_nimbus_cloud</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>SPEED</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -22528,24 +22528,19 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10, 14, 18, 22, 26, 32</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Tăng {0}% HP và {0}% Phòng Thủ. Mỗi khi chịu sát thương, Phòng Thủ tăng thêm {1}%, tối đa cộng dồn 5 tầng. Khi đạt 5 tầng, hồi phục 10% HP Tối Đa.</t>
+          <t>4.0, 5.0, 6.0, 7.0, 8.5, 10.0</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>psv_nine_toothed_rake</t>
+          <t>psv_nimbus_cloud</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>ATK</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -22555,24 +22550,19 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10, 14, 18, 22, 26, 32</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Tăng {0}% HP và {0}% Phòng Thủ. Mỗi khi chịu sát thương, Phòng Thủ tăng thêm {1}%, tối đa cộng dồn 5 tầng. Khi đạt 5 tầng, hồi phục 10% HP Tối Đa.</t>
+          <t>5.0, 6.5, 8.0, 10.0, 12.0, 15.0</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>psv_sunburst_spade</t>
+          <t>psv_plantain_fan</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ATK</t>
+          <t>CRIT_DMG</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -22582,24 +22572,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>5, 7.5, 10, 12.5, 15, 20</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Tấn công tăng {0}%.</t>
+          <t>20.0, 25.0, 30.0, 35.0, 40.0, 50.0</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>psv_vanguard_of_volition</t>
+          <t>psv_plantain_fan</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CRIT_DMG</t>
+          <t>ATK</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -22609,39 +22594,169 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>20, 25, 30, 35, 40, 50</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {2}% Điểm Hành Động của bản thân. Sau khi tấn công đơn mục tiêu, nếu mục tiêu còn sống, có {3}% xác suất lập tức tung đòn Đánh Thường để truy kích.</t>
+          <t>10.0, 12.0, 14.0, 17.0, 20.0, 25.0</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>psv_vanguard_of_volition</t>
+          <t>psv_triple_edged_blade</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>CRIT_DMG</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>30.0, 36.0, 42.0, 48.0, 54.0, 60.0</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Sau khi thi triển kỹ năng tấn công đơn đánh bại mục tiêu, có {2}% xác suất hiệp hồi chiêu kỹ năng của bản thân -1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>psv_triple_edged_blade</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>ATK</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Percent</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>10, 12, 14, 17, 20, 25</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {2}% Điểm Hành Động của bản thân. Sau khi tấn công đơn mục tiêu, nếu mục tiêu còn sống, có {3}% xác suất lập tức tung đòn Đánh Thường để truy kích.</t>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>10.0, 12.0, 14.0, 17.0, 20.0, 25.0</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Sau khi thi triển kỹ năng tấn công đơn đánh bại mục tiêu, có {2}% xác suất hiệp hồi chiêu kỹ năng của bản thân -1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>psv_moonlit_firefly</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SPEED</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>8.0, 10.0, 12.0, 15.0, 18.0, 25.0</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Tăng {0}% Tốc Độ và {1}% Tấn Công. Tăng thêm {2}% hiệu quả cho các kỹ năng Cường Hóa và Hỗ Trợ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>psv_moonlit_firefly</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ATK</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>10.0, 12.0, 14.0, 17.0, 20.0, 25.0</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Tăng {0}% Tốc Độ và {1}% Tấn Công. Tăng thêm {2}% hiệu quả cho các kỹ năng Cường Hóa và Hỗ Trợ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>psv_wings_of_phoenix</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>15.0, 18.0, 21.0, 25.0, 30.0, 40.0</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Tăng {0}% HP và {1}% Phòng Thủ. Tăng thêm {2}% hiệu quả cho các kỹ năng Hồi Máu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>psv_wings_of_phoenix</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>10.0, 12.0, 14.0, 17.0, 20.0, 25.0</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Tăng {0}% HP và {1}% Phòng Thủ. Tăng thêm {2}% hiệu quả cho các kỹ năng Hồi Máu.</t>
         </is>
       </c>
     </row>
@@ -22661,7 +22776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26.7109375" customWidth="1" style="35" min="1" max="1"/>
@@ -22799,7 +22914,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ST Bạo kích tăng {0}%. Sau khi thi triển kỹ năng tấn công đơn đánh bại mục tiêu, có {1}% xác suất hiệp hồi chiêu kỹ năng của bản thân -1.</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Sau khi thi triển kỹ năng tấn công đơn đánh bại mục tiêu, có {2}% xác suất hiệp hồi chiêu kỹ năng của bản thân -1.</t>
         </is>
       </c>
     </row>
@@ -22842,34 +22957,34 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Tăng {0}% Tốc độ. Tăng thêm {1}% hiệu quả cho các kỹ năng Cường Hóa và Buff.</t>
+          <t>Tăng {0}% Tốc Độ. Tăng thêm {1}% hiệu quả cho các kỹ năng Cường Hóa và Hỗ Trợ.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>psv_nimbus_cloud</t>
+          <t>psv_reincarnation</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OnAfterTakeDamage</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Eff_Action_Point_Boost</t>
+          <t>Eff_IncreaseAttack</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10.0, 15.0, 20.0, 25.0, 30.0, 40.0</t>
+          <t>10.0, 13.0, 16.0, 19.0, 22.0, 25.0</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AoEAttack</t>
+          <t>SingleTarget</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -22885,34 +23000,34 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Khi bị tấn công phạm vi, điểm hành động của bản thân tăng {0)%.</t>
+          <t>Tấn công tăng {0}%. Đòn tấn công đơn mục tiêu gây thêm {1}% Sát thương.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>psv_reincarnation</t>
+          <t>psv_sunwukong_major</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>OnBeforeDealDamage</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Eff_IncreaseAttack</t>
+          <t>Eff_Lifesteal</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.0, 13.0, 16.0, 19.0, 22.0, 25.0</t>
+          <t>20, 25, 30, 30, 30, 30</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SingleTarget</t>
+          <t>MajorSkill</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -22928,38 +23043,38 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Tấn công tăng {0}%. Đòn tấn công đơn mục tiêu gây thêm {1}% Sát thương.</t>
+          <t>Kỹ năng Major hút máu 25%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>psv_moonlit_firefly</t>
+          <t>psv_erlangshen_major</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OnAfterSkillExecute</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eff_Reduce_Cooldown</t>
+          <t>Eff_IncreaseCritDmg</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>30.0, 40.0, 50.0, 60.0, 70.0, 80.0</t>
+          <t>60, 80, 100, 100, 100, 100</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>NonAttackSkill</t>
+          <t>MajorSkill</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -22971,84 +23086,84 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Tấn công và phòng thủ tăng {0}%. Sau khi thi triển kỹ năng không phải tấn công, có {1}% xác suất hiệp hồi chiêu -1.</t>
+          <t>Kỹ năng Major tăng 100% Crit DMG</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>psv_plantain_fan</t>
+          <t>psv_lijing_base</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>OnAfterSkillExecute</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Eff_Apply_Mark_Debuff</t>
+          <t>Eff_AddShield</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>40.0, 50.0, 60.0, 70.0, 80.0, 90.0</t>
+          <t>5, 5, 5, 5, 5, 5</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SingleTarget</t>
+          <t>BasicAttack</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>self</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Tăng {0}% Hiệu quả Chính Xác.Các đòn tấn công đơn mục tiêu có {1}% cơ hội gây hiệu ứng Đánh Dấu lên mục tiêu trong 1 lượt.</t>
+          <t>Đánh thường nhận khiên 5% Max HP (max 5 tầng)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>psv_wings_of_phoenix</t>
+          <t>psv_lijing_ultimate</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>OnAfterSkillExecute</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Eff_Dispel_Self_Debuff</t>
+          <t>Eff_HPScalingDamage</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>40.0, 50.0, 60.0, 70.0, 80.0, 90.0</t>
+          <t>30, 30, 30, 30, 30, 30</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>HasDebuff</t>
+          <t>UltimateSkill</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -23057,34 +23172,34 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Kháng hiệu ứng tăng {0}%. Sau khi bị kĩ năng tấn công, nếu bản thân tồn tại hiệu ứng suy yếu, có {1}% xác xuất xóa 2 hiệu ứng suy yếu cảu bản thân, cứ 2 hiệp kích hoạt tối đa 1 lần.</t>
+          <t>Tuyệt kỹ nộ tăng 30% Max HP vào Base Damage</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>psv_sunwukong_major</t>
+          <t>psv_erlangshen_ultimate</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>OnAfterDealDamage</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Eff_Lifesteal</t>
+          <t>Eff_ArmorPenetration</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>20, 25, 30, 30, 30, 30</t>
+          <t>30, 30, 30, 30, 30, 30</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MajorSkill</t>
+          <t>UltimateSkill</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -23100,34 +23215,34 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Kỹ năng Major hút máu 25%</t>
+          <t>Tuyệt kỹ tăng 30% Xuyên Giáp</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>psv_erlangshen_major</t>
+          <t>psv_sunwukong_ultiamte</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>OnBeforeDealDamage</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Eff_IncreaseCritDmg</t>
+          <t>Eff_ReduceDefense</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>60, 80, 100, 100, 100, 100</t>
+          <t>15, 20, 25, 25, 25, 25</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>MajorSkill</t>
+          <t>UltimateSkill</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -23138,34 +23253,34 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>enemy</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Kỹ năng Major tăng 100% Crit DMG</t>
+          <t>Tuyệt kỹ giảm 25% DEF mục tiêu</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>psv_lijing_base</t>
+          <t>psv_bulldemonking_counter</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>OnAfterDealDamage</t>
+          <t>OnTakeDamage</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Eff_AddShield</t>
+          <t>Eff_CounterAttack</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5, 5, 5, 5, 5, 5</t>
+          <t>50, 75, 100, 100, 100, 100</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -23174,26 +23289,26 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>enemy</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Đánh thường nhận khiên 5% Max HP (max 5 tầng)</t>
+          <t>Có 50%, 75%, 100% cơ hội phản kích khi bị đánh thường, gây 100% ATK</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>psv_lijing_ultimate</t>
+          <t>psv_ferrous_chaos</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -23203,17 +23318,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Eff_HPScalingDamage</t>
+          <t>Eff_IncreaseAttack</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>30, 30, 30, 30, 30, 30</t>
+          <t>16, 16, 16, 16, 16, 16</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>UltimateSkill</t>
+          <t>IsSkill, HP_Above_50</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -23229,34 +23344,34 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Tuyệt kỹ nộ tăng 30% Max HP vào Base Damage</t>
+          <t>Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>psv_erlangshen_ultimate</t>
+          <t>psv_ferrous_chaos</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OnBeforeDealDamage</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eff_ArmorPenetration</t>
+          <t>Eff_Lifesteal</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>30, 30, 30, 30, 30, 30</t>
+          <t>16, 16, 16, 16, 16, 16</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>UltimateSkill</t>
+          <t>HP_BelowOrEqual_50</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -23272,14 +23387,14 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Tuyệt kỹ tăng 30% Xuyên Giáp</t>
+          <t>Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>psv_sunwukong_ultiamte</t>
+          <t>psv_nezha_ultimate</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -23289,17 +23404,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Eff_ReduceDefense</t>
+          <t>Eff_FollowUp_BasicAttack</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>15, 20, 25, 25, 25, 25</t>
+          <t>100, 120, 150, 200, 200, 200</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>UltimateSkill</t>
+          <t>UltimateSkill, TargetDead</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -23310,86 +23425,86 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>self</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Tuyệt kỹ giảm 25% DEF mục tiêu</t>
+          <t>Khi kết liễu kẻ địch bằng chiêu cuối, kích hoạt hiệu ứng [Càn Quét] tấn công 1 kẻ địch khác với 120% ATK.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>psv_bulldemonking_counter</t>
+          <t>psv_windfire_wheel</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>OnTakeDamage</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Eff_CounterAttack</t>
+          <t>Eff_Action_Point_Boost</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>50, 75, 100, 100, 100, 100</t>
+          <t>10, 12, 14, 16, 18, 20</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BasicAttack</t>
+          <t>IsCritical</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>enemy</t>
+          <t>self</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Có 50%, 75%, 100% cơ hội phản kích khi bị đánh thường, gây 100% ATK</t>
+          <t>Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>psv_ferrous_chaos</t>
+          <t>psv_nine_toothed_rake</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>OnBeforeDealDamage</t>
+          <t>OnTakeDamage</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Eff_IncreaseAttack</t>
+          <t>Eff_Stackable_DEF_Buff</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>16, 16, 16, 16, 16, 16</t>
+          <t>4.0, 5.0, 6.0, 7.0, 8.0, 10.0</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>IsSkill, HP_Above_50</t>
+          <t>None</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -23401,14 +23516,14 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng</t>
+          <t>Mỗi khi chịu sát thương, Phòng Thủ tăng thêm {1}%, tối đa cộng dồn 5 tầng. Khi đạt 5 tầng, hồi phục 10% HP Tối Đa.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>psv_ferrous_chaos</t>
+          <t>psv_vanguard_of_volition</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -23418,17 +23533,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Eff_Lifesteal</t>
+          <t>Eff_Action_Point_Boost</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>16, 16, 16, 16, 16, 16</t>
+          <t>15.0, 18.0, 21.0, 24.0, 27.0, 30.0</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>HP_BelowOrEqual_50</t>
+          <t>IsCritical</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -23444,19 +23559,19 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {2}% Điểm Hành Động của bản thân. Sau khi tấn công đơn mục tiêu, nếu mục tiêu còn sống, có {3}% xác suất lập tức tung đòn Đánh Thường để truy kích.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>psv_nezha_ultimate</t>
+          <t>psv_vanguard_of_volition</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>OnAfterDealDamage</t>
+          <t>OnAfterSkillExecute</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -23466,12 +23581,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>100, 120, 150, 200, 200, 200</t>
+          <t>50.0, 60.0, 70.0, 80.0, 90.0, 100.0</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>UltimateSkill, TargetDead</t>
+          <t>SingleTarget, TargetAlive</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -23487,19 +23602,19 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Khi kết liễu kẻ địch bằng chiêu cuối, kích hoạt hiệu ứng [Càn Quét] tấn công 1 kẻ địch khác với 120% ATK.</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {2}% Điểm Hành Động của bản thân. Sau khi tấn công đơn mục tiêu, nếu mục tiêu còn sống, có {3}% xác suất lập tức tung đòn Đánh Thường để truy kích.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>psv_windfire_wheel</t>
+          <t>psv_nimbus_cloud</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>OnAfterDealDamage</t>
+          <t>OnTurnStart</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -23509,12 +23624,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10, 12, 14, 16, 18, 20</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>IsCritical</t>
+          <t>10.0, 12.0, 14.0, 16.0, 18.0, 20.0</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -23530,67 +23640,67 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Khi gây sát thương Bạo Kích, tăng {1}% Điểm Hành Động của bản thân.</t>
+          <t>Tăng {0}% Tốc Độ và {1}% Tấn Công. Khi bắt đầu lượt, tăng {2}% Điểm Hành Động của bản thân.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>psv_nine_toothed_rake</t>
+          <t>psv_plantain_fan</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>OnTakeDamage</t>
+          <t>OnAfterDealDamage</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Eff_Stackable_DEF_Buff</t>
+          <t>Eff_ReduceDefense</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>4.0, 5.0, 6.0, 7.0, 8.0, 10.0</t>
+          <t>15.0, 18.0, 21.0, 24.0, 27.0, 30.0</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>IsSkill</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>enemy</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Mỗi khi chịu sát thương, Phòng Thủ tăng thêm {1}%, tối đa cộng dồn 5 tầng. Khi đạt 5 tầng, hồi phục 10% HP Tối Đa.</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Đòn tấn công kỹ năng có 60% xác suất giảm {2}% Phòng Thủ của mục tiêu trong 2 hiệp và gây thêm {3}% Sát Thương lên kẻ địch đang chịu hiệu ứng bất lợi.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>psv_vanguard_of_volition</t>
+          <t>psv_plantain_fan</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>OnAfterDealDamage</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Eff_Action_Point_Boost</t>
+          <t>Eff_DamageBonus</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -23600,7 +23710,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>IsCritical</t>
+          <t>TargetHasDebuff</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -23616,34 +23726,34 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {2}% Điểm Hành Động của bản thân. Sau khi tấn công đơn mục tiêu, nếu mục tiêu còn sống, có {3}% xác suất lập tức tung đòn Đánh Thường để truy kích.</t>
+          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Đòn tấn công kỹ năng có 60% xác suất giảm {2}% Phòng Thủ của mục tiêu trong 2 hiệp và gây thêm {3}% Sát Thương lên kẻ địch đang chịu hiệu ứng bất lợi.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>psv_vanguard_of_volition</t>
+          <t>psv_moonlit_firefly</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>OnAfterSkillExecute</t>
+          <t>OnBeforeDealDamage</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Eff_FollowUp_BasicAttack</t>
+          <t>Eff_Buff_Enhance</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>50.0, 60.0, 70.0, 80.0, 90.0, 100.0</t>
+          <t>40.0, 50.0, 60.0, 70.0, 80.0, 100.0</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SingleTarget, TargetAlive</t>
+          <t>None</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -23659,7 +23769,50 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Tăng {0}% Sát Thương Bạo Kích và {1}% Tấn Công. Khi gây sát thương Bạo Kích, tăng {2}% Điểm Hành Động của bản thân. Sau khi tấn công đơn mục tiêu, nếu mục tiêu còn sống, có {3}% xác suất lập tức tung đòn Đánh Thường để truy kích.</t>
+          <t>Tăng {0}% Tốc Độ và {1}% Tấn Công. Tăng thêm {2}% hiệu quả cho các kỹ năng Cường Hóa và Hỗ Trợ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>psv_wings_of_phoenix</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>OnBeforeDealDamage</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Eff_Buff_Enhance</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>30.0, 40.0, 50.0, 60.0, 70.0, 80.0</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Tăng {0}% HP và {1}% Phòng Thủ. Tăng thêm {2}% hiệu quả cho các kỹ năng Hồi Máu.</t>
         </is>
       </c>
     </row>

</xml_diff>